<commit_message>
Jury1 Integration updated tasks with additional fields
- added additional fields to all tasks and changed schema accordingly
- need method or classname to run for syntax check
- New Display for Points and Unit-Tests (still needs work)
- changed execution logic for python

ToDos:
- Java Jury1 not working yet
</commit_message>
<xml_diff>
--- a/files/programming-tasks/programmieraufgaben_JACK_SOSE23_WORKSHOP_WISE2324.xlsx
+++ b/files/programming-tasks/programmieraufgaben_JACK_SOSE23_WORKSHOP_WISE2324.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\hefl\files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\hefl\files\programming-tasks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65A1172F-019F-4F59-AE3C-C1EDF83F3CFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E67EF1F7-96C1-4D75-BEAC-3987EF670435}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-15" yWindow="90" windowWidth="25860" windowHeight="20805" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Aufgaben" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="290">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="449" uniqueCount="336">
   <si>
     <t>id</t>
   </si>
@@ -9046,12 +9046,150 @@
 }
 </t>
   </si>
+  <si>
+    <t>runMethod</t>
+  </si>
+  <si>
+    <t>input</t>
+  </si>
+  <si>
+    <t>kapitalWert</t>
+  </si>
+  <si>
+    <t>biblio</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> [["34587", "Learning", 4, 40.95], ["98762", "Programming", 5, 56.80], ["77226", "Head", 3, 32.00]]</t>
+  </si>
+  <si>
+    <t>querSum</t>
+  </si>
+  <si>
+    <t>AlterTest.java</t>
+  </si>
+  <si>
+    <t>SummenwertTest.java</t>
+  </si>
+  <si>
+    <t>DiscountTest.java</t>
+  </si>
+  <si>
+    <t>StarterTest.java</t>
+  </si>
+  <si>
+    <t>ArrayWorkTest.java</t>
+  </si>
+  <si>
+    <t>SchachTest.java</t>
+  </si>
+  <si>
+    <t>RestTest.java</t>
+  </si>
+  <si>
+    <t>BibVerwaltungTest.java</t>
+  </si>
+  <si>
+    <t>GGTTest.java</t>
+  </si>
+  <si>
+    <t>UniTest.java</t>
+  </si>
+  <si>
+    <t>VektorWorkTest.java</t>
+  </si>
+  <si>
+    <t>AppAutoTest.java</t>
+  </si>
+  <si>
+    <t>AppPunktTest.java</t>
+  </si>
+  <si>
+    <t>AppBankTest.java</t>
+  </si>
+  <si>
+    <t>AppRadioTest.java</t>
+  </si>
+  <si>
+    <t>LeserTest.java</t>
+  </si>
+  <si>
+    <t>AirlineTest.java</t>
+  </si>
+  <si>
+    <t>FormenTest.java</t>
+  </si>
+  <si>
+    <t>MyThreadTest.java</t>
+  </si>
+  <si>
+    <t>WettrennenTest.java</t>
+  </si>
+  <si>
+    <t>SortierenTest.java</t>
+  </si>
+  <si>
+    <t>AutoTest.java</t>
+  </si>
+  <si>
+    <t>test_main.py</t>
+  </si>
+  <si>
+    <t>testClassName</t>
+  </si>
+  <si>
+    <t>2000, 5, 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> fib_index</t>
+  </si>
+  <si>
+    <t>charFrequenz</t>
+  </si>
+  <si>
+    <t>"Wie du mir so ich dir"</t>
+  </si>
+  <si>
+    <t>summe</t>
+  </si>
+  <si>
+    <t>ggT</t>
+  </si>
+  <si>
+    <t>56, 98</t>
+  </si>
+  <si>
+    <t>sieb</t>
+  </si>
+  <si>
+    <t>make_matrix</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> potenz</t>
+  </si>
+  <si>
+    <t>2, 0</t>
+  </si>
+  <si>
+    <t>drehe_string</t>
+  </si>
+  <si>
+    <t>"hello"</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> reduziere_liste</t>
+  </si>
+  <si>
+    <t>lambda x1, x2: x1 + x2, list(range(10))</t>
+  </si>
+  <si>
+    <t>fib</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -9114,16 +9252,28 @@
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C5700"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -9138,11 +9288,27 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -9172,8 +9338,38 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Neutral" xfId="1" builtinId="28"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -9477,7 +9673,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:L39"/>
+  <dimension ref="A1:Q39"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
@@ -9489,12 +9685,13 @@
     <col min="8" max="8" width="105.5703125" style="2" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="23.7109375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="49.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="74.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="13" max="16" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="50.7109375" style="1" customWidth="1"/>
+    <col min="12" max="12" width="49.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="74.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="17" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>115</v>
       </c>
@@ -9525,8 +9722,17 @@
       <c r="J1" s="1" t="s">
         <v>124</v>
       </c>
+      <c r="K1" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>290</v>
+      </c>
+      <c r="M1" t="s">
+        <v>291</v>
+      </c>
     </row>
-    <row r="2" spans="1:10" ht="409.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -9545,7 +9751,7 @@
       <c r="F2" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="G2" s="9" t="s">
+      <c r="G2" s="11" t="s">
         <v>252</v>
       </c>
       <c r="H2" s="5" t="s">
@@ -9557,8 +9763,17 @@
       <c r="J2" s="3">
         <v>0</v>
       </c>
+      <c r="K2" s="12" t="s">
+        <v>318</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="M2" t="s">
+        <v>320</v>
+      </c>
     </row>
-    <row r="3" spans="1:10" ht="409.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -9577,7 +9792,7 @@
       <c r="F3" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="G3" s="9" t="s">
+      <c r="G3" s="11" t="s">
         <v>253</v>
       </c>
       <c r="H3" s="5" t="s">
@@ -9589,8 +9804,17 @@
       <c r="J3" s="3">
         <v>0</v>
       </c>
+      <c r="K3" s="12" t="s">
+        <v>318</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="M3" t="s">
+        <v>294</v>
+      </c>
     </row>
-    <row r="4" spans="1:10" ht="409.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -9609,7 +9833,7 @@
       <c r="F4" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="G4" s="11" t="s">
         <v>254</v>
       </c>
       <c r="H4" s="5" t="s">
@@ -9621,8 +9845,17 @@
       <c r="J4" s="3">
         <v>0</v>
       </c>
+      <c r="K4" s="12" t="s">
+        <v>318</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>295</v>
+      </c>
+      <c r="M4">
+        <v>174</v>
+      </c>
     </row>
-    <row r="5" spans="1:10" ht="409.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -9641,7 +9874,7 @@
       <c r="F5" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="G5" s="9" t="s">
+      <c r="G5" s="13" t="s">
         <v>255</v>
       </c>
       <c r="H5" s="5" t="s">
@@ -9653,8 +9886,17 @@
       <c r="J5" s="3">
         <v>0</v>
       </c>
+      <c r="K5" s="12" t="s">
+        <v>318</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>321</v>
+      </c>
+      <c r="M5">
+        <v>47</v>
+      </c>
     </row>
-    <row r="6" spans="1:10" ht="409.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -9673,7 +9915,7 @@
       <c r="F6" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="G6" s="9" t="s">
+      <c r="G6" s="13" t="s">
         <v>256</v>
       </c>
       <c r="H6" s="5" t="s">
@@ -9685,8 +9927,17 @@
       <c r="J6" s="3">
         <v>0</v>
       </c>
+      <c r="K6" s="12" t="s">
+        <v>318</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="M6" t="s">
+        <v>323</v>
+      </c>
     </row>
-    <row r="7" spans="1:10" ht="409.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -9705,7 +9956,7 @@
       <c r="F7" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="G7" s="9" t="s">
+      <c r="G7" s="13" t="s">
         <v>257</v>
       </c>
       <c r="H7" s="5" t="s">
@@ -9717,8 +9968,17 @@
       <c r="J7" s="3">
         <v>0</v>
       </c>
+      <c r="K7" s="12" t="s">
+        <v>318</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>324</v>
+      </c>
+      <c r="M7">
+        <v>6.7</v>
+      </c>
     </row>
-    <row r="8" spans="1:10" ht="409.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -9737,7 +9997,7 @@
       <c r="F8" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="G8" s="9" t="s">
+      <c r="G8" s="13" t="s">
         <v>258</v>
       </c>
       <c r="H8" s="5" t="s">
@@ -9749,8 +10009,17 @@
       <c r="J8" s="3">
         <v>0</v>
       </c>
+      <c r="K8" s="12" t="s">
+        <v>318</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>325</v>
+      </c>
+      <c r="M8" t="s">
+        <v>326</v>
+      </c>
     </row>
-    <row r="9" spans="1:10" ht="409.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3">
         <v>8</v>
       </c>
@@ -9769,7 +10038,7 @@
       <c r="F9" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="G9" s="9" t="s">
+      <c r="G9" s="13" t="s">
         <v>259</v>
       </c>
       <c r="H9" s="5" t="s">
@@ -9781,8 +10050,17 @@
       <c r="J9" s="3">
         <v>0</v>
       </c>
+      <c r="K9" s="12" t="s">
+        <v>318</v>
+      </c>
+      <c r="L9" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="M9">
+        <v>10</v>
+      </c>
     </row>
-    <row r="10" spans="1:10" ht="409.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3">
         <v>9</v>
       </c>
@@ -9813,8 +10091,11 @@
       <c r="J10" s="3">
         <v>0</v>
       </c>
+      <c r="K10" s="12" t="s">
+        <v>296</v>
+      </c>
     </row>
-    <row r="11" spans="1:10" ht="409.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3">
         <v>10</v>
       </c>
@@ -9845,8 +10126,11 @@
       <c r="J11" s="3">
         <v>0</v>
       </c>
+      <c r="K11" s="12" t="s">
+        <v>297</v>
+      </c>
     </row>
-    <row r="12" spans="1:10" ht="409.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3">
         <v>11</v>
       </c>
@@ -9877,8 +10161,11 @@
       <c r="J12" s="3">
         <v>1</v>
       </c>
+      <c r="K12" s="12" t="s">
+        <v>298</v>
+      </c>
     </row>
-    <row r="13" spans="1:10" ht="409.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3">
         <v>12</v>
       </c>
@@ -9897,7 +10184,7 @@
       <c r="F13" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="G13" s="9" t="s">
+      <c r="G13" s="13" t="s">
         <v>263</v>
       </c>
       <c r="H13" s="5" t="s">
@@ -9909,8 +10196,11 @@
       <c r="J13" s="3">
         <v>0</v>
       </c>
+      <c r="K13" s="12" t="s">
+        <v>299</v>
+      </c>
     </row>
-    <row r="14" spans="1:10" ht="409.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="3">
         <v>13</v>
       </c>
@@ -9941,8 +10231,11 @@
       <c r="J14" s="3">
         <v>1</v>
       </c>
+      <c r="K14" s="12" t="s">
+        <v>300</v>
+      </c>
     </row>
-    <row r="15" spans="1:10" ht="409.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="3">
         <v>14</v>
       </c>
@@ -9973,8 +10266,11 @@
       <c r="J15" s="3">
         <v>0</v>
       </c>
+      <c r="K15" s="12" t="s">
+        <v>301</v>
+      </c>
     </row>
-    <row r="16" spans="1:10" ht="409.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3">
         <v>15</v>
       </c>
@@ -10005,8 +10301,11 @@
       <c r="J16" s="3">
         <v>2</v>
       </c>
+      <c r="K16" s="12" t="s">
+        <v>302</v>
+      </c>
     </row>
-    <row r="17" spans="1:12" ht="409.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:17" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="3">
         <v>16</v>
       </c>
@@ -10037,8 +10336,11 @@
       <c r="J17" s="3">
         <v>0</v>
       </c>
+      <c r="K17" s="12" t="s">
+        <v>303</v>
+      </c>
     </row>
-    <row r="18" spans="1:12" ht="409.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:17" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="3">
         <v>17</v>
       </c>
@@ -10069,8 +10371,11 @@
       <c r="J18" s="3">
         <v>0</v>
       </c>
+      <c r="K18" s="12" t="s">
+        <v>304</v>
+      </c>
     </row>
-    <row r="19" spans="1:12" ht="409.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:17" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="3">
         <v>18</v>
       </c>
@@ -10101,8 +10406,11 @@
       <c r="J19" s="3">
         <v>0</v>
       </c>
+      <c r="K19" s="12" t="s">
+        <v>305</v>
+      </c>
     </row>
-    <row r="20" spans="1:12" ht="409.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:17" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="8">
         <v>19</v>
       </c>
@@ -10133,8 +10441,11 @@
       <c r="J20" s="3">
         <v>0</v>
       </c>
+      <c r="K20" s="12" t="s">
+        <v>306</v>
+      </c>
     </row>
-    <row r="21" spans="1:12" ht="409.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:17" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="3">
         <v>20</v>
       </c>
@@ -10165,8 +10476,11 @@
       <c r="J21" s="3">
         <v>0</v>
       </c>
+      <c r="K21" s="12" t="s">
+        <v>307</v>
+      </c>
     </row>
-    <row r="22" spans="1:12" ht="409.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:17" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="3">
         <v>21</v>
       </c>
@@ -10197,8 +10511,11 @@
       <c r="J22" s="3">
         <v>0</v>
       </c>
+      <c r="K22" s="12" t="s">
+        <v>308</v>
+      </c>
     </row>
-    <row r="23" spans="1:12" ht="409.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:17" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="3">
         <v>22</v>
       </c>
@@ -10229,8 +10546,11 @@
       <c r="J23" s="3">
         <v>0</v>
       </c>
+      <c r="K23" s="12" t="s">
+        <v>309</v>
+      </c>
     </row>
-    <row r="24" spans="1:12" ht="409.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:17" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="3">
         <v>23</v>
       </c>
@@ -10261,8 +10581,11 @@
       <c r="J24" s="3">
         <v>0</v>
       </c>
+      <c r="K24" s="12" t="s">
+        <v>310</v>
+      </c>
     </row>
-    <row r="25" spans="1:12" ht="261" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:17" ht="261" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="3">
         <v>24</v>
       </c>
@@ -10293,8 +10616,11 @@
       <c r="J25" s="3">
         <v>0</v>
       </c>
+      <c r="K25" s="12" t="s">
+        <v>311</v>
+      </c>
     </row>
-    <row r="26" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:17" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="3">
         <v>25</v>
       </c>
@@ -10325,8 +10651,11 @@
       <c r="J26" s="3">
         <v>0</v>
       </c>
+      <c r="K26" s="12" t="s">
+        <v>312</v>
+      </c>
     </row>
-    <row r="27" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:17" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="3">
         <v>26</v>
       </c>
@@ -10357,8 +10686,11 @@
       <c r="J27" s="3">
         <v>0</v>
       </c>
+      <c r="K27" s="12" t="s">
+        <v>313</v>
+      </c>
     </row>
-    <row r="28" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:17" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="3">
         <v>27</v>
       </c>
@@ -10389,8 +10721,11 @@
       <c r="J28" s="3">
         <v>0</v>
       </c>
+      <c r="K28" s="12" t="s">
+        <v>314</v>
+      </c>
     </row>
-    <row r="29" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:17" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="3">
         <v>28</v>
       </c>
@@ -10409,7 +10744,7 @@
       <c r="F29" s="5" t="s">
         <v>209</v>
       </c>
-      <c r="G29" s="10" t="s">
+      <c r="G29" s="14" t="s">
         <v>279</v>
       </c>
       <c r="H29" s="5" t="s">
@@ -10421,52 +10756,64 @@
       <c r="J29" s="3">
         <v>0</v>
       </c>
-      <c r="K29" s="5" t="s">
+      <c r="K29" s="12" t="s">
+        <v>318</v>
+      </c>
+      <c r="L29" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="M29">
+        <v>3</v>
+      </c>
+      <c r="P29" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="L29" s="5" t="s">
+      <c r="Q29" s="6" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="30" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="3">
+    <row r="30" spans="1:17" s="16" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="15">
         <v>29</v>
       </c>
-      <c r="B30" s="3">
+      <c r="B30" s="15">
         <v>0</v>
       </c>
-      <c r="C30" t="s">
+      <c r="C30" s="16" t="s">
         <v>125</v>
       </c>
-      <c r="D30" s="3">
+      <c r="D30" s="15">
         <v>26</v>
       </c>
-      <c r="E30" s="6" t="s">
+      <c r="E30" s="17" t="s">
         <v>212</v>
       </c>
-      <c r="F30" s="5" t="s">
+      <c r="F30" s="18" t="s">
         <v>213</v>
       </c>
-      <c r="G30" s="10" t="s">
+      <c r="G30" s="19" t="s">
         <v>280</v>
       </c>
-      <c r="H30" s="5" t="s">
+      <c r="H30" s="18" t="s">
         <v>214</v>
       </c>
-      <c r="I30" t="s">
+      <c r="I30" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="J30" s="3">
+      <c r="J30" s="15">
         <v>0</v>
       </c>
-      <c r="K30" s="5" t="s">
+      <c r="K30" s="20" t="s">
+        <v>318</v>
+      </c>
+      <c r="P30" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="L30" s="5" t="s">
+      <c r="Q30" s="17" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="31" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:17" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="3">
         <v>30</v>
       </c>
@@ -10485,7 +10832,7 @@
       <c r="F31" s="5" t="s">
         <v>217</v>
       </c>
-      <c r="G31" s="10" t="s">
+      <c r="G31" s="14" t="s">
         <v>281</v>
       </c>
       <c r="H31" s="5" t="s">
@@ -10497,14 +10844,23 @@
       <c r="J31" s="3">
         <v>0</v>
       </c>
-      <c r="K31" s="5" t="s">
+      <c r="K31" s="12" t="s">
+        <v>318</v>
+      </c>
+      <c r="L31" s="21" t="s">
+        <v>329</v>
+      </c>
+      <c r="M31" s="21" t="s">
+        <v>330</v>
+      </c>
+      <c r="P31" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="L31" s="5" t="s">
+      <c r="Q31" s="6" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="32" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:17" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="3">
         <v>31</v>
       </c>
@@ -10523,7 +10879,7 @@
       <c r="F32" s="5" t="s">
         <v>221</v>
       </c>
-      <c r="G32" s="10" t="s">
+      <c r="G32" s="14" t="s">
         <v>282</v>
       </c>
       <c r="H32" s="5" t="s">
@@ -10535,90 +10891,107 @@
       <c r="J32" s="3">
         <v>0</v>
       </c>
-      <c r="K32" s="5" t="s">
+      <c r="K32" s="12" t="s">
+        <v>318</v>
+      </c>
+      <c r="L32" s="2" t="s">
+        <v>331</v>
+      </c>
+      <c r="M32" t="s">
+        <v>332</v>
+      </c>
+      <c r="P32" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="L32" s="5" t="s">
+      <c r="Q32" s="6" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="33" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="3">
+    <row r="33" spans="1:17" s="16" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="15">
         <v>32</v>
       </c>
-      <c r="B33" s="3">
+      <c r="B33" s="15">
         <v>0</v>
       </c>
-      <c r="C33" t="s">
+      <c r="C33" s="16" t="s">
         <v>125</v>
       </c>
-      <c r="D33" s="3">
+      <c r="D33" s="15">
         <v>26</v>
       </c>
-      <c r="E33" t="s">
+      <c r="E33" s="16" t="s">
         <v>224</v>
       </c>
-      <c r="F33" s="5" t="s">
+      <c r="F33" s="18" t="s">
         <v>225</v>
       </c>
-      <c r="G33" s="10" t="s">
+      <c r="G33" s="19" t="s">
         <v>283</v>
       </c>
-      <c r="H33" s="5" t="s">
+      <c r="H33" s="18" t="s">
         <v>226</v>
       </c>
-      <c r="I33" t="s">
+      <c r="I33" s="16" t="s">
         <v>95</v>
       </c>
-      <c r="J33" s="3">
+      <c r="J33" s="15">
         <v>0</v>
       </c>
-      <c r="K33" s="5" t="s">
+      <c r="K33" s="20" t="s">
+        <v>318</v>
+      </c>
+      <c r="L33" s="19"/>
+      <c r="P33" s="18" t="s">
         <v>96</v>
       </c>
-      <c r="L33" s="5" t="s">
+      <c r="Q33" s="17" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="34" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="3">
+    <row r="34" spans="1:17" s="16" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="15">
         <v>33</v>
       </c>
-      <c r="B34" s="3">
+      <c r="B34" s="15">
         <v>0</v>
       </c>
-      <c r="C34" t="s">
+      <c r="C34" s="16" t="s">
         <v>125</v>
       </c>
-      <c r="D34" s="3">
+      <c r="D34" s="15">
         <v>28</v>
       </c>
-      <c r="E34" t="s">
+      <c r="E34" s="16" t="s">
         <v>228</v>
       </c>
-      <c r="F34" s="5" t="s">
+      <c r="F34" s="18" t="s">
         <v>229</v>
       </c>
-      <c r="G34" s="10" t="s">
+      <c r="G34" s="19" t="s">
         <v>284</v>
       </c>
-      <c r="H34" s="5" t="s">
+      <c r="H34" s="18" t="s">
         <v>230</v>
       </c>
-      <c r="I34" t="s">
+      <c r="I34" s="16" t="s">
         <v>97</v>
       </c>
-      <c r="J34" s="3">
+      <c r="J34" s="15">
         <v>0</v>
       </c>
-      <c r="K34" s="5" t="s">
+      <c r="K34" s="20" t="s">
+        <v>318</v>
+      </c>
+      <c r="L34" s="19"/>
+      <c r="P34" s="18" t="s">
         <v>98</v>
       </c>
-      <c r="L34" s="5" t="s">
+      <c r="Q34" s="17" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="35" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:17" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="3">
         <v>34</v>
       </c>
@@ -10637,7 +11010,7 @@
       <c r="F35" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="G35" s="10" t="s">
+      <c r="G35" s="14" t="s">
         <v>285</v>
       </c>
       <c r="H35" s="5" t="s">
@@ -10649,14 +11022,23 @@
       <c r="J35" s="3">
         <v>0</v>
       </c>
-      <c r="K35" s="5" t="s">
+      <c r="K35" s="12" t="s">
+        <v>318</v>
+      </c>
+      <c r="L35" s="2" t="s">
+        <v>333</v>
+      </c>
+      <c r="M35" t="s">
+        <v>334</v>
+      </c>
+      <c r="P35" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="L35" s="5" t="s">
+      <c r="Q35" s="6" t="s">
         <v>235</v>
       </c>
     </row>
-    <row r="36" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:17" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A36" s="3">
         <v>35</v>
       </c>
@@ -10675,7 +11057,7 @@
       <c r="F36" s="5" t="s">
         <v>237</v>
       </c>
-      <c r="G36" s="10" t="s">
+      <c r="G36" s="14" t="s">
         <v>286</v>
       </c>
       <c r="H36" s="5" t="s">
@@ -10687,14 +11069,23 @@
       <c r="J36" s="3">
         <v>0</v>
       </c>
-      <c r="K36" s="5" t="s">
+      <c r="K36" s="12" t="s">
+        <v>318</v>
+      </c>
+      <c r="L36" s="2" t="s">
+        <v>335</v>
+      </c>
+      <c r="M36">
+        <v>5</v>
+      </c>
+      <c r="P36" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="L36" s="5" t="s">
+      <c r="Q36" s="6" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="37" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:17" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="3">
         <v>36</v>
       </c>
@@ -10713,7 +11104,7 @@
       <c r="F37" s="5" t="s">
         <v>241</v>
       </c>
-      <c r="G37" s="10" t="s">
+      <c r="G37" s="14" t="s">
         <v>287</v>
       </c>
       <c r="H37" s="5" t="s">
@@ -10725,14 +11116,17 @@
       <c r="J37" s="3">
         <v>0</v>
       </c>
-      <c r="K37" s="5" t="s">
+      <c r="K37" s="12" t="s">
+        <v>315</v>
+      </c>
+      <c r="P37" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="L37" s="5" t="s">
+      <c r="Q37" s="6" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="38" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:17" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="3">
         <v>37</v>
       </c>
@@ -10763,14 +11157,17 @@
       <c r="J38" s="3">
         <v>0</v>
       </c>
-      <c r="K38" s="5" t="s">
+      <c r="K38" s="12" t="s">
+        <v>316</v>
+      </c>
+      <c r="P38" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="L38" s="5" t="s">
+      <c r="Q38" s="6" t="s">
         <v>247</v>
       </c>
     </row>
-    <row r="39" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:17" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="3">
         <v>38</v>
       </c>
@@ -10801,15 +11198,19 @@
       <c r="J39" s="3">
         <v>0</v>
       </c>
-      <c r="K39" s="2" t="s">
+      <c r="K39" s="12" t="s">
+        <v>317</v>
+      </c>
+      <c r="P39" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="L39" s="5" t="s">
+      <c r="Q39" s="6" t="s">
         <v>251</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Fixed Unit-Tests for Python Codingquestion
3 Unittests for Higher Functions still missing
</commit_message>
<xml_diff>
--- a/files/programming-tasks/programmieraufgaben_JACK_SOSE23_WORKSHOP_WISE2324.xlsx
+++ b/files/programming-tasks/programmieraufgaben_JACK_SOSE23_WORKSHOP_WISE2324.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\hefl\files\programming-tasks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB36739A-47A4-4BBF-B900-0C053C888D96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BCC36E3-E6EB-423F-B9F2-20F97FAB44AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="77040" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Aufgaben" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="449" uniqueCount="339">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="469" uniqueCount="352">
   <si>
     <t>id</t>
   </si>
@@ -414,30 +414,6 @@
 Weil 1+7+4=12 ist. </t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>Schreiben Sie &amp;nbsp;eine rekursive Funktion&amp;nbsp;&lt;code&gt;querSum(n)&lt;/code&gt;, die eine positive Ganzzahl&amp;nbsp;&lt;code&gt;n&lt;/code&gt;&amp;nbsp;als Parameter erh&amp;auml;lt und ihre Quersumme ausgibt.&lt;br /&gt;
-Hinweis:&amp;nbsp;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>Bsp.:&lt;br /&gt;
-&amp;gt;&amp;gt;&amp;gt;&amp;nbsp;&lt;code&gt;querSum(174)&lt;/code&gt;&amp;nbsp;&lt;br /&gt;
-&amp;gt;&amp;gt;&amp;gt;&amp;nbsp;12&lt;br /&gt;
-Weil&amp;nbsp;1+7+4=12 ist.&amp;nbsp;</t>
-    </r>
-  </si>
-  <si>
     <t>Python_Fibonacci Index</t>
   </si>
   <si>
@@ -449,732 +425,6 @@
 0,1,1,2,3,5,8,13,21,...
 Tipp:
 In den Übungen haben Sie ja bereits eine Funktion zur Bestimmung der Fibonacci Folge geschrieben, die sie jetzt wiederverwenden können!</t>
-  </si>
-  <si>
-    <r>
-      <t>style="font-size:12px;"&gt;style="font-family:Calibri, sans-serif"&gt;style="caret-color:#000000"&gt;style="font-style: normal;"&gt;style="font-variant-caps: normal;"&gt;style="font-weight: 400;"&gt;style="letter-spacing: normal;"&gt;style="text-transform: none;"&gt;style="white-space: normal;"&gt;style="word-spacing: 0px;"&gt;style="text-decoration: none;"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF222222"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Schreiben Sie eine rekursive Funktion </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>fib_index()</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="color: rgb(34, 34, 34);"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, die den Index einer Zahl in der Fibonacci-Folge (&lt;a href="https://de.wikipedia.org/wiki/Fibonacci-Folge" style="color:#954f72; text-decoration:underline"&gt;https://de.wikipedia.org/wiki/Fibonacci-Folge&lt;/a&gt;) zur&amp;uuml;ckgibt, wenn die Zahl ein Element dieser Folge ist, und -1 zur&amp;uuml;ckgibt, wenn die Zahl nicht darin enthalten ist.&amp;nbsp;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="font-family:Calibri, sans-serif"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="caret-color:#000000"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="color:#000000"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="font-style:normal"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="font-variant-caps:normal"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="font-weight:400"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="letter-spacing:normal"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="text-transform:none"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="white-space:normal"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="word-spacing:0px"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="text-decoration:none"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="color:#222222"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Bsp.:&lt;br /&gt;
-&amp;gt;&amp;gt;&amp;gt; fib_index(13)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="font-family:Calibri, sans-serif"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="caret-color:#000000"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="color:#000000"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="font-style:normal"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="font-variant-caps:normal"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="font-weight:400"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="letter-spacing:normal"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="text-transform:none"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="white-space:normal"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="word-spacing:0px"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>&amp;gt;&amp;gt;&amp;gt; 7</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="font-family:Calibri, sans-serif"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="caret-color:#000000"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="color:#000000"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="font-style:normal"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="font-variant-caps:normal"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="font-weight:400"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="letter-spacing:normal"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="text-transform:none"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="white-space:normal"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="word-spacing:0px"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>In der Fibonacci-Folge ist die 13 an der 7. Position:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="font-family:Calibri, sans-serif"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="caret-color:#000000"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="color:#000000"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="font-style:normal"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="font-variant-caps:normal"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="font-weight:400"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="letter-spacing:normal"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="text-transform:none"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="white-space:normal"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="word-spacing:0px"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0,1,1,2,3,5,8,13,21,...</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="font-family:Calibri, sans-serif"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="caret-color:#000000"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="color:#000000"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="font-style:normal"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="font-variant-caps:normal"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="font-weight:400"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="letter-spacing:normal"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="text-transform:none"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="white-space:normal"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="word-spacing:0px"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Tipp:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="font-family:Calibri, sans-serif"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="caret-color:#000000"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="color:#000000"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="font-style:normal"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="font-variant-caps:normal"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="font-weight:400"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="letter-spacing:normal"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="text-transform:none"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="white-space:normal"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>style="word-spacing:0px"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>In den &amp;Uuml;bungen haben Sie ja bereits eine Funktion zur Bestimmung der Fibonacci Folge geschrieben, die sie jetzt wiederverwenden k&amp;ouml;nnen!</t>
-    </r>
   </si>
   <si>
     <t>Buchstabenfrequenz</t>
@@ -1252,28 +502,6 @@
   </si>
   <si>
     <t>Sieb des Erathostenes</t>
-  </si>
-  <si>
-    <t>Das Sieb des Erathostenes ist ein Algorithmus der eine Liste alle Primzahlen von 2 bis zu einer gegebenen Zahl n berechnet (siehe u.a. https://de.wikipedia.org/wiki/Sieb_des_Eratosthenes). 
-Implementieren Sie den Algorithmus dazu in einer Funktion sieb(). Die Funktion erhält als Parameter den Wert n der angibt bis zu welcher Zahl die Primzahlen berechnet werden sollen. Die Funktion gibt die Liste mit allen Primzahlen von 2 bis n zurück!
-Gehen Sie dazu wie folgt vor:
-    Der Algorithmus berechnet jeweils die Vielfachen von 2, 3, 5 und 7 aus der gegebenen Liste und entfernt diese. Schreiben Sie deshalb zuerst eine Funktion vielfaches(). Die Funktion erhält als Parameter die Zahl zu denen die Vielfachen entfernt werden sollen. Dazu die Liste auf die Operation durchgeführt wird.
-    Bsp:: vielfach(2, liste) 
-    Entfernt alle Vielfachen von 2 aus liste
-    Implementieren sie dann die Funktion sieb() mit Hilfe der Funktion vielfaches().</t>
-  </si>
-  <si>
-    <t>Das &lt;strong&gt;Sieb des Erathostenes&lt;/strong&gt; ist ein Algorithmus der eine Liste alle Primzahlen von &lt;em&gt;2&lt;/em&gt; bis zu einer gegebenen Zahl &lt;em&gt;n&lt;/em&gt; berechnet (siehe u.a.&amp;nbsp;&lt;em&gt;https://de.wikipedia.org/wiki/Sieb_des_Eratosthenes&lt;/em&gt;).&amp;nbsp;&lt;br /&gt;
-&lt;br /&gt;
-Implementieren Sie den Algorithmus dazu in einer Funktion &lt;em&gt;sieb()&lt;/em&gt;. Die Funktion erh&amp;auml;lt als Parameter den Wert n der angibt bis zu welcher Zahl die Primzahlen berechnet werden sollen. Die Funktion gibt die Liste mit allen Primzahlen von 2 bis n zur&amp;uuml;ck!&lt;br /&gt;
-&lt;br /&gt;
-Gehen Sie dazu wie folgt vor:
-&lt;ol&gt;
-	&lt;li&gt;Der Algorithmus berechnet jeweils die Vielfachen von 2, 3, 5 und 7 aus der gegebenen Liste und entfernt diese. Schreiben Sie deshalb zuerst eine Funktion vielfaches(). Die Funktion erh&amp;auml;lt als Parameter die Zahl zu denen die Vielfachen entfernt werden sollen. Dazu die Liste auf die Operation durchgef&amp;uuml;hrt wird.&lt;br /&gt;
-	&lt;em&gt;Bsp:: vielfach(2, liste)&amp;nbsp;&lt;br /&gt;
-	Entfernt alle Vielfachen von 2 aus liste&lt;/em&gt;&lt;/li&gt;
-	&lt;li&gt;Implementieren sie dann die Funktion &lt;em&gt;sieb()&lt;/em&gt; mit Hilfe der Funktion &lt;em&gt;vielfaches()&lt;/em&gt;.&lt;/li&gt;
-&lt;/ol&gt;</t>
   </si>
   <si>
     <t>java</t>
@@ -2203,53 +1431,6 @@
   </si>
   <si>
     <t xml:space="preserve">import unittest
-import math
-def concatenate_functions(f1, f2):
-    def concatenated_function(x):
-        return f1(f2(x))
-    return concatenated_function
-class TestConcatenateFunctions(unittest.TestCase):
-    def test_case1(self):
-        f1 = lambda x: math.sin(x)
-        f2 = lambda x: 2 * math.pi * x
-        concatenated_func = concatenate_functions(f1, f2)
-        expected = math.sin(2 * math.pi * 0)
-        result = concatenated_func(0)
-        self.assertAlmostEqual(result, expected, delta=1e-7)
-    def test_case2(self):
-        f1 = lambda x: math.sin(x)
-        f2 = lambda x: 2 * math.pi * x
-        concatenated_func = concatenate_functions(f1, f2)
-        expected = math.sin(2 * math.pi * 1)
-        result = concatenated_func(1)
-        self.assertAlmostEqual(result, expected, delta=1e-7)
-    def test_case3(self):
-        f1 = lambda x: math.sin(x)
-        f2 = lambda x: 2 * math.pi * x
-        concatenated_func = concatenate_functions(f1, f2)
-        expected = math.sin(2 * math.pi * 2)
-        result = concatenated_func(2)
-        self.assertAlmostEqual(result, expected, delta=1e-7)
-    def test_case4(self):
-        f1 = lambda x: math.sin(x)
-        f2 = lambda x: 2 * math.pi * x
-        concatenated_func = concatenate_functions(f1, f2)
-        expected = math.sin(2 * math.pi * 3)
-        result = concatenated_func(3)
-        self.assertAlmostEqual(result, expected, delta=1e-7)
-    def test_case5(self):
-        f1 = lambda x: math.sin(x)
-        f2 = lambda x: 2 * math.pi * x
-        concatenated_func = concatenate_functions(f1, f2)
-        expected = math.sin(2 * math.pi * 4)
-        result = concatenated_func(4)
-        self.assertAlmostEqual(result, expected, delta=1e-7)
-if __name__ == '__main__':
-    unittest.main()
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">import unittest
 from potenz import potenz
 class TestPotenzFunction(unittest.TestCase):
     def test_potenz_case1(self):
@@ -4013,12 +3194,119 @@
 &lt;strong&gt;Hinweis zur Bewertung: Ihre main()-Klasse Airline wird durch Tutor Kai durch eine Testklasse ersetzt. Ihre main()-Klasse dient nur dazu das Sie Ihre Implementierungen der Klassen Verkehrsflugzeug und Doppeldecker testen k&amp;ouml;nnen. Laden Sie dennoch auch die Airline.java mit hoch!&lt;br /&gt;
 &lt;br /&gt;&lt;/strong&gt;</t>
   </si>
+  <si>
+    <t>6, 7</t>
+  </si>
+  <si>
+    <t>Das Sieb des Erathostenes ist ein Algorithmus der eine Liste alle Primzahlen von 2 bis zu einer gegebenen Zahl n berechnet (siehe u.a. https://de.wikipedia.org/wiki/Sieb_des_Eratosthenes). 
+Implementieren Sie den Algorithmus dazu in einer Funktion sieb(). Die Funktion erhält als Parameter den Wert n der angibt bis zu welcher Zahl die Primzahlen berechnet werden sollen. Die Funktion gibt die Liste mit allen Primzahlen von 2 bis n zurück!
+Gehen Sie dazu wie folgt vor:
+    Der Algorithmus berechnet jeweils die Vielfachen von 2, 3, 5 und 7 aus der gegebenen Liste und entfernt diese. Schreiben Sie deshalb zuerst eine Funktion vielfach(). Die Funktion erhält als Parameter die Zahl zu denen die Vielfachen entfernt werden sollen. Dazu die Liste auf die Operation durchgeführt wird.
+    Bsp:: vielfach(2, liste) 
+    Entfernt alle Vielfachen von 2 aus liste
+    Implementieren sie dann die Funktion sieb() mit Hilfe der Funktion vielfaches().</t>
+  </si>
+  <si>
+    <t>Das &lt;strong&gt;Sieb des Erathostenes&lt;/strong&gt; ist ein Algorithmus der eine Liste alle Primzahlen von &lt;em&gt;2&lt;/em&gt; bis zu einer gegebenen Zahl &lt;em&gt;n&lt;/em&gt; berechnet (siehe u.a.&amp;nbsp;&lt;em&gt;https://de.wikipedia.org/wiki/Sieb_des_Eratosthenes&lt;/em&gt;).&amp;nbsp;&lt;br /&gt;
+&lt;br /&gt;
+Implementieren Sie den Algorithmus dazu in einer Funktion &lt;em&gt;sieb()&lt;/em&gt;. Die Funktion erh&amp;auml;lt als Parameter den Wert n der angibt bis zu welcher Zahl die Primzahlen berechnet werden sollen. Die Funktion gibt die Liste mit allen Primzahlen von 2 bis n zur&amp;uuml;ck!&lt;br /&gt;
+&lt;br /&gt;
+Gehen Sie dazu wie folgt vor:
+&lt;ol&gt;
+	&lt;li&gt;Der Algorithmus berechnet jeweils die Vielfachen von 2, 3, 5 und 7 aus der gegebenen Liste und entfernt diese. Schreiben Sie deshalb zuerst eine Funktion vielfach(). Die Funktion erh&amp;auml;lt als Parameter die Zahl zu denen die Vielfachen entfernt werden sollen. Dazu die Liste auf die Operation durchgef&amp;uuml;hrt wird.&lt;br /&gt;
+	&lt;em&gt;Bsp:: vielfach(2, liste)&amp;nbsp;&lt;br /&gt;
+	Entfernt alle Vielfachen von 2 aus liste&lt;/em&gt;&lt;/li&gt;
+	&lt;li&gt;Implementieren sie dann die Funktion &lt;em&gt;sieb()&lt;/em&gt; mit Hilfe der Funktion &lt;em&gt;vielfaches()&lt;/em&gt;.&lt;/li&gt;
+&lt;/ol&gt;</t>
+  </si>
+  <si>
+    <t>Comment</t>
+  </si>
+  <si>
+    <t>Streng genommen wird der Fall 0 Jahre nicht überprüft, sonst gut.</t>
+  </si>
+  <si>
+    <t>Streng genommen wird der Fall exakt 100 Euro nicht richtig überprüft, sonst gut.</t>
+  </si>
+  <si>
+    <t>gut</t>
+  </si>
+  <si>
+    <t>Fehler in Anzeige der Aufgabenstellung. Welche Antwort wird für 1 erwartet? Sonst gut.</t>
+  </si>
+  <si>
+    <t>nicht in Goals(?)</t>
+  </si>
+  <si>
+    <t>Traceback (most recent call last):
+  File "&lt;string&gt;", line 1, in &lt;module&gt;
+TypeError: summe() missing 1 required positional argument: 'n' in Ausgabe, sonst gut</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Funktion heißt einmal in Aufgabenstellung vielfaches() statt vielfach() wie sonst und im Test</t>
+  </si>
+  <si>
+    <t>liefert 100% bei leerem Code (no program to run)</t>
+  </si>
+  <si>
+    <t>no program to run als Ausgabe, Rest scheint zu funktionieren</t>
+  </si>
+  <si>
+    <t>Schreiben Sie &amp;nbsp;eine rekursive Funktion&amp;nbsp;&lt;code&gt;querSum(n)&lt;/code&gt;, die eine positive Ganzzahl&amp;nbsp;&lt;code&gt;n&lt;/code&gt;&amp;nbsp;als Parameter erh&amp;auml;lt und ihre Quersumme ausgibt.&lt;br /&gt;
+Hinweis:&amp;nbsp;Bsp.:&lt;br /&gt;
+&amp;gt;&amp;gt;&amp;gt;&amp;nbsp;&lt;code&gt;querSum(174)&lt;/code&gt;&amp;nbsp;&lt;br /&gt;
+&amp;gt;&amp;gt;&amp;gt;&amp;nbsp;12&lt;br /&gt;
+Weil&amp;nbsp;1+7+4=12 ist.&amp;nbsp;</t>
+  </si>
+  <si>
+    <t>style="font-size:12px;"&gt;style="font-family:Calibri, sans-serif"&gt;style="caret-color:#000000"&gt;style="font-style: normal;"&gt;style="font-variant-caps: normal;"&gt;style="font-weight: 400;"&gt;style="letter-spacing: normal;"&gt;style="text-transform: none;"&gt;style="white-space: normal;"&gt;style="word-spacing: 0px;"&gt;style="text-decoration: none;"&gt;Schreiben Sie eine rekursive Funktion fib_index()style="color: rgb(34, 34, 34);"&gt;, die den Index einer Zahl in der Fibonacci-Folge (&lt;a href="https://de.wikipedia.org/wiki/Fibonacci-Folge" style="color:#954f72; text-decoration:underline"&gt;https://de.wikipedia.org/wiki/Fibonacci-Folge&lt;/a&gt;) zur&amp;uuml;ckgibt, wenn die Zahl ein Element dieser Folge ist, und -1 zur&amp;uuml;ckgibt, wenn die Zahl nicht darin enthalten ist.&amp;nbsp;style="font-family:Calibri, sans-serif"&gt;style="caret-color:#000000"&gt;style="color:#000000"&gt;style="font-style:normal"&gt;style="font-variant-caps:normal"&gt;style="font-weight:400"&gt;style="letter-spacing:normal"&gt;style="text-transform:none"&gt;style="white-space:normal"&gt;style="word-spacing:0px"&gt;style="text-decoration:none"&gt;style="color:#222222"&gt;Bsp.:&lt;br /&gt;
+&amp;gt;&amp;gt;&amp;gt; fib_index(13)style="font-family:Calibri, sans-serif"&gt;style="caret-color:#000000"&gt;style="color:#000000"&gt;style="font-style:normal"&gt;style="font-variant-caps:normal"&gt;style="font-weight:400"&gt;style="letter-spacing:normal"&gt;style="text-transform:none"&gt;style="white-space:normal"&gt;style="word-spacing:0px"&gt;&amp;gt;&amp;gt;&amp;gt; 7style="font-family:Calibri, sans-serif"&gt;style="caret-color:#000000"&gt;style="color:#000000"&gt;style="font-style:normal"&gt;style="font-variant-caps:normal"&gt;style="font-weight:400"&gt;style="letter-spacing:normal"&gt;style="text-transform:none"&gt;style="white-space:normal"&gt;style="word-spacing:0px"&gt;In der Fibonacci-Folge ist die 13 an der 7. Position:style="font-family:Calibri, sans-serif"&gt;style="caret-color:#000000"&gt;style="color:#000000"&gt;style="font-style:normal"&gt;style="font-variant-caps:normal"&gt;style="font-weight:400"&gt;style="letter-spacing:normal"&gt;style="text-transform:none"&gt;style="white-space:normal"&gt;style="word-spacing:0px"&gt;0,1,1,2,3,5,8,13,21,...style="font-family:Calibri, sans-serif"&gt;style="caret-color:#000000"&gt;style="color:#000000"&gt;style="font-style:normal"&gt;style="font-variant-caps:normal"&gt;style="font-weight:400"&gt;style="letter-spacing:normal"&gt;style="text-transform:none"&gt;style="white-space:normal"&gt;style="word-spacing:0px"&gt;Tipp:style="font-family:Calibri, sans-serif"&gt;style="caret-color:#000000"&gt;style="color:#000000"&gt;style="font-style:normal"&gt;style="font-variant-caps:normal"&gt;style="font-weight:400"&gt;style="letter-spacing:normal"&gt;style="text-transform:none"&gt;style="white-space:normal"&gt;style="word-spacing:0px"&gt;In den &amp;Uuml;bungen haben Sie ja bereits eine Funktion zur Bestimmung der Fibonacci Folge geschrieben, die sie jetzt wiederverwenden k&amp;ouml;nnen!</t>
+  </si>
+  <si>
+    <t>concatenate_functions</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> lambda x: math.sin(x),  lambda x: 2 * math.pi * x</t>
+  </si>
+  <si>
+    <t xml:space="preserve">import unittest
+import math
+from funktionen import concatenate_functions
+class TestConcatenateFunctions(unittest.TestCase):
+     def test_direct_math_functions(self):
+        """Testet die Verkettung von zwei direkten mathematischen Funktionen."""
+        f1 = math.sqrt  # Erste Funktion: Quadratwurzel
+        f2 = math.exp   # Zweite Funktion: Exponentialfunktion
+        concatenated_func = concatenate_functions(f1, f2)
+        x = 2  # Beispielwert
+        expected = math.sqrt(math.exp(x))
+        self.assertAlmostEqual(concatenated_func(x), expected, delta=1e-7)
+    def test_identity_function(self):
+        """Überprüft die Verkettung mit einer Identitätsfunktion."""
+        f1 = lambda x: x  # Identitätsfunktion
+        f2 = math.sin     # Zweite Funktion: Sinus
+        concatenated_func = concatenate_functions(f1, f2)
+        x = math.pi / 2  # Beispielwert
+        expected = math.sin(x)
+        self.assertEqual(concatenated_func(x), expected)
+    def test_custom_functions(self):
+        """Testet die Verkettung von benutzerdefinierten Funktionen."""
+        f1 = lambda x: x ** 2  # Quadrieren
+        f2 = lambda x: x + 2   # Addiere 2
+        concatenated_func = concatenate_functions(f1, f2)
+        x = 3  # Beispielwert
+        expected = (x + 2) ** 2
+        self.assertEqual(concatenated_func(x), expected)
+if __name__ == '__main__':
+    unittest.main()
+</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4043,19 +3331,6 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF222222"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -4088,8 +3363,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -4099,6 +3381,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -4133,11 +3420,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -4163,37 +3451,60 @@
     <xf numFmtId="3" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="10" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="8" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="2" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="3" fontId="9" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="2" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="2" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
+    <cellStyle name="Gut" xfId="2" builtinId="26"/>
     <cellStyle name="Neutral" xfId="1" builtinId="28"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
@@ -4499,393 +3810,421 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:Q39"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="13.54296875" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="23.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.1796875" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="37.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="66.7265625" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="143.1796875" style="2" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="105.54296875" style="2" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="23.7265625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.54296875" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="50.7265625" style="1" customWidth="1"/>
-    <col min="12" max="12" width="49.81640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="74.54296875" bestFit="1" customWidth="1"/>
-    <col min="14" max="17" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="37.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="66.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="143.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="105.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="23.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="50.7109375" style="1" customWidth="1"/>
+    <col min="12" max="12" width="49.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="74.5703125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="170.7109375" customWidth="1"/>
+    <col min="15" max="17" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:14" s="18" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="20" t="s">
         <v>76</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="20" t="s">
         <v>77</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="20" t="s">
         <v>79</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="18" t="s">
         <v>80</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="19" t="s">
         <v>81</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="19" t="s">
         <v>82</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="19" t="s">
         <v>83</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="20" t="s">
         <v>85</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="20" t="s">
+        <v>227</v>
+      </c>
+      <c r="L1" s="19" t="s">
+        <v>198</v>
+      </c>
+      <c r="M1" s="18" t="s">
+        <v>199</v>
+      </c>
+      <c r="N1" s="18" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" s="18" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="21">
+        <v>1</v>
+      </c>
+      <c r="B2" s="21">
+        <v>5</v>
+      </c>
+      <c r="C2" s="18" t="s">
+        <v>86</v>
+      </c>
+      <c r="D2" s="21">
+        <v>34</v>
+      </c>
+      <c r="E2" s="22" t="s">
+        <v>87</v>
+      </c>
+      <c r="F2" s="22" t="s">
+        <v>88</v>
+      </c>
+      <c r="G2" s="23" t="s">
+        <v>183</v>
+      </c>
+      <c r="H2" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="I2" s="18" t="s">
+        <v>4</v>
+      </c>
+      <c r="J2" s="21">
+        <v>0</v>
+      </c>
+      <c r="K2" s="24" t="s">
+        <v>226</v>
+      </c>
+      <c r="L2" s="19" t="s">
+        <v>200</v>
+      </c>
+      <c r="M2" s="18" t="s">
+        <v>228</v>
+      </c>
+      <c r="N2" s="18" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" s="18" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="21">
+        <v>2</v>
+      </c>
+      <c r="B3" s="21">
+        <v>5</v>
+      </c>
+      <c r="C3" s="18" t="s">
+        <v>86</v>
+      </c>
+      <c r="D3" s="21">
+        <v>36</v>
+      </c>
+      <c r="E3" s="25" t="s">
+        <v>90</v>
+      </c>
+      <c r="F3" s="22" t="s">
+        <v>91</v>
+      </c>
+      <c r="G3" s="23" t="s">
+        <v>184</v>
+      </c>
+      <c r="H3" s="22" t="s">
+        <v>92</v>
+      </c>
+      <c r="I3" s="18" t="s">
+        <v>6</v>
+      </c>
+      <c r="J3" s="21">
+        <v>0</v>
+      </c>
+      <c r="K3" s="24" t="s">
+        <v>226</v>
+      </c>
+      <c r="L3" s="19" t="s">
+        <v>201</v>
+      </c>
+      <c r="M3" s="18" t="s">
+        <v>202</v>
+      </c>
+      <c r="N3" s="18" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" s="18" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="21">
+        <v>3</v>
+      </c>
+      <c r="B4" s="21">
+        <v>5</v>
+      </c>
+      <c r="C4" s="18" t="s">
+        <v>86</v>
+      </c>
+      <c r="D4" s="21">
+        <v>34</v>
+      </c>
+      <c r="E4" s="25" t="s">
+        <v>93</v>
+      </c>
+      <c r="F4" s="22" t="s">
+        <v>94</v>
+      </c>
+      <c r="G4" s="23" t="s">
+        <v>185</v>
+      </c>
+      <c r="H4" s="22" t="s">
+        <v>347</v>
+      </c>
+      <c r="I4" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="J4" s="21">
+        <v>0</v>
+      </c>
+      <c r="K4" s="24" t="s">
+        <v>226</v>
+      </c>
+      <c r="L4" s="19" t="s">
+        <v>203</v>
+      </c>
+      <c r="M4" s="18">
+        <v>174</v>
+      </c>
+      <c r="N4" s="18" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" s="13" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="12">
+        <v>4</v>
+      </c>
+      <c r="B5" s="12">
+        <v>5</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="D5" s="12">
+        <v>34</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="F5" s="15" t="s">
+        <v>96</v>
+      </c>
+      <c r="G5" s="26" t="s">
+        <v>186</v>
+      </c>
+      <c r="H5" s="15" t="s">
+        <v>348</v>
+      </c>
+      <c r="I5" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="J5" s="12">
+        <v>0</v>
+      </c>
+      <c r="K5" s="17" t="s">
+        <v>226</v>
+      </c>
+      <c r="L5" s="16" t="s">
+        <v>229</v>
+      </c>
+      <c r="M5" s="13">
+        <v>47</v>
+      </c>
+      <c r="N5" s="13" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" s="13" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="12">
+        <v>5</v>
+      </c>
+      <c r="B6" s="12">
+        <v>4</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="D6" s="12">
+        <v>52</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="F6" s="15" t="s">
+        <v>98</v>
+      </c>
+      <c r="G6" s="26" t="s">
+        <v>187</v>
+      </c>
+      <c r="H6" s="15" t="s">
+        <v>99</v>
+      </c>
+      <c r="I6" s="13" t="s">
+        <v>9</v>
+      </c>
+      <c r="J6" s="12">
+        <v>0</v>
+      </c>
+      <c r="K6" s="17" t="s">
+        <v>226</v>
+      </c>
+      <c r="L6" s="16" t="s">
+        <v>230</v>
+      </c>
+      <c r="M6" s="13" t="s">
+        <v>231</v>
+      </c>
+      <c r="N6" s="13" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" s="18" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="21">
+        <v>6</v>
+      </c>
+      <c r="B7" s="21">
+        <v>4</v>
+      </c>
+      <c r="C7" s="18" t="s">
+        <v>86</v>
+      </c>
+      <c r="D7" s="21">
+        <v>34</v>
+      </c>
+      <c r="E7" s="18" t="s">
+        <v>100</v>
+      </c>
+      <c r="F7" s="22" t="s">
+        <v>101</v>
+      </c>
+      <c r="G7" s="23" t="s">
+        <v>188</v>
+      </c>
+      <c r="H7" s="22" t="s">
+        <v>102</v>
+      </c>
+      <c r="I7" s="18" t="s">
+        <v>10</v>
+      </c>
+      <c r="J7" s="21">
+        <v>0</v>
+      </c>
+      <c r="K7" s="24" t="s">
+        <v>226</v>
+      </c>
+      <c r="L7" s="19" t="s">
         <v>232</v>
       </c>
-      <c r="L1" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="M1" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A2" s="3">
-        <v>1</v>
-      </c>
-      <c r="B2" s="3">
-        <v>5</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="M7" s="18" t="s">
+        <v>334</v>
+      </c>
+      <c r="N7" s="19" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" s="18" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="21">
+        <v>7</v>
+      </c>
+      <c r="B8" s="21">
+        <v>4</v>
+      </c>
+      <c r="C8" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D8" s="21">
         <v>34</v>
       </c>
-      <c r="E2" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="G2" s="9" t="s">
-        <v>187</v>
-      </c>
-      <c r="H2" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="I2" t="s">
+      <c r="E8" s="18" t="s">
+        <v>103</v>
+      </c>
+      <c r="F8" s="22" t="s">
+        <v>104</v>
+      </c>
+      <c r="G8" s="23" t="s">
+        <v>189</v>
+      </c>
+      <c r="H8" s="22" t="s">
+        <v>105</v>
+      </c>
+      <c r="I8" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="J8" s="21">
+        <v>0</v>
+      </c>
+      <c r="K8" s="24" t="s">
+        <v>226</v>
+      </c>
+      <c r="L8" s="19" t="s">
+        <v>233</v>
+      </c>
+      <c r="M8" s="18" t="s">
+        <v>234</v>
+      </c>
+      <c r="N8" s="18" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" s="18" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="21">
+        <v>8</v>
+      </c>
+      <c r="B9" s="21">
         <v>4</v>
       </c>
-      <c r="J2" s="3">
+      <c r="C9" s="18" t="s">
+        <v>86</v>
+      </c>
+      <c r="D9" s="21">
+        <v>26</v>
+      </c>
+      <c r="E9" s="18" t="s">
+        <v>106</v>
+      </c>
+      <c r="F9" s="22" t="s">
+        <v>335</v>
+      </c>
+      <c r="G9" s="23" t="s">
+        <v>190</v>
+      </c>
+      <c r="H9" s="22" t="s">
+        <v>336</v>
+      </c>
+      <c r="I9" s="18" t="s">
+        <v>12</v>
+      </c>
+      <c r="J9" s="21">
         <v>0</v>
       </c>
-      <c r="K2" s="10" t="s">
-        <v>231</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="M2" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="3">
-        <v>2</v>
-      </c>
-      <c r="B3" s="3">
-        <v>5</v>
-      </c>
-      <c r="C3" t="s">
-        <v>86</v>
-      </c>
-      <c r="D3" s="3">
-        <v>36</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="G3" s="9" t="s">
-        <v>188</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="I3" t="s">
-        <v>6</v>
-      </c>
-      <c r="J3" s="3">
-        <v>0</v>
-      </c>
-      <c r="K3" s="10" t="s">
-        <v>231</v>
-      </c>
-      <c r="L3" s="2" t="s">
-        <v>206</v>
-      </c>
-      <c r="M3" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A4" s="3">
-        <v>3</v>
-      </c>
-      <c r="B4" s="3">
-        <v>5</v>
-      </c>
-      <c r="C4" t="s">
-        <v>86</v>
-      </c>
-      <c r="D4" s="3">
-        <v>34</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="G4" s="9" t="s">
-        <v>189</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="I4" t="s">
-        <v>7</v>
-      </c>
-      <c r="J4" s="3">
-        <v>0</v>
-      </c>
-      <c r="K4" s="10" t="s">
-        <v>231</v>
-      </c>
-      <c r="L4" s="2" t="s">
-        <v>208</v>
-      </c>
-      <c r="M4">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A5" s="3">
-        <v>4</v>
-      </c>
-      <c r="B5" s="3">
-        <v>5</v>
-      </c>
-      <c r="C5" t="s">
-        <v>86</v>
-      </c>
-      <c r="D5" s="3">
-        <v>34</v>
-      </c>
-      <c r="E5" t="s">
-        <v>96</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="G5" s="11" t="s">
-        <v>190</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="I5" t="s">
-        <v>8</v>
-      </c>
-      <c r="J5" s="3">
-        <v>0</v>
-      </c>
-      <c r="K5" s="10" t="s">
-        <v>231</v>
-      </c>
-      <c r="L5" s="2" t="s">
-        <v>234</v>
-      </c>
-      <c r="M5">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="3">
-        <v>5</v>
-      </c>
-      <c r="B6" s="3">
-        <v>4</v>
-      </c>
-      <c r="C6" t="s">
-        <v>86</v>
-      </c>
-      <c r="D6" s="3">
-        <v>52</v>
-      </c>
-      <c r="E6" t="s">
-        <v>99</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="G6" s="11" t="s">
-        <v>191</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="I6" t="s">
-        <v>9</v>
-      </c>
-      <c r="J6" s="3">
-        <v>0</v>
-      </c>
-      <c r="K6" s="10" t="s">
-        <v>231</v>
-      </c>
-      <c r="L6" s="2" t="s">
+      <c r="K9" s="24" t="s">
+        <v>226</v>
+      </c>
+      <c r="L9" s="19" t="s">
         <v>235</v>
       </c>
-      <c r="M6" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="3">
-        <v>6</v>
-      </c>
-      <c r="B7" s="3">
-        <v>4</v>
-      </c>
-      <c r="C7" t="s">
-        <v>86</v>
-      </c>
-      <c r="D7" s="3">
-        <v>34</v>
-      </c>
-      <c r="E7" t="s">
-        <v>102</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="G7" s="11" t="s">
-        <v>192</v>
-      </c>
-      <c r="H7" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="I7" t="s">
+      <c r="M9" s="18">
         <v>10</v>
       </c>
-      <c r="J7" s="3">
-        <v>0</v>
-      </c>
-      <c r="K7" s="10" t="s">
-        <v>231</v>
-      </c>
-      <c r="L7" s="2" t="s">
-        <v>237</v>
-      </c>
-      <c r="M7">
-        <v>6.7</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="3">
-        <v>7</v>
-      </c>
-      <c r="B8" s="3">
-        <v>4</v>
-      </c>
-      <c r="C8" t="s">
-        <v>86</v>
-      </c>
-      <c r="D8" s="3">
-        <v>34</v>
-      </c>
-      <c r="E8" t="s">
-        <v>105</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="G8" s="11" t="s">
-        <v>193</v>
-      </c>
-      <c r="H8" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="I8" t="s">
-        <v>11</v>
-      </c>
-      <c r="J8" s="3">
-        <v>0</v>
-      </c>
-      <c r="K8" s="10" t="s">
-        <v>231</v>
-      </c>
-      <c r="L8" s="2" t="s">
-        <v>238</v>
-      </c>
-      <c r="M8" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A9" s="3">
-        <v>8</v>
-      </c>
-      <c r="B9" s="3">
-        <v>4</v>
-      </c>
-      <c r="C9" t="s">
-        <v>86</v>
-      </c>
-      <c r="D9" s="3">
-        <v>26</v>
-      </c>
-      <c r="E9" t="s">
-        <v>108</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="G9" s="11" t="s">
-        <v>194</v>
-      </c>
-      <c r="H9" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="I9" t="s">
-        <v>12</v>
-      </c>
-      <c r="J9" s="3">
-        <v>0</v>
-      </c>
-      <c r="K9" s="10" t="s">
-        <v>231</v>
-      </c>
-      <c r="L9" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="M9">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="N9" s="18" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3">
         <v>9</v>
       </c>
@@ -4893,22 +4232,22 @@
         <v>6</v>
       </c>
       <c r="C10" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D10" s="3">
         <v>63</v>
       </c>
       <c r="E10" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="G10" s="11" t="s">
-        <v>249</v>
+        <v>109</v>
+      </c>
+      <c r="G10" s="10" t="s">
+        <v>244</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="I10" t="s">
         <v>13</v>
@@ -4916,11 +4255,11 @@
       <c r="J10" s="3">
         <v>0</v>
       </c>
-      <c r="K10" s="10" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="K10" s="9" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3">
         <v>10</v>
       </c>
@@ -4928,22 +4267,22 @@
         <v>6</v>
       </c>
       <c r="C11" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D11" s="3">
         <v>65</v>
       </c>
       <c r="E11" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>313</v>
-      </c>
-      <c r="G11" s="11" t="s">
-        <v>250</v>
+        <v>308</v>
+      </c>
+      <c r="G11" s="10" t="s">
+        <v>245</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>314</v>
+        <v>309</v>
       </c>
       <c r="I11" t="s">
         <v>14</v>
@@ -4951,11 +4290,11 @@
       <c r="J11" s="3">
         <v>0</v>
       </c>
-      <c r="K11" s="10" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="K11" s="9" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3">
         <v>11</v>
       </c>
@@ -4963,22 +4302,22 @@
         <v>6</v>
       </c>
       <c r="C12" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D12" s="3">
         <v>63</v>
       </c>
       <c r="E12" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="G12" s="11" t="s">
-        <v>251</v>
+        <v>113</v>
+      </c>
+      <c r="G12" s="10" t="s">
+        <v>246</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="I12" t="s">
         <v>15</v>
@@ -4986,11 +4325,11 @@
       <c r="J12" s="3">
         <v>1</v>
       </c>
-      <c r="K12" s="10" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="K12" s="9" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3">
         <v>12</v>
       </c>
@@ -4998,22 +4337,22 @@
         <v>6</v>
       </c>
       <c r="C13" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D13" s="3">
         <v>63</v>
       </c>
       <c r="E13" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="G13" s="11" t="s">
-        <v>252</v>
+        <v>116</v>
+      </c>
+      <c r="G13" s="10" t="s">
+        <v>247</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="I13" t="s">
         <v>16</v>
@@ -5021,11 +4360,11 @@
       <c r="J13" s="3">
         <v>0</v>
       </c>
-      <c r="K13" s="10" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="K13" s="9" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="3">
         <v>13</v>
       </c>
@@ -5033,22 +4372,22 @@
         <v>7</v>
       </c>
       <c r="C14" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D14" s="3">
         <v>69</v>
       </c>
       <c r="E14" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="F14" s="7" t="s">
-        <v>315</v>
-      </c>
-      <c r="G14" s="12" t="s">
-        <v>253</v>
+        <v>310</v>
+      </c>
+      <c r="G14" s="11" t="s">
+        <v>248</v>
       </c>
       <c r="H14" s="7" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="I14" t="s">
         <v>17</v>
@@ -5056,11 +4395,11 @@
       <c r="J14" s="3">
         <v>1</v>
       </c>
-      <c r="K14" s="10" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="K14" s="9" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="3">
         <v>14</v>
       </c>
@@ -5068,22 +4407,22 @@
         <v>7</v>
       </c>
       <c r="C15" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D15" s="3">
         <v>70</v>
       </c>
       <c r="E15" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>124</v>
-      </c>
-      <c r="G15" s="12" t="s">
-        <v>254</v>
+        <v>120</v>
+      </c>
+      <c r="G15" s="11" t="s">
+        <v>249</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="I15" t="s">
         <v>18</v>
@@ -5091,11 +4430,11 @@
       <c r="J15" s="3">
         <v>0</v>
       </c>
-      <c r="K15" s="10" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="K15" s="9" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3">
         <v>15</v>
       </c>
@@ -5103,22 +4442,22 @@
         <v>7</v>
       </c>
       <c r="C16" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D16" s="3">
         <v>64</v>
       </c>
       <c r="E16" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>317</v>
-      </c>
-      <c r="G16" s="12" t="s">
-        <v>255</v>
+        <v>312</v>
+      </c>
+      <c r="G16" s="11" t="s">
+        <v>250</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
       <c r="I16" t="s">
         <v>19</v>
@@ -5126,11 +4465,11 @@
       <c r="J16" s="3">
         <v>2</v>
       </c>
-      <c r="K16" s="10" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="17" spans="1:17" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="K16" s="9" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="3">
         <v>16</v>
       </c>
@@ -5138,22 +4477,22 @@
         <v>8</v>
       </c>
       <c r="C17" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D17" s="3">
         <v>85</v>
       </c>
       <c r="E17" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>319</v>
-      </c>
-      <c r="G17" s="12" t="s">
-        <v>256</v>
+        <v>314</v>
+      </c>
+      <c r="G17" s="11" t="s">
+        <v>251</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>320</v>
+        <v>315</v>
       </c>
       <c r="I17" s="5" t="s">
         <v>20</v>
@@ -5161,11 +4500,11 @@
       <c r="J17" s="3">
         <v>0</v>
       </c>
-      <c r="K17" s="10" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="18" spans="1:17" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="K17" s="9" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="3">
         <v>17</v>
       </c>
@@ -5173,22 +4512,22 @@
         <v>8</v>
       </c>
       <c r="C18" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D18" s="3">
         <v>84</v>
       </c>
       <c r="E18" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>321</v>
-      </c>
-      <c r="G18" s="12" t="s">
-        <v>257</v>
+        <v>316</v>
+      </c>
+      <c r="G18" s="11" t="s">
+        <v>252</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="I18" t="s">
         <v>25</v>
@@ -5196,11 +4535,11 @@
       <c r="J18" s="3">
         <v>0</v>
       </c>
-      <c r="K18" s="10" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="19" spans="1:17" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="K18" s="9" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="3">
         <v>18</v>
       </c>
@@ -5208,22 +4547,22 @@
         <v>8</v>
       </c>
       <c r="C19" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D19" s="3">
         <v>93</v>
       </c>
       <c r="E19" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>323</v>
-      </c>
-      <c r="G19" s="12" t="s">
-        <v>258</v>
+        <v>318</v>
+      </c>
+      <c r="G19" s="11" t="s">
+        <v>253</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>324</v>
+        <v>319</v>
       </c>
       <c r="I19" t="s">
         <v>29</v>
@@ -5231,11 +4570,11 @@
       <c r="J19" s="3">
         <v>0</v>
       </c>
-      <c r="K19" s="10" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="20" spans="1:17" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="K19" s="9" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="8">
         <v>19</v>
       </c>
@@ -5243,22 +4582,22 @@
         <v>8</v>
       </c>
       <c r="C20" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D20" s="3">
         <v>69</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="G20" s="12" t="s">
-        <v>259</v>
+        <v>127</v>
+      </c>
+      <c r="G20" s="11" t="s">
+        <v>254</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="I20" s="6" t="s">
         <v>30</v>
@@ -5266,11 +4605,11 @@
       <c r="J20" s="3">
         <v>0</v>
       </c>
-      <c r="K20" s="10" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="21" spans="1:17" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="K20" s="9" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="3">
         <v>20</v>
       </c>
@@ -5278,22 +4617,22 @@
         <v>9</v>
       </c>
       <c r="C21" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D21" s="3">
         <v>78</v>
       </c>
       <c r="E21" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="G21" s="12" t="s">
-        <v>260</v>
+        <v>320</v>
+      </c>
+      <c r="G21" s="11" t="s">
+        <v>255</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>326</v>
+        <v>321</v>
       </c>
       <c r="I21" t="s">
         <v>32</v>
@@ -5301,11 +4640,11 @@
       <c r="J21" s="3">
         <v>0</v>
       </c>
-      <c r="K21" s="10" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="22" spans="1:17" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="K21" s="9" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="3">
         <v>21</v>
       </c>
@@ -5313,22 +4652,22 @@
         <v>9</v>
       </c>
       <c r="C22" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D22" s="3">
         <v>75</v>
       </c>
       <c r="E22" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>331</v>
-      </c>
-      <c r="G22" s="12" t="s">
-        <v>261</v>
+        <v>326</v>
+      </c>
+      <c r="G22" s="11" t="s">
+        <v>256</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="I22" s="5" t="s">
         <v>34</v>
@@ -5336,11 +4675,11 @@
       <c r="J22" s="3">
         <v>0</v>
       </c>
-      <c r="K22" s="10" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="23" spans="1:17" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="K22" s="9" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="3">
         <v>22</v>
       </c>
@@ -5348,22 +4687,22 @@
         <v>9</v>
       </c>
       <c r="C23" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D23" s="3">
         <v>78</v>
       </c>
       <c r="E23" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>327</v>
-      </c>
-      <c r="G23" s="12" t="s">
-        <v>262</v>
+        <v>322</v>
+      </c>
+      <c r="G23" s="11" t="s">
+        <v>257</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>328</v>
+        <v>323</v>
       </c>
       <c r="I23" s="5" t="s">
         <v>36</v>
@@ -5371,11 +4710,11 @@
       <c r="J23" s="3">
         <v>0</v>
       </c>
-      <c r="K23" s="10" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="24" spans="1:17" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="K23" s="9" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="3">
         <v>23</v>
       </c>
@@ -5383,22 +4722,22 @@
         <v>9</v>
       </c>
       <c r="C24" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D24" s="3">
         <v>1</v>
       </c>
       <c r="E24" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>332</v>
-      </c>
-      <c r="G24" s="12" t="s">
-        <v>263</v>
+        <v>327</v>
+      </c>
+      <c r="G24" s="11" t="s">
+        <v>258</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>333</v>
+        <v>328</v>
       </c>
       <c r="I24" s="5" t="s">
         <v>38</v>
@@ -5406,11 +4745,11 @@
       <c r="J24" s="3">
         <v>0</v>
       </c>
-      <c r="K24" s="10" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="25" spans="1:17" ht="261" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="K24" s="9" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" ht="261" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="3">
         <v>24</v>
       </c>
@@ -5418,22 +4757,22 @@
         <v>11</v>
       </c>
       <c r="C25" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D25" s="3">
         <v>1</v>
       </c>
       <c r="E25" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>329</v>
-      </c>
-      <c r="G25" s="12" t="s">
-        <v>264</v>
+        <v>324</v>
+      </c>
+      <c r="G25" s="11" t="s">
+        <v>259</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>330</v>
+        <v>325</v>
       </c>
       <c r="I25" s="5" t="s">
         <v>39</v>
@@ -5441,11 +4780,11 @@
       <c r="J25" s="3">
         <v>0</v>
       </c>
-      <c r="K25" s="10" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="26" spans="1:17" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="K25" s="9" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="3">
         <v>25</v>
       </c>
@@ -5453,22 +4792,22 @@
         <v>11</v>
       </c>
       <c r="C26" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D26" s="3">
         <v>1</v>
       </c>
       <c r="E26" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>334</v>
-      </c>
-      <c r="G26" s="12" t="s">
-        <v>265</v>
+        <v>329</v>
+      </c>
+      <c r="G26" s="11" t="s">
+        <v>260</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="I26" s="5" t="s">
         <v>41</v>
@@ -5476,11 +4815,11 @@
       <c r="J26" s="3">
         <v>0</v>
       </c>
-      <c r="K26" s="10" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="27" spans="1:17" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="K26" s="9" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="3">
         <v>26</v>
       </c>
@@ -5488,22 +4827,22 @@
         <v>11</v>
       </c>
       <c r="C27" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D27" s="3">
         <v>1</v>
       </c>
       <c r="E27" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>335</v>
-      </c>
-      <c r="G27" s="12" t="s">
-        <v>266</v>
+        <v>330</v>
+      </c>
+      <c r="G27" s="11" t="s">
+        <v>261</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="I27" s="5" t="s">
         <v>46</v>
@@ -5511,11 +4850,11 @@
       <c r="J27" s="3">
         <v>0</v>
       </c>
-      <c r="K27" s="10" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="28" spans="1:17" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="K27" s="9" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="3">
         <v>27</v>
       </c>
@@ -5523,22 +4862,22 @@
         <v>11</v>
       </c>
       <c r="C28" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D28" s="3">
         <v>1</v>
       </c>
       <c r="E28" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>336</v>
-      </c>
-      <c r="G28" s="12" t="s">
-        <v>267</v>
+        <v>331</v>
+      </c>
+      <c r="G28" s="11" t="s">
+        <v>262</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="I28" s="5" t="s">
         <v>48</v>
@@ -5546,371 +4885,401 @@
       <c r="J28" s="3">
         <v>0</v>
       </c>
-      <c r="K28" s="10" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="29" spans="1:17" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A29" s="3">
+      <c r="K28" s="9" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="29" spans="1:17" s="18" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29" s="21">
         <v>28</v>
       </c>
-      <c r="B29" s="3">
+      <c r="B29" s="21">
         <v>0</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C29" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="D29" s="3">
+      <c r="D29" s="21">
         <v>40</v>
       </c>
-      <c r="E29" s="5" t="s">
+      <c r="E29" s="22" t="s">
+        <v>139</v>
+      </c>
+      <c r="F29" s="22" t="s">
+        <v>140</v>
+      </c>
+      <c r="G29" s="19" t="s">
+        <v>191</v>
+      </c>
+      <c r="H29" s="22" t="s">
+        <v>141</v>
+      </c>
+      <c r="I29" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="J29" s="21">
+        <v>0</v>
+      </c>
+      <c r="K29" s="24" t="s">
+        <v>226</v>
+      </c>
+      <c r="L29" s="19" t="s">
+        <v>236</v>
+      </c>
+      <c r="M29" s="18">
+        <v>3</v>
+      </c>
+      <c r="N29" s="18" t="s">
+        <v>340</v>
+      </c>
+      <c r="P29" s="22" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q29" s="25" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17" s="13" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="12">
+        <v>29</v>
+      </c>
+      <c r="B30" s="12">
+        <v>0</v>
+      </c>
+      <c r="C30" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="D30" s="12">
+        <v>26</v>
+      </c>
+      <c r="E30" s="14" t="s">
         <v>143</v>
       </c>
-      <c r="F29" s="5" t="s">
+      <c r="F30" s="15" t="s">
         <v>144</v>
       </c>
-      <c r="G29" s="12" t="s">
+      <c r="G30" s="16" t="s">
+        <v>351</v>
+      </c>
+      <c r="H30" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="I30" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="J30" s="12">
+        <v>0</v>
+      </c>
+      <c r="K30" s="17" t="s">
+        <v>226</v>
+      </c>
+      <c r="L30" s="13" t="s">
+        <v>349</v>
+      </c>
+      <c r="M30" s="13" t="s">
+        <v>350</v>
+      </c>
+      <c r="N30" s="13" t="s">
+        <v>345</v>
+      </c>
+      <c r="P30" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q30" s="14" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="31" spans="1:17" s="18" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="21">
+        <v>30</v>
+      </c>
+      <c r="B31" s="21">
+        <v>0</v>
+      </c>
+      <c r="C31" s="18" t="s">
+        <v>86</v>
+      </c>
+      <c r="D31" s="21">
+        <v>34</v>
+      </c>
+      <c r="E31" s="25" t="s">
+        <v>147</v>
+      </c>
+      <c r="F31" s="22" t="s">
+        <v>148</v>
+      </c>
+      <c r="G31" s="19" t="s">
+        <v>192</v>
+      </c>
+      <c r="H31" s="22" t="s">
+        <v>149</v>
+      </c>
+      <c r="I31" s="18" t="s">
+        <v>54</v>
+      </c>
+      <c r="J31" s="21">
+        <v>0</v>
+      </c>
+      <c r="K31" s="24" t="s">
+        <v>226</v>
+      </c>
+      <c r="L31" s="27" t="s">
+        <v>237</v>
+      </c>
+      <c r="M31" s="27" t="s">
+        <v>238</v>
+      </c>
+      <c r="N31" s="27" t="s">
+        <v>340</v>
+      </c>
+      <c r="P31" s="22" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q31" s="25" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="32" spans="1:17" s="18" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="21">
+        <v>31</v>
+      </c>
+      <c r="B32" s="21">
+        <v>0</v>
+      </c>
+      <c r="C32" s="18" t="s">
+        <v>86</v>
+      </c>
+      <c r="D32" s="21">
+        <v>34</v>
+      </c>
+      <c r="E32" s="18" t="s">
+        <v>151</v>
+      </c>
+      <c r="F32" s="22" t="s">
+        <v>152</v>
+      </c>
+      <c r="G32" s="19" t="s">
+        <v>193</v>
+      </c>
+      <c r="H32" s="22" t="s">
+        <v>153</v>
+      </c>
+      <c r="I32" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="J32" s="21">
+        <v>0</v>
+      </c>
+      <c r="K32" s="24" t="s">
+        <v>226</v>
+      </c>
+      <c r="L32" s="19" t="s">
+        <v>239</v>
+      </c>
+      <c r="M32" s="18" t="s">
+        <v>240</v>
+      </c>
+      <c r="N32" s="18" t="s">
+        <v>340</v>
+      </c>
+      <c r="P32" s="22" t="s">
+        <v>57</v>
+      </c>
+      <c r="Q32" s="25" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="33" spans="1:17" s="13" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="12">
+        <v>32</v>
+      </c>
+      <c r="B33" s="12">
+        <v>0</v>
+      </c>
+      <c r="C33" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="D33" s="12">
+        <v>26</v>
+      </c>
+      <c r="E33" s="13" t="s">
+        <v>155</v>
+      </c>
+      <c r="F33" s="15" t="s">
+        <v>156</v>
+      </c>
+      <c r="G33" s="16" t="s">
+        <v>194</v>
+      </c>
+      <c r="H33" s="15" t="s">
+        <v>157</v>
+      </c>
+      <c r="I33" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="J33" s="12">
+        <v>0</v>
+      </c>
+      <c r="K33" s="17" t="s">
+        <v>226</v>
+      </c>
+      <c r="L33" s="16"/>
+      <c r="N33" s="13" t="s">
+        <v>346</v>
+      </c>
+      <c r="P33" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q33" s="14" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="34" spans="1:17" s="13" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="12">
+        <v>33</v>
+      </c>
+      <c r="B34" s="12">
+        <v>0</v>
+      </c>
+      <c r="C34" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="D34" s="12">
+        <v>28</v>
+      </c>
+      <c r="E34" s="13" t="s">
+        <v>159</v>
+      </c>
+      <c r="F34" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="G34" s="16" t="s">
         <v>195</v>
       </c>
-      <c r="H29" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="I29" t="s">
-        <v>50</v>
-      </c>
-      <c r="J29" s="3">
+      <c r="H34" s="15" t="s">
+        <v>161</v>
+      </c>
+      <c r="I34" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="J34" s="12">
         <v>0</v>
       </c>
-      <c r="K29" s="10" t="s">
-        <v>231</v>
-      </c>
-      <c r="L29" s="2" t="s">
+      <c r="K34" s="17" t="s">
+        <v>226</v>
+      </c>
+      <c r="L34" s="16"/>
+      <c r="N34" s="13" t="s">
+        <v>346</v>
+      </c>
+      <c r="P34" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q34" s="14" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="35" spans="1:17" s="18" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A35" s="21">
+        <v>34</v>
+      </c>
+      <c r="B35" s="21">
+        <v>0</v>
+      </c>
+      <c r="C35" s="18" t="s">
+        <v>86</v>
+      </c>
+      <c r="D35" s="21">
+        <v>26</v>
+      </c>
+      <c r="E35" s="18" t="s">
+        <v>163</v>
+      </c>
+      <c r="F35" s="22" t="s">
+        <v>164</v>
+      </c>
+      <c r="G35" s="19" t="s">
+        <v>196</v>
+      </c>
+      <c r="H35" s="22" t="s">
+        <v>165</v>
+      </c>
+      <c r="I35" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="J35" s="21">
+        <v>0</v>
+      </c>
+      <c r="K35" s="24" t="s">
+        <v>226</v>
+      </c>
+      <c r="L35" s="19" t="s">
         <v>241</v>
       </c>
-      <c r="M29">
-        <v>3</v>
-      </c>
-      <c r="P29" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="Q29" s="6" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="30" spans="1:17" s="14" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A30" s="13">
-        <v>29</v>
-      </c>
-      <c r="B30" s="13">
+      <c r="M35" s="18" t="s">
+        <v>242</v>
+      </c>
+      <c r="N35" s="18" t="s">
+        <v>340</v>
+      </c>
+      <c r="P35" s="22" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q35" s="25" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="36" spans="1:17" s="18" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="21">
+        <v>35</v>
+      </c>
+      <c r="B36" s="21">
         <v>0</v>
       </c>
-      <c r="C30" s="14" t="s">
+      <c r="C36" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="D30" s="13">
-        <v>26</v>
-      </c>
-      <c r="E30" s="15" t="s">
-        <v>147</v>
-      </c>
-      <c r="F30" s="16" t="s">
-        <v>148</v>
-      </c>
-      <c r="G30" s="17" t="s">
-        <v>196</v>
-      </c>
-      <c r="H30" s="16" t="s">
-        <v>149</v>
-      </c>
-      <c r="I30" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="J30" s="13">
+      <c r="D36" s="21">
+        <v>34</v>
+      </c>
+      <c r="E36" s="18" t="s">
+        <v>167</v>
+      </c>
+      <c r="F36" s="22" t="s">
+        <v>168</v>
+      </c>
+      <c r="G36" s="19" t="s">
+        <v>197</v>
+      </c>
+      <c r="H36" s="22" t="s">
+        <v>169</v>
+      </c>
+      <c r="I36" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="J36" s="21">
         <v>0</v>
       </c>
-      <c r="K30" s="18" t="s">
-        <v>231</v>
-      </c>
-      <c r="P30" s="16" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q30" s="15" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="31" spans="1:17" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A31" s="3">
-        <v>30</v>
-      </c>
-      <c r="B31" s="3">
-        <v>0</v>
-      </c>
-      <c r="C31" t="s">
-        <v>86</v>
-      </c>
-      <c r="D31" s="3">
-        <v>34</v>
-      </c>
-      <c r="E31" s="6" t="s">
-        <v>151</v>
-      </c>
-      <c r="F31" s="5" t="s">
-        <v>152</v>
-      </c>
-      <c r="G31" s="12" t="s">
-        <v>197</v>
-      </c>
-      <c r="H31" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="I31" t="s">
-        <v>54</v>
-      </c>
-      <c r="J31" s="3">
-        <v>0</v>
-      </c>
-      <c r="K31" s="10" t="s">
-        <v>231</v>
-      </c>
-      <c r="L31" s="19" t="s">
-        <v>242</v>
-      </c>
-      <c r="M31" s="19" t="s">
+      <c r="K36" s="24" t="s">
+        <v>226</v>
+      </c>
+      <c r="L36" s="19" t="s">
         <v>243</v>
       </c>
-      <c r="P31" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="Q31" s="6" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="32" spans="1:17" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A32" s="3">
-        <v>31</v>
-      </c>
-      <c r="B32" s="3">
-        <v>0</v>
-      </c>
-      <c r="C32" t="s">
-        <v>86</v>
-      </c>
-      <c r="D32" s="3">
-        <v>34</v>
-      </c>
-      <c r="E32" t="s">
-        <v>155</v>
-      </c>
-      <c r="F32" s="5" t="s">
-        <v>156</v>
-      </c>
-      <c r="G32" s="12" t="s">
-        <v>198</v>
-      </c>
-      <c r="H32" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="I32" t="s">
-        <v>56</v>
-      </c>
-      <c r="J32" s="3">
-        <v>0</v>
-      </c>
-      <c r="K32" s="10" t="s">
-        <v>231</v>
-      </c>
-      <c r="L32" s="2" t="s">
-        <v>244</v>
-      </c>
-      <c r="M32" t="s">
-        <v>245</v>
-      </c>
-      <c r="P32" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="Q32" s="6" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="33" spans="1:17" s="14" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A33" s="13">
-        <v>32</v>
-      </c>
-      <c r="B33" s="13">
-        <v>0</v>
-      </c>
-      <c r="C33" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="D33" s="13">
-        <v>26</v>
-      </c>
-      <c r="E33" s="14" t="s">
-        <v>159</v>
-      </c>
-      <c r="F33" s="16" t="s">
-        <v>160</v>
-      </c>
-      <c r="G33" s="17" t="s">
-        <v>199</v>
-      </c>
-      <c r="H33" s="16" t="s">
-        <v>161</v>
-      </c>
-      <c r="I33" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="J33" s="13">
-        <v>0</v>
-      </c>
-      <c r="K33" s="18" t="s">
-        <v>231</v>
-      </c>
-      <c r="L33" s="17"/>
-      <c r="P33" s="16" t="s">
-        <v>59</v>
-      </c>
-      <c r="Q33" s="15" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="34" spans="1:17" s="14" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A34" s="13">
-        <v>33</v>
-      </c>
-      <c r="B34" s="13">
-        <v>0</v>
-      </c>
-      <c r="C34" s="14" t="s">
-        <v>86</v>
-      </c>
-      <c r="D34" s="13">
-        <v>28</v>
-      </c>
-      <c r="E34" s="14" t="s">
-        <v>163</v>
-      </c>
-      <c r="F34" s="16" t="s">
-        <v>164</v>
-      </c>
-      <c r="G34" s="17" t="s">
-        <v>200</v>
-      </c>
-      <c r="H34" s="16" t="s">
-        <v>165</v>
-      </c>
-      <c r="I34" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="J34" s="13">
-        <v>0</v>
-      </c>
-      <c r="K34" s="18" t="s">
-        <v>231</v>
-      </c>
-      <c r="L34" s="17"/>
-      <c r="P34" s="16" t="s">
-        <v>61</v>
-      </c>
-      <c r="Q34" s="15" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="35" spans="1:17" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A35" s="3">
-        <v>34</v>
-      </c>
-      <c r="B35" s="3">
-        <v>0</v>
-      </c>
-      <c r="C35" t="s">
-        <v>86</v>
-      </c>
-      <c r="D35" s="3">
-        <v>26</v>
-      </c>
-      <c r="E35" t="s">
-        <v>167</v>
-      </c>
-      <c r="F35" s="5" t="s">
-        <v>168</v>
-      </c>
-      <c r="G35" s="12" t="s">
-        <v>201</v>
-      </c>
-      <c r="H35" s="5" t="s">
-        <v>169</v>
-      </c>
-      <c r="I35" t="s">
-        <v>62</v>
-      </c>
-      <c r="J35" s="3">
-        <v>0</v>
-      </c>
-      <c r="K35" s="10" t="s">
-        <v>231</v>
-      </c>
-      <c r="L35" s="2" t="s">
-        <v>246</v>
-      </c>
-      <c r="M35" t="s">
-        <v>247</v>
-      </c>
-      <c r="P35" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="Q35" s="6" t="s">
+      <c r="M36" s="18">
+        <v>5</v>
+      </c>
+      <c r="N36" s="18" t="s">
+        <v>340</v>
+      </c>
+      <c r="P36" s="22" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q36" s="25" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="36" spans="1:17" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A36" s="3">
-        <v>35</v>
-      </c>
-      <c r="B36" s="3">
-        <v>0</v>
-      </c>
-      <c r="C36" t="s">
-        <v>86</v>
-      </c>
-      <c r="D36" s="3">
-        <v>34</v>
-      </c>
-      <c r="E36" t="s">
-        <v>171</v>
-      </c>
-      <c r="F36" s="5" t="s">
-        <v>172</v>
-      </c>
-      <c r="G36" s="12" t="s">
-        <v>202</v>
-      </c>
-      <c r="H36" s="5" t="s">
-        <v>173</v>
-      </c>
-      <c r="I36" t="s">
-        <v>64</v>
-      </c>
-      <c r="J36" s="3">
-        <v>0</v>
-      </c>
-      <c r="K36" s="10" t="s">
-        <v>231</v>
-      </c>
-      <c r="L36" s="2" t="s">
-        <v>248</v>
-      </c>
-      <c r="M36">
-        <v>5</v>
-      </c>
-      <c r="P36" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="Q36" s="6" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="37" spans="1:17" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:17" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="3">
         <v>36</v>
       </c>
@@ -5918,22 +5287,22 @@
         <v>0</v>
       </c>
       <c r="C37" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D37" s="3">
         <v>1</v>
       </c>
       <c r="E37" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="F37" s="5" t="s">
-        <v>176</v>
-      </c>
-      <c r="G37" s="12" t="s">
-        <v>268</v>
+        <v>172</v>
+      </c>
+      <c r="G37" s="11" t="s">
+        <v>263</v>
       </c>
       <c r="H37" s="5" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="I37" t="s">
         <v>73</v>
@@ -5941,17 +5310,17 @@
       <c r="J37" s="3">
         <v>0</v>
       </c>
-      <c r="K37" s="10" t="s">
-        <v>228</v>
+      <c r="K37" s="9" t="s">
+        <v>223</v>
       </c>
       <c r="P37" s="5" t="s">
         <v>67</v>
       </c>
       <c r="Q37" s="6" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="38" spans="1:17" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="38" spans="1:17" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="3">
         <v>37</v>
       </c>
@@ -5959,22 +5328,22 @@
         <v>0</v>
       </c>
       <c r="C38" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D38" s="3">
         <v>1</v>
       </c>
       <c r="E38" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="F38" s="7" t="s">
-        <v>180</v>
-      </c>
-      <c r="G38" s="12" t="s">
-        <v>269</v>
+        <v>176</v>
+      </c>
+      <c r="G38" s="11" t="s">
+        <v>264</v>
       </c>
       <c r="H38" s="7" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="I38" t="s">
         <v>74</v>
@@ -5982,17 +5351,17 @@
       <c r="J38" s="3">
         <v>0</v>
       </c>
-      <c r="K38" s="10" t="s">
-        <v>229</v>
+      <c r="K38" s="9" t="s">
+        <v>224</v>
       </c>
       <c r="P38" s="5" t="s">
         <v>75</v>
       </c>
       <c r="Q38" s="6" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="39" spans="1:17" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="39" spans="1:17" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="3">
         <v>38</v>
       </c>
@@ -6000,22 +5369,22 @@
         <v>0</v>
       </c>
       <c r="C39" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="D39" s="3">
         <v>1</v>
       </c>
       <c r="E39" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>184</v>
-      </c>
-      <c r="G39" s="12" t="s">
-        <v>270</v>
+        <v>180</v>
+      </c>
+      <c r="G39" s="11" t="s">
+        <v>265</v>
       </c>
       <c r="H39" s="5" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="I39" s="5" t="s">
         <v>68</v>
@@ -6023,14 +5392,14 @@
       <c r="J39" s="3">
         <v>0</v>
       </c>
-      <c r="K39" s="10" t="s">
-        <v>230</v>
+      <c r="K39" s="9" t="s">
+        <v>225</v>
       </c>
       <c r="P39" s="2" t="s">
         <v>69</v>
       </c>
       <c r="Q39" s="6" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
     </row>
   </sheetData>
@@ -6045,14 +5414,14 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:D63"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="60" customHeight="1" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="60" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="13.54296875" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.26953125" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="129.7265625" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="129.7109375" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6066,7 +5435,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <f t="shared" ref="A2:A27" si="0">ROW()-1</f>
         <v>1</v>
@@ -6081,7 +5450,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <f t="shared" si="0"/>
         <v>2</v>
@@ -6096,7 +5465,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -6111,7 +5480,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -6126,7 +5495,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -6141,7 +5510,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -6156,7 +5525,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -6171,7 +5540,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -6186,7 +5555,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -6198,10 +5567,10 @@
         <v>13</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -6213,10 +5582,10 @@
         <v>14</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -6228,10 +5597,10 @@
         <v>15</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -6243,10 +5612,10 @@
         <v>16</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -6258,10 +5627,10 @@
         <v>17</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -6273,10 +5642,10 @@
         <v>18</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -6288,10 +5657,10 @@
         <v>19</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -6303,10 +5672,10 @@
         <v>20</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -6318,10 +5687,10 @@
         <v>21</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -6333,10 +5702,10 @@
         <v>22</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3">
         <f t="shared" si="0"/>
         <v>19</v>
@@ -6348,10 +5717,10 @@
         <v>23</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3">
         <f t="shared" si="0"/>
         <v>20</v>
@@ -6363,10 +5732,10 @@
         <v>24</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3">
         <f t="shared" si="0"/>
         <v>21</v>
@@ -6378,10 +5747,10 @@
         <v>25</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
         <f t="shared" si="0"/>
         <v>22</v>
@@ -6393,10 +5762,10 @@
         <v>26</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3">
         <f t="shared" si="0"/>
         <v>23</v>
@@ -6408,10 +5777,10 @@
         <v>27</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3">
         <f t="shared" si="0"/>
         <v>24</v>
@@ -6423,10 +5792,10 @@
         <v>28</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="3">
         <f t="shared" si="0"/>
         <v>25</v>
@@ -6438,10 +5807,10 @@
         <v>29</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3">
         <f t="shared" si="0"/>
         <v>26</v>
@@ -6453,10 +5822,10 @@
         <v>30</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="3">
         <v>27</v>
       </c>
@@ -6467,10 +5836,10 @@
         <v>31</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="3">
         <v>28</v>
       </c>
@@ -6481,10 +5850,10 @@
         <v>32</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="3">
         <v>29</v>
       </c>
@@ -6495,10 +5864,10 @@
         <v>33</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="3">
         <v>30</v>
       </c>
@@ -6509,10 +5878,10 @@
         <v>34</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="3">
         <v>31</v>
       </c>
@@ -6523,10 +5892,10 @@
         <v>35</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="3">
         <v>32</v>
       </c>
@@ -6537,10 +5906,10 @@
         <v>36</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3">
         <v>33</v>
       </c>
@@ -6551,10 +5920,10 @@
         <v>37</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="3">
         <v>34</v>
       </c>
@@ -6565,10 +5934,10 @@
         <v>38</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="3">
         <v>35</v>
       </c>
@@ -6579,10 +5948,10 @@
         <v>39</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="3">
         <v>36</v>
       </c>
@@ -6593,10 +5962,10 @@
         <v>40</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="3">
         <v>37</v>
       </c>
@@ -6607,10 +5976,10 @@
         <v>41</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="3">
         <v>38</v>
       </c>
@@ -6621,10 +5990,10 @@
         <v>42</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="3">
         <v>39</v>
       </c>
@@ -6635,10 +6004,10 @@
         <v>43</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="3">
         <v>40</v>
       </c>
@@ -6649,10 +6018,10 @@
         <v>44</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="3">
         <v>41</v>
       </c>
@@ -6663,10 +6032,10 @@
         <v>45</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="3">
         <v>42</v>
       </c>
@@ -6677,10 +6046,10 @@
         <v>46</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3">
         <v>43</v>
       </c>
@@ -6691,10 +6060,10 @@
         <v>47</v>
       </c>
       <c r="D44" s="5" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="3">
         <v>44</v>
       </c>
@@ -6705,10 +6074,10 @@
         <v>48</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="3">
         <v>45</v>
       </c>
@@ -6719,10 +6088,10 @@
         <v>49</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="3">
         <v>46</v>
       </c>
@@ -6736,7 +6105,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="48" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="3">
         <v>47</v>
       </c>
@@ -6750,7 +6119,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="49" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="3">
         <v>48</v>
       </c>
@@ -6764,7 +6133,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="50" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="3">
         <v>49</v>
       </c>
@@ -6778,7 +6147,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="51" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="3">
         <v>50</v>
       </c>
@@ -6792,7 +6161,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="52" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="3">
         <v>51</v>
       </c>
@@ -6806,7 +6175,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="53" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="3">
         <v>52</v>
       </c>
@@ -6820,7 +6189,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="54" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="3">
         <v>53</v>
       </c>
@@ -6834,7 +6203,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="55" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="3">
         <v>54</v>
       </c>
@@ -6845,10 +6214,10 @@
         <v>66</v>
       </c>
       <c r="D55" s="5" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="56" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3">
         <v>55</v>
       </c>
@@ -6859,10 +6228,10 @@
         <v>68</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="57" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="3">
         <v>56</v>
       </c>
@@ -6873,10 +6242,10 @@
         <v>70</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="58" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="3">
         <v>57</v>
       </c>
@@ -6887,10 +6256,10 @@
         <v>71</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="3">
         <v>58</v>
       </c>
@@ -6901,10 +6270,10 @@
         <v>72</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="3">
         <v>59</v>
       </c>
@@ -6915,10 +6284,10 @@
         <v>73</v>
       </c>
       <c r="D60" s="5" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="3">
         <v>60</v>
       </c>
@@ -6929,10 +6298,10 @@
         <v>74</v>
       </c>
       <c r="D61" s="5" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="62" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="3">
         <v>61</v>
       </c>
@@ -6943,10 +6312,10 @@
         <v>68</v>
       </c>
       <c r="D62" s="5" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.35">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="3">
         <v>62</v>
       </c>
@@ -6957,7 +6326,7 @@
         <v>66</v>
       </c>
       <c r="D63" s="5" t="s">
-        <v>312</v>
+        <v>307</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Replace input args with standard args in 3 Java tasks
- concerns 3 tasks
- We can support this again next semester with JURY1.
</commit_message>
<xml_diff>
--- a/files/programming-tasks/programmieraufgaben_JACK_SOSE23_WORKSHOP_WISE2324.xlsx
+++ b/files/programming-tasks/programmieraufgaben_JACK_SOSE23_WORKSHOP_WISE2324.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\hefl\files\programming-tasks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BCC36E3-E6EB-423F-B9F2-20F97FAB44AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB9DC980-F00D-4721-ACE9-B3764C5F1215}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="77040" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Aufgaben" sheetId="1" r:id="rId1"/>
@@ -534,34 +534,6 @@
   </si>
   <si>
     <t>Java Discount</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-Vervollständigen Sie die Methode berechneRabatt() des Java-Programms Discount.java, das als Kommandozeilenargument einen Geldbertrag erhält. Die Methode berechneRabatt() erhält als Parameter einen Euro-Wert.
-Falls der Betrag größer als 1000 EUR ist, soll ein Rabatt von 8 Prozent gewährt werden. In diesem Falle soll die Methode den String "Betrag mit Rabatt: " zurückgeben und anschließend den zu zahlenden Betrag (siehe Beispiele unten). Falls der Betrag kleiner oder gleich 1000 EUR ist, soll nur der Betrag zurückgegeben werden.
-Die eigentliche Ausgabe erfolgt dann im main-Part.
-Bsp. 1:
-java Discount 1234.45
-Betrag mit Rabattt: 1135.69
----------
-Bsp.: 2:
-java Discount 999
-Zu zahlender Betrag: 999.00
-Verwenden Sie exakt das vorgegebene Code-Gerüst</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;&amp;nbsp;&lt;/p&gt;
-&lt;p&gt;Vervollst&amp;auml;ndigen Sie die Methode &lt;i&gt;berechneRabatt() &lt;/i&gt;des Java-Programms &lt;b&gt;&lt;i&gt;Discount.java&lt;/i&gt;&lt;/b&gt;, das als Kommandozeilenargument einen Geldbertrag erh&amp;auml;lt. Die Methode &lt;i&gt;berechneRabatt() &lt;/i&gt;erh&amp;auml;lt als Parameter einen Euro-Wert.&lt;/p&gt;
-&lt;p&gt;Falls der Betrag gr&amp;ouml;&amp;szlig;er als 1000 EUR ist, soll ein Rabatt von 8 Prozent gew&amp;auml;hrt werden. In diesem Falle soll die Methode den String "Betrag mit Rabatt:&amp;nbsp;" zur&amp;uuml;ckgeben und anschlie&amp;szlig;end den zu zahlenden Betrag (siehe Beispiele unten). Falls der Betrag kleiner oder gleich 1000 EUR ist, soll nur der Betrag zur&amp;uuml;ckgegeben werden.&lt;/p&gt;
-&lt;p&gt;Die eigentliche Ausgabe erfolgt dann im main-Part.&lt;/p&gt;
-&lt;p&gt;&lt;b&gt;Bsp. 1: &lt;/b&gt;&lt;/p&gt;
-&lt;p&gt;java Discount 1234.45&lt;/p&gt;
-&lt;p&gt;Betrag mit Rabattt:&amp;nbsp;1135.69&lt;/p&gt;
-&lt;p&gt;---------&lt;/p&gt;
-&lt;p&gt;&lt;b&gt;Bsp.: 2: &lt;/b&gt;&lt;/p&gt;
-&lt;p&gt;java Discount 999&lt;/p&gt;
-&lt;p&gt;Zu zahlender Betrag: 999.00&lt;/p&gt;
-&lt;p&gt;Verwenden Sie exakt das vorgegebene Code-Ger&amp;uuml;st&lt;/p&gt;</t>
   </si>
   <si>
     <t>Java Maximalwert</t>
@@ -2477,23 +2449,6 @@
   </si>
   <si>
     <t>package de.goals.testing; // nicht entfernen
-public class Discount
-{
-	public static String berechneRabatt(double betrag) {
-		//Hier steht Ihre Loesung
-	}
-    public static void main(String[] args)
-    {
-        double rechnungsBetrag = 0.0; //Rechnungsbetrag
-        rechnungsBetrag = Double.parseDouble(args[0]); //Kommandozeilenargument als Gleit-
-                                                       //kommazahl auswerten (Umwandlung in
-                            						   //eine double-Zahl)
-        System.out.println(berechneRabatt(rechnungsBetrag));
-    }    
-}</t>
-  </si>
-  <si>
-    <t>package de.goals.testing; // nicht entfernen
 import java.io.*;
 public class Starter {
 	public int max(int a, int b) {
@@ -2503,20 +2458,6 @@
 		Starter s = new Starter();
 		System.out.println("Ausgabe: "+s.max(12,13)); //Beispielausgabe
 	}
-}</t>
-  </si>
-  <si>
-    <t>package de.goals.testing; // nicht entfernen
-public class ArrayWork {  
-    public double ArrayFunc(double[] w, int func) {
- 	//Ihre Loesung  
-    }  
-    public static void main(String[] args) {    
-      int arg=Integer.parseInt(args[0]);    
-      ArrayWork aw = new ArrayWork();
-      double werte[] = {1.9, 4.6, 99.0, 12.49, 78.99, 0.5, 56.98, 8.90, 119.90, 2.20};
-      System.out.println(aw.ArrayFunc(werte, arg));
-    }
 }</t>
   </si>
   <si>
@@ -2540,22 +2481,6 @@
     <t>package de.goals.testing; // nicht entfernen
 public class BibVerwaltung {
     // Ihre Loesung
-}</t>
-  </si>
-  <si>
-    <t>package de.goals.testing; // nicht entfernen
-import java.io.*;
-import java.lang.Integer;
-public class Rest {	
-    public String checkModulo(int i, int j){
-       // Ihre Lösung
-     }
-    public static void main(String[] args) {		
-        int i = Integer.parseInt(args[0]);		
-        int j = Integer.parseInt(args[1]);
-        Rest r = new Rest();
-        System.out.println(r.checkModulo(i,j));
-    }
 }</t>
   </si>
   <si>
@@ -2863,57 +2788,6 @@
 Erstellen Sie eine Java-Klasse &lt;em&gt;Summenwert&lt;/em&gt; mit einer Methode &lt;em&gt;public double bruchSumme(int n)&lt;/em&gt;.&amp;nbsp;&lt;br /&gt;
 Verwenden Sie eine Schleife!!!&lt;br /&gt;
 &lt;br /&gt;</t>
-  </si>
-  <si>
-    <t>Betrachten Sie den Quellcode der Datei ArrayWork.java.
-Das Programm ArrayWork.java soll verschiedene Operationen auf ein Array mit double-Werten realisieren. Das Array ist bereits vorgegeben (double werte[]) und die entsprechende Operation wird per Programmparameter als int-Wert angegeben (int arg).
-Bei Tutor-Kai kann dieser Wert direkt in das Input-Feld eingegeben werden (args[0]).
-Das Array und der Parameter werden einer Funktion ArrayFunc übergeben in der die folgenden Funktionen implementiert werden sollen:
-- func=1: Gib den kleinsten Wert aus dem Array zurück
-- func=2: Gib den größten Wert aus dem Array zurück
-- func=3: Gib den arithmetischen Mittelwert aus dem Array zurück
-- func=4: Addiere alle Elemente des Arrays, addiere 19 % MwSt. und gib das Ergebnis zurück.
-- Für alle anderen Werte von func soll 0 zurückgegeben werden.
-Implementieren Sie die gewünschte Funktionalität unter der Verwendung von Schleifen und ggf. weiteren Funktionen.
-Verwenden Sie exakt das vorgegebene Code-Gerüst!</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Betrachten Sie den Quellcode der Datei &lt;strong&gt;ArrayWork.java&lt;/strong&gt;.&lt;/p&gt;
-&lt;p&gt;Das Programm ArrayWork.java soll verschiedene Operationen auf ein Array mit&amp;nbsp;double-Werten realisieren. Das Array ist bereits vorgegeben (double werte[]) und die&amp;nbsp;entsprechende Operation wird per Programmparameter als int-Wert angegeben (int arg).&lt;/p&gt;
-&lt;p&gt;Bei Tutor-Kai kann dieser Wert direkt in das Input-Feld eingegeben werden (args[0]).&lt;/p&gt;
-&lt;p&gt;Das Array und der Parameter werden einer Funktion ArrayFunc übergeben in der die&amp;nbsp;folgenden Funktionen implementiert werden sollen:&lt;/p&gt;
-&lt;p&gt;- func=1: Gib den kleinsten Wert aus dem Array zurück&lt;br /&gt;
-- func=2: Gib den gr&amp;ouml;&amp;szlig;ten Wert aus dem Array zurück&lt;br /&gt;
-- func=3: Gib den arithmetischen Mittelwert aus dem Array zurück&lt;br /&gt;
-- func=4: Addiere alle Elemente des Arrays, addiere 19 % MwSt. und gib das Ergebnis&amp;nbsp;zurück.&lt;br /&gt;
-- Für alle anderen Werte von func soll 0 zurückgegeben werden.&lt;/p&gt;
-&lt;p&gt;Implementieren Sie die gewünschte Funktionalit&amp;auml;t unter der Verwendung von Schleifen und&amp;nbsp;ggf. weiteren Funktionen.&lt;/p&gt;
-&lt;p&gt;Verwenden Sie exakt das vorgegebene Code-Gerüst!&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>Erstellen Sie ein Java-Programm mit Hilfe des Programmgerüst aus Rest.java:
-Das Programm erhält als Kommandozeilenparameter zwei int-Werte. Ein Beispielaufruf könnte wie folgt aussehen:
-java Rest 23 44
-Bei Tutor-Kai können diese Werte direkt in die Input-Felder eingegeben werden(args[0] und args[1]). Vervollständigen Sie die Methode checkModulo() die als Parameter die beiden int-Werte erhält, durch die Umsetzung der folgenden Bedingungen:
-Es soll zunächst der Rest der Division von i durch j berechnet werden (modulo). Implementieren Sie nun eine switch-Anweisung, die unterscheidet ob die folgenden Bedingungen erfüllt sind:
-· der Rest ist null. ("Der Rest ist null")
-· der Rest ist eine einstellige Primzahl ("Der Rest ist eine einstellige Primzahl")
-· oder Rest ist ungerade (aber keine einstellige Primzahl) ("Der Rest ist ungerade")
-· keine der Bedingungen trifft zu. ("Keine der Aussagen trifft zu")
-In allen Fällen soll der jeweils angegebene Text (exakt diese Text!) von der Methode checkModulo urückgegeben werden. Nutzen Sie daher insbesondere die break-Anweisung!!! Verwenden Sie exakt das vorgegebene Code-Gerüst!</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Erstellen Sie ein Java-Programm mit Hilfe des Programmgerüst aus Rest.java:&lt;/p&gt;
-&lt;p&gt;Das Programm erh&amp;auml;lt als Kommandozeilenparameter zwei int-Werte. Ein Beispielaufruf&amp;nbsp;k&amp;ouml;nnte wie folgt aussehen:&lt;/p&gt;
-&lt;p&gt;&lt;em&gt;java Rest 23 44&lt;/em&gt;&lt;/p&gt;
-&lt;p&gt;Bei Tutor-Kai können diese Werte direkt in die Input-Felder eingegeben werden(args[0] und args[1]).&lt;/p&gt;
-&lt;p&gt;Vervollst&amp;auml;ndigen Sie die Methode checkModulo() die als Parameter die beiden int-Werte erh&amp;auml;lt,&amp;nbsp;durch die Umsetzung der folgenden Bedingungen:&lt;/p&gt;
-&lt;p&gt;Es soll zun&amp;auml;chst der Rest der Division von i durch j berechnet werden (modulo).&amp;nbsp;Implementieren Sie nun eine switch-Anweisung, die unterscheidet ob die folgenden&amp;nbsp;Bedingungen erfüllt sind:&lt;/p&gt;
-&lt;p&gt;&amp;middot; der Rest ist null. ("Der Rest ist null")&lt;br /&gt;
-&amp;middot; der Rest ist eine einstellige Primzahl ("Der Rest ist eine einstellige&amp;nbsp;Primzahl")&lt;br /&gt;
-&amp;middot; oder Rest ist ungerade (aber keine einstellige Primzahl) ("Der Rest ist ungerade")&lt;br /&gt;
-&amp;middot; keine der Bedingungen trifft zu. ("Keine der Aussagen trifft zu")&lt;/p&gt;
-&lt;p&gt;In allen F&amp;auml;llen soll der jeweils angegebene Text (exakt diese Text!) von der Methode checkModulo ur&amp;uuml;ckgegeben werden. Nutzen Sie daher insbesondere die break-Anweisung!!!&amp;nbsp;Verwenden Sie exakt das vorgegebene Code-Gerüst!&lt;/p&gt;</t>
   </si>
   <si>
     <t>Betrachten Sie das folgende Klassendiagramm:
@@ -3259,10 +3133,6 @@
 Weil&amp;nbsp;1+7+4=12 ist.&amp;nbsp;</t>
   </si>
   <si>
-    <t>style="font-size:12px;"&gt;style="font-family:Calibri, sans-serif"&gt;style="caret-color:#000000"&gt;style="font-style: normal;"&gt;style="font-variant-caps: normal;"&gt;style="font-weight: 400;"&gt;style="letter-spacing: normal;"&gt;style="text-transform: none;"&gt;style="white-space: normal;"&gt;style="word-spacing: 0px;"&gt;style="text-decoration: none;"&gt;Schreiben Sie eine rekursive Funktion fib_index()style="color: rgb(34, 34, 34);"&gt;, die den Index einer Zahl in der Fibonacci-Folge (&lt;a href="https://de.wikipedia.org/wiki/Fibonacci-Folge" style="color:#954f72; text-decoration:underline"&gt;https://de.wikipedia.org/wiki/Fibonacci-Folge&lt;/a&gt;) zur&amp;uuml;ckgibt, wenn die Zahl ein Element dieser Folge ist, und -1 zur&amp;uuml;ckgibt, wenn die Zahl nicht darin enthalten ist.&amp;nbsp;style="font-family:Calibri, sans-serif"&gt;style="caret-color:#000000"&gt;style="color:#000000"&gt;style="font-style:normal"&gt;style="font-variant-caps:normal"&gt;style="font-weight:400"&gt;style="letter-spacing:normal"&gt;style="text-transform:none"&gt;style="white-space:normal"&gt;style="word-spacing:0px"&gt;style="text-decoration:none"&gt;style="color:#222222"&gt;Bsp.:&lt;br /&gt;
-&amp;gt;&amp;gt;&amp;gt; fib_index(13)style="font-family:Calibri, sans-serif"&gt;style="caret-color:#000000"&gt;style="color:#000000"&gt;style="font-style:normal"&gt;style="font-variant-caps:normal"&gt;style="font-weight:400"&gt;style="letter-spacing:normal"&gt;style="text-transform:none"&gt;style="white-space:normal"&gt;style="word-spacing:0px"&gt;&amp;gt;&amp;gt;&amp;gt; 7style="font-family:Calibri, sans-serif"&gt;style="caret-color:#000000"&gt;style="color:#000000"&gt;style="font-style:normal"&gt;style="font-variant-caps:normal"&gt;style="font-weight:400"&gt;style="letter-spacing:normal"&gt;style="text-transform:none"&gt;style="white-space:normal"&gt;style="word-spacing:0px"&gt;In der Fibonacci-Folge ist die 13 an der 7. Position:style="font-family:Calibri, sans-serif"&gt;style="caret-color:#000000"&gt;style="color:#000000"&gt;style="font-style:normal"&gt;style="font-variant-caps:normal"&gt;style="font-weight:400"&gt;style="letter-spacing:normal"&gt;style="text-transform:none"&gt;style="white-space:normal"&gt;style="word-spacing:0px"&gt;0,1,1,2,3,5,8,13,21,...style="font-family:Calibri, sans-serif"&gt;style="caret-color:#000000"&gt;style="color:#000000"&gt;style="font-style:normal"&gt;style="font-variant-caps:normal"&gt;style="font-weight:400"&gt;style="letter-spacing:normal"&gt;style="text-transform:none"&gt;style="white-space:normal"&gt;style="word-spacing:0px"&gt;Tipp:style="font-family:Calibri, sans-serif"&gt;style="caret-color:#000000"&gt;style="color:#000000"&gt;style="font-style:normal"&gt;style="font-variant-caps:normal"&gt;style="font-weight:400"&gt;style="letter-spacing:normal"&gt;style="text-transform:none"&gt;style="white-space:normal"&gt;style="word-spacing:0px"&gt;In den &amp;Uuml;bungen haben Sie ja bereits eine Funktion zur Bestimmung der Fibonacci Folge geschrieben, die sie jetzt wiederverwenden k&amp;ouml;nnen!</t>
-  </si>
-  <si>
     <t>concatenate_functions</t>
   </si>
   <si>
@@ -3300,6 +3170,128 @@
 if __name__ == '__main__':
     unittest.main()
 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  &lt;h1&gt;Fibonacci-Folge Index Finder&lt;/h1&gt;
+        &lt;p&gt;Schreiben Sie eine rekursive Funktion &lt;code&gt;fib_index()&lt;/code&gt;, die den Index einer Zahl in der &lt;a href="https://de.wikipedia.org/wiki/Fibonacci-Folge" target="_blank"&gt;Fibonacci-Folge&lt;/a&gt; zurückgibt, wenn die Zahl ein Element dieser Folge ist, und &lt;code&gt;-1&lt;/code&gt; zurückgibt, wenn die Zahl nicht darin enthalten ist.&lt;/p&gt;
+        &lt;p&gt;&lt;strong&gt;Beispiel:&lt;/strong&gt;&lt;/p&gt;
+        &lt;pre&gt;&lt;code&gt;&amp;gt;&amp;gt;&amp;gt; fib_index(13)
+&amp;gt;&amp;gt;&amp;gt; 7&lt;/code&gt;&lt;/pre&gt;
+        &lt;p&gt;In der Fibonacci-Folge ist die &lt;code&gt;13&lt;/code&gt; an der &lt;code&gt;7.&lt;/code&gt; Position:
+        &lt;code&gt;0, 1, 1, 2, 3, 5, 8, 13, 21, ...&lt;/code&gt;&lt;/p&gt;
+        &lt;p&gt;&lt;strong&gt;Tipp:&lt;/strong&gt; In den Übungen haben Sie ja bereits eine Funktion zur Bestimmung der Fibonacci Folge geschrieben, die sie jetzt wiederverwenden können!&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+Vervollständigen Sie die Methode berechneRabatt() des Java-Programms Discount.java, das als Argument einen Geldbertrag erhält. Die Methode berechneRabatt() erhält als Parameter einen Euro-Wert.
+Falls der Betrag größer als 1000 EUR ist, soll ein Rabatt von 8 Prozent gewährt werden. In diesem Falle soll die Methode den String "Betrag mit Rabatt: " zurückgeben und anschließend den zu zahlenden Betrag (siehe Beispiele unten). Falls der Betrag kleiner oder gleich 1000 EUR ist, soll nur der Betrag zurückgegeben werden.
+Die eigentliche Ausgabe erfolgt dann im main-Part.
+Bsp. 1:
+java Discount 1234.45
+Betrag mit Rabattt: 1135.69
+---------
+Bsp.: 2:
+java Discount 999
+Zu zahlender Betrag: 999.00</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;&amp;nbsp;&lt;/p&gt;
+&lt;p&gt;Vervollst&amp;auml;ndigen Sie die Methode &lt;i&gt;berechneRabatt() &lt;/i&gt;des Java-Programms &lt;b&gt;&lt;i&gt;Discount.java&lt;/i&gt;&lt;/b&gt;, das als Argument einen Geldbertrag erh&amp;auml;lt. Die Methode &lt;i&gt;berechneRabatt() &lt;/i&gt;erh&amp;auml;lt als Parameter einen Euro-Wert.&lt;/p&gt;
+&lt;p&gt;Falls der Betrag gr&amp;ouml;&amp;szlig;er als 1000 EUR ist, soll ein Rabatt von 8 Prozent gew&amp;auml;hrt werden. In diesem Falle soll die Methode den String "Betrag mit Rabatt:&amp;nbsp;" zur&amp;uuml;ckgeben und anschlie&amp;szlig;end den zu zahlenden Betrag (siehe Beispiele unten). Falls der Betrag kleiner oder gleich 1000 EUR ist, soll nur der Betrag zur&amp;uuml;ckgegeben werden.&lt;/p&gt;
+&lt;p&gt;Die eigentliche Ausgabe erfolgt dann im main-Part.&lt;/p&gt;
+&lt;p&gt;&lt;b&gt;Bsp. 1: &lt;/b&gt;&lt;/p&gt;
+&lt;p&gt;java Discount 1234.45&lt;/p&gt;
+&lt;p&gt;Betrag mit Rabattt:&amp;nbsp;1135.69&lt;/p&gt;
+&lt;p&gt;---------&lt;/p&gt;
+&lt;p&gt;&lt;b&gt;Bsp.: 2: &lt;/b&gt;&lt;/p&gt;
+&lt;p&gt;java Discount 999&lt;/p&gt;
+&lt;p&gt;Zu zahlender Betrag: 999.00&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>package de.goals.testing; // nicht entfernen
+public class Discount
+{
+	public static String berechneRabatt(double betrag) {
+		//Hier steht Ihre Loesung
+	}
+    public static void main(String[] args)
+    {
+        double rechnungsBetrag = 100.0; //Rechnungsbetrag    
+        System.out.println(berechneRabatt(rechnungsBetrag));
+    }    
+}</t>
+  </si>
+  <si>
+    <t>package de.goals.testing; // nicht entfernen
+public class ArrayWork {  
+    public double ArrayFunc(double[] w, int func) {
+ 	//Ihre Loesung  
+    }  
+    public static void main(String[] args) {    
+      int arg=1; // Diesen Wert anpassen, um die verschiedenen Funktionen zu testen
+      ArrayWork aw = new ArrayWork();
+      double werte[] = {1.9, 4.6, 99.0, 12.49, 78.99, 0.5, 56.98, 8.90, 119.90, 2.20};
+      System.out.println(aw.ArrayFunc(werte, arg));
+    }
+}</t>
+  </si>
+  <si>
+    <t>Betrachten Sie den Quellcode der Datei ArrayWork.java.
+Das Programm ArrayWork.java soll verschiedene Operationen auf ein Array mit double-Werten realisieren. Das Array ist bereits vorgegeben (double werte[]) und die entsprechende Operation wird per Parameter als int-Wert angegeben (int arg).
+Das Array und der Parameter werden einer Funktion ArrayFunc übergeben in der die folgenden Funktionen implementiert werden sollen:
+- func=1: Gib den kleinsten Wert aus dem Array zurück
+- func=2: Gib den größten Wert aus dem Array zurück
+- func=3: Gib den arithmetischen Mittelwert aus dem Array zurück
+- func=4: Addiere alle Elemente des Arrays, addiere 19 % MwSt. und gib das Ergebnis zurück.
+- Für alle anderen Werte von func soll 0 zurückgegeben werden.
+Implementieren Sie die gewünschte Funktionalität unter der Verwendung von Schleifen und ggf. weiteren Funktionen.
+Verwenden Sie exakt das vorgegebene Code-Gerüst!</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Betrachten Sie den Quellcode der Datei &lt;strong&gt;ArrayWork.java&lt;/strong&gt;.&lt;/p&gt;
+&lt;p&gt;Das Programm ArrayWork.java soll verschiedene Operationen auf ein Array mit&amp;nbsp;double-Werten realisieren. Das Array ist bereits vorgegeben (double werte[]) und die&amp;nbsp;entsprechende Operation wird per Parameter als int-Wert angegeben (int arg).&lt;/p&gt;
+&lt;p&gt;Das Array und der Parameter werden einer Funktion ArrayFunc übergeben in der die&amp;nbsp;folgenden Funktionen implementiert werden sollen:&lt;/p&gt;
+&lt;p&gt;- func=1: Gib den kleinsten Wert aus dem Array zurück&lt;br /&gt;
+- func=2: Gib den gr&amp;ouml;&amp;szlig;ten Wert aus dem Array zurück&lt;br /&gt;
+- func=3: Gib den arithmetischen Mittelwert aus dem Array zurück&lt;br /&gt;
+- func=4: Addiere alle Elemente des Arrays, addiere 19 % MwSt. und gib das Ergebnis&amp;nbsp;zurück.&lt;br /&gt;
+- Für alle anderen Werte von func soll 0 zurückgegeben werden.&lt;/p&gt;
+&lt;p&gt;Implementieren Sie die gewünschte Funktionalit&amp;auml;t unter der Verwendung von Schleifen und&amp;nbsp;ggf. weiteren Funktionen.&lt;/p&gt;
+&lt;p&gt;Verwenden Sie exakt das vorgegebene Code-Gerüst!&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>Vervollständigen Sie die Methode checkModulo() die als Parameter zwei int-Werte erhält, durch die Umsetzung der folgenden Bedingungen:
+Es soll zunächst der Rest der Division von i durch j berechnet werden (modulo). Implementieren Sie nun eine switch-Anweisung, die unterscheidet ob die folgenden Bedingungen erfüllt sind:
+· der Rest ist null. ("Der Rest ist null")
+· der Rest ist eine einstellige Primzahl ("Der Rest ist eine einstellige Primzahl")
+· oder Rest ist ungerade (aber keine einstellige Primzahl) ("Der Rest ist ungerade")
+· keine der Bedingungen trifft zu. ("Keine der Aussagen trifft zu")
+In allen Fällen soll der jeweils angegebene Text (exakt diese Text!) von der Methode checkModulo urückgegeben werden. Nutzen Sie daher insbesondere die break-Anweisung!!! Verwenden Sie exakt das vorgegebene Code-Gerüst!</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Vervollständigen Sie die Methode checkModulo() die als Parameter zwei int-Werte erhält, durch die Umsetzung der folgenden Bedingungen:&lt;/p&gt;
+&lt;p&gt;Es soll zun&amp;auml;chst der Rest der Division von i durch j berechnet werden (modulo).&amp;nbsp;Implementieren Sie nun eine switch-Anweisung, die unterscheidet ob die folgenden&amp;nbsp;Bedingungen erfüllt sind:&lt;/p&gt;
+&lt;p&gt;&amp;middot; der Rest ist null. ("Der Rest ist null")&lt;br /&gt;
+&amp;middot; der Rest ist eine einstellige Primzahl ("Der Rest ist eine einstellige&amp;nbsp;Primzahl")&lt;br /&gt;
+&amp;middot; oder Rest ist ungerade (aber keine einstellige Primzahl) ("Der Rest ist ungerade")&lt;br /&gt;
+&amp;middot; keine der Bedingungen trifft zu. ("Keine der Aussagen trifft zu")&lt;/p&gt;
+&lt;p&gt;In allen F&amp;auml;llen soll der jeweils angegebene Text (exakt diese Text!) von der Methode checkModulo ur&amp;uuml;ckgegeben werden. Nutzen Sie daher insbesondere die break-Anweisung!!!&amp;nbsp;Verwenden Sie exakt das vorgegebene Code-Gerüst!&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>package de.goals.testing; // nicht entfernen
+import java.io.*;
+import java.lang.Integer;
+public class Rest {	
+    public String checkModulo(int i, int j){
+       // Ihre Lösung
+     }
+    public static void main(String[] args) {		
+        int i = 7;		
+        int j = 3;
+        Rest r = new Rest();
+        System.out.println(r.checkModulo(i,j));
+    }
+}</t>
   </si>
 </sst>
 </file>
@@ -3425,7 +3417,7 @@
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -3502,6 +3494,10 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="2" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Gut" xfId="2" builtinId="26"/>
@@ -3860,16 +3856,16 @@
         <v>85</v>
       </c>
       <c r="K1" s="20" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="L1" s="19" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="M1" s="18" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="N1" s="18" t="s">
-        <v>337</v>
+        <v>328</v>
       </c>
     </row>
     <row r="2" spans="1:14" s="18" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -3892,7 +3888,7 @@
         <v>88</v>
       </c>
       <c r="G2" s="23" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="H2" s="22" t="s">
         <v>89</v>
@@ -3904,16 +3900,16 @@
         <v>0</v>
       </c>
       <c r="K2" s="24" t="s">
+        <v>224</v>
+      </c>
+      <c r="L2" s="19" t="s">
+        <v>198</v>
+      </c>
+      <c r="M2" s="18" t="s">
         <v>226</v>
       </c>
-      <c r="L2" s="19" t="s">
-        <v>200</v>
-      </c>
-      <c r="M2" s="18" t="s">
-        <v>228</v>
-      </c>
       <c r="N2" s="18" t="s">
-        <v>338</v>
+        <v>329</v>
       </c>
     </row>
     <row r="3" spans="1:14" s="18" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -3936,7 +3932,7 @@
         <v>91</v>
       </c>
       <c r="G3" s="23" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="H3" s="22" t="s">
         <v>92</v>
@@ -3948,16 +3944,16 @@
         <v>0</v>
       </c>
       <c r="K3" s="24" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="L3" s="19" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="M3" s="18" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="N3" s="18" t="s">
-        <v>339</v>
+        <v>330</v>
       </c>
     </row>
     <row r="4" spans="1:14" s="18" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -3980,10 +3976,10 @@
         <v>94</v>
       </c>
       <c r="G4" s="23" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="H4" s="22" t="s">
-        <v>347</v>
+        <v>338</v>
       </c>
       <c r="I4" s="18" t="s">
         <v>7</v>
@@ -3992,16 +3988,16 @@
         <v>0</v>
       </c>
       <c r="K4" s="24" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="L4" s="19" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="M4" s="18">
         <v>174</v>
       </c>
       <c r="N4" s="18" t="s">
-        <v>340</v>
+        <v>331</v>
       </c>
     </row>
     <row r="5" spans="1:14" s="13" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4024,10 +4020,10 @@
         <v>96</v>
       </c>
       <c r="G5" s="26" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="H5" s="15" t="s">
-        <v>348</v>
+        <v>342</v>
       </c>
       <c r="I5" s="13" t="s">
         <v>8</v>
@@ -4036,16 +4032,16 @@
         <v>0</v>
       </c>
       <c r="K5" s="17" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="L5" s="16" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="M5" s="13">
         <v>47</v>
       </c>
       <c r="N5" s="13" t="s">
-        <v>341</v>
+        <v>332</v>
       </c>
     </row>
     <row r="6" spans="1:14" s="13" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4068,7 +4064,7 @@
         <v>98</v>
       </c>
       <c r="G6" s="26" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="H6" s="15" t="s">
         <v>99</v>
@@ -4080,16 +4076,16 @@
         <v>0</v>
       </c>
       <c r="K6" s="17" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="L6" s="16" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="M6" s="13" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="N6" s="13" t="s">
-        <v>342</v>
+        <v>333</v>
       </c>
     </row>
     <row r="7" spans="1:14" s="18" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4112,7 +4108,7 @@
         <v>101</v>
       </c>
       <c r="G7" s="23" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="H7" s="22" t="s">
         <v>102</v>
@@ -4124,16 +4120,16 @@
         <v>0</v>
       </c>
       <c r="K7" s="24" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="L7" s="19" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="M7" s="18" t="s">
+        <v>325</v>
+      </c>
+      <c r="N7" s="19" t="s">
         <v>334</v>
-      </c>
-      <c r="N7" s="19" t="s">
-        <v>343</v>
       </c>
     </row>
     <row r="8" spans="1:14" s="18" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4156,7 +4152,7 @@
         <v>104</v>
       </c>
       <c r="G8" s="23" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="H8" s="22" t="s">
         <v>105</v>
@@ -4168,16 +4164,16 @@
         <v>0</v>
       </c>
       <c r="K8" s="24" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="L8" s="19" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="M8" s="18" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="N8" s="18" t="s">
-        <v>340</v>
+        <v>331</v>
       </c>
     </row>
     <row r="9" spans="1:14" s="18" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4197,13 +4193,13 @@
         <v>106</v>
       </c>
       <c r="F9" s="22" t="s">
-        <v>335</v>
+        <v>326</v>
       </c>
       <c r="G9" s="23" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="H9" s="22" t="s">
-        <v>336</v>
+        <v>327</v>
       </c>
       <c r="I9" s="18" t="s">
         <v>12</v>
@@ -4212,16 +4208,16 @@
         <v>0</v>
       </c>
       <c r="K9" s="24" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="L9" s="19" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="M9" s="18">
         <v>10</v>
       </c>
       <c r="N9" s="18" t="s">
-        <v>344</v>
+        <v>335</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4244,7 +4240,7 @@
         <v>109</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="H10" s="5" t="s">
         <v>110</v>
@@ -4256,7 +4252,7 @@
         <v>0</v>
       </c>
       <c r="K10" s="9" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
     </row>
     <row r="11" spans="1:14" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4276,13 +4272,13 @@
         <v>111</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>308</v>
+        <v>303</v>
       </c>
       <c r="G11" s="10" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
       <c r="I11" t="s">
         <v>14</v>
@@ -4291,42 +4287,42 @@
         <v>0</v>
       </c>
       <c r="K11" s="9" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="3">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" s="28" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="28">
         <v>11</v>
       </c>
-      <c r="B12" s="3">
+      <c r="B12" s="28">
         <v>6</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="28" t="s">
         <v>107</v>
       </c>
-      <c r="D12" s="3">
+      <c r="D12" s="28">
         <v>63</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" s="28" t="s">
         <v>112</v>
       </c>
-      <c r="F12" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="G12" s="10" t="s">
-        <v>246</v>
-      </c>
-      <c r="H12" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="I12" t="s">
+      <c r="F12" s="28" t="s">
+        <v>343</v>
+      </c>
+      <c r="G12" s="28" t="s">
+        <v>244</v>
+      </c>
+      <c r="H12" s="28" t="s">
+        <v>344</v>
+      </c>
+      <c r="I12" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="J12" s="3">
+      <c r="J12" s="27">
         <v>1</v>
       </c>
-      <c r="K12" s="9" t="s">
-        <v>206</v>
+      <c r="K12" s="28" t="s">
+        <v>204</v>
       </c>
     </row>
     <row r="13" spans="1:14" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4343,16 +4339,16 @@
         <v>63</v>
       </c>
       <c r="E13" t="s">
+        <v>113</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="G13" s="10" t="s">
+        <v>245</v>
+      </c>
+      <c r="H13" s="5" t="s">
         <v>115</v>
-      </c>
-      <c r="F13" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="G13" s="10" t="s">
-        <v>247</v>
-      </c>
-      <c r="H13" s="5" t="s">
-        <v>117</v>
       </c>
       <c r="I13" t="s">
         <v>16</v>
@@ -4361,42 +4357,42 @@
         <v>0</v>
       </c>
       <c r="K13" s="9" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="3">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" s="28" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="28">
         <v>13</v>
       </c>
-      <c r="B14" s="3">
+      <c r="B14" s="28">
         <v>7</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="28" t="s">
         <v>107</v>
       </c>
-      <c r="D14" s="3">
+      <c r="D14" s="28">
         <v>69</v>
       </c>
-      <c r="E14" t="s">
-        <v>118</v>
-      </c>
-      <c r="F14" s="7" t="s">
-        <v>310</v>
-      </c>
-      <c r="G14" s="11" t="s">
-        <v>248</v>
-      </c>
-      <c r="H14" s="7" t="s">
-        <v>311</v>
-      </c>
-      <c r="I14" t="s">
+      <c r="E14" s="28" t="s">
+        <v>116</v>
+      </c>
+      <c r="F14" s="28" t="s">
+        <v>347</v>
+      </c>
+      <c r="G14" s="28" t="s">
+        <v>246</v>
+      </c>
+      <c r="H14" s="28" t="s">
+        <v>348</v>
+      </c>
+      <c r="I14" s="28" t="s">
         <v>17</v>
       </c>
-      <c r="J14" s="3">
+      <c r="J14" s="28">
         <v>1</v>
       </c>
-      <c r="K14" s="9" t="s">
-        <v>208</v>
+      <c r="K14" s="28" t="s">
+        <v>206</v>
       </c>
     </row>
     <row r="15" spans="1:14" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4413,16 +4409,16 @@
         <v>70</v>
       </c>
       <c r="E15" t="s">
+        <v>117</v>
+      </c>
+      <c r="F15" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="G15" s="11" t="s">
+        <v>247</v>
+      </c>
+      <c r="H15" s="7" t="s">
         <v>119</v>
-      </c>
-      <c r="F15" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="G15" s="11" t="s">
-        <v>249</v>
-      </c>
-      <c r="H15" s="7" t="s">
-        <v>121</v>
       </c>
       <c r="I15" t="s">
         <v>18</v>
@@ -4431,42 +4427,42 @@
         <v>0</v>
       </c>
       <c r="K15" s="9" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="3">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" s="28" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="28">
         <v>15</v>
       </c>
-      <c r="B16" s="3">
+      <c r="B16" s="28">
         <v>7</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="28" t="s">
         <v>107</v>
       </c>
-      <c r="D16" s="3">
+      <c r="D16" s="28">
         <v>64</v>
       </c>
-      <c r="E16" t="s">
-        <v>122</v>
-      </c>
-      <c r="F16" s="7" t="s">
-        <v>312</v>
-      </c>
-      <c r="G16" s="11" t="s">
-        <v>250</v>
-      </c>
-      <c r="H16" s="7" t="s">
-        <v>313</v>
-      </c>
-      <c r="I16" t="s">
+      <c r="E16" s="28" t="s">
+        <v>120</v>
+      </c>
+      <c r="F16" s="29" t="s">
+        <v>349</v>
+      </c>
+      <c r="G16" s="28" t="s">
+        <v>248</v>
+      </c>
+      <c r="H16" s="28" t="s">
+        <v>350</v>
+      </c>
+      <c r="I16" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="J16" s="3">
+      <c r="J16" s="28">
         <v>2</v>
       </c>
-      <c r="K16" s="9" t="s">
-        <v>210</v>
+      <c r="K16" s="28" t="s">
+        <v>208</v>
       </c>
     </row>
     <row r="17" spans="1:17" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4483,16 +4479,16 @@
         <v>85</v>
       </c>
       <c r="E17" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>314</v>
+        <v>305</v>
       </c>
       <c r="G17" s="11" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>315</v>
+        <v>306</v>
       </c>
       <c r="I17" s="5" t="s">
         <v>20</v>
@@ -4501,7 +4497,7 @@
         <v>0</v>
       </c>
       <c r="K17" s="9" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
     </row>
     <row r="18" spans="1:17" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4518,16 +4514,16 @@
         <v>84</v>
       </c>
       <c r="E18" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>316</v>
+        <v>307</v>
       </c>
       <c r="G18" s="11" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>317</v>
+        <v>308</v>
       </c>
       <c r="I18" t="s">
         <v>25</v>
@@ -4536,7 +4532,7 @@
         <v>0</v>
       </c>
       <c r="K18" s="9" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
     </row>
     <row r="19" spans="1:17" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4553,16 +4549,16 @@
         <v>93</v>
       </c>
       <c r="E19" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>318</v>
+        <v>309</v>
       </c>
       <c r="G19" s="11" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>319</v>
+        <v>310</v>
       </c>
       <c r="I19" t="s">
         <v>29</v>
@@ -4571,7 +4567,7 @@
         <v>0</v>
       </c>
       <c r="K19" s="9" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
     </row>
     <row r="20" spans="1:17" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4588,16 +4584,16 @@
         <v>69</v>
       </c>
       <c r="E20" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="F20" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="G20" s="11" t="s">
+        <v>252</v>
+      </c>
+      <c r="H20" s="5" t="s">
         <v>126</v>
-      </c>
-      <c r="F20" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="G20" s="11" t="s">
-        <v>254</v>
-      </c>
-      <c r="H20" s="5" t="s">
-        <v>128</v>
       </c>
       <c r="I20" s="6" t="s">
         <v>30</v>
@@ -4606,7 +4602,7 @@
         <v>0</v>
       </c>
       <c r="K20" s="9" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
     </row>
     <row r="21" spans="1:17" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4623,16 +4619,16 @@
         <v>78</v>
       </c>
       <c r="E21" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>320</v>
+        <v>311</v>
       </c>
       <c r="G21" s="11" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>321</v>
+        <v>312</v>
       </c>
       <c r="I21" t="s">
         <v>32</v>
@@ -4641,7 +4637,7 @@
         <v>0</v>
       </c>
       <c r="K21" s="9" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
     </row>
     <row r="22" spans="1:17" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4658,16 +4654,16 @@
         <v>75</v>
       </c>
       <c r="E22" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>326</v>
+        <v>317</v>
       </c>
       <c r="G22" s="11" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>332</v>
+        <v>323</v>
       </c>
       <c r="I22" s="5" t="s">
         <v>34</v>
@@ -4676,7 +4672,7 @@
         <v>0</v>
       </c>
       <c r="K22" s="9" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
     </row>
     <row r="23" spans="1:17" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4693,16 +4689,16 @@
         <v>78</v>
       </c>
       <c r="E23" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>322</v>
+        <v>313</v>
       </c>
       <c r="G23" s="11" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>323</v>
+        <v>314</v>
       </c>
       <c r="I23" s="5" t="s">
         <v>36</v>
@@ -4711,7 +4707,7 @@
         <v>0</v>
       </c>
       <c r="K23" s="9" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
     </row>
     <row r="24" spans="1:17" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4728,16 +4724,16 @@
         <v>1</v>
       </c>
       <c r="E24" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>327</v>
+        <v>318</v>
       </c>
       <c r="G24" s="11" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>328</v>
+        <v>319</v>
       </c>
       <c r="I24" s="5" t="s">
         <v>38</v>
@@ -4746,7 +4742,7 @@
         <v>0</v>
       </c>
       <c r="K24" s="9" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
     </row>
     <row r="25" spans="1:17" ht="261" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4763,16 +4759,16 @@
         <v>1</v>
       </c>
       <c r="E25" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>324</v>
+        <v>315</v>
       </c>
       <c r="G25" s="11" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>325</v>
+        <v>316</v>
       </c>
       <c r="I25" s="5" t="s">
         <v>39</v>
@@ -4781,7 +4777,7 @@
         <v>0</v>
       </c>
       <c r="K25" s="9" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
     </row>
     <row r="26" spans="1:17" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4798,16 +4794,16 @@
         <v>1</v>
       </c>
       <c r="E26" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>329</v>
+        <v>320</v>
       </c>
       <c r="G26" s="11" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>333</v>
+        <v>324</v>
       </c>
       <c r="I26" s="5" t="s">
         <v>41</v>
@@ -4816,7 +4812,7 @@
         <v>0</v>
       </c>
       <c r="K26" s="9" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
     <row r="27" spans="1:17" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4833,16 +4829,16 @@
         <v>1</v>
       </c>
       <c r="E27" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>330</v>
+        <v>321</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I27" s="5" t="s">
         <v>46</v>
@@ -4851,7 +4847,7 @@
         <v>0</v>
       </c>
       <c r="K27" s="9" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="28" spans="1:17" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4868,16 +4864,16 @@
         <v>1</v>
       </c>
       <c r="E28" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>331</v>
+        <v>322</v>
       </c>
       <c r="G28" s="11" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="I28" s="5" t="s">
         <v>48</v>
@@ -4886,7 +4882,7 @@
         <v>0</v>
       </c>
       <c r="K28" s="9" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
     </row>
     <row r="29" spans="1:17" s="18" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4903,16 +4899,16 @@
         <v>40</v>
       </c>
       <c r="E29" s="22" t="s">
+        <v>137</v>
+      </c>
+      <c r="F29" s="22" t="s">
+        <v>138</v>
+      </c>
+      <c r="G29" s="19" t="s">
+        <v>189</v>
+      </c>
+      <c r="H29" s="22" t="s">
         <v>139</v>
-      </c>
-      <c r="F29" s="22" t="s">
-        <v>140</v>
-      </c>
-      <c r="G29" s="19" t="s">
-        <v>191</v>
-      </c>
-      <c r="H29" s="22" t="s">
-        <v>141</v>
       </c>
       <c r="I29" s="18" t="s">
         <v>50</v>
@@ -4921,22 +4917,22 @@
         <v>0</v>
       </c>
       <c r="K29" s="24" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="L29" s="19" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="M29" s="18">
         <v>3</v>
       </c>
       <c r="N29" s="18" t="s">
-        <v>340</v>
+        <v>331</v>
       </c>
       <c r="P29" s="22" t="s">
         <v>51</v>
       </c>
       <c r="Q29" s="25" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="30" spans="1:17" s="13" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4953,16 +4949,16 @@
         <v>26</v>
       </c>
       <c r="E30" s="14" t="s">
+        <v>141</v>
+      </c>
+      <c r="F30" s="15" t="s">
+        <v>142</v>
+      </c>
+      <c r="G30" s="16" t="s">
+        <v>341</v>
+      </c>
+      <c r="H30" s="15" t="s">
         <v>143</v>
-      </c>
-      <c r="F30" s="15" t="s">
-        <v>144</v>
-      </c>
-      <c r="G30" s="16" t="s">
-        <v>351</v>
-      </c>
-      <c r="H30" s="15" t="s">
-        <v>145</v>
       </c>
       <c r="I30" s="13" t="s">
         <v>52</v>
@@ -4971,22 +4967,22 @@
         <v>0</v>
       </c>
       <c r="K30" s="17" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="L30" s="13" t="s">
-        <v>349</v>
+        <v>339</v>
       </c>
       <c r="M30" s="13" t="s">
-        <v>350</v>
+        <v>340</v>
       </c>
       <c r="N30" s="13" t="s">
-        <v>345</v>
+        <v>336</v>
       </c>
       <c r="P30" s="15" t="s">
         <v>53</v>
       </c>
       <c r="Q30" s="14" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="31" spans="1:17" s="18" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -5003,16 +4999,16 @@
         <v>34</v>
       </c>
       <c r="E31" s="25" t="s">
+        <v>145</v>
+      </c>
+      <c r="F31" s="22" t="s">
+        <v>146</v>
+      </c>
+      <c r="G31" s="19" t="s">
+        <v>190</v>
+      </c>
+      <c r="H31" s="22" t="s">
         <v>147</v>
-      </c>
-      <c r="F31" s="22" t="s">
-        <v>148</v>
-      </c>
-      <c r="G31" s="19" t="s">
-        <v>192</v>
-      </c>
-      <c r="H31" s="22" t="s">
-        <v>149</v>
       </c>
       <c r="I31" s="18" t="s">
         <v>54</v>
@@ -5021,22 +5017,22 @@
         <v>0</v>
       </c>
       <c r="K31" s="24" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="L31" s="27" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="M31" s="27" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="N31" s="27" t="s">
-        <v>340</v>
+        <v>331</v>
       </c>
       <c r="P31" s="22" t="s">
         <v>55</v>
       </c>
       <c r="Q31" s="25" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="32" spans="1:17" s="18" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -5053,16 +5049,16 @@
         <v>34</v>
       </c>
       <c r="E32" s="18" t="s">
+        <v>149</v>
+      </c>
+      <c r="F32" s="22" t="s">
+        <v>150</v>
+      </c>
+      <c r="G32" s="19" t="s">
+        <v>191</v>
+      </c>
+      <c r="H32" s="22" t="s">
         <v>151</v>
-      </c>
-      <c r="F32" s="22" t="s">
-        <v>152</v>
-      </c>
-      <c r="G32" s="19" t="s">
-        <v>193</v>
-      </c>
-      <c r="H32" s="22" t="s">
-        <v>153</v>
       </c>
       <c r="I32" s="18" t="s">
         <v>56</v>
@@ -5071,22 +5067,22 @@
         <v>0</v>
       </c>
       <c r="K32" s="24" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="L32" s="19" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="M32" s="18" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="N32" s="18" t="s">
-        <v>340</v>
+        <v>331</v>
       </c>
       <c r="P32" s="22" t="s">
         <v>57</v>
       </c>
       <c r="Q32" s="25" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="33" spans="1:17" s="13" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -5103,16 +5099,16 @@
         <v>26</v>
       </c>
       <c r="E33" s="13" t="s">
+        <v>153</v>
+      </c>
+      <c r="F33" s="15" t="s">
+        <v>154</v>
+      </c>
+      <c r="G33" s="16" t="s">
+        <v>192</v>
+      </c>
+      <c r="H33" s="15" t="s">
         <v>155</v>
-      </c>
-      <c r="F33" s="15" t="s">
-        <v>156</v>
-      </c>
-      <c r="G33" s="16" t="s">
-        <v>194</v>
-      </c>
-      <c r="H33" s="15" t="s">
-        <v>157</v>
       </c>
       <c r="I33" s="13" t="s">
         <v>58</v>
@@ -5121,17 +5117,17 @@
         <v>0</v>
       </c>
       <c r="K33" s="17" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="L33" s="16"/>
       <c r="N33" s="13" t="s">
-        <v>346</v>
+        <v>337</v>
       </c>
       <c r="P33" s="15" t="s">
         <v>59</v>
       </c>
       <c r="Q33" s="14" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="34" spans="1:17" s="13" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -5148,16 +5144,16 @@
         <v>28</v>
       </c>
       <c r="E34" s="13" t="s">
+        <v>157</v>
+      </c>
+      <c r="F34" s="15" t="s">
+        <v>158</v>
+      </c>
+      <c r="G34" s="16" t="s">
+        <v>193</v>
+      </c>
+      <c r="H34" s="15" t="s">
         <v>159</v>
-      </c>
-      <c r="F34" s="15" t="s">
-        <v>160</v>
-      </c>
-      <c r="G34" s="16" t="s">
-        <v>195</v>
-      </c>
-      <c r="H34" s="15" t="s">
-        <v>161</v>
       </c>
       <c r="I34" s="13" t="s">
         <v>60</v>
@@ -5166,17 +5162,17 @@
         <v>0</v>
       </c>
       <c r="K34" s="17" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="L34" s="16"/>
       <c r="N34" s="13" t="s">
-        <v>346</v>
+        <v>337</v>
       </c>
       <c r="P34" s="15" t="s">
         <v>61</v>
       </c>
       <c r="Q34" s="14" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="35" spans="1:17" s="18" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -5193,16 +5189,16 @@
         <v>26</v>
       </c>
       <c r="E35" s="18" t="s">
+        <v>161</v>
+      </c>
+      <c r="F35" s="22" t="s">
+        <v>162</v>
+      </c>
+      <c r="G35" s="19" t="s">
+        <v>194</v>
+      </c>
+      <c r="H35" s="22" t="s">
         <v>163</v>
-      </c>
-      <c r="F35" s="22" t="s">
-        <v>164</v>
-      </c>
-      <c r="G35" s="19" t="s">
-        <v>196</v>
-      </c>
-      <c r="H35" s="22" t="s">
-        <v>165</v>
       </c>
       <c r="I35" s="18" t="s">
         <v>62</v>
@@ -5211,22 +5207,22 @@
         <v>0</v>
       </c>
       <c r="K35" s="24" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="L35" s="19" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="M35" s="18" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="N35" s="18" t="s">
-        <v>340</v>
+        <v>331</v>
       </c>
       <c r="P35" s="22" t="s">
         <v>63</v>
       </c>
       <c r="Q35" s="25" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="36" spans="1:17" s="18" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -5243,16 +5239,16 @@
         <v>34</v>
       </c>
       <c r="E36" s="18" t="s">
+        <v>165</v>
+      </c>
+      <c r="F36" s="22" t="s">
+        <v>166</v>
+      </c>
+      <c r="G36" s="19" t="s">
+        <v>195</v>
+      </c>
+      <c r="H36" s="22" t="s">
         <v>167</v>
-      </c>
-      <c r="F36" s="22" t="s">
-        <v>168</v>
-      </c>
-      <c r="G36" s="19" t="s">
-        <v>197</v>
-      </c>
-      <c r="H36" s="22" t="s">
-        <v>169</v>
       </c>
       <c r="I36" s="18" t="s">
         <v>64</v>
@@ -5261,22 +5257,22 @@
         <v>0</v>
       </c>
       <c r="K36" s="24" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="L36" s="19" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="M36" s="18">
         <v>5</v>
       </c>
       <c r="N36" s="18" t="s">
-        <v>340</v>
+        <v>331</v>
       </c>
       <c r="P36" s="22" t="s">
         <v>65</v>
       </c>
       <c r="Q36" s="25" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
     </row>
     <row r="37" spans="1:17" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -5293,16 +5289,16 @@
         <v>1</v>
       </c>
       <c r="E37" t="s">
+        <v>169</v>
+      </c>
+      <c r="F37" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="G37" s="11" t="s">
+        <v>261</v>
+      </c>
+      <c r="H37" s="5" t="s">
         <v>171</v>
-      </c>
-      <c r="F37" s="5" t="s">
-        <v>172</v>
-      </c>
-      <c r="G37" s="11" t="s">
-        <v>263</v>
-      </c>
-      <c r="H37" s="5" t="s">
-        <v>173</v>
       </c>
       <c r="I37" t="s">
         <v>73</v>
@@ -5311,13 +5307,13 @@
         <v>0</v>
       </c>
       <c r="K37" s="9" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="P37" s="5" t="s">
         <v>67</v>
       </c>
       <c r="Q37" s="6" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="38" spans="1:17" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -5334,16 +5330,16 @@
         <v>1</v>
       </c>
       <c r="E38" t="s">
+        <v>173</v>
+      </c>
+      <c r="F38" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="G38" s="11" t="s">
+        <v>262</v>
+      </c>
+      <c r="H38" s="7" t="s">
         <v>175</v>
-      </c>
-      <c r="F38" s="7" t="s">
-        <v>176</v>
-      </c>
-      <c r="G38" s="11" t="s">
-        <v>264</v>
-      </c>
-      <c r="H38" s="7" t="s">
-        <v>177</v>
       </c>
       <c r="I38" t="s">
         <v>74</v>
@@ -5352,13 +5348,13 @@
         <v>0</v>
       </c>
       <c r="K38" s="9" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="P38" s="5" t="s">
         <v>75</v>
       </c>
       <c r="Q38" s="6" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="39" spans="1:17" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -5375,16 +5371,16 @@
         <v>1</v>
       </c>
       <c r="E39" t="s">
+        <v>177</v>
+      </c>
+      <c r="F39" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="G39" s="11" t="s">
+        <v>263</v>
+      </c>
+      <c r="H39" s="5" t="s">
         <v>179</v>
-      </c>
-      <c r="F39" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="G39" s="11" t="s">
-        <v>265</v>
-      </c>
-      <c r="H39" s="5" t="s">
-        <v>181</v>
       </c>
       <c r="I39" s="5" t="s">
         <v>68</v>
@@ -5393,13 +5389,13 @@
         <v>0</v>
       </c>
       <c r="K39" s="9" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="P39" s="2" t="s">
         <v>69</v>
       </c>
       <c r="Q39" s="6" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
   </sheetData>
@@ -5567,7 +5563,7 @@
         <v>13</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5582,7 +5578,7 @@
         <v>14</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5597,7 +5593,7 @@
         <v>15</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>268</v>
+        <v>345</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5612,7 +5608,7 @@
         <v>16</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5627,7 +5623,7 @@
         <v>17</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>270</v>
+        <v>346</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5642,7 +5638,7 @@
         <v>18</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5657,7 +5653,7 @@
         <v>19</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>273</v>
+        <v>351</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5672,7 +5668,7 @@
         <v>20</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5687,7 +5683,7 @@
         <v>21</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5702,7 +5698,7 @@
         <v>22</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5717,7 +5713,7 @@
         <v>23</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5732,7 +5728,7 @@
         <v>24</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5747,7 +5743,7 @@
         <v>25</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>278</v>
+        <v>273</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5762,7 +5758,7 @@
         <v>26</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>279</v>
+        <v>274</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5777,7 +5773,7 @@
         <v>27</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5792,7 +5788,7 @@
         <v>28</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5807,7 +5803,7 @@
         <v>29</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5822,7 +5818,7 @@
         <v>30</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5836,7 +5832,7 @@
         <v>31</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5850,7 +5846,7 @@
         <v>32</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5864,7 +5860,7 @@
         <v>33</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5878,7 +5874,7 @@
         <v>34</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5892,7 +5888,7 @@
         <v>35</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5906,7 +5902,7 @@
         <v>36</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5920,7 +5916,7 @@
         <v>37</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>290</v>
+        <v>285</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5934,7 +5930,7 @@
         <v>38</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>291</v>
+        <v>286</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5948,7 +5944,7 @@
         <v>39</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5962,7 +5958,7 @@
         <v>40</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>293</v>
+        <v>288</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5976,7 +5972,7 @@
         <v>41</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>294</v>
+        <v>289</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5990,7 +5986,7 @@
         <v>42</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>295</v>
+        <v>290</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6004,7 +6000,7 @@
         <v>43</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>296</v>
+        <v>291</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6018,7 +6014,7 @@
         <v>44</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>297</v>
+        <v>292</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6032,7 +6028,7 @@
         <v>45</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>298</v>
+        <v>293</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6046,7 +6042,7 @@
         <v>46</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>299</v>
+        <v>294</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6060,7 +6056,7 @@
         <v>47</v>
       </c>
       <c r="D44" s="5" t="s">
-        <v>300</v>
+        <v>295</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6074,7 +6070,7 @@
         <v>48</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>301</v>
+        <v>296</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6088,7 +6084,7 @@
         <v>49</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>302</v>
+        <v>297</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6214,7 +6210,7 @@
         <v>66</v>
       </c>
       <c r="D55" s="5" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6228,7 +6224,7 @@
         <v>68</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6242,7 +6238,7 @@
         <v>70</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
     </row>
     <row r="58" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6256,7 +6252,7 @@
         <v>71</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6270,7 +6266,7 @@
         <v>72</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
     </row>
     <row r="60" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6284,7 +6280,7 @@
         <v>73</v>
       </c>
       <c r="D60" s="5" t="s">
-        <v>305</v>
+        <v>300</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6298,7 +6294,7 @@
         <v>74</v>
       </c>
       <c r="D61" s="5" t="s">
-        <v>306</v>
+        <v>301</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6312,7 +6308,7 @@
         <v>68</v>
       </c>
       <c r="D62" s="5" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
     </row>
     <row r="63" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6326,7 +6322,7 @@
         <v>66</v>
       </c>
       <c r="D63" s="5" t="s">
-        <v>307</v>
+        <v>302</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Matched missing Codingquestions to concepts
</commit_message>
<xml_diff>
--- a/files/programming-tasks/programmieraufgaben_JACK_SOSE23_WORKSHOP_WISE2324.xlsx
+++ b/files/programming-tasks/programmieraufgaben_JACK_SOSE23_WORKSHOP_WISE2324.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\hefl\files\programming-tasks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB9DC980-F00D-4721-ACE9-B3764C5F1215}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F81C6378-78D8-401E-AD6F-7524A226DDFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="90" windowWidth="25860" windowHeight="20805" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Aufgaben" sheetId="1" r:id="rId1"/>
@@ -773,9 +773,6 @@
     </r>
   </si>
   <si>
-    <t>1 Python Matrix</t>
-  </si>
-  <si>
     <t>Schreiben sie ein Funktion, welche eine n x n Matrix A  als Liste von Listen erstellt, wobei der (i,j)-te Eintrag, A_{i,j}, gleich i+j ist. Verwenden sie hierfür zwei verschachtelte for-Schleifen.</t>
   </si>
   <si>
@@ -802,9 +799,6 @@
     return matrix</t>
   </si>
   <si>
-    <t>2 Python Funktionen</t>
-  </si>
-  <si>
     <t>&lt;p&gt;Schreiben Sie eine Funktion "concatenate_functions", die als Eingabeargument zwei Funktionen "f1" und "f2" bekommt und als Rückgabe eine Funktion liefert, die f1(f2(x)) auswertet. Testen Sie Ihr Programm mit f1(x) = sin(x) und f2(x) = 2*pi*x. 
 &lt;/p&gt;
 &lt;br&gt;
@@ -827,9 +821,6 @@
     return concat</t>
   </si>
   <si>
-    <t>3 Python Potenz</t>
-  </si>
-  <si>
     <t>Schreiben Sie eine Funktion namens potenz, die die Potenz von x hoch a rekursiv berechnet.</t>
   </si>
   <si>
@@ -845,9 +836,6 @@
         return x*potenz(x, a-1)</t>
   </si>
   <si>
-    <t>4 Python Drehe String</t>
-  </si>
-  <si>
     <t>Schreiben Sie eine Funktion namens drehe_string, die einen String rekursiv umdreht.</t>
   </si>
   <si>
@@ -861,9 +849,6 @@
         return ''
     else:
         return drehe_string(s[1:]) + s[0]</t>
-  </si>
-  <si>
-    <t>5 Python Steuer</t>
   </si>
   <si>
     <t>Schreiben sie eine Funktion "mehrwertsteuer(betrag)", die 19% des Betrages
@@ -887,9 +872,6 @@
     return steuer_mit_freibetrag</t>
   </si>
   <si>
-    <t>6 Python Filter Liste</t>
-  </si>
-  <si>
     <t>Schreiben sie eine Funktion höherer Ordnung "filter_liste",
     die eine Funktion mit boolschem Rückgabewert und eine Liste als Eingabe entgegennimmt.
     Sie soll auf jedem Element der Liste die Funktion aufrufen und alle diejenigen Elemente
@@ -909,9 +891,6 @@
             liste.remove(element)</t>
   </si>
   <si>
-    <t>7 Python Reduziere Liste</t>
-  </si>
-  <si>
     <t>Schreiben sie eine Funktion höherer Ordnung "reduziere_liste", die eine Funktion
     mit zwei Eingabeargumenten sowie eine Liste entgegennimmt.
     Hat die Liste nur ein Element, soll dieses Element zurückgegeben werden.
@@ -930,9 +909,6 @@
     for i in range (1, len(liste)):
         result = funktion(result, liste[i])
     return result</t>
-  </si>
-  <si>
-    <t>8 Python Fibonacci</t>
   </si>
   <si>
     <t>Schreiben Sie eine Funktion namens fib, die die n-te Zahl der Fibonacci-Folge rekursiv berechnet.</t>
@@ -951,9 +927,6 @@
     else:
         return fib(n-1)+fib(n-2)
 </t>
-  </si>
-  <si>
-    <t>9 Java Wettrennen</t>
   </si>
   <si>
     <t>Für die Simulation eines Wettrennens sollen verschiedene Fahrzeugarten objektorientiert modelliert werden. Da alle Fahrzeugtypen gemeinsame Eigenschaften haben, definieren wir uns zunächst eine Basisklasse Fahrzeug, die als Oberklasse für die anderen Klassen dienen soll. Ein Fahrzeug hat folgende allgemeinen Merkmale:
@@ -1052,9 +1025,6 @@
 }</t>
   </si>
   <si>
-    <t>10 Java BubbleSort</t>
-  </si>
-  <si>
     <t>In dieser Aufgabe sollst du den Bubblesort-Algorithmus in Java implementieren. Dieser Algorithmus ist ein einfaches Verfahren zum Sortieren einer Liste von Elementen (z.B. Zahlen). Bubblesort ist ein Sortieralgorithmus, der durch wiederholtes Durchlaufen der zu sortierenden Liste arbeitet. Bei jedem Durchlauf werden benachbarte Elemente miteinander verglichen und gegebenenfalls vertauscht. Das Besondere am Bubblesort ist, dass mit jedem Durchgang das größte Element der noch zu sortierenden Elemente an das Ende der Liste "aufsteigt".</t>
   </si>
   <si>
@@ -1095,50 +1065,6 @@
         }
     }
 }</t>
-  </si>
-  <si>
-    <t>11 Java UML to Java</t>
-  </si>
-  <si>
-    <r>
-      <t>Schreiben Sie den Java Code für beide Klassen des UML-Diagramms</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, in eine Datei, erst Fahrzeug, dann Auto.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Klasse Fahrzeug:
-    Attribute:
-        marke: privates Attribut vom Typ String
-        modell: privates Attribut vom Typ String
-    Konstruktor:
-        Öffentlicher Konstruktor Fahrzeug, der die Parameter marke und modell vom Typ String nimmt.
-    Methoden:
-        Öffentliche Methode getMarke(): gibt einen String zurück.
-        Öffentliche Methode getModell(): gibt einen String zurück.
-Klasse Auto:
-    Attribute:
-        jahr: privates Attribut vom Typ int
-    Konstruktor:
-        Öffentlicher Konstruktor Auto, der die Parameter marke, modell vom Typ String und jahr vom Typ int nimmt.
-    Methoden:
-        Öffentliche Methode getJahr(): gibt einen int zurück.
-Die Klasse Auto erbt die Attribute und Methoden von der Klasse Fahrzeug. Darauf weist der Vererbungspfeil im Diagramm hin.</t>
-    </r>
   </si>
   <si>
     <r>
@@ -3292,6 +3218,70 @@
         System.out.println(r.checkModulo(i,j));
     }
 }</t>
+  </si>
+  <si>
+    <r>
+      <t>Schreiben Sie den Java Code für beide Klassen des UML-Diagramms</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, in eine Datei, erst Fahrzeug, dann Auto. Klasse Fahrzeug:
+    Attribute:
+        marke: privates Attribut vom Typ String
+        modell: privates Attribut vom Typ String
+    Konstruktor:
+        Öffentlicher Konstruktor Fahrzeug, der die Parameter marke und modell vom Typ String nimmt.
+    Methoden:
+        Öffentliche Methode getMarke(): gibt einen String zurück.
+        Öffentliche Methode getModell(): gibt einen String zurück.
+Klasse Auto:
+    Attribute:
+        jahr: privates Attribut vom Typ int
+    Konstruktor:
+        Öffentlicher Konstruktor Auto, der die Parameter marke, modell vom Typ String und jahr vom Typ int nimmt.
+    Methoden:
+        Öffentliche Methode getJahr(): gibt einen int zurück.
+Die Klasse Auto erbt die Attribute und Methoden von der Klasse Fahrzeug. Darauf weist der Vererbungspfeil im Diagramm hin.</t>
+    </r>
+  </si>
+  <si>
+    <t>Java BubbleSort</t>
+  </si>
+  <si>
+    <t>Java UML to Java</t>
+  </si>
+  <si>
+    <t>Java Wettrennen</t>
+  </si>
+  <si>
+    <t>Python Fibonacci</t>
+  </si>
+  <si>
+    <t>Python Matrix</t>
+  </si>
+  <si>
+    <t>Python Funktionen</t>
+  </si>
+  <si>
+    <t>Python Potenz</t>
+  </si>
+  <si>
+    <t>Python Drehe String</t>
+  </si>
+  <si>
+    <t>Python Steuer</t>
+  </si>
+  <si>
+    <t>Python Filter Liste</t>
+  </si>
+  <si>
+    <t>Python Reduziere Liste</t>
   </si>
 </sst>
 </file>
@@ -3856,16 +3846,16 @@
         <v>85</v>
       </c>
       <c r="K1" s="20" t="s">
-        <v>225</v>
+        <v>213</v>
       </c>
       <c r="L1" s="19" t="s">
-        <v>196</v>
+        <v>184</v>
       </c>
       <c r="M1" s="18" t="s">
-        <v>197</v>
+        <v>185</v>
       </c>
       <c r="N1" s="18" t="s">
-        <v>328</v>
+        <v>316</v>
       </c>
     </row>
     <row r="2" spans="1:14" s="18" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -3888,7 +3878,7 @@
         <v>88</v>
       </c>
       <c r="G2" s="23" t="s">
-        <v>181</v>
+        <v>169</v>
       </c>
       <c r="H2" s="22" t="s">
         <v>89</v>
@@ -3900,16 +3890,16 @@
         <v>0</v>
       </c>
       <c r="K2" s="24" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
       <c r="L2" s="19" t="s">
-        <v>198</v>
+        <v>186</v>
       </c>
       <c r="M2" s="18" t="s">
-        <v>226</v>
+        <v>214</v>
       </c>
       <c r="N2" s="18" t="s">
-        <v>329</v>
+        <v>317</v>
       </c>
     </row>
     <row r="3" spans="1:14" s="18" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -3932,7 +3922,7 @@
         <v>91</v>
       </c>
       <c r="G3" s="23" t="s">
-        <v>182</v>
+        <v>170</v>
       </c>
       <c r="H3" s="22" t="s">
         <v>92</v>
@@ -3944,16 +3934,16 @@
         <v>0</v>
       </c>
       <c r="K3" s="24" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
       <c r="L3" s="19" t="s">
-        <v>199</v>
+        <v>187</v>
       </c>
       <c r="M3" s="18" t="s">
-        <v>200</v>
+        <v>188</v>
       </c>
       <c r="N3" s="18" t="s">
-        <v>330</v>
+        <v>318</v>
       </c>
     </row>
     <row r="4" spans="1:14" s="18" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -3976,10 +3966,10 @@
         <v>94</v>
       </c>
       <c r="G4" s="23" t="s">
-        <v>183</v>
+        <v>171</v>
       </c>
       <c r="H4" s="22" t="s">
-        <v>338</v>
+        <v>326</v>
       </c>
       <c r="I4" s="18" t="s">
         <v>7</v>
@@ -3988,16 +3978,16 @@
         <v>0</v>
       </c>
       <c r="K4" s="24" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
       <c r="L4" s="19" t="s">
-        <v>201</v>
+        <v>189</v>
       </c>
       <c r="M4" s="18">
         <v>174</v>
       </c>
       <c r="N4" s="18" t="s">
-        <v>331</v>
+        <v>319</v>
       </c>
     </row>
     <row r="5" spans="1:14" s="13" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4020,10 +4010,10 @@
         <v>96</v>
       </c>
       <c r="G5" s="26" t="s">
-        <v>184</v>
+        <v>172</v>
       </c>
       <c r="H5" s="15" t="s">
-        <v>342</v>
+        <v>330</v>
       </c>
       <c r="I5" s="13" t="s">
         <v>8</v>
@@ -4032,16 +4022,16 @@
         <v>0</v>
       </c>
       <c r="K5" s="17" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
       <c r="L5" s="16" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="M5" s="13">
         <v>47</v>
       </c>
       <c r="N5" s="13" t="s">
-        <v>332</v>
+        <v>320</v>
       </c>
     </row>
     <row r="6" spans="1:14" s="13" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4055,7 +4045,7 @@
         <v>86</v>
       </c>
       <c r="D6" s="12">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="E6" s="13" t="s">
         <v>97</v>
@@ -4064,7 +4054,7 @@
         <v>98</v>
       </c>
       <c r="G6" s="26" t="s">
-        <v>185</v>
+        <v>173</v>
       </c>
       <c r="H6" s="15" t="s">
         <v>99</v>
@@ -4076,16 +4066,16 @@
         <v>0</v>
       </c>
       <c r="K6" s="17" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
       <c r="L6" s="16" t="s">
-        <v>228</v>
+        <v>216</v>
       </c>
       <c r="M6" s="13" t="s">
-        <v>229</v>
+        <v>217</v>
       </c>
       <c r="N6" s="13" t="s">
-        <v>333</v>
+        <v>321</v>
       </c>
     </row>
     <row r="7" spans="1:14" s="18" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4108,7 +4098,7 @@
         <v>101</v>
       </c>
       <c r="G7" s="23" t="s">
-        <v>186</v>
+        <v>174</v>
       </c>
       <c r="H7" s="22" t="s">
         <v>102</v>
@@ -4120,16 +4110,16 @@
         <v>0</v>
       </c>
       <c r="K7" s="24" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
       <c r="L7" s="19" t="s">
-        <v>230</v>
+        <v>218</v>
       </c>
       <c r="M7" s="18" t="s">
-        <v>325</v>
+        <v>313</v>
       </c>
       <c r="N7" s="19" t="s">
-        <v>334</v>
+        <v>322</v>
       </c>
     </row>
     <row r="8" spans="1:14" s="18" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4152,7 +4142,7 @@
         <v>104</v>
       </c>
       <c r="G8" s="23" t="s">
-        <v>187</v>
+        <v>175</v>
       </c>
       <c r="H8" s="22" t="s">
         <v>105</v>
@@ -4164,16 +4154,16 @@
         <v>0</v>
       </c>
       <c r="K8" s="24" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
       <c r="L8" s="19" t="s">
-        <v>231</v>
+        <v>219</v>
       </c>
       <c r="M8" s="18" t="s">
-        <v>232</v>
+        <v>220</v>
       </c>
       <c r="N8" s="18" t="s">
-        <v>331</v>
+        <v>319</v>
       </c>
     </row>
     <row r="9" spans="1:14" s="18" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4193,13 +4183,13 @@
         <v>106</v>
       </c>
       <c r="F9" s="22" t="s">
-        <v>326</v>
+        <v>314</v>
       </c>
       <c r="G9" s="23" t="s">
-        <v>188</v>
+        <v>176</v>
       </c>
       <c r="H9" s="22" t="s">
-        <v>327</v>
+        <v>315</v>
       </c>
       <c r="I9" s="18" t="s">
         <v>12</v>
@@ -4208,16 +4198,16 @@
         <v>0</v>
       </c>
       <c r="K9" s="24" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
       <c r="L9" s="19" t="s">
-        <v>233</v>
+        <v>221</v>
       </c>
       <c r="M9" s="18">
         <v>10</v>
       </c>
       <c r="N9" s="18" t="s">
-        <v>335</v>
+        <v>323</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4240,7 +4230,7 @@
         <v>109</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>242</v>
+        <v>230</v>
       </c>
       <c r="H10" s="5" t="s">
         <v>110</v>
@@ -4252,7 +4242,7 @@
         <v>0</v>
       </c>
       <c r="K10" s="9" t="s">
-        <v>202</v>
+        <v>190</v>
       </c>
     </row>
     <row r="11" spans="1:14" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4272,13 +4262,13 @@
         <v>111</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>303</v>
+        <v>291</v>
       </c>
       <c r="G11" s="10" t="s">
-        <v>243</v>
+        <v>231</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>304</v>
+        <v>292</v>
       </c>
       <c r="I11" t="s">
         <v>14</v>
@@ -4287,7 +4277,7 @@
         <v>0</v>
       </c>
       <c r="K11" s="9" t="s">
-        <v>203</v>
+        <v>191</v>
       </c>
     </row>
     <row r="12" spans="1:14" s="28" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4307,13 +4297,13 @@
         <v>112</v>
       </c>
       <c r="F12" s="28" t="s">
-        <v>343</v>
+        <v>331</v>
       </c>
       <c r="G12" s="28" t="s">
-        <v>244</v>
+        <v>232</v>
       </c>
       <c r="H12" s="28" t="s">
-        <v>344</v>
+        <v>332</v>
       </c>
       <c r="I12" s="28" t="s">
         <v>15</v>
@@ -4322,7 +4312,7 @@
         <v>1</v>
       </c>
       <c r="K12" s="28" t="s">
-        <v>204</v>
+        <v>192</v>
       </c>
     </row>
     <row r="13" spans="1:14" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4345,7 +4335,7 @@
         <v>114</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>245</v>
+        <v>233</v>
       </c>
       <c r="H13" s="5" t="s">
         <v>115</v>
@@ -4357,7 +4347,7 @@
         <v>0</v>
       </c>
       <c r="K13" s="9" t="s">
-        <v>205</v>
+        <v>193</v>
       </c>
     </row>
     <row r="14" spans="1:14" s="28" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4377,13 +4367,13 @@
         <v>116</v>
       </c>
       <c r="F14" s="28" t="s">
-        <v>347</v>
+        <v>335</v>
       </c>
       <c r="G14" s="28" t="s">
-        <v>246</v>
+        <v>234</v>
       </c>
       <c r="H14" s="28" t="s">
-        <v>348</v>
+        <v>336</v>
       </c>
       <c r="I14" s="28" t="s">
         <v>17</v>
@@ -4392,7 +4382,7 @@
         <v>1</v>
       </c>
       <c r="K14" s="28" t="s">
-        <v>206</v>
+        <v>194</v>
       </c>
     </row>
     <row r="15" spans="1:14" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4415,7 +4405,7 @@
         <v>118</v>
       </c>
       <c r="G15" s="11" t="s">
-        <v>247</v>
+        <v>235</v>
       </c>
       <c r="H15" s="7" t="s">
         <v>119</v>
@@ -4427,7 +4417,7 @@
         <v>0</v>
       </c>
       <c r="K15" s="9" t="s">
-        <v>207</v>
+        <v>195</v>
       </c>
     </row>
     <row r="16" spans="1:14" s="28" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4447,13 +4437,13 @@
         <v>120</v>
       </c>
       <c r="F16" s="29" t="s">
-        <v>349</v>
+        <v>337</v>
       </c>
       <c r="G16" s="28" t="s">
-        <v>248</v>
+        <v>236</v>
       </c>
       <c r="H16" s="28" t="s">
-        <v>350</v>
+        <v>338</v>
       </c>
       <c r="I16" s="28" t="s">
         <v>19</v>
@@ -4462,7 +4452,7 @@
         <v>2</v>
       </c>
       <c r="K16" s="28" t="s">
-        <v>208</v>
+        <v>196</v>
       </c>
     </row>
     <row r="17" spans="1:17" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4482,13 +4472,13 @@
         <v>121</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>305</v>
+        <v>293</v>
       </c>
       <c r="G17" s="11" t="s">
-        <v>249</v>
+        <v>237</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>306</v>
+        <v>294</v>
       </c>
       <c r="I17" s="5" t="s">
         <v>20</v>
@@ -4497,7 +4487,7 @@
         <v>0</v>
       </c>
       <c r="K17" s="9" t="s">
-        <v>209</v>
+        <v>197</v>
       </c>
     </row>
     <row r="18" spans="1:17" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4517,13 +4507,13 @@
         <v>122</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>307</v>
+        <v>295</v>
       </c>
       <c r="G18" s="11" t="s">
-        <v>250</v>
+        <v>238</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>308</v>
+        <v>296</v>
       </c>
       <c r="I18" t="s">
         <v>25</v>
@@ -4532,7 +4522,7 @@
         <v>0</v>
       </c>
       <c r="K18" s="9" t="s">
-        <v>210</v>
+        <v>198</v>
       </c>
     </row>
     <row r="19" spans="1:17" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4552,13 +4542,13 @@
         <v>123</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>309</v>
+        <v>297</v>
       </c>
       <c r="G19" s="11" t="s">
-        <v>251</v>
+        <v>239</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>310</v>
+        <v>298</v>
       </c>
       <c r="I19" t="s">
         <v>29</v>
@@ -4567,7 +4557,7 @@
         <v>0</v>
       </c>
       <c r="K19" s="9" t="s">
-        <v>211</v>
+        <v>199</v>
       </c>
     </row>
     <row r="20" spans="1:17" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4590,7 +4580,7 @@
         <v>125</v>
       </c>
       <c r="G20" s="11" t="s">
-        <v>252</v>
+        <v>240</v>
       </c>
       <c r="H20" s="5" t="s">
         <v>126</v>
@@ -4602,7 +4592,7 @@
         <v>0</v>
       </c>
       <c r="K20" s="9" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
     </row>
     <row r="21" spans="1:17" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4622,13 +4612,13 @@
         <v>127</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>311</v>
+        <v>299</v>
       </c>
       <c r="G21" s="11" t="s">
-        <v>253</v>
+        <v>241</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>312</v>
+        <v>300</v>
       </c>
       <c r="I21" t="s">
         <v>32</v>
@@ -4637,7 +4627,7 @@
         <v>0</v>
       </c>
       <c r="K21" s="9" t="s">
-        <v>213</v>
+        <v>201</v>
       </c>
     </row>
     <row r="22" spans="1:17" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4657,13 +4647,13 @@
         <v>128</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>317</v>
+        <v>305</v>
       </c>
       <c r="G22" s="11" t="s">
-        <v>254</v>
+        <v>242</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>323</v>
+        <v>311</v>
       </c>
       <c r="I22" s="5" t="s">
         <v>34</v>
@@ -4672,7 +4662,7 @@
         <v>0</v>
       </c>
       <c r="K22" s="9" t="s">
-        <v>214</v>
+        <v>202</v>
       </c>
     </row>
     <row r="23" spans="1:17" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4692,13 +4682,13 @@
         <v>129</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>313</v>
+        <v>301</v>
       </c>
       <c r="G23" s="11" t="s">
-        <v>255</v>
+        <v>243</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>314</v>
+        <v>302</v>
       </c>
       <c r="I23" s="5" t="s">
         <v>36</v>
@@ -4707,7 +4697,7 @@
         <v>0</v>
       </c>
       <c r="K23" s="9" t="s">
-        <v>215</v>
+        <v>203</v>
       </c>
     </row>
     <row r="24" spans="1:17" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4721,19 +4711,19 @@
         <v>107</v>
       </c>
       <c r="D24" s="3">
-        <v>1</v>
+        <v>75</v>
       </c>
       <c r="E24" t="s">
         <v>130</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>318</v>
+        <v>306</v>
       </c>
       <c r="G24" s="11" t="s">
-        <v>256</v>
+        <v>244</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>319</v>
+        <v>307</v>
       </c>
       <c r="I24" s="5" t="s">
         <v>38</v>
@@ -4742,7 +4732,7 @@
         <v>0</v>
       </c>
       <c r="K24" s="9" t="s">
-        <v>216</v>
+        <v>204</v>
       </c>
     </row>
     <row r="25" spans="1:17" ht="261" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4756,19 +4746,19 @@
         <v>107</v>
       </c>
       <c r="D25" s="3">
-        <v>1</v>
+        <v>85</v>
       </c>
       <c r="E25" t="s">
         <v>131</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>315</v>
+        <v>303</v>
       </c>
       <c r="G25" s="11" t="s">
-        <v>257</v>
+        <v>245</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>316</v>
+        <v>304</v>
       </c>
       <c r="I25" s="5" t="s">
         <v>39</v>
@@ -4777,7 +4767,7 @@
         <v>0</v>
       </c>
       <c r="K25" s="9" t="s">
-        <v>217</v>
+        <v>205</v>
       </c>
     </row>
     <row r="26" spans="1:17" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4791,19 +4781,19 @@
         <v>107</v>
       </c>
       <c r="D26" s="3">
-        <v>1</v>
+        <v>78</v>
       </c>
       <c r="E26" t="s">
         <v>132</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>320</v>
+        <v>308</v>
       </c>
       <c r="G26" s="11" t="s">
-        <v>258</v>
+        <v>246</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>324</v>
+        <v>312</v>
       </c>
       <c r="I26" s="5" t="s">
         <v>41</v>
@@ -4812,7 +4802,7 @@
         <v>0</v>
       </c>
       <c r="K26" s="9" t="s">
-        <v>218</v>
+        <v>206</v>
       </c>
     </row>
     <row r="27" spans="1:17" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4826,16 +4816,16 @@
         <v>107</v>
       </c>
       <c r="D27" s="3">
-        <v>1</v>
+        <v>95</v>
       </c>
       <c r="E27" t="s">
         <v>133</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>321</v>
+        <v>309</v>
       </c>
       <c r="G27" s="11" t="s">
-        <v>259</v>
+        <v>247</v>
       </c>
       <c r="H27" s="5" t="s">
         <v>134</v>
@@ -4847,7 +4837,7 @@
         <v>0</v>
       </c>
       <c r="K27" s="9" t="s">
-        <v>219</v>
+        <v>207</v>
       </c>
     </row>
     <row r="28" spans="1:17" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4861,16 +4851,16 @@
         <v>107</v>
       </c>
       <c r="D28" s="3">
-        <v>1</v>
+        <v>107</v>
       </c>
       <c r="E28" t="s">
         <v>135</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>322</v>
+        <v>310</v>
       </c>
       <c r="G28" s="11" t="s">
-        <v>260</v>
+        <v>248</v>
       </c>
       <c r="H28" s="5" t="s">
         <v>136</v>
@@ -4882,7 +4872,7 @@
         <v>0</v>
       </c>
       <c r="K28" s="9" t="s">
-        <v>220</v>
+        <v>208</v>
       </c>
     </row>
     <row r="29" spans="1:17" s="18" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4899,16 +4889,16 @@
         <v>40</v>
       </c>
       <c r="E29" s="22" t="s">
+        <v>345</v>
+      </c>
+      <c r="F29" s="22" t="s">
         <v>137</v>
       </c>
-      <c r="F29" s="22" t="s">
+      <c r="G29" s="19" t="s">
+        <v>177</v>
+      </c>
+      <c r="H29" s="22" t="s">
         <v>138</v>
-      </c>
-      <c r="G29" s="19" t="s">
-        <v>189</v>
-      </c>
-      <c r="H29" s="22" t="s">
-        <v>139</v>
       </c>
       <c r="I29" s="18" t="s">
         <v>50</v>
@@ -4917,22 +4907,22 @@
         <v>0</v>
       </c>
       <c r="K29" s="24" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
       <c r="L29" s="19" t="s">
-        <v>234</v>
+        <v>222</v>
       </c>
       <c r="M29" s="18">
         <v>3</v>
       </c>
       <c r="N29" s="18" t="s">
-        <v>331</v>
+        <v>319</v>
       </c>
       <c r="P29" s="22" t="s">
         <v>51</v>
       </c>
       <c r="Q29" s="25" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="30" spans="1:17" s="13" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4949,16 +4939,16 @@
         <v>26</v>
       </c>
       <c r="E30" s="14" t="s">
+        <v>346</v>
+      </c>
+      <c r="F30" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="G30" s="16" t="s">
+        <v>329</v>
+      </c>
+      <c r="H30" s="15" t="s">
         <v>141</v>
-      </c>
-      <c r="F30" s="15" t="s">
-        <v>142</v>
-      </c>
-      <c r="G30" s="16" t="s">
-        <v>341</v>
-      </c>
-      <c r="H30" s="15" t="s">
-        <v>143</v>
       </c>
       <c r="I30" s="13" t="s">
         <v>52</v>
@@ -4967,22 +4957,22 @@
         <v>0</v>
       </c>
       <c r="K30" s="17" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
       <c r="L30" s="13" t="s">
-        <v>339</v>
+        <v>327</v>
       </c>
       <c r="M30" s="13" t="s">
-        <v>340</v>
+        <v>328</v>
       </c>
       <c r="N30" s="13" t="s">
-        <v>336</v>
+        <v>324</v>
       </c>
       <c r="P30" s="15" t="s">
         <v>53</v>
       </c>
       <c r="Q30" s="14" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="31" spans="1:17" s="18" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4999,16 +4989,16 @@
         <v>34</v>
       </c>
       <c r="E31" s="25" t="s">
-        <v>145</v>
+        <v>347</v>
       </c>
       <c r="F31" s="22" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="G31" s="19" t="s">
-        <v>190</v>
+        <v>178</v>
       </c>
       <c r="H31" s="22" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="I31" s="18" t="s">
         <v>54</v>
@@ -5017,22 +5007,22 @@
         <v>0</v>
       </c>
       <c r="K31" s="24" t="s">
+        <v>212</v>
+      </c>
+      <c r="L31" s="27" t="s">
+        <v>223</v>
+      </c>
+      <c r="M31" s="27" t="s">
         <v>224</v>
       </c>
-      <c r="L31" s="27" t="s">
-        <v>235</v>
-      </c>
-      <c r="M31" s="27" t="s">
-        <v>236</v>
-      </c>
       <c r="N31" s="27" t="s">
-        <v>331</v>
+        <v>319</v>
       </c>
       <c r="P31" s="22" t="s">
         <v>55</v>
       </c>
       <c r="Q31" s="25" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="32" spans="1:17" s="18" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -5049,16 +5039,16 @@
         <v>34</v>
       </c>
       <c r="E32" s="18" t="s">
-        <v>149</v>
+        <v>348</v>
       </c>
       <c r="F32" s="22" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="G32" s="19" t="s">
-        <v>191</v>
+        <v>179</v>
       </c>
       <c r="H32" s="22" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="I32" s="18" t="s">
         <v>56</v>
@@ -5067,22 +5057,22 @@
         <v>0</v>
       </c>
       <c r="K32" s="24" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
       <c r="L32" s="19" t="s">
-        <v>237</v>
+        <v>225</v>
       </c>
       <c r="M32" s="18" t="s">
-        <v>238</v>
+        <v>226</v>
       </c>
       <c r="N32" s="18" t="s">
-        <v>331</v>
+        <v>319</v>
       </c>
       <c r="P32" s="22" t="s">
         <v>57</v>
       </c>
       <c r="Q32" s="25" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
     </row>
     <row r="33" spans="1:17" s="13" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -5099,16 +5089,16 @@
         <v>26</v>
       </c>
       <c r="E33" s="13" t="s">
-        <v>153</v>
+        <v>349</v>
       </c>
       <c r="F33" s="15" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="G33" s="16" t="s">
-        <v>192</v>
+        <v>180</v>
       </c>
       <c r="H33" s="15" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="I33" s="13" t="s">
         <v>58</v>
@@ -5117,17 +5107,17 @@
         <v>0</v>
       </c>
       <c r="K33" s="17" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
       <c r="L33" s="16"/>
       <c r="N33" s="13" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="P33" s="15" t="s">
         <v>59</v>
       </c>
       <c r="Q33" s="14" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
     </row>
     <row r="34" spans="1:17" s="13" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -5144,16 +5134,16 @@
         <v>28</v>
       </c>
       <c r="E34" s="13" t="s">
-        <v>157</v>
+        <v>350</v>
       </c>
       <c r="F34" s="15" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="G34" s="16" t="s">
-        <v>193</v>
+        <v>181</v>
       </c>
       <c r="H34" s="15" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="I34" s="13" t="s">
         <v>60</v>
@@ -5162,17 +5152,17 @@
         <v>0</v>
       </c>
       <c r="K34" s="17" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
       <c r="L34" s="16"/>
       <c r="N34" s="13" t="s">
-        <v>337</v>
+        <v>325</v>
       </c>
       <c r="P34" s="15" t="s">
         <v>61</v>
       </c>
       <c r="Q34" s="14" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
     </row>
     <row r="35" spans="1:17" s="18" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -5189,16 +5179,16 @@
         <v>26</v>
       </c>
       <c r="E35" s="18" t="s">
-        <v>161</v>
+        <v>351</v>
       </c>
       <c r="F35" s="22" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="G35" s="19" t="s">
-        <v>194</v>
+        <v>182</v>
       </c>
       <c r="H35" s="22" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="I35" s="18" t="s">
         <v>62</v>
@@ -5207,22 +5197,22 @@
         <v>0</v>
       </c>
       <c r="K35" s="24" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
       <c r="L35" s="19" t="s">
-        <v>239</v>
+        <v>227</v>
       </c>
       <c r="M35" s="18" t="s">
-        <v>240</v>
+        <v>228</v>
       </c>
       <c r="N35" s="18" t="s">
-        <v>331</v>
+        <v>319</v>
       </c>
       <c r="P35" s="22" t="s">
         <v>63</v>
       </c>
       <c r="Q35" s="25" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
     </row>
     <row r="36" spans="1:17" s="18" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -5239,16 +5229,16 @@
         <v>34</v>
       </c>
       <c r="E36" s="18" t="s">
-        <v>165</v>
+        <v>344</v>
       </c>
       <c r="F36" s="22" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="G36" s="19" t="s">
-        <v>195</v>
+        <v>183</v>
       </c>
       <c r="H36" s="22" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="I36" s="18" t="s">
         <v>64</v>
@@ -5257,22 +5247,22 @@
         <v>0</v>
       </c>
       <c r="K36" s="24" t="s">
-        <v>224</v>
+        <v>212</v>
       </c>
       <c r="L36" s="19" t="s">
-        <v>241</v>
+        <v>229</v>
       </c>
       <c r="M36" s="18">
         <v>5</v>
       </c>
       <c r="N36" s="18" t="s">
-        <v>331</v>
+        <v>319</v>
       </c>
       <c r="P36" s="22" t="s">
         <v>65</v>
       </c>
       <c r="Q36" s="25" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
     </row>
     <row r="37" spans="1:17" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -5286,19 +5276,19 @@
         <v>107</v>
       </c>
       <c r="D37" s="3">
-        <v>1</v>
+        <v>97</v>
       </c>
       <c r="E37" t="s">
-        <v>169</v>
+        <v>343</v>
       </c>
       <c r="F37" s="5" t="s">
-        <v>170</v>
+        <v>161</v>
       </c>
       <c r="G37" s="11" t="s">
-        <v>261</v>
+        <v>249</v>
       </c>
       <c r="H37" s="5" t="s">
-        <v>171</v>
+        <v>162</v>
       </c>
       <c r="I37" t="s">
         <v>73</v>
@@ -5307,13 +5297,13 @@
         <v>0</v>
       </c>
       <c r="K37" s="9" t="s">
-        <v>221</v>
+        <v>209</v>
       </c>
       <c r="P37" s="5" t="s">
         <v>67</v>
       </c>
       <c r="Q37" s="6" t="s">
-        <v>172</v>
+        <v>163</v>
       </c>
     </row>
     <row r="38" spans="1:17" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -5327,19 +5317,19 @@
         <v>107</v>
       </c>
       <c r="D38" s="3">
-        <v>1</v>
+        <v>67</v>
       </c>
       <c r="E38" t="s">
-        <v>173</v>
+        <v>341</v>
       </c>
       <c r="F38" s="7" t="s">
-        <v>174</v>
+        <v>164</v>
       </c>
       <c r="G38" s="11" t="s">
-        <v>262</v>
+        <v>250</v>
       </c>
       <c r="H38" s="7" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="I38" t="s">
         <v>74</v>
@@ -5348,13 +5338,13 @@
         <v>0</v>
       </c>
       <c r="K38" s="9" t="s">
-        <v>222</v>
+        <v>210</v>
       </c>
       <c r="P38" s="5" t="s">
         <v>75</v>
       </c>
       <c r="Q38" s="6" t="s">
-        <v>176</v>
+        <v>166</v>
       </c>
     </row>
     <row r="39" spans="1:17" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -5368,19 +5358,19 @@
         <v>107</v>
       </c>
       <c r="D39" s="3">
-        <v>1</v>
+        <v>85</v>
       </c>
       <c r="E39" t="s">
-        <v>177</v>
+        <v>342</v>
       </c>
       <c r="F39" s="5" t="s">
-        <v>178</v>
+        <v>340</v>
       </c>
       <c r="G39" s="11" t="s">
-        <v>263</v>
+        <v>251</v>
       </c>
       <c r="H39" s="5" t="s">
-        <v>179</v>
+        <v>167</v>
       </c>
       <c r="I39" s="5" t="s">
         <v>68</v>
@@ -5389,13 +5379,13 @@
         <v>0</v>
       </c>
       <c r="K39" s="9" t="s">
-        <v>223</v>
+        <v>211</v>
       </c>
       <c r="P39" s="2" t="s">
         <v>69</v>
       </c>
       <c r="Q39" s="6" t="s">
-        <v>180</v>
+        <v>168</v>
       </c>
     </row>
   </sheetData>
@@ -5563,7 +5553,7 @@
         <v>13</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>264</v>
+        <v>252</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5578,7 +5568,7 @@
         <v>14</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>265</v>
+        <v>253</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5593,7 +5583,7 @@
         <v>15</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>345</v>
+        <v>333</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5608,7 +5598,7 @@
         <v>16</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>266</v>
+        <v>254</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5623,7 +5613,7 @@
         <v>17</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>346</v>
+        <v>334</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5638,7 +5628,7 @@
         <v>18</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>267</v>
+        <v>255</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5653,7 +5643,7 @@
         <v>19</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>351</v>
+        <v>339</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5668,7 +5658,7 @@
         <v>20</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>268</v>
+        <v>256</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5683,7 +5673,7 @@
         <v>21</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>269</v>
+        <v>257</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5698,7 +5688,7 @@
         <v>22</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>270</v>
+        <v>258</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5713,7 +5703,7 @@
         <v>23</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>271</v>
+        <v>259</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5728,7 +5718,7 @@
         <v>24</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>272</v>
+        <v>260</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5743,7 +5733,7 @@
         <v>25</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>273</v>
+        <v>261</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5758,7 +5748,7 @@
         <v>26</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>274</v>
+        <v>262</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5773,7 +5763,7 @@
         <v>27</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>275</v>
+        <v>263</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5788,7 +5778,7 @@
         <v>28</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>276</v>
+        <v>264</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5803,7 +5793,7 @@
         <v>29</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>277</v>
+        <v>265</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5818,7 +5808,7 @@
         <v>30</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>278</v>
+        <v>266</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5832,7 +5822,7 @@
         <v>31</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>279</v>
+        <v>267</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5846,7 +5836,7 @@
         <v>32</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>280</v>
+        <v>268</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5860,7 +5850,7 @@
         <v>33</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>281</v>
+        <v>269</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5874,7 +5864,7 @@
         <v>34</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>282</v>
+        <v>270</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5888,7 +5878,7 @@
         <v>35</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>283</v>
+        <v>271</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5902,7 +5892,7 @@
         <v>36</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>284</v>
+        <v>272</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5916,7 +5906,7 @@
         <v>37</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>285</v>
+        <v>273</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5930,7 +5920,7 @@
         <v>38</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>286</v>
+        <v>274</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5944,7 +5934,7 @@
         <v>39</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>287</v>
+        <v>275</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5958,7 +5948,7 @@
         <v>40</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>288</v>
+        <v>276</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5972,7 +5962,7 @@
         <v>41</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>289</v>
+        <v>277</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5986,7 +5976,7 @@
         <v>42</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>290</v>
+        <v>278</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6000,7 +5990,7 @@
         <v>43</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>291</v>
+        <v>279</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6014,7 +6004,7 @@
         <v>44</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>292</v>
+        <v>280</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6028,7 +6018,7 @@
         <v>45</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>293</v>
+        <v>281</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6042,7 +6032,7 @@
         <v>46</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>294</v>
+        <v>282</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6056,7 +6046,7 @@
         <v>47</v>
       </c>
       <c r="D44" s="5" t="s">
-        <v>295</v>
+        <v>283</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6070,7 +6060,7 @@
         <v>48</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>296</v>
+        <v>284</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6084,7 +6074,7 @@
         <v>49</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>297</v>
+        <v>285</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6210,7 +6200,7 @@
         <v>66</v>
       </c>
       <c r="D55" s="5" t="s">
-        <v>298</v>
+        <v>286</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6224,7 +6214,7 @@
         <v>68</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>299</v>
+        <v>287</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6238,7 +6228,7 @@
         <v>70</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>299</v>
+        <v>287</v>
       </c>
     </row>
     <row r="58" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6252,7 +6242,7 @@
         <v>71</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>299</v>
+        <v>287</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6266,7 +6256,7 @@
         <v>72</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>299</v>
+        <v>287</v>
       </c>
     </row>
     <row r="60" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6280,7 +6270,7 @@
         <v>73</v>
       </c>
       <c r="D60" s="5" t="s">
-        <v>300</v>
+        <v>288</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6294,7 +6284,7 @@
         <v>74</v>
       </c>
       <c r="D61" s="5" t="s">
-        <v>301</v>
+        <v>289</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6308,7 +6298,7 @@
         <v>68</v>
       </c>
       <c r="D62" s="5" t="s">
-        <v>302</v>
+        <v>290</v>
       </c>
     </row>
     <row r="63" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6322,7 +6312,7 @@
         <v>66</v>
       </c>
       <c r="D63" s="5" t="s">
-        <v>302</v>
+        <v>290</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix:  Programmingtasks: Java Testfile names
</commit_message>
<xml_diff>
--- a/files/programming-tasks/programmieraufgaben_JACK_SOSE23_WORKSHOP_WISE2324.xlsx
+++ b/files/programming-tasks/programmieraufgaben_JACK_SOSE23_WORKSHOP_WISE2324.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\hefl\files\programming-tasks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A586511-387F-4E24-AF33-787F9C060FEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3B583EC-8942-46C2-B8C5-FC8C62AE54E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25650" yWindow="240" windowWidth="45780" windowHeight="20505" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Aufgaben" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="487" uniqueCount="364">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="346">
   <si>
     <t>id</t>
   </si>
@@ -1328,12 +1328,6 @@
     <t>WettrennenTest.java</t>
   </si>
   <si>
-    <t>SortierenTest.java</t>
-  </si>
-  <si>
-    <t>AutoTest.java</t>
-  </si>
-  <si>
     <t>test_main.py</t>
   </si>
   <si>
@@ -1719,40 +1713,6 @@
     <t xml:space="preserve">package de.goals.testing;
 import org.junit.jupiter.api.Test;
 import static org.junit.jupiter.api.Assertions.assertEquals;
-public class KFZTest {
-    private int punkte = 0;
-    private KFZ porsche = new KFZ("AK-CA 740", 24500, 50, 8, 0);
-    public int getResult() {
-        return punkte;
-    }
-    @Test
-    public void testGetKMstand() {
-        assertEquals(24500, porsche.getKMstand(), "Fehler beim Aufruf der Methode getKMstand()");
-        punkte += 25;
-        System.out.println("Test 1 erfolgreich " + porsche.getKMstand());
-    }
-    @Test
-    public void testTanken() {
-        porsche.tanken(60);
-        assertEquals(50, porsche.getTankinhalt(), "Fehler beim Aufruf der Methode getTankinhalt()");
-        punkte += 25;
-        System.out.println("Test 2 erfolgreich " + porsche.getTankinhalt());
-    }
-    @Test
-    public void testFahren() {
-        porsche.tanken(60);
-        boolean ret = porsche.fahren(150);
-        assertEquals(24650, porsche.getKMstand(), "Fehler beim Aufruf der Methode getKMstand() oder fahren()");
-        punkte += 50;
-        System.out.println("Test 3 erfolgreich " + porsche.getKMstand());
-    }
-}
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">package de.goals.testing;
-import org.junit.jupiter.api.Test;
-import static org.junit.jupiter.api.Assertions.assertEquals;
 public class AppPunktTest {
     private int punkte = 0;
     public int getResult() {
@@ -1791,52 +1751,6 @@
     <t xml:space="preserve">package de.goals.testing;
 import org.junit.jupiter.api.Test;
 import static org.junit.jupiter.api.Assertions.assertEquals;
-public class KontoTest {
-    @Test
-    public void testToString() {
-        Konto konto = new Konto("Andreas", "Hoffmann", "DE232212442");
-        konto.einzahlen(100);
-        String expected = "Kunde: Andreas Hoffmann, Konto: DE232212442, Stand: 100.0, Limit: 0.0";
-        assertEquals(expected, konto.toString(), "Fehler in der toString() Methode");
-    }
-    @Test
-    public void testEinzahlen() {
-        Konto konto = new Konto("Max", "Mustermann", "DE12345678901234567890");
-        konto.einzahlen(100);
-        double expectedKontostand = 100.0;
-        assertEquals(expectedKontostand, konto.kontostand(), "Fehler in der Einzahlen-Methode");
-    }
-    @Test
-    public void testAuszahlenWithinLimit() {
-        Konto konto = new Konto("Max", "Mustermann", "DE12345678901234567890");
-        konto.einzahlen(1000);
-        konto.auszahlen(500);
-        double expectedKontostand = 500.0;
-        assertEquals(expectedKontostand, konto.kontostand(), "Fehler in der Auszahlen-Methode mit Betrag innerhalb des Limits");
-    }
-    @Test
-    public void testAuszahlenExceedingLimit() {
-        Konto konto = new Konto("Max", "Mustermann", "DE12345678901234567890");
-        konto.einzahlen(1000);
-        konto.setLimit(500); // Set the limit before withdrawing
-        konto.auszahlen(1000);
-        double expectedKontostand = konto.getLimit();
-        assertEquals(expectedKontostand, konto.kontostand(), "Fehler in der Auszahlen-Methode mit Betrag, der das Limit überschreitet");
-    }
-    @Test
-    public void testSetLimit() {
-        Konto konto = new Konto("Max", "Mustermann", "DE12345678901234567890");
-        konto.setLimit(1000);
-        double expectedLimit = 1000.0;
-        assertEquals(expectedLimit, konto.getLimit(), "Fehler in der SetLimit-Methode");
-    }
-}
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">package de.goals.testing;
-import org.junit.jupiter.api.Test;
-import static org.junit.jupiter.api.Assertions.assertEquals;
 public class AppRadioTest {
     private int punkte = 0;
     public int getResult() {
@@ -1863,26 +1777,6 @@
         assertEquals("Radio an: Freq=89.8, Laut=10", r3.toString());
         punkte += 34;
         System.out.println("Test 3 erfolgreich");
-    }
-}
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">package de.goals.testing;
-import org.junit.jupiter.api.Test;
-import static org.junit.jupiter.api.Assertions.assertEquals;
-public class AppLeserTest {
-    private int punkte = 0;
-    public int getResult() {
-        return punkte;
-    }
-    @Test
-    public void test1() {
-        Leser l = new Leser(1, 56534, "Hoffmann");
-        String out = l.getName();
-        assertEquals("Hoffmann", out);
-        punkte += 100;
-        System.out.println("Test 1 erfolgreich");
     }
 }
 </t>
@@ -2620,38 +2514,6 @@
 	Entfernt alle Vielfachen von 2 aus liste&lt;/em&gt;&lt;/li&gt;
 	&lt;li&gt;Implementieren sie dann die Funktion &lt;em&gt;sieb()&lt;/em&gt; mit Hilfe der Funktion &lt;em&gt;vielfaches()&lt;/em&gt;.&lt;/li&gt;
 &lt;/ol&gt;</t>
-  </si>
-  <si>
-    <t>Comment</t>
-  </si>
-  <si>
-    <t>Streng genommen wird der Fall 0 Jahre nicht überprüft, sonst gut.</t>
-  </si>
-  <si>
-    <t>Streng genommen wird der Fall exakt 100 Euro nicht richtig überprüft, sonst gut.</t>
-  </si>
-  <si>
-    <t>gut</t>
-  </si>
-  <si>
-    <t>Fehler in Anzeige der Aufgabenstellung. Welche Antwort wird für 1 erwartet? Sonst gut.</t>
-  </si>
-  <si>
-    <t>nicht in Goals(?)</t>
-  </si>
-  <si>
-    <t>Traceback (most recent call last):
-  File "&lt;string&gt;", line 1, in &lt;module&gt;
-TypeError: summe() missing 1 required positional argument: 'n' in Ausgabe, sonst gut</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Funktion heißt einmal in Aufgabenstellung vielfaches() statt vielfach() wie sonst und im Test</t>
-  </si>
-  <si>
-    <t>liefert 100% bei leerem Code (no program to run)</t>
-  </si>
-  <si>
-    <t>no program to run als Ausgabe, Rest scheint zu funktionieren</t>
   </si>
   <si>
     <t>Schreiben Sie &amp;nbsp;eine rekursive Funktion&amp;nbsp;&lt;code&gt;querSum(n)&lt;/code&gt;, die eine positive Ganzzahl&amp;nbsp;&lt;code&gt;n&lt;/code&gt;&amp;nbsp;als Parameter erh&amp;auml;lt und ihre Quersumme ausgibt.&lt;br /&gt;
@@ -2840,35 +2702,6 @@
   </si>
   <si>
     <t>Python Reduziere Liste</t>
-  </si>
-  <si>
-    <t>Klassenname scheint vertauscht zu sein, daher nicht testbar.</t>
-  </si>
-  <si>
-    <t>Kommandozeilenparameter führen noch zu Fehler, aber funktioniert sonst.</t>
-  </si>
-  <si>
-    <t>Scheint noch nicht richtig zu laufen: Es sieht so aus, als ob es ein Problem mit der Kompilierung deines Codes gibt. Überprüfe, ob alle Klassen korrekt definiert sind und ob die Zugriffsrechte und Konstruktoren richtig gesetzt sind. Achte darauf, dass alle benötigten Klassen importiert sind und keine Tippfehler in den Klassennamen oder Methodenaufrufen vorhanden sind.
-Stelle sicher, dass die Klassen und Methoden richtig miteinander interagieren. Überprüfe insbesondere die Verwendung der Datum Klasse in den Methoden berechneUeberziehungsgeld in den Klassen Buch und DVD. Es könnte hilfreich sein, die Logik und die Berechnungen in diesen Methoden noch einmal zu überdenken, um sicherzustellen, dass alles logisch und korrekt abläuft.
-Vergewissere dich auch, dass die Klassen Buch und DVD korrekt von der Klasse Medium erben und dass alle abstrakten Methoden, die in Medium definiert sind, in den Unterklassen implementiert werden. Dies ist entscheidend für die korrekte Funktionsweise des Programms.</t>
-  </si>
-  <si>
-    <t>gut, Error: Could not find or load main class de.goals.testing.Uni
-Caused by: java.lang.ClassNotFoundException: de.goals.testing.Uni</t>
-  </si>
-  <si>
-    <t>Error: Main method not found in class de.goals.testing.VektorWork, please define the main method as:
-   public static void main(String[] args)
-or a JavaFX application class must extend javafx.application.Application</t>
-  </si>
-  <si>
-    <t>markdown Fehler oder so etwas, Aufgabe wird nicht angezeigt. lösung gibt auch 0 punkte, egal was man schreibt. (feedback sagt "es sieht richtig aus aber es gibt kompilierfehler"</t>
-  </si>
-  <si>
-    <t>markdown Fehler oder so etwas, Aufgabe wird nicht angezeigt</t>
-  </si>
-  <si>
-    <t>Markdown Fehler, außerdem: Es scheint, dass es ein Problem mit der Kompilierung deines Codes gibt. Überprüfe, ob alle Klassen korrekt definiert sind und ob die Paketnamen und Importe korrekt sind. Achte auch darauf, dass die Methodensignaturen und Konstruktoren wie in der Aufgabenstellung beschrieben implementiert sind.</t>
   </si>
   <si>
     <t xml:space="preserve">package de.goals.testing;
@@ -3297,12 +3130,118 @@
   Schreiben Sie den Java Code für beide Klassen des UML-Diagramms, in eine Datei, erst Fahrzeug, dann Auto.
 &lt;/p&gt;</t>
   </si>
+  <si>
+    <t>BubbleSortTest.java</t>
+  </si>
+  <si>
+    <t>FahrzeugTest.java</t>
+  </si>
+  <si>
+    <t xml:space="preserve">package de.goals.testing;
+import org.junit.jupiter.api.Test;
+import static org.junit.jupiter.api.Assertions.assertEquals;
+public class LeserTest {
+    private int punkte = 0;
+    public int getResult() {
+        return punkte;
+    }
+    @Test
+    public void test1() {
+        Leser l = new Leser(1, 56534, "Hoffmann");
+        String out = l.getName();
+        assertEquals("Hoffmann", out);
+        punkte += 100;
+        System.out.println("Test 1 erfolgreich");
+    }
+}
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">package de.goals.testing;
+import org.junit.jupiter.api.Test;
+import static org.junit.jupiter.api.Assertions.assertEquals;
+public class AppBankTest {
+    @Test
+    public void testToString() {
+        Konto konto = new Konto("Andreas", "Hoffmann", "DE232212442");
+        konto.einzahlen(100);
+        String expected = "Kunde: Andreas Hoffmann, Konto: DE232212442, Stand: 100.0, Limit: 0.0";
+        assertEquals(expected, konto.toString(), "Fehler in der toString() Methode");
+    }
+    @Test
+    public void testEinzahlen() {
+        Konto konto = new Konto("Max", "Mustermann", "DE12345678901234567890");
+        konto.einzahlen(100);
+        double expectedKontostand = 100.0;
+        assertEquals(expectedKontostand, konto.kontostand(), "Fehler in der Einzahlen-Methode");
+    }
+    @Test
+    public void testAuszahlenWithinLimit() {
+        Konto konto = new Konto("Max", "Mustermann", "DE12345678901234567890");
+        konto.einzahlen(1000);
+        konto.auszahlen(500);
+        double expectedKontostand = 500.0;
+        assertEquals(expectedKontostand, konto.kontostand(), "Fehler in der Auszahlen-Methode mit Betrag innerhalb des Limits");
+    }
+    @Test
+    public void testAuszahlenExceedingLimit() {
+        Konto konto = new Konto("Max", "Mustermann", "DE12345678901234567890");
+        konto.einzahlen(1000);
+        konto.setLimit(500); // Set the limit before withdrawing
+        konto.auszahlen(1000);
+        double expectedKontostand = konto.getLimit();
+        assertEquals(expectedKontostand, konto.kontostand(), "Fehler in der Auszahlen-Methode mit Betrag, der das Limit überschreitet");
+    }
+    @Test
+    public void testSetLimit() {
+        Konto konto = new Konto("Max", "Mustermann", "DE12345678901234567890");
+        konto.setLimit(1000);
+        double expectedLimit = 1000.0;
+        assertEquals(expectedLimit, konto.getLimit(), "Fehler in der SetLimit-Methode");
+    }
+}
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">package de.goals.testing;
+import org.junit.jupiter.api.Test;
+import static org.junit.jupiter.api.Assertions.assertEquals;
+public class AppAutoTest {
+    private int punkte = 0;
+    private KFZ porsche = new KFZ("AK-CA 740", 24500, 50, 8, 0);
+    public int getResult() {
+        return punkte;
+    }
+    @Test
+    public void testGetKMstand() {
+        assertEquals(24500, porsche.getKMstand(), "Fehler beim Aufruf der Methode getKMstand()");
+        punkte += 25;
+        System.out.println("Test 1 erfolgreich " + porsche.getKMstand());
+    }
+    @Test
+    public void testTanken() {
+        porsche.tanken(60);
+        assertEquals(50, porsche.getTankinhalt(), "Fehler beim Aufruf der Methode getTankinhalt()");
+        punkte += 25;
+        System.out.println("Test 2 erfolgreich " + porsche.getTankinhalt());
+    }
+    @Test
+    public void testFahren() {
+        porsche.tanken(60);
+        boolean ret = porsche.fahren(150);
+        assertEquals(24650, porsche.getKMstand(), "Fehler beim Aufruf der Methode getKMstand() oder fahren()");
+        punkte += 50;
+        System.out.println("Test 3 erfolgreich " + porsche.getKMstand());
+    }
+}
+</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3345,13 +3284,6 @@
     </font>
     <font>
       <sz val="24"/>
-      <color rgb="FF9C5700"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="24"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -3360,13 +3292,6 @@
     <font>
       <sz val="14"/>
       <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <color rgb="FF9C5700"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -3387,20 +3312,20 @@
     </font>
     <font>
       <sz val="22"/>
-      <color rgb="FF9C5700"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="22"/>
-      <color theme="1"/>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3415,6 +3340,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -3464,12 +3394,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -3526,37 +3457,27 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="2" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="11" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="9" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
@@ -3567,10 +3488,27 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="11" fillId="4" borderId="1" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="3"/>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="3" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="2" xfId="3" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="4">
     <cellStyle name="Gut" xfId="2" builtinId="26"/>
     <cellStyle name="Neutral" xfId="1" builtinId="28"/>
+    <cellStyle name="Schlecht" xfId="3" builtinId="27"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -3882,14 +3820,14 @@
     <col min="4" max="4" width="23.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="37.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="66.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="143.140625" style="33" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="143.140625" style="30" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="105.5703125" style="2" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="23.7109375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="50.7109375" style="29" customWidth="1"/>
+    <col min="11" max="11" width="50.7109375" style="27" customWidth="1"/>
     <col min="12" max="12" width="49.85546875" style="2" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="74.5703125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="170.7109375" style="24" customWidth="1"/>
+    <col min="14" max="14" width="170.7109375" style="23" customWidth="1"/>
     <col min="15" max="17" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3912,7 +3850,7 @@
       <c r="F1" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="G1" s="30" t="s">
+      <c r="G1" s="28" t="s">
         <v>82</v>
       </c>
       <c r="H1" s="13" t="s">
@@ -3924,8 +3862,8 @@
       <c r="J1" s="14" t="s">
         <v>85</v>
       </c>
-      <c r="K1" s="26" t="s">
-        <v>208</v>
+      <c r="K1" s="25" t="s">
+        <v>206</v>
       </c>
       <c r="L1" s="13" t="s">
         <v>179</v>
@@ -3933,9 +3871,7 @@
       <c r="M1" s="12" t="s">
         <v>180</v>
       </c>
-      <c r="N1" s="21" t="s">
-        <v>299</v>
-      </c>
+      <c r="N1" s="21"/>
     </row>
     <row r="2" spans="1:18" s="12" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="15">
@@ -3956,7 +3892,7 @@
       <c r="F2" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="G2" s="31" t="s">
+      <c r="G2" s="29" t="s">
         <v>164</v>
       </c>
       <c r="H2" s="16" t="s">
@@ -3968,18 +3904,16 @@
       <c r="J2" s="15">
         <v>0</v>
       </c>
-      <c r="K2" s="27" t="s">
-        <v>207</v>
+      <c r="K2" s="26" t="s">
+        <v>205</v>
       </c>
       <c r="L2" s="13" t="s">
         <v>181</v>
       </c>
       <c r="M2" s="12" t="s">
-        <v>209</v>
-      </c>
-      <c r="N2" s="21" t="s">
-        <v>300</v>
-      </c>
+        <v>207</v>
+      </c>
+      <c r="N2" s="21"/>
     </row>
     <row r="3" spans="1:18" s="12" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="15">
@@ -4000,7 +3934,7 @@
       <c r="F3" s="16" t="s">
         <v>91</v>
       </c>
-      <c r="G3" s="31" t="s">
+      <c r="G3" s="29" t="s">
         <v>165</v>
       </c>
       <c r="H3" s="16" t="s">
@@ -4012,8 +3946,8 @@
       <c r="J3" s="15">
         <v>0</v>
       </c>
-      <c r="K3" s="27" t="s">
-        <v>207</v>
+      <c r="K3" s="26" t="s">
+        <v>205</v>
       </c>
       <c r="L3" s="13" t="s">
         <v>182</v>
@@ -4021,9 +3955,7 @@
       <c r="M3" s="12" t="s">
         <v>183</v>
       </c>
-      <c r="N3" s="21" t="s">
-        <v>301</v>
-      </c>
+      <c r="N3" s="21"/>
     </row>
     <row r="4" spans="1:18" s="12" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="15">
@@ -4044,11 +3976,11 @@
       <c r="F4" s="16" t="s">
         <v>94</v>
       </c>
-      <c r="G4" s="31" t="s">
+      <c r="G4" s="29" t="s">
         <v>166</v>
       </c>
       <c r="H4" s="16" t="s">
-        <v>309</v>
+        <v>294</v>
       </c>
       <c r="I4" s="12" t="s">
         <v>7</v>
@@ -4056,8 +3988,8 @@
       <c r="J4" s="15">
         <v>0</v>
       </c>
-      <c r="K4" s="27" t="s">
-        <v>207</v>
+      <c r="K4" s="26" t="s">
+        <v>205</v>
       </c>
       <c r="L4" s="13" t="s">
         <v>184</v>
@@ -4065,98 +3997,89 @@
       <c r="M4" s="12">
         <v>174</v>
       </c>
-      <c r="N4" s="21" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="5" spans="1:18" s="7" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A5" s="6">
+      <c r="N4" s="21"/>
+    </row>
+    <row r="5" spans="1:18" s="12" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="15">
         <v>4</v>
       </c>
-      <c r="B5" s="6">
+      <c r="B5" s="15">
         <v>5</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="D5" s="6">
+      <c r="D5" s="15">
         <v>34</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="12" t="s">
         <v>95</v>
       </c>
-      <c r="F5" s="9" t="s">
+      <c r="F5" s="16" t="s">
         <v>96</v>
       </c>
-      <c r="G5" s="32" t="s">
+      <c r="G5" s="17" t="s">
         <v>167</v>
       </c>
-      <c r="H5" s="9" t="s">
-        <v>313</v>
-      </c>
-      <c r="I5" s="7" t="s">
+      <c r="H5" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="I5" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="J5" s="6">
+      <c r="J5" s="15">
         <v>0</v>
       </c>
-      <c r="K5" s="28" t="s">
-        <v>207</v>
-      </c>
-      <c r="L5" s="10" t="s">
+      <c r="K5" s="18" t="s">
+        <v>205</v>
+      </c>
+      <c r="L5" s="13" t="s">
+        <v>208</v>
+      </c>
+      <c r="M5" s="12">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" s="12" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="15">
+        <v>5</v>
+      </c>
+      <c r="B6" s="15">
+        <v>4</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="D6" s="15">
+        <v>23</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="F6" s="16" t="s">
+        <v>98</v>
+      </c>
+      <c r="G6" s="17" t="s">
+        <v>168</v>
+      </c>
+      <c r="H6" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="I6" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="J6" s="15">
+        <v>0</v>
+      </c>
+      <c r="K6" s="18" t="s">
+        <v>205</v>
+      </c>
+      <c r="L6" s="13" t="s">
+        <v>209</v>
+      </c>
+      <c r="M6" s="12" t="s">
         <v>210</v>
       </c>
-      <c r="M5" s="7">
-        <v>47</v>
-      </c>
-      <c r="N5" s="22" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="6" spans="1:18" s="7" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A6" s="6">
-        <v>5</v>
-      </c>
-      <c r="B6" s="6">
-        <v>4</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="D6" s="6">
-        <v>23</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="F6" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="G6" s="32" t="s">
-        <v>168</v>
-      </c>
-      <c r="H6" s="9" t="s">
-        <v>99</v>
-      </c>
-      <c r="I6" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="J6" s="6">
-        <v>0</v>
-      </c>
-      <c r="K6" s="28" t="s">
-        <v>207</v>
-      </c>
-      <c r="L6" s="10" t="s">
-        <v>211</v>
-      </c>
-      <c r="M6" s="7" t="s">
-        <v>212</v>
-      </c>
-      <c r="N6" s="22" t="s">
-        <v>304</v>
-      </c>
-      <c r="Q6" s="12"/>
     </row>
     <row r="7" spans="1:18" s="12" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="15">
@@ -4177,7 +4100,7 @@
       <c r="F7" s="16" t="s">
         <v>101</v>
       </c>
-      <c r="G7" s="31" t="s">
+      <c r="G7" s="29" t="s">
         <v>169</v>
       </c>
       <c r="H7" s="16" t="s">
@@ -4189,18 +4112,16 @@
       <c r="J7" s="15">
         <v>0</v>
       </c>
-      <c r="K7" s="27" t="s">
-        <v>207</v>
+      <c r="K7" s="26" t="s">
+        <v>205</v>
       </c>
       <c r="L7" s="13" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="M7" s="12" t="s">
-        <v>296</v>
-      </c>
-      <c r="N7" s="23" t="s">
-        <v>305</v>
-      </c>
+        <v>291</v>
+      </c>
+      <c r="N7" s="22"/>
     </row>
     <row r="8" spans="1:18" s="12" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="15">
@@ -4221,11 +4142,11 @@
       <c r="F8" s="16" t="s">
         <v>104</v>
       </c>
-      <c r="G8" s="31" t="s">
+      <c r="G8" s="29" t="s">
         <v>170</v>
       </c>
       <c r="H8" s="16" t="s">
-        <v>353</v>
+        <v>330</v>
       </c>
       <c r="I8" s="12" t="s">
         <v>11</v>
@@ -4233,18 +4154,16 @@
       <c r="J8" s="15">
         <v>0</v>
       </c>
-      <c r="K8" s="27" t="s">
-        <v>207</v>
+      <c r="K8" s="26" t="s">
+        <v>205</v>
       </c>
       <c r="L8" s="13" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="M8" s="12" t="s">
-        <v>215</v>
-      </c>
-      <c r="N8" s="21" t="s">
-        <v>302</v>
-      </c>
+        <v>213</v>
+      </c>
+      <c r="N8" s="21"/>
     </row>
     <row r="9" spans="1:18" s="12" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="15">
@@ -4263,13 +4182,13 @@
         <v>105</v>
       </c>
       <c r="F9" s="16" t="s">
-        <v>297</v>
-      </c>
-      <c r="G9" s="31" t="s">
+        <v>292</v>
+      </c>
+      <c r="G9" s="29" t="s">
         <v>171</v>
       </c>
       <c r="H9" s="16" t="s">
-        <v>298</v>
+        <v>293</v>
       </c>
       <c r="I9" s="12" t="s">
         <v>12</v>
@@ -4277,18 +4196,16 @@
       <c r="J9" s="15">
         <v>0</v>
       </c>
-      <c r="K9" s="27" t="s">
-        <v>207</v>
+      <c r="K9" s="26" t="s">
+        <v>205</v>
       </c>
       <c r="L9" s="13" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="M9" s="12">
         <v>10</v>
       </c>
-      <c r="N9" s="21" t="s">
-        <v>306</v>
-      </c>
+      <c r="N9" s="21"/>
     </row>
     <row r="10" spans="1:18" s="12" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="15">
@@ -4310,7 +4227,7 @@
         <v>108</v>
       </c>
       <c r="G10" s="17" t="s">
-        <v>341</v>
+        <v>318</v>
       </c>
       <c r="H10" s="16" t="s">
         <v>109</v>
@@ -4325,11 +4242,8 @@
         <v>185</v>
       </c>
       <c r="L10" s="13"/>
-      <c r="N10" s="12" t="s">
-        <v>333</v>
-      </c>
       <c r="R10" s="13" t="s">
-        <v>349</v>
+        <v>326</v>
       </c>
     </row>
     <row r="11" spans="1:18" s="12" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4349,13 +4263,13 @@
         <v>110</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
       <c r="G11" s="17" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="H11" s="16" t="s">
-        <v>282</v>
+        <v>277</v>
       </c>
       <c r="I11" s="12" t="s">
         <v>14</v>
@@ -4368,7 +4282,7 @@
       </c>
       <c r="L11" s="13"/>
       <c r="R11" s="13" t="s">
-        <v>343</v>
+        <v>320</v>
       </c>
     </row>
     <row r="12" spans="1:18" s="20" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4388,13 +4302,13 @@
         <v>111</v>
       </c>
       <c r="F12" s="20" t="s">
-        <v>314</v>
-      </c>
-      <c r="G12" s="35" t="s">
-        <v>226</v>
-      </c>
-      <c r="H12" s="35" t="s">
-        <v>344</v>
+        <v>299</v>
+      </c>
+      <c r="G12" s="31" t="s">
+        <v>224</v>
+      </c>
+      <c r="H12" s="31" t="s">
+        <v>321</v>
       </c>
       <c r="I12" s="20" t="s">
         <v>15</v>
@@ -4405,11 +4319,9 @@
       <c r="K12" s="20" t="s">
         <v>187</v>
       </c>
-      <c r="N12" s="12" t="s">
-        <v>334</v>
-      </c>
-      <c r="R12" s="35" t="s">
-        <v>345</v>
+      <c r="N12" s="12"/>
+      <c r="R12" s="31" t="s">
+        <v>322</v>
       </c>
     </row>
     <row r="13" spans="1:18" s="12" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4432,7 +4344,7 @@
         <v>113</v>
       </c>
       <c r="G13" s="17" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="H13" s="16" t="s">
         <v>114</v>
@@ -4447,9 +4359,6 @@
         <v>188</v>
       </c>
       <c r="L13" s="13"/>
-      <c r="N13" s="12" t="s">
-        <v>302</v>
-      </c>
     </row>
     <row r="14" spans="1:18" s="20" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="20">
@@ -4468,13 +4377,13 @@
         <v>115</v>
       </c>
       <c r="F14" s="20" t="s">
-        <v>317</v>
+        <v>302</v>
       </c>
       <c r="G14" s="20" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="H14" s="20" t="s">
-        <v>318</v>
+        <v>303</v>
       </c>
       <c r="I14" s="20" t="s">
         <v>17</v>
@@ -4485,11 +4394,9 @@
       <c r="K14" s="20" t="s">
         <v>189</v>
       </c>
-      <c r="N14" s="12" t="s">
-        <v>334</v>
-      </c>
-      <c r="R14" s="35" t="s">
-        <v>350</v>
+      <c r="N14" s="12"/>
+      <c r="R14" s="31" t="s">
+        <v>327</v>
       </c>
     </row>
     <row r="15" spans="1:18" s="12" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4512,7 +4419,7 @@
         <v>117</v>
       </c>
       <c r="G15" s="13" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="H15" s="16" t="s">
         <v>118</v>
@@ -4527,9 +4434,6 @@
         <v>190</v>
       </c>
       <c r="L15" s="13"/>
-      <c r="N15" s="12" t="s">
-        <v>302</v>
-      </c>
     </row>
     <row r="16" spans="1:18" s="20" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="20">
@@ -4547,14 +4451,14 @@
       <c r="E16" s="20" t="s">
         <v>119</v>
       </c>
-      <c r="F16" s="35" t="s">
-        <v>319</v>
+      <c r="F16" s="31" t="s">
+        <v>304</v>
       </c>
       <c r="G16" s="20" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="H16" s="20" t="s">
-        <v>320</v>
+        <v>305</v>
       </c>
       <c r="I16" s="20" t="s">
         <v>19</v>
@@ -4565,9 +4469,7 @@
       <c r="K16" s="20" t="s">
         <v>191</v>
       </c>
-      <c r="N16" s="12" t="s">
-        <v>302</v>
-      </c>
+      <c r="N16" s="12"/>
     </row>
     <row r="17" spans="1:17" s="7" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="6">
@@ -4586,13 +4488,13 @@
         <v>120</v>
       </c>
       <c r="F17" s="9" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="G17" s="10" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="H17" s="9" t="s">
-        <v>284</v>
+        <v>279</v>
       </c>
       <c r="I17" s="9" t="s">
         <v>20</v>
@@ -4604,9 +4506,7 @@
         <v>192</v>
       </c>
       <c r="L17" s="10"/>
-      <c r="N17" s="10" t="s">
-        <v>335</v>
-      </c>
+      <c r="N17" s="10"/>
     </row>
     <row r="18" spans="1:17" s="12" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="15">
@@ -4625,13 +4525,13 @@
         <v>121</v>
       </c>
       <c r="F18" s="16" t="s">
-        <v>285</v>
+        <v>280</v>
       </c>
       <c r="G18" s="13" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="H18" s="16" t="s">
-        <v>286</v>
+        <v>281</v>
       </c>
       <c r="I18" s="12" t="s">
         <v>25</v>
@@ -4643,9 +4543,6 @@
         <v>193</v>
       </c>
       <c r="L18" s="13"/>
-      <c r="N18" s="12" t="s">
-        <v>302</v>
-      </c>
     </row>
     <row r="19" spans="1:17" s="7" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="6">
@@ -4664,13 +4561,13 @@
         <v>122</v>
       </c>
       <c r="F19" s="9" t="s">
-        <v>346</v>
+        <v>323</v>
       </c>
       <c r="G19" s="10" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="H19" s="9" t="s">
-        <v>347</v>
+        <v>324</v>
       </c>
       <c r="I19" s="7" t="s">
         <v>29</v>
@@ -4682,15 +4579,13 @@
         <v>194</v>
       </c>
       <c r="L19" s="10"/>
-      <c r="N19" s="10" t="s">
-        <v>336</v>
-      </c>
+      <c r="N19" s="10"/>
     </row>
     <row r="20" spans="1:17" s="12" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="36">
+      <c r="A20" s="32">
         <v>19</v>
       </c>
-      <c r="B20" s="36">
+      <c r="B20" s="32">
         <v>8</v>
       </c>
       <c r="C20" s="12" t="s">
@@ -4706,7 +4601,7 @@
         <v>124</v>
       </c>
       <c r="G20" s="13" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="H20" s="16" t="s">
         <v>125</v>
@@ -4721,9 +4616,7 @@
         <v>195</v>
       </c>
       <c r="L20" s="13"/>
-      <c r="N20" s="13" t="s">
-        <v>337</v>
-      </c>
+      <c r="N20" s="13"/>
     </row>
     <row r="21" spans="1:17" s="7" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6">
@@ -4742,13 +4635,13 @@
         <v>126</v>
       </c>
       <c r="F21" s="9" t="s">
-        <v>287</v>
+        <v>282</v>
       </c>
       <c r="G21" s="10" t="s">
-        <v>235</v>
-      </c>
-      <c r="H21" s="38" t="s">
-        <v>356</v>
+        <v>345</v>
+      </c>
+      <c r="H21" s="34" t="s">
+        <v>333</v>
       </c>
       <c r="I21" s="7" t="s">
         <v>32</v>
@@ -4760,9 +4653,6 @@
         <v>196</v>
       </c>
       <c r="L21" s="10"/>
-      <c r="N21" s="7" t="s">
-        <v>338</v>
-      </c>
     </row>
     <row r="22" spans="1:17" s="7" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="6">
@@ -4781,13 +4671,13 @@
         <v>127</v>
       </c>
       <c r="F22" s="9" t="s">
-        <v>291</v>
+        <v>286</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>236</v>
-      </c>
-      <c r="H22" s="38" t="s">
-        <v>357</v>
+        <v>233</v>
+      </c>
+      <c r="H22" s="34" t="s">
+        <v>334</v>
       </c>
       <c r="I22" s="9" t="s">
         <v>34</v>
@@ -4799,9 +4689,6 @@
         <v>197</v>
       </c>
       <c r="L22" s="10"/>
-      <c r="N22" s="7" t="s">
-        <v>339</v>
-      </c>
     </row>
     <row r="23" spans="1:17" s="7" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="6">
@@ -4820,13 +4707,13 @@
         <v>128</v>
       </c>
       <c r="F23" s="9" t="s">
-        <v>288</v>
+        <v>283</v>
       </c>
       <c r="G23" s="10" t="s">
-        <v>237</v>
-      </c>
-      <c r="H23" s="38" t="s">
-        <v>358</v>
+        <v>344</v>
+      </c>
+      <c r="H23" s="34" t="s">
+        <v>335</v>
       </c>
       <c r="I23" s="9" t="s">
         <v>36</v>
@@ -4838,9 +4725,6 @@
         <v>198</v>
       </c>
       <c r="L23" s="10"/>
-      <c r="N23" s="7" t="s">
-        <v>338</v>
-      </c>
     </row>
     <row r="24" spans="1:17" s="7" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="6">
@@ -4859,13 +4743,13 @@
         <v>129</v>
       </c>
       <c r="F24" s="9" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>238</v>
-      </c>
-      <c r="H24" s="38" t="s">
-        <v>359</v>
+        <v>234</v>
+      </c>
+      <c r="H24" s="34" t="s">
+        <v>336</v>
       </c>
       <c r="I24" s="9" t="s">
         <v>38</v>
@@ -4877,9 +4761,7 @@
         <v>199</v>
       </c>
       <c r="L24" s="10"/>
-      <c r="N24" s="37" t="s">
-        <v>340</v>
-      </c>
+      <c r="N24" s="33"/>
     </row>
     <row r="25" spans="1:17" s="7" customFormat="1" ht="261" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="6">
@@ -4898,13 +4780,13 @@
         <v>130</v>
       </c>
       <c r="F25" s="9" t="s">
-        <v>289</v>
+        <v>284</v>
       </c>
       <c r="G25" s="10" t="s">
-        <v>239</v>
+        <v>343</v>
       </c>
       <c r="H25" s="9" t="s">
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="I25" s="9" t="s">
         <v>39</v>
@@ -4934,13 +4816,13 @@
         <v>131</v>
       </c>
       <c r="F26" s="9" t="s">
-        <v>293</v>
+        <v>288</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="H26" s="9" t="s">
-        <v>354</v>
+        <v>331</v>
       </c>
       <c r="I26" s="9" t="s">
         <v>41</v>
@@ -4970,13 +4852,13 @@
         <v>132</v>
       </c>
       <c r="F27" s="9" t="s">
-        <v>294</v>
+        <v>289</v>
       </c>
       <c r="G27" s="10" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="H27" s="9" t="s">
-        <v>360</v>
+        <v>337</v>
       </c>
       <c r="I27" s="9" t="s">
         <v>46</v>
@@ -5006,13 +4888,13 @@
         <v>133</v>
       </c>
       <c r="F28" s="9" t="s">
-        <v>295</v>
+        <v>290</v>
       </c>
       <c r="G28" s="10" t="s">
-        <v>242</v>
+        <v>237</v>
       </c>
       <c r="H28" s="9" t="s">
-        <v>361</v>
+        <v>338</v>
       </c>
       <c r="I28" s="9" t="s">
         <v>48</v>
@@ -5039,12 +4921,12 @@
         <v>40</v>
       </c>
       <c r="E29" s="16" t="s">
-        <v>326</v>
+        <v>311</v>
       </c>
       <c r="F29" s="16" t="s">
         <v>134</v>
       </c>
-      <c r="G29" s="30" t="s">
+      <c r="G29" s="28" t="s">
         <v>172</v>
       </c>
       <c r="H29" s="16" t="s">
@@ -5056,18 +4938,16 @@
       <c r="J29" s="15">
         <v>0</v>
       </c>
-      <c r="K29" s="27" t="s">
-        <v>207</v>
+      <c r="K29" s="26" t="s">
+        <v>205</v>
       </c>
       <c r="L29" s="13" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="M29" s="12">
         <v>3</v>
       </c>
-      <c r="N29" s="21" t="s">
-        <v>302</v>
-      </c>
+      <c r="N29" s="21"/>
       <c r="P29" s="16" t="s">
         <v>51</v>
       </c>
@@ -5075,53 +4955,50 @@
         <v>136</v>
       </c>
     </row>
-    <row r="30" spans="1:17" s="7" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A30" s="6">
+    <row r="30" spans="1:17" s="36" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="35">
         <v>29</v>
       </c>
-      <c r="B30" s="6">
+      <c r="B30" s="35">
         <v>0</v>
       </c>
-      <c r="C30" s="7" t="s">
+      <c r="C30" s="36" t="s">
         <v>86</v>
       </c>
-      <c r="D30" s="6">
+      <c r="D30" s="35">
         <v>26</v>
       </c>
-      <c r="E30" s="8" t="s">
-        <v>327</v>
-      </c>
-      <c r="F30" s="9" t="s">
+      <c r="E30" s="37" t="s">
+        <v>312</v>
+      </c>
+      <c r="F30" s="38" t="s">
         <v>137</v>
       </c>
-      <c r="G30" s="34" t="s">
-        <v>312</v>
-      </c>
-      <c r="H30" s="9" t="s">
+      <c r="G30" s="39" t="s">
+        <v>297</v>
+      </c>
+      <c r="H30" s="38" t="s">
         <v>138</v>
       </c>
-      <c r="I30" s="7" t="s">
+      <c r="I30" s="36" t="s">
         <v>52</v>
       </c>
-      <c r="J30" s="6">
+      <c r="J30" s="35">
         <v>0</v>
       </c>
-      <c r="K30" s="28" t="s">
-        <v>207</v>
-      </c>
-      <c r="L30" s="7" t="s">
-        <v>310</v>
-      </c>
-      <c r="M30" s="7" t="s">
-        <v>311</v>
-      </c>
-      <c r="N30" s="22" t="s">
-        <v>307</v>
-      </c>
-      <c r="P30" s="9" t="s">
+      <c r="K30" s="40" t="s">
+        <v>205</v>
+      </c>
+      <c r="L30" s="36" t="s">
+        <v>295</v>
+      </c>
+      <c r="M30" s="36" t="s">
+        <v>296</v>
+      </c>
+      <c r="P30" s="38" t="s">
         <v>53</v>
       </c>
-      <c r="Q30" s="8" t="s">
+      <c r="Q30" s="37" t="s">
         <v>139</v>
       </c>
     </row>
@@ -5139,12 +5016,12 @@
         <v>34</v>
       </c>
       <c r="E31" s="19" t="s">
-        <v>328</v>
+        <v>313</v>
       </c>
       <c r="F31" s="16" t="s">
         <v>140</v>
       </c>
-      <c r="G31" s="30" t="s">
+      <c r="G31" s="28" t="s">
         <v>173</v>
       </c>
       <c r="H31" s="16" t="s">
@@ -5156,18 +5033,16 @@
       <c r="J31" s="15">
         <v>0</v>
       </c>
-      <c r="K31" s="27" t="s">
-        <v>207</v>
+      <c r="K31" s="26" t="s">
+        <v>205</v>
       </c>
       <c r="L31" s="20" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="M31" s="20" t="s">
-        <v>219</v>
-      </c>
-      <c r="N31" s="25" t="s">
-        <v>302</v>
-      </c>
+        <v>217</v>
+      </c>
+      <c r="N31" s="24"/>
       <c r="P31" s="16" t="s">
         <v>55</v>
       </c>
@@ -5189,12 +5064,12 @@
         <v>34</v>
       </c>
       <c r="E32" s="12" t="s">
-        <v>329</v>
+        <v>314</v>
       </c>
       <c r="F32" s="16" t="s">
         <v>143</v>
       </c>
-      <c r="G32" s="30" t="s">
+      <c r="G32" s="28" t="s">
         <v>174</v>
       </c>
       <c r="H32" s="16" t="s">
@@ -5206,18 +5081,16 @@
       <c r="J32" s="15">
         <v>0</v>
       </c>
-      <c r="K32" s="27" t="s">
-        <v>207</v>
+      <c r="K32" s="26" t="s">
+        <v>205</v>
       </c>
       <c r="L32" s="13" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="M32" s="12" t="s">
-        <v>221</v>
-      </c>
-      <c r="N32" s="21" t="s">
-        <v>302</v>
-      </c>
+        <v>219</v>
+      </c>
+      <c r="N32" s="21"/>
       <c r="P32" s="16" t="s">
         <v>57</v>
       </c>
@@ -5225,93 +5098,87 @@
         <v>145</v>
       </c>
     </row>
-    <row r="33" spans="1:17" s="7" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A33" s="6">
+    <row r="33" spans="1:17" s="36" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="35">
         <v>32</v>
       </c>
-      <c r="B33" s="6">
+      <c r="B33" s="35">
         <v>0</v>
       </c>
-      <c r="C33" s="7" t="s">
+      <c r="C33" s="36" t="s">
         <v>86</v>
       </c>
-      <c r="D33" s="6">
+      <c r="D33" s="35">
         <v>26</v>
       </c>
-      <c r="E33" s="7" t="s">
-        <v>330</v>
-      </c>
-      <c r="F33" s="9" t="s">
+      <c r="E33" s="36" t="s">
+        <v>315</v>
+      </c>
+      <c r="F33" s="38" t="s">
         <v>146</v>
       </c>
-      <c r="G33" s="34" t="s">
+      <c r="G33" s="39" t="s">
         <v>175</v>
       </c>
-      <c r="H33" s="9" t="s">
+      <c r="H33" s="38" t="s">
         <v>147</v>
       </c>
-      <c r="I33" s="7" t="s">
+      <c r="I33" s="36" t="s">
         <v>58</v>
       </c>
-      <c r="J33" s="6">
+      <c r="J33" s="35">
         <v>0</v>
       </c>
-      <c r="K33" s="28" t="s">
-        <v>207</v>
-      </c>
-      <c r="L33" s="10"/>
-      <c r="N33" s="22" t="s">
-        <v>308</v>
-      </c>
-      <c r="P33" s="9" t="s">
+      <c r="K33" s="40" t="s">
+        <v>205</v>
+      </c>
+      <c r="L33" s="39"/>
+      <c r="P33" s="38" t="s">
         <v>59</v>
       </c>
-      <c r="Q33" s="8" t="s">
+      <c r="Q33" s="37" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="34" spans="1:17" s="7" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A34" s="6">
+    <row r="34" spans="1:17" s="36" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="35">
         <v>33</v>
       </c>
-      <c r="B34" s="6">
+      <c r="B34" s="35">
         <v>0</v>
       </c>
-      <c r="C34" s="7" t="s">
+      <c r="C34" s="36" t="s">
         <v>86</v>
       </c>
-      <c r="D34" s="6">
+      <c r="D34" s="35">
         <v>28</v>
       </c>
-      <c r="E34" s="7" t="s">
-        <v>331</v>
-      </c>
-      <c r="F34" s="9" t="s">
+      <c r="E34" s="36" t="s">
+        <v>316</v>
+      </c>
+      <c r="F34" s="38" t="s">
         <v>149</v>
       </c>
-      <c r="G34" s="34" t="s">
+      <c r="G34" s="39" t="s">
         <v>176</v>
       </c>
-      <c r="H34" s="9" t="s">
+      <c r="H34" s="38" t="s">
         <v>150</v>
       </c>
-      <c r="I34" s="7" t="s">
+      <c r="I34" s="36" t="s">
         <v>60</v>
       </c>
-      <c r="J34" s="6">
+      <c r="J34" s="35">
         <v>0</v>
       </c>
-      <c r="K34" s="28" t="s">
-        <v>207</v>
-      </c>
-      <c r="L34" s="10"/>
-      <c r="N34" s="22" t="s">
-        <v>308</v>
-      </c>
-      <c r="P34" s="9" t="s">
+      <c r="K34" s="40" t="s">
+        <v>205</v>
+      </c>
+      <c r="L34" s="39"/>
+      <c r="P34" s="38" t="s">
         <v>61</v>
       </c>
-      <c r="Q34" s="8" t="s">
+      <c r="Q34" s="37" t="s">
         <v>151</v>
       </c>
     </row>
@@ -5329,12 +5196,12 @@
         <v>26</v>
       </c>
       <c r="E35" s="12" t="s">
-        <v>332</v>
+        <v>317</v>
       </c>
       <c r="F35" s="16" t="s">
         <v>152</v>
       </c>
-      <c r="G35" s="30" t="s">
+      <c r="G35" s="28" t="s">
         <v>177</v>
       </c>
       <c r="H35" s="16" t="s">
@@ -5346,18 +5213,16 @@
       <c r="J35" s="15">
         <v>0</v>
       </c>
-      <c r="K35" s="27" t="s">
-        <v>207</v>
+      <c r="K35" s="26" t="s">
+        <v>205</v>
       </c>
       <c r="L35" s="13" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="M35" s="12" t="s">
-        <v>223</v>
-      </c>
-      <c r="N35" s="21" t="s">
-        <v>302</v>
-      </c>
+        <v>221</v>
+      </c>
+      <c r="N35" s="21"/>
       <c r="P35" s="16" t="s">
         <v>63</v>
       </c>
@@ -5379,12 +5244,12 @@
         <v>34</v>
       </c>
       <c r="E36" s="12" t="s">
-        <v>325</v>
+        <v>310</v>
       </c>
       <c r="F36" s="16" t="s">
         <v>155</v>
       </c>
-      <c r="G36" s="30" t="s">
+      <c r="G36" s="28" t="s">
         <v>178</v>
       </c>
       <c r="H36" s="16" t="s">
@@ -5396,18 +5261,16 @@
       <c r="J36" s="15">
         <v>0</v>
       </c>
-      <c r="K36" s="27" t="s">
-        <v>207</v>
+      <c r="K36" s="26" t="s">
+        <v>205</v>
       </c>
       <c r="L36" s="13" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="M36" s="12">
         <v>5</v>
       </c>
-      <c r="N36" s="21" t="s">
-        <v>302</v>
-      </c>
+      <c r="N36" s="21"/>
       <c r="P36" s="16" t="s">
         <v>65</v>
       </c>
@@ -5429,16 +5292,16 @@
         <v>97</v>
       </c>
       <c r="E37" s="7" t="s">
-        <v>324</v>
+        <v>309</v>
       </c>
       <c r="F37" s="9" t="s">
         <v>158</v>
       </c>
       <c r="G37" s="10" t="s">
-        <v>243</v>
+        <v>238</v>
       </c>
       <c r="H37" s="9" t="s">
-        <v>355</v>
+        <v>332</v>
       </c>
       <c r="I37" s="7" t="s">
         <v>73</v>
@@ -5471,13 +5334,13 @@
         <v>67</v>
       </c>
       <c r="E38" s="7" t="s">
-        <v>322</v>
+        <v>307</v>
       </c>
       <c r="F38" s="9" t="s">
         <v>160</v>
       </c>
       <c r="G38" s="10" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="H38" s="9" t="s">
         <v>161</v>
@@ -5489,7 +5352,7 @@
         <v>0</v>
       </c>
       <c r="K38" s="11" t="s">
-        <v>205</v>
+        <v>341</v>
       </c>
       <c r="L38" s="10"/>
       <c r="P38" s="9" t="s">
@@ -5513,16 +5376,16 @@
         <v>85</v>
       </c>
       <c r="E39" s="7" t="s">
-        <v>323</v>
+        <v>308</v>
       </c>
       <c r="F39" s="9" t="s">
-        <v>362</v>
+        <v>339</v>
       </c>
       <c r="G39" s="10" t="s">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="H39" s="9" t="s">
-        <v>363</v>
+        <v>340</v>
       </c>
       <c r="I39" s="9" t="s">
         <v>68</v>
@@ -5531,7 +5394,7 @@
         <v>0</v>
       </c>
       <c r="K39" s="11" t="s">
-        <v>206</v>
+        <v>342</v>
       </c>
       <c r="L39" s="10"/>
       <c r="P39" s="10" t="s">
@@ -5706,7 +5569,7 @@
         <v>13</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>348</v>
+        <v>325</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5721,7 +5584,7 @@
         <v>14</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>342</v>
+        <v>319</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5736,7 +5599,7 @@
         <v>15</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>315</v>
+        <v>300</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5751,7 +5614,7 @@
         <v>16</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>246</v>
+        <v>241</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5766,7 +5629,7 @@
         <v>17</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>316</v>
+        <v>301</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5781,7 +5644,7 @@
         <v>18</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>247</v>
+        <v>242</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5796,7 +5659,7 @@
         <v>19</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>321</v>
+        <v>306</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5811,7 +5674,7 @@
         <v>20</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>351</v>
+        <v>328</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5826,7 +5689,7 @@
         <v>21</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>248</v>
+        <v>243</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5841,7 +5704,7 @@
         <v>22</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5856,7 +5719,7 @@
         <v>23</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5871,7 +5734,7 @@
         <v>24</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5886,7 +5749,7 @@
         <v>25</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>252</v>
+        <v>247</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5901,7 +5764,7 @@
         <v>26</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>253</v>
+        <v>248</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5916,7 +5779,7 @@
         <v>27</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5931,7 +5794,7 @@
         <v>28</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5946,7 +5809,7 @@
         <v>29</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5961,7 +5824,7 @@
         <v>30</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>352</v>
+        <v>329</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5975,7 +5838,7 @@
         <v>31</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>257</v>
+        <v>252</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5989,7 +5852,7 @@
         <v>32</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6003,7 +5866,7 @@
         <v>33</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6017,7 +5880,7 @@
         <v>34</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6031,7 +5894,7 @@
         <v>35</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6045,7 +5908,7 @@
         <v>36</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6059,7 +5922,7 @@
         <v>37</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>263</v>
+        <v>258</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6073,7 +5936,7 @@
         <v>38</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>264</v>
+        <v>259</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6087,7 +5950,7 @@
         <v>39</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>265</v>
+        <v>260</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6101,7 +5964,7 @@
         <v>40</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>266</v>
+        <v>261</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6115,7 +5978,7 @@
         <v>41</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>267</v>
+        <v>262</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6129,7 +5992,7 @@
         <v>42</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>268</v>
+        <v>263</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6143,7 +6006,7 @@
         <v>43</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>269</v>
+        <v>264</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6157,7 +6020,7 @@
         <v>44</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>270</v>
+        <v>265</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6171,7 +6034,7 @@
         <v>45</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>271</v>
+        <v>266</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6185,7 +6048,7 @@
         <v>46</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>272</v>
+        <v>267</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6199,7 +6062,7 @@
         <v>47</v>
       </c>
       <c r="D44" s="5" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6213,7 +6076,7 @@
         <v>48</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6227,7 +6090,7 @@
         <v>49</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6353,7 +6216,7 @@
         <v>66</v>
       </c>
       <c r="D55" s="5" t="s">
-        <v>276</v>
+        <v>271</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6367,7 +6230,7 @@
         <v>68</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6381,7 +6244,7 @@
         <v>70</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
     </row>
     <row r="58" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6395,7 +6258,7 @@
         <v>71</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6409,7 +6272,7 @@
         <v>72</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>277</v>
+        <v>272</v>
       </c>
     </row>
     <row r="60" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6423,7 +6286,7 @@
         <v>73</v>
       </c>
       <c r="D60" s="5" t="s">
-        <v>278</v>
+        <v>273</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6437,7 +6300,7 @@
         <v>74</v>
       </c>
       <c r="D61" s="5" t="s">
-        <v>279</v>
+        <v>274</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6451,7 +6314,7 @@
         <v>68</v>
       </c>
       <c r="D62" s="5" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
     </row>
     <row r="63" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6465,7 +6328,7 @@
         <v>66</v>
       </c>
       <c r="D63" s="5" t="s">
-        <v>280</v>
+        <v>275</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed 13 Java Programming Tasks (check desc)
- Almost all Java Tasks work now (Bank Task still wip)
- New Unit-Tests still had some problems...
Changes:
1. Java Bibliothek -  - Testcase verbessert
2. Java Uni -  Fehler in Tabelle verbessert
3. Java KFZ -  Fehler in Tabelle verbessert
4. Java Punkt -  - Testcase verbessert
5. Java Bank -  - Testcase verbessert FUNKTIONIERT NOCH NICHT
6. Java Radio -  Fehler in Tabelle verbessert
7. UMLtoJava -  - Testcase erweitert
8. Java Airline -  - HTML verbessert und 3 weitere Testcases für Polymorphie
9. Java Koerper -  HTML an gepasst. Main Methode hinzugefügt
10. Java Threads -  HTML und Testcases angepasst
11. Java Wettrennen -  war bereits korrekt
12. Java Sortieren -  Test angepasst
13. Java UML to Java -  Neue Klasse mit Main Methode hinzugefügt
</commit_message>
<xml_diff>
--- a/files/programming-tasks/programmieraufgaben_JACK_SOSE23_WORKSHOP_WISE2324.xlsx
+++ b/files/programming-tasks/programmieraufgaben_JACK_SOSE23_WORKSHOP_WISE2324.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\hefl\files\programming-tasks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3B583EC-8942-46C2-B8C5-FC8C62AE54E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72D76F82-293F-48EF-B565-F7F61FF8CCC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="51480" yWindow="-645" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Aufgaben" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="456" uniqueCount="346">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="461" uniqueCount="350">
   <si>
     <t>id</t>
   </si>
@@ -833,11 +833,6 @@
     <t>In dieser Aufgabe sollst du den Bubblesort-Algorithmus in Java implementieren. Dieser Algorithmus ist ein einfaches Verfahren zum Sortieren einer Liste von Elementen (z.B. Zahlen). Bubblesort ist ein Sortieralgorithmus, der durch wiederholtes Durchlaufen der zu sortierenden Liste arbeitet. Bei jedem Durchlauf werden benachbarte Elemente miteinander verglichen und gegebenenfalls vertauscht. Das Besondere am Bubblesort ist, dass mit jedem Durchgang das größte Element der noch zu sortierenden Elemente an das Ende der Liste "aufsteigt".</t>
   </si>
   <si>
-    <t>&lt;p&gt; In dieser Aufgabe sollst du den Bubblesort-Algorithmus in Java implementieren. Dieser Algorithmus ist ein einfaches Verfahren zum Sortieren einer Liste von Elementen (z.B. Zahlen).&lt;/p&gt;
-&lt;br&gt;
-&lt;p&gt;Bubblesort ist ein Sortieralgorithmus, der durch wiederholtes Durchlaufen der zu sortierenden Liste arbeitet. Bei jedem Durchlauf werden benachbarte Elemente miteinander verglichen und gegebenenfalls vertauscht. Das Besondere am Bubblesort ist, dass mit jedem Durchgang das gr\u00f6\u00dfte Element der noch zu sortierenden Elemente an das Ende der Liste "aufsteigt".&lt;/p&gt;</t>
-  </si>
-  <si>
     <t>public class Sortieren {
     // Methode, um ein Array von Zahlen zu sortieren und zurückzugeben
     public static int[] bubbleSort(int[] arr) {
@@ -1568,49 +1563,6 @@
   </si>
   <si>
     <t xml:space="preserve">package de.goals.testing;
-import org.junit.Test;
-import static org.junit.Assert.assertEquals;
-public class BibVerwaltungTest {
-    @Test
-    public void testBerechneStrafgeldBuch() {
-        Buch buch = new Buch("Fussballfieber", "Manuel Neuer", 75);
-        buch.setAusleihdatum(new Datum(2020, 2, 1));
-        Datum currentDate = new Datum();
-        double expectedStrafgeld = calculateFineForBuch(buch.getAusleihdatum(), currentDate);
-        assertEquals(expectedStrafgeld, buch.berechneStrafgeld(), 0.01);
-    }
-    @Test
-    public void testBerechneStrafgeldDVD() {
-        DVD dvd = new DVD("FussballfieberderFilm", "Manuel Neuer", 120);
-        dvd.setAusleihdatum(new Datum(2019, 2, 1));
-        Datum currentDate = new Datum();
-        double expectedStrafgeld = calculateFineForDVD(dvd.getAusleihdatum(), currentDate);
-        assertEquals(expectedStrafgeld, dvd.berechneStrafgeld(), 0.01);
-    }
-    private double calculateFineForBuch(Datum ausleihDatum, Datum currentDate) {
-        int daysDiff = calcDiffDaysTest(ausleihDatum, currentDate);
-        int daysOverdue = Math.max(0, daysDiff - 28); // Calculate the number of days overdue
-        return daysOverdue * 1.0; // 1 EUR per day fine
-    }
-    private double calculateFineForDVD(Datum ausleihDatum, Datum currentDate) {
-        int daysDiff = calcDiffDaysTest(ausleihDatum, currentDate);
-        int daysOverdue = Math.max(0, daysDiff - 7); // Calculate the number of days overdue
-        return daysOverdue * 2.0; // 2 EUR per day fine
-    }
-    private int calcDiffDaysTest(Datum ausleih, Datum currentDate) {
-        int daysHeute = currentDate.getMonat();
-        daysHeute--;
-        daysHeute = ((daysHeute * 30) + currentDate.getTag()) + (365 * currentDate.getJahr());
-        int daysAusleih = ausleih.getMonat();
-        daysAusleih--;
-        daysAusleih = ((daysAusleih * 30) + ausleih.getTag()) + (365 * ausleih.getJahr());
-        return daysHeute - daysAusleih;
-    }
-}
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">package de.goals.testing;
 import org.junit.jupiter.api.Test;
 import static org.junit.jupiter.api.Assertions.assertEquals;
 public class GGTTest {
@@ -1713,44 +1665,6 @@
     <t xml:space="preserve">package de.goals.testing;
 import org.junit.jupiter.api.Test;
 import static org.junit.jupiter.api.Assertions.assertEquals;
-public class AppPunktTest {
-    private int punkte = 0;
-    public int getResult() {
-        return punkte;
-    }
-    @Test
-    public void test1() {
-        AppPunkt p = new AppPunkt(3, 4);
-        String s = p.toString();
-        assertEquals("3/4", s);
-        punkte += 25;
-        System.out.println("Test 1 erfolgreich " + s);
-    }
-    @Test
-    public void test2() {
-        AppPunkt p2 = new AppPunkt(3, 4);
-        AppPunkt spiegelx = p2.spiegelX();
-        String s2 = spiegelx.toString();
-        assertEquals("3/-4", s2);
-        punkte += 25;
-        System.out.println("Test 2 erfolgreich " + s2);
-    }
-    @Test
-    public void test3() {
-        AppPunkt p3 = new AppPunkt(3, 4);
-        AppPunkt spiegelUr = p3.spiegelUrsprung();
-        String s3 = spiegelUr.toString();
-        assertEquals("-3/-4", s3);
-        punkte += 50;
-        System.out.println("Test 3 erfolgreich " + s3);
-    }
-}
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">package de.goals.testing;
-import org.junit.jupiter.api.Test;
-import static org.junit.jupiter.api.Assertions.assertEquals;
 public class AppRadioTest {
     private int punkte = 0;
     public int getResult() {
@@ -1777,34 +1691,6 @@
         assertEquals("Radio an: Freq=89.8, Laut=10", r3.toString());
         punkte += 34;
         System.out.println("Test 3 erfolgreich");
-    }
-}
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">package de.goals.testing;
-import org.junit.jupiter.api.Test;
-import static org.junit.jupiter.api.Assertions.assertEquals;
-public class AirlineTest {
-    private int punkte = 0;
-    public int getResult() {
-        return punkte;
-    }
-    @Test
-    public void test1() {
-        Flugzeug f1 = new Doppeldecker("New", 123,  "98765GHS");
-        String immat = f1.getImmatNummer();
-        assertEquals("98765GHS", immat);
-        punkte += 50;
-        System.out.println("Test 1 erfolgreich");
-    }
-    @Test
-    public void test2() {
-        Flugzeug f2 = new Verkehrsflugzeug("Airbus", 900, "A8789HHU", 490);
-        int speed = f2.getMaxSpeed();
-        assertEquals(900, speed);
-        punkte += 50;
-        System.out.println("Test 2 erfolgreich");
     }
 }
 </t>
@@ -1854,52 +1740,6 @@
     <t xml:space="preserve">package de.goals.testing;
 import org.junit.jupiter.api.Test;
 import static org.junit.jupiter.api.Assertions.assertEquals;
-public class MyThreadTest {
-    private int punkte = 0;
-    public int getResult() {
-        return punkte;
-    }
-    @Test
-    public void test1() {
-        int[] a = {1, 2, 3, 4, 5, 6, 7, 8, 9, 10};
-        ArrayCalc a1 = new ArrayCalc(a, 0, 4);
-        ArrayCalc a2 = new ArrayCalc(a, 5, 9);
-        a1.start();
-        a2.start();
-        try {
-            a1.join();
-            a2.join();
-        } catch (InterruptedException e) {
-            e.printStackTrace();
-        }
-        assertEquals(55, a1.getSumme() + a2.getSumme());
-        punkte += 50;
-        System.out.println("Test 1 erfolgreich");
-    }
-    @Test
-    public void test2() {
-        int[] a = {10, 23, 11, 18, 4, 9, 12, 21};
-        ArrayCalc a1 = new ArrayCalc(a, 0, 3);
-        ArrayCalc a2 = new ArrayCalc(a, 4, 7);
-        a1.start();
-        a2.start();
-        try {
-            a1.join();
-            a2.join();
-        } catch (InterruptedException e) {
-            e.printStackTrace();
-        }
-        assertEquals(108, a1.getSumme() + a2.getSumme());
-        punkte += 50;
-        System.out.println("Test 2 erfolgreich");
-    }
-}
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">package de.goals.testing;
-import org.junit.jupiter.api.Test;
-import static org.junit.jupiter.api.Assertions.assertEquals;
 import static org.junit.jupiter.api.Assertions.assertTrue;
 public class WettrennenTest {
     @Test
@@ -1935,46 +1775,6 @@
         assertEquals(4, kw.getAnzahlRaeder());
         assertEquals(80, kw.position, 0.01);
         assertTrue(kw.isBlaulichtAn());
-    }
-}
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">package de.goals.testing;
-import org.junit.jupiter.api.Test;
-import static org.junit.jupiter.api.Assertions.assertArrayEquals;
-public class BubbleSortTest {
-    @Test
-    public void testBubbleSort1() {
-        BubbleSort sorter = new BubbleSort();
-        int[] arr = {64, 34, 25, 12, 22, 11, 90};
-        int[] expected = {11, 12, 22, 25, 34, 64, 90};
-        sorter.bubbleSort(arr);
-        assertArrayEquals(expected, arr);
-    }
-    @Test
-    public void testBubbleSort2() {
-        BubbleSort sorter = new BubbleSort();
-        int[] arr = {5, 1, 9, 3, 7, 6, 8, 2, 4};
-        int[] expected = {1, 2, 3, 4, 5, 6, 7, 8, 9};
-        sorter.bubbleSort(arr);
-        assertArrayEquals(expected, arr);
-    }
-    @Test
-    public void testBubbleSort3() {
-        BubbleSort sorter = new BubbleSort();
-        int[] arr = {10, -2, 0, -10, -20};
-        int[] expected = {-20, -10, -2, 0, 10};
-        sorter.bubbleSort(arr);
-        assertArrayEquals(expected, arr);
-    }
-    @Test
-    public void testBubbleSort4() {
-        BubbleSort sorter = new BubbleSort();
-        int[] arr = {1, 1, 1, 1, 1, 1};
-        int[] expected = {1, 1, 1, 1, 1, 1};
-        sorter.bubbleSort(arr);
-        assertArrayEquals(expected, arr);
     }
 }
 </t>
@@ -2187,12 +1987,6 @@
   </si>
   <si>
     <t>package de.goals.testing; // nicht entfernen
-public class Leser {
-// Ihre Loesung
-}</t>
-  </si>
-  <si>
-    <t>package de.goals.testing; // nicht entfernen
 public abstract class Flugzeug {
     protected String hersteller;            // Herstellername
     protected int maxSpeed;                 // Max. Geschwindigkeit
@@ -2244,12 +2038,6 @@
   <si>
     <t>package de.goals.testing; // nicht entfernen
 public class Kegel {
-// Ihre Loesung
-}</t>
-  </si>
-  <si>
-    <t>package de.goals.testing; // nicht entfernen
-public class Formen {
 // Ihre Loesung
 }</t>
   </si>
@@ -2334,26 +2122,6 @@
 &lt;br /&gt;</t>
   </si>
   <si>
-    <t>Betrachten Sie das folgende Klassendiagramm:
-a) Laden Sie sich die Klasse Datum (Datum.java) herunter. Machen Sie sich mit den Eigenschaften der Klasse vertraut, in dem Sie sich den Quelltext anschauen. Schauen Sie sich die Eigenschaften der Klasse Calendar in der Java-API an.
-b) Setzen Sie nun das oben stehende UML-Klassendiagramm in Java um, unter der Verwendung der Klasse Datum. Implementieren Sie auch die Methoden der Klassen Medium, Buch und DVD. Für die Berechnung des Strafgeldes bei Überziehung der Leihfristen gelten folgende Bestimmungen:
-- Bücher können 4 Wochen ausgeliehen werden, bei Überziehung 1 EUR Strafgeld pro angefangenen Überziehungstag.
-- DVDs können 1 Woche ausgeliehen werden, bei Überziehung 2 EUR Strafgeld pro angefangenen Überziehungstag
-Für die Berechnung der Differenztage zwischen dem Ausleihdatum und Heute implementieren Sie bitte die Methode calcDiffDays() der Klasse Datum. Nehmen Sie dazu an, dass jeder Monat 30 Tage hat und das Jahr 365 Tage.
-c) Schreiben Sie ein kleines Testprogramm (BibVerwaltung.java), das Objekte von den beiden Medien Buch und DVD erzeugt.</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Betrachten Sie das folgende Klassendiagramm:&lt;br /&gt;
-&lt;img src="/assets/taskImgs/Java_Bibliothek_Bib.jpg" alt="image"&gt;
-&lt;br /&gt;
-a) Laden Sie sich die Klasse Datum (Datum.java) herunter. Machen Sie sich mit den&amp;nbsp;Eigenschaften der Klasse vertraut, in dem Sie sich den Quelltext anschauen. Schauen Sie sich&amp;nbsp;die Eigenschaften der Klasse Calendar in der Java-API an.&lt;/p&gt;
-&lt;p&gt;b) Setzen Sie nun das oben stehende UML-Klassendiagramm in Java um, unter der&amp;nbsp;Verwendung der Klasse Datum. Implementieren Sie auch die Methoden der Klassen&amp;nbsp;Medium, Buch und DVD. Für die Berechnung des Strafgeldes bei &amp;Uuml;berziehung der&amp;nbsp;Leihfristen gelten folgende Bestimmungen:&lt;/p&gt;
-&lt;p&gt;- Bücher k&amp;ouml;nnen 4 Wochen ausgeliehen werden, bei &amp;Uuml;berziehung 1 EUR Strafgeld pro&amp;nbsp;angefangenen &amp;Uuml;berziehungstag.&lt;br /&gt;
-- DVDs k&amp;ouml;nnen 1 Woche ausgeliehen werden, bei &amp;Uuml;berziehung 2 EUR Strafgeld pro&amp;nbsp;angefangenen &amp;Uuml;berziehungstag&lt;/p&gt;
-&lt;p&gt;Für die Berechnung der Differenztage zwischen dem Ausleihdatum und Heute&amp;nbsp;implementieren Sie bitte die Methode calcDiffDays() der Klasse Datum. Nehmen Sie&amp;nbsp;dazu an, dass jeder Monat 30 Tage hat und das Jahr 365 Tage.&lt;/p&gt;
-&lt;p&gt;c) Schreiben Sie ein kleines Testprogramm (BibVerwaltung.java), das Objekte von den&amp;nbsp;beiden Medien Buch und DVD erzeugt.&lt;/p&gt;</t>
-  </si>
-  <si>
     <t>Verwenden Sie das Code-Gerüst aus Java_GGT.java und implementieren Sie die Methode ggT().
 Die Methode ggT berechnet den größten gemeinsamen Teiler zweier natürlicher Zahlen a und b. Verwenden Sie dazu den folgenden Algorithmus:
 1. setze m=a und n=b
@@ -2386,20 +2154,6 @@
     fahren() erhält die Strecke als Parameter und errechnet dann ob der aktuelle Tankinhalt ausreicht die Strecke zu fahren. Wenn das nicht der Fall ist, gibt die Methode false zurück. Wenn es möglich ist, dann berechnet die Methode den Kraftstoffverbrauch für die gefahrenen Kilometer und zieht die Liter von der aktuellen Kraftstoffmenge ab. Außerdem wird der Kilometerstand entsprechend erhöht. Die Methode gibt dann true zurück. 
 Implementieren Sie die Klasse KFZ in Java. Selbstverständlich können Sie auch noch weitere Methoden implementieren. 
 Implementieren Sie eine neue Test-Klasse AppAuto, in der Autos erzeugt werden und diese fahren bzw. tanken lässt. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Schreiben Sie eine Klasse Konto, die ein Bankkonto realisiert. Attribute für das Bankkonto sind der Name und Vorname des Kontoinhabers, die Kontonummer (IBAN), der Kontostand, sowie ein Limit, bis zu dem das Konto überzogen werden darf.
-Erstellen Sie einen oder mehrere geeignete Konstruktoren! Auf jeden Fall erstellen Sie einen Konstruktor:
-Konto(String Vorname, String Name, String kontonummer)
-Dieser Konstruktor dient dazu einen Neukunden zu initialisieren. 
-Erstellen Sie Methoden für folgende Operationen:
-    String toString(): Rückgabe aller Kontodaten eines Kunden in der Form (z.B.):
-    Kunde: Sarah Müller, Konto: DE87123456782435465711, Stand: 123.45, Limit: 1000.00
-    einzahlen(Betrag): Einzahlung eines Betrages
-    auszahlen(): Auszahlung eines Betrages mit Überprüfung ob ggf. Limit überschritten wurde. In dem Falle wird dann nur die Summe bis zum Limit ausgezahlt.
-    double Kontostand(): Abfrage des Kontostandes.
-    setLimit(Limit): setzte das Limit auf einen neuen Betrag. 
-Erstellen Sie eine Test-Klasse AppBank in der die Konten der Kunden verwaltet werden. </t>
   </si>
   <si>
     <t xml:space="preserve">Betrachten Sie das folgende UML-Diagramm:
@@ -2447,48 +2201,9 @@
 Schreiben Sie eine neue Test-Klasse AppRadio die in ihrem main()-Part ein Objekt der Klasse Radio erzeugt und in der Sie dann die Methoden testweise aufrufen können. </t>
   </si>
   <si>
-    <t>Im Rahmen einer Softwareentwicklung für die einheitliche Verwaltung von Flugzeugen wurde die Klasse Flugzeug entwickelt (siehe Flugzeug.java). 
-Ausgehend von dieser Klasse sind zwei Klassen Verkehrsflugzeug und Doppeldecker zu erzeugen. Diese sollen folgende Spezifikationen erfüllen:
-Klasse Verkehrsflugzeug:
-    Ein Verkehrsflugzeug ist ein Flugzeug, das genau ein Flügelpaar sowie eine zusätzliche Variable für die Anzahl der Passagiere hat. 
-    Ein Verkehrsflugzeug fliegt keine Loopings. Stellen Sie deshalb sicher, dass die Methode getLooping immer false zurückgibt, auch in allen Unterklassen von Verkehrsflugzeug.
-    Ein Verkehrsflugzeug-Objekt kann mit Angabe des Herstellers (String), der maximalen Geschwindigkeit (int), der Immatrikulationsnummer (String) und der Anzahl der Passagiere (int) erzeugt werden.
-    Die Klasse Verkehrsflugzeug hat die Methoden getAnzahlPassagiere und setAnzahlPassagiere zum Abfragen und Setzen der Anzahl der Passagiere.
-Klasse Doppeldecker:
-    Ein Doppeldecker ist ein Flugzeug, das genau zwei Flügelpaare hat.
-    Weiter ist ein Doppeldecker akrobatiktauglich, d.h. man kann damit Loopings fliegen. Für einen Looping muss der Doppeldecker eine Mindestgeschwindigkeit von 320 km/h erreichen. Definieren Sie dafür eine Konstante LOOPINGSPEED. Die Methode getLooping soll true zurückgeben, falls die zulässige max. Geschwindigkeit (maxSpeed) grösser LOOPINGSPEED ist.
-    Die Klasse Doppeldecker hat eine Variable offenesCockpit vom Typ boolean. Sie gibt an, ob der Doppeldecker ein offenes oder geschlossenes Cockpit hat. Nachdem offenesCockpit gesetzt worden ist, darf sie nicht mehr verändert werden. Der Wert des Attributes darf gelesen werden.
-    Ein Doppeldecker-Objekt kann durch 2 Konstruktoren initianlisert werden:
-        Der 1. Konstruktor hat folgende Parameter: Hersteller (String), maximale Geschwindigkeit (int), die Immatrikulationsnummer (String) und einen boolean offenesCockpit, der angibt, ob der Doppeldecker ein offenes oder geschlossenes Cockpit hat.
-        Der 2. Konstruktor hat folgende Parameter: Hersteller (String), maximale Geschwindigkeit (int), die Immatrikulationsnummer (int). Der Defaultwert für offenesCockpit bei einem Doppeldecker ist true.
-    Die Klasse Doppeldecker soll nicht erweiterbar sein.
-    Modellieren Sie die beschriebenen Klassen in einem UML-Klassendiagramm.
-    Implementieren Sie die Klassen Verkehrsflugzeug und Doppeldecker anhand der o.a. Eigenschaften.
-    Implementieren Sie eine main-Klasse Airline in der Sie beliebig Objekte der Klassen Verkehrsflugzeug und Doppeldecker anlegen. Des Weiteren legen Sie eine ArrayList flug wie folgt an:
-       ArrayList&lt;Flugzeug&gt; flug= new ArrayList&lt;Flugzeug&gt;();
-    Fügen Sie der Arraylist per flug.add() die zuvor erzeugten Objekte der Klassen Verkehrsflugzeug und Doppeldecker hinzu! Sollte dies zu Fehlern führen, dann ist ihre Implementierung der Klassen nicht korrekt!! :-) 
-    Geben Sie die Daten der in der ArrayList gespeicherten Objekten aus, in dem Sie die entsprechenden Methoden aufrufen. 
-Hinweis zur Bewertung: Ihre main()-Klasse Airline wird in Tutor Kai durch eine Testklasse ersetzt. Ihre main()-Klasse dient nur dazu das Sie Ihre Implementierungen der Klassen Verkehrsflugzeug und Doppeldecker testen können. Laden Sie dennoch auch die Airline.java mit hoch!</t>
-  </si>
-  <si>
     <t xml:space="preserve">Eine quadratische Pyramide und Kegel besitzen eine Grundfläche, die durch die Angabe einer einzigen Länge bestimmt ist (beim Kegel der Radius), und eine Höhe. Aus diesen Größen lassen sich Volumen und Oberfläche dieser Körper berechnen.
 Implementieren Sie eine geeignete abstrakte Klasse Koerper und leiten Sie die Klassen Pyramide und Kegel ab. Implementieren Sie in der Klasse Koerper einen Konstruktor mit den beiden Werten für die Länge und die Höhe. 
 Die Berechnung des Volumens und der Oberfläche und die Rückgabe der Ergebnisse (double-Werte) erfolgt durch getVolumen() und getFlaeche(), die als abstrakte Methoden in der Klasse Koerper definiert sind und in den jeweiligen Klassen implementiert werden! Erstellen Sie ein main() Programm  Formen.java zum Testen der Klassen. </t>
-  </si>
-  <si>
-    <t>Schreiben Sie ein Java-Programm MyThread.java, das die Summe aller Zahlen eines vorgegebenen int-Arrays mit Hilfe von zwei Threads berechnet. Dazu wird das Array jeweils zur Hälfte auf die beiden Threads verteilt. Jeder Thread berechnet seinen Bereich für sich. Nach Beendigung der Threads soll das Hauptprogramm die Ergebnisse aus dem Objekt lesen, die Summe berechnen und das Ergebnis ausgeben.
-Verwenden Sie das Programmgerüst aus MyThread.java für Ihre Lösung:
-public class MyThread {
-    public static void main(String[] args) {
-        int[] a={1,2,3,4,5,6,7,8,9,10};
-        ArrayCalc a1 = new ArrayCalc(a,0,6);
-        ArrayCalc a2 = new ArrayCalc(a,7,9);
-            //Ihre Loesung
-        System.out.println("Summe:"+(a1.getSumme()+a2.getSumme()));
-    }
-}
-Erstellen Sie eine Klasse ArrayCalc (ArrayCalc.java), die die Berechnung für einen Teil des Arrays übernimmt!
-Hinweis: Machen Sie sich mit der join()-Methode der Klasse Thread vertraut!</t>
   </si>
   <si>
     <t>6, 7</t>
@@ -2951,40 +2666,6 @@
 &lt;/ul&gt;
 &lt;p&gt;&lt;br /&gt;
 &amp;nbsp;&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>Im Rahmen einer Softwareentwicklung f&amp;uuml;r die einheitliche Verwaltung von Flugzeugen wurde die Klasse&amp;nbsp;&lt;em&gt;Flugzeug&amp;nbsp;&lt;/em&gt;entwickelt&amp;nbsp;(siehe Flugzeug.java).&amp;nbsp;
-&lt;p&gt;Ausgehend von dieser Klasse sind zwei Klassen&amp;nbsp;&lt;em&gt;Verkehrsflugzeug&amp;nbsp;&lt;/em&gt;und&amp;nbsp;&lt;em&gt;Doppeldecker&amp;nbsp;&lt;/em&gt;zu erzeugen. Diese sollen folgende Spezifikationen erf&amp;uuml;llen:&lt;/p&gt;
-&lt;p&gt;Klasse&amp;nbsp;&lt;em&gt;Verkehrsflugzeug&lt;/em&gt;:&lt;/p&gt;
-&lt;ul&gt;
-	&lt;li&gt;Ein Verkehrsflugzeug ist ein Flugzeug, das genau ein Fl&amp;uuml;gelpaar sowie eine zus&amp;auml;tzliche Variable f&amp;uuml;r die Anzahl der Passagiere hat.&amp;nbsp;&lt;/li&gt;
-	&lt;li&gt;Ein Verkehrsflugzeug fliegt keine Loopings. Stellen Sie deshalb sicher, dass die Methode&amp;nbsp;&lt;em&gt;getLooping&amp;nbsp;&lt;/em&gt;immer false zur&amp;uuml;ckgibt, auch in allen Unterklassen von Verkehrsflugzeug.&lt;/li&gt;
-	&lt;li&gt;Ein Verkehrsflugzeug-Objekt kann mit Angabe des Herstellers (String), der maximalen Geschwindigkeit (int), der Immatrikulationsnummer (String) und der Anzahl der Passagiere (int) erzeugt werden.&lt;/li&gt;
-	&lt;li&gt;Die Klasse Verkehrsflugzeug hat die Methoden&amp;nbsp;&lt;em&gt;getAnzahlPassagiere&amp;nbsp;&lt;/em&gt;und&amp;nbsp;&lt;em&gt;setAnzahlPassagiere&amp;nbsp;&lt;/em&gt;zum Abfragen und Setzen der Anzahl der Passagiere.&lt;/li&gt;
-&lt;/ul&gt;
-&lt;p&gt;Klasse&amp;nbsp;&lt;em&gt;Doppeldecker&lt;/em&gt;:&lt;/p&gt;
-&lt;ul&gt;
-	&lt;li&gt;Ein Doppeldecker ist ein Flugzeug, das genau zwei Fl&amp;uuml;gelpaare hat.&lt;/li&gt;
-	&lt;li&gt;Weiter ist ein Doppeldecker akrobatiktauglich, d.h. man kann damit Loopings fliegen. F&amp;uuml;r einen Looping muss der Doppeldecker eine Mindestgeschwindigkeit von 320 km/h erreichen. Definieren Sie daf&amp;uuml;r eine Konstante&amp;nbsp;&lt;em&gt;LOOPINGSPEED&lt;/em&gt;. Die Methode&amp;nbsp;&lt;em&gt;getLooping&amp;nbsp;&lt;/em&gt;soll true zur&amp;uuml;ckgeben, falls die zul&amp;auml;ssige max. Geschwindigkeit (&lt;em&gt;maxSpeed&lt;/em&gt;) gr&amp;ouml;sser LOOPINGSPEED ist.&lt;/li&gt;
-	&lt;li&gt;Die Klasse Doppeldecker hat eine Variable&amp;nbsp;&lt;em&gt;offenesCockpit&amp;nbsp;&lt;/em&gt;vom Typ boolean. Sie gibt an, ob der Doppeldecker ein offenes oder geschlossenes Cockpit hat. Nachdem&amp;nbsp;&lt;em&gt;offenesCockpit&amp;nbsp;&lt;/em&gt;gesetzt worden ist, darf sie nicht mehr ver&amp;auml;ndert werden. Der Wert des Attributes darf gelesen werden.&lt;/li&gt;
-	&lt;li&gt;Ein Doppeldecker-Objekt kann durch 2 Konstruktoren initianlisert werden:
-	&lt;ul&gt;
-		&lt;li&gt;Der 1. Konstruktor hat folgende Parameter: Hersteller (String), maximale Geschwindigkeit (int), die Immatrikulationsnummer (String) und einen boolean offenesCockpit, der angibt, ob der Doppeldecker ein offenes oder geschlossenes Cockpit hat.&lt;/li&gt;
-		&lt;li&gt;Der 2. Konstruktor hat folgende Parameter: Hersteller (String), maximale Geschwindigkeit (int), die Immatrikulationsnummer (int). Der Defaultwert f&amp;uuml;r offenesCockpit bei einem Doppeldecker ist true.&lt;/li&gt;
-	&lt;/ul&gt;
-	&lt;/li&gt;
-	&lt;li&gt;Die Klasse Doppeldecker soll nicht erweiterbar sein.&lt;/li&gt;
-&lt;/ul&gt;
-&lt;ol&gt;
-	&lt;li&gt;Modellieren Sie die beschriebenen Klassen in einem UML-Klassendiagramm.;&lt;/li&gt;
-	&lt;li&gt;Implementieren Sie die Klassen&amp;nbsp;&lt;em&gt;Verkehrsflugzeug&amp;nbsp;&lt;/em&gt;und&amp;nbsp;&lt;em&gt;Doppeldecker &lt;/em&gt;anhand der o.a. Eigenschaften.&lt;/li&gt;
-	&lt;li&gt;Implementieren Sie eine main-Klasse Airline in der Sie beliebig Objekte der Klassen Verkehrsflugzeug und Doppeldecker anlegen. Des Weiteren legen Sie eine ArrayList flug wie folgt an:&lt;br /&gt;
-	&amp;nbsp; &amp;nbsp;ArrayList&lt;Flugzeug&gt; flug= new ArrayList&lt;Flugzeug&gt;();&lt;br /&gt;
-	F&amp;uuml;gen Sie der Arraylist per flug.add() die zuvor erzeugten Objekte der Klassen Verkehrsflugzeug und Doppeldecker hinzu! Sollte dies zu Fehlern f&amp;uuml;hren, dann ist ihre Implementierung der Klassen nicht korrekt!! :-)&amp;nbsp;&lt;/li&gt;
-	&lt;li&gt;Geben Sie die Daten der in der ArrayList gespeicherten Objekten aus, in dem Sie die entsprechenden Methoden aufrufen.&amp;nbsp;&lt;/li&gt;
-&lt;/ol&gt;
-&lt;strong&gt;Hinweis zur Bewertung: Ihre main()-Klasse Airline wird durch Tutor Kai durch eine Testklasse ersetzt. Ihre main()-Klasse dient nur dazu das Sie Ihre Implementierungen der Klassen Verkehrsflugzeug und Doppeldecker testen k&amp;ouml;nnen. Laden Sie dennoch auch die Airline.java mit hoch!&lt;br /&gt;
-&lt;br /&gt;&lt;/strong&gt;</t>
   </si>
   <si>
     <t>&lt;div&gt;
@@ -3059,19 +2740,6 @@
   </si>
   <si>
     <t>&lt;div&gt;
-  &lt;p&gt;&lt;strong&gt;Schreiben Sie eine Klasse Konto, die ein Bankkonto realisiert.&lt;/strong&gt; Attribute für das Bankkonto sind der Name und Vorname des Kontoinhabers, die Kontonummer (IBAN), der Kontostand, sowie ein Limit, bis zu dem das Konto überzogen werden darf.&lt;/p&gt;
-  &lt;p&gt;&lt;strong&gt;Erstellen Sie einen oder mehrere geeignete Konstruktoren!&lt;/strong&gt; Auf jeden Fall erstellen Sie einen Konstruktor:&lt;br&gt;Konto(String Vorname, String Name, String kontonummer)&lt;br&gt;Dieser Konstruktor dient dazu einen Neukunden zu initialisieren.&lt;/p&gt;
-  &lt;p&gt;&lt;strong&gt;Erstellen Sie Methoden für folgende Operationen:&lt;/strong&gt;&lt;/p&gt;
-  &lt;p&gt;&lt;em&gt;String toString():&lt;/em&gt; Rückgabe aller Kontodaten eines Kunden in der Form (z.B.):&lt;br&gt;Kunde: Sarah Müller, Konto: DE87123456782435465711, Stand: 123.45, Limit: 1000.00&lt;/p&gt;
-  &lt;p&gt;&lt;em&gt;einzahlen(Betrag):&lt;/em&gt; Einzahlung eines Betrages&lt;/p&gt;
-  &lt;p&gt;&lt;em&gt;auszahlen():&lt;/em&gt; Auszahlung eines Betrages mit Überprüfung ob ggf. Limit überschritten wurde. In dem Falle wird dann nur die Summe bis zum Limit ausgezahlt.&lt;/p&gt;
-  &lt;p&gt;&lt;em&gt;double Kontostand():&lt;/em&gt; Abfrage des Kontostandes.&lt;/p&gt;
-  &lt;p&gt;&lt;em&gt;setLimit(Limit):&lt;/em&gt; setzte das Limit auf einen neuen Betrag.&lt;/p&gt;
-  &lt;p&gt;&lt;strong&gt;Erstellen Sie eine Test-Klasse AppBank in der die Konten der Kunden verwaltet werden.&lt;/strong&gt;&lt;/p&gt;
-&lt;/div&gt;</t>
-  </si>
-  <si>
-    <t>&lt;div&gt;
     &lt;p&gt;&lt;strong&gt;Implementieren Sie eine Klasse Radio mit folgenden Attributen:&lt;/strong&gt;&lt;/p&gt;
     &lt;p&gt;eingeschaltet, wenn ein Radio an oder aus ist.&lt;br&gt;
     lautstaerke, wie laut spielt das Radio Musik? (Die Lautstärke soll nur im Bereich von 0 bis 10 liegen.)&lt;br&gt;
@@ -3089,24 +2757,486 @@
 &lt;/div&gt;</t>
   </si>
   <si>
-    <t>&lt;p&gt;Eine quadratische Pyramide&amp;nbsp;und Kegel besitzen eine Grundfl&amp;auml;che, die durch die Angabe einer einzigen L&amp;auml;nge bestimmt ist (beim Kegel der Radius), und eine H&amp;ouml;he.&amp;nbsp;Aus diesen Gr&amp;ouml;&amp;szlig;en lassen sich Volumen und Oberfl&amp;auml;che dieser K&amp;ouml;rper&amp;nbsp;berechnen.&lt;/p&gt;
-&lt;p&gt;Implementieren Sie eine geeignete abstrakte Klasse KoerperPyramideKegelKoerpergetVolumen()getFlaeche()main()Formen.java Formen.javaKoerper.java,Pyramide.javaKegel.java</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Schreiben Sie ein Java-Programm MyThread.java, das die Summe aller Zahlen eines vorgegebenen int-Arrays mit Hilfe von zwei Threads berechnet. Dazu wird das Array jeweils zur H&amp;auml;lfte auf die beiden Threads verteilt. Jeder Thread berechnet seinen Bereich f&amp;uuml;r sich. Nach Beendigung der Threads soll das Hauptprogramm die Ergebnisse aus dem Objekt lesen, die Summe berechnen und das Ergebnis ausgeben.&lt;/p&gt;
-&lt;p&gt;Verwenden Sie das Programmger&amp;uuml;st aus MyThread.java f&amp;uuml;r Ihre L&amp;ouml;sung:&lt;/p&gt;
-&lt;p&gt;public class MyThread {&lt;br /&gt;
-&amp;nbsp;&amp;nbsp; &amp;nbsp;public static void main(String[] args) {&lt;br /&gt;
-&amp;nbsp;&amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp;int[] a={1,2,3,4,5,6,7,8,9,10};&lt;br /&gt;
-&amp;nbsp;&amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp;ArrayCalc a1 = new ArrayCalc(a,0,6);&lt;br /&gt;
-&amp;nbsp;&amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp;ArrayCalc a2 = new ArrayCalc(a,7,9);&lt;br /&gt;
-&amp;nbsp;&amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp;&lt;b&gt;//Ihre Loesung&lt;br /&gt;
-&amp;nbsp;&amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp;&lt;/b&gt;System.out.println(&amp;quot;Summe:&amp;quot;+(a1.getSumme()+a2.getSumme()));&lt;br /&gt;
-&amp;nbsp;&amp;nbsp; &amp;nbsp;}&lt;br /&gt;
+    <t>BubbleSortTest.java</t>
+  </si>
+  <si>
+    <t>FahrzeugTest.java</t>
+  </si>
+  <si>
+    <t xml:space="preserve">package de.goals.testing;
+import org.junit.jupiter.api.Test;
+import static org.junit.jupiter.api.Assertions.assertEquals;
+public class AppAutoTest {
+    private int punkte = 0;
+    private KFZ porsche = new KFZ("AK-CA 740", 24500, 50, 8, 0);
+    public int getResult() {
+        return punkte;
+    }
+    @Test
+    public void testGetKMstand() {
+        assertEquals(24500, porsche.getKMstand(), "Fehler beim Aufruf der Methode getKMstand()");
+        punkte += 25;
+        System.out.println("Test 1 erfolgreich " + porsche.getKMstand());
+    }
+    @Test
+    public void testTanken() {
+        porsche.tanken(60);
+        assertEquals(50, porsche.getTankinhalt(), "Fehler beim Aufruf der Methode getTankinhalt()");
+        punkte += 25;
+        System.out.println("Test 2 erfolgreich " + porsche.getTankinhalt());
+    }
+    @Test
+    public void testFahren() {
+        porsche.tanken(60);
+        boolean ret = porsche.fahren(150);
+        assertEquals(24650, porsche.getKMstand(), "Fehler beim Aufruf der Methode getKMstand() oder fahren()");
+        punkte += 50;
+        System.out.println("Test 3 erfolgreich " + porsche.getKMstand());
+    }
+}
+</t>
+  </si>
+  <si>
+    <t>Betrachten Sie das folgende Klassendiagramm:
+a) Machen Sie sich mit den Eigenschaften der  Klasse Datum  vertraut, in dem Sie sich den Quelltext anschauen. Schauen Sie sich die Eigenschaften der Klasse Calendar in der Java-API an.
+b) Setzen Sie nun das oben stehende UML-Klassendiagramm in Java um, unter der Verwendung der Klasse Datum. Implementieren Sie auch die Methoden der Klassen Medium, Buch und DVD. Für die Berechnung des Strafgeldes bei Überziehung der Leihfristen gelten folgende Bestimmungen:
+- Bücher können 4 Wochen ausgeliehen werden, bei Überziehung 1 EUR Strafgeld pro angefangenen Überziehungstag.
+- DVDs können 1 Woche ausgeliehen werden, bei Überziehung 2 EUR Strafgeld pro angefangenen Überziehungstag
+Für die Berechnung der Differenztage zwischen dem Ausleihdatum und Heute implementieren Sie bitte die Methode calcDiffDays() der Klasse Datum. Nehmen Sie dazu an, dass jeder Monat 30 Tage hat und das Jahr 365 Tage.
+c) Schreiben Sie ein kleines Testprogramm (BibVerwaltung.java), das Objekte von den beiden Medien Buch und DVD erzeugt.</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Betrachten Sie das folgende Klassendiagramm:&lt;br /&gt;
+&lt;img src="/assets/taskImgs/Java_Bibliothek_Bib.jpg" alt="image"&gt;
+&lt;br /&gt;
+a) Machen Sie sich mit den&amp;nbsp;Eigenschaften der  Klasse Datum vertraut, in dem Sie sich den Quelltext anschauen. Schauen Sie sich&amp;nbsp;die Eigenschaften der Klasse Calendar in der Java-API an.&lt;/p&gt;
+&lt;p&gt;b) Setzen Sie nun das oben stehende UML-Klassendiagramm in Java um, unter der&amp;nbsp;Verwendung der Klasse Datum. Implementieren Sie auch die Methoden der Klassen&amp;nbsp;Medium, Buch und DVD. Für die Berechnung des Strafgeldes bei &amp;Uuml;berziehung der&amp;nbsp;Leihfristen gelten folgende Bestimmungen:&lt;/p&gt;
+&lt;p&gt;- Bücher k&amp;ouml;nnen 4 Wochen ausgeliehen werden, bei &amp;Uuml;berziehung 1 EUR Strafgeld pro&amp;nbsp;angefangenen &amp;Uuml;berziehungstag.&lt;br /&gt;
+- DVDs k&amp;ouml;nnen 1 Woche ausgeliehen werden, bei &amp;Uuml;berziehung 2 EUR Strafgeld pro&amp;nbsp;angefangenen &amp;Uuml;berziehungstag&lt;/p&gt;
+&lt;p&gt;Für die Berechnung der Differenztage zwischen dem Ausleihdatum und Heute&amp;nbsp;implementieren Sie bitte die Methode calcDiffDays() der Klasse Datum. Nehmen Sie&amp;nbsp;dazu an, dass jeder Monat 30 Tage hat und das Jahr 365 Tage.&lt;/p&gt;
+&lt;p&gt;c) Schreiben Sie ein kleines Testprogramm (BibVerwaltung.java), das Objekte von den&amp;nbsp;beiden Medien Buch und DVD erzeugt.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Schreiben Sie eine Klasse Konto, die ein Bankkonto realisiert. Attribute für das Bankkonto sind der Name und Vorname des Kontoinhabers, die Kontonummer (IBAN), der Kontostand, sowie ein Limit, bis zu dem das Konto überzogen werden darf.
+Erstellen Sie einen oder mehrere geeignete Konstruktoren! Auf jeden Fall erstellen Sie einen Konstruktor:
+Konto(String Vorname, String Name, String kontonummer)
+Dieser Konstruktor dient dazu einen Neukunden zu initialisieren. 
+Erstellen Sie Methoden für folgende Operationen:
+    String toString(): Rückgabe aller Kontodaten eines Kunden in der Form (z.B.):
+    Kunde: Sarah Müller, Konto: DE87123456782435465711, Stand: 123.45, Limit: 1000.00
+    einzahlen(Betrag): Einzahlung eines Betrages
+    auszahlen(): Auszahlung eines Betrages mit Überprüfung ob ggf. Limit überschritten wurde. In dem Falle wird dann nur die Summe bis zum Limit ausgezahlt.
+    double getKontostand(): Abfrage des Kontostandes.
+    setLimit(Limit): setzte das Limit auf einen neuen Betrag. 
+Erstellen Sie eine Test-Klasse AppBank in der die Konten der Kunden verwaltet werden. </t>
+  </si>
+  <si>
+    <t>&lt;div&gt;
+  &lt;p&gt;&lt;strong&gt;Schreiben Sie eine Klasse Konto, die ein Bankkonto realisiert.&lt;/strong&gt; Attribute für das Bankkonto sind der Name und Vorname des Kontoinhabers, die Kontonummer (IBAN), der Kontostand, sowie ein Limit, bis zu dem das Konto überzogen werden darf.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Erstellen Sie einen oder mehrere geeignete Konstruktoren!&lt;/strong&gt; Auf jeden Fall erstellen Sie einen Konstruktor:&lt;br&gt;Konto(String Vorname, String Name, String kontonummer)&lt;br&gt;Dieser Konstruktor dient dazu einen Neukunden zu initialisieren.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Erstellen Sie Methoden für folgende Operationen:&lt;/strong&gt;&lt;/p&gt;
+  &lt;p&gt;&lt;em&gt;String toString():&lt;/em&gt; Rückgabe aller Kontodaten eines Kunden in der Form (z.B.):&lt;br&gt;Kunde: Sarah Müller, Konto: DE87123456782435465711, Stand: 123.45, Limit: 1000.00&lt;/p&gt;
+  &lt;p&gt;&lt;em&gt;einzahlen(Betrag):&lt;/em&gt; Einzahlung eines Betrages&lt;/p&gt;
+  &lt;p&gt;&lt;em&gt;auszahlen():&lt;/em&gt; Auszahlung eines Betrages mit Überprüfung ob ggf. Limit überschritten wurde. In dem Falle wird dann nur die Summe bis zum Limit ausgezahlt.&lt;/p&gt;
+  &lt;p&gt;&lt;em&gt;double getKontostand():&lt;/em&gt; Abfrage des Kontostandes.&lt;/p&gt;
+  &lt;p&gt;&lt;em&gt;setLimit(Limit):&lt;/em&gt; setzte das Limit auf einen neuen Betrag.&lt;/p&gt;
+  &lt;p&gt;&lt;strong&gt;Erstellen Sie eine Test-Klasse AppBank in der die Konten der Kunden verwaltet werden.&lt;/strong&gt;&lt;/p&gt;
+&lt;/div&gt;</t>
+  </si>
+  <si>
+    <t>package de.goals.testing;
+import org.junit.jupiter.api.Test;
+import static org.junit.jupiter.api.Assertions.assertEquals;
+public class AppBankTest {
+    @Test
+    public void testToString() {
+        Konto konto = new Konto("Andreas", "Hoffmann", "DE232212442");
+        konto.einzahlen(100);
+        konto.setLimit(500);
+        String expected = "Kunde: Andreas Hoffmann, Konto: DE232212442, Stand: 100.00, Limit: 500.00";
+        assertEquals(expected, konto.toString(), "Fehler in der toString() Methode");
+    }
+    @Test
+    public void testEinzahlen() {
+        Konto konto = new Konto("Max", "Mustermann", "DE12345678901234567890");
+        konto.einzahlen(100);
+        double expectedKontostand = 100.00;
+        assertEquals(expectedKontostand, konto.getKontostand(), "Fehler in der Einzahlen-Methode");
+    }
+    @Test
+    public void testAuszahlenWithinLimit() {
+        Konto konto = new Konto("Max", "Mustermann", "DE12345678901234567890");
+        konto.einzahlen(1000);
+        konto.auszahlen(500);
+        double expectedKontostand = 500.0;
+        assertEquals(expectedKontostand, konto.getKontostand(), "Fehler in der Auszahlen-Methode mit Betrag innerhalb des Limits");
+    }
+    @Test
+    public void testAuszahlenExceedingLimit() {
+        Konto konto = new Konto("Max", "Mustermann", "DE12345678901234567890");
+        konto.einzahlen(1000);
+        konto.setLimit(500); // Set the limit before withdrawing
+        konto.auszahlen(1500); // Versucht 1500 auszuzahlen, was über das Limit geht
+        double expectedKontostand = -500.0; // Kontostand sollte -Limit sein
+        assertEquals(expectedKontostand, konto.getKontostand(), "Fehler in der Auszahlen-Methode bei Überschreitung des Limits");
+    }
+    @Test
+    public void testSetLimit() {
+        Konto konto = new Konto("Max", "Mustermann", "DE12345678901234567890");
+        konto.setLimit(1000);
+        double expectedLimit = 1000.0;
+        assertEquals(expectedLimit, konto.getLimit(), "Fehler in der SetLimit-Methode");
+    }
 }</t>
   </si>
   <si>
-    <t>Schreiben Sie den Java Code für beide Klassen des UML-Diagramms, in eine Datei, erst Fahrzeug, dann Auto. Klasse Fahrzeug:
+    <t>Syntaxfehler: JA, Tests: NEIN
+Tests angepasst: Erneut überprüfen</t>
+  </si>
+  <si>
+    <t>package de.goals.testing;
+import org.junit.jupiter.api.Test;
+import static org.junit.jupiter.api.Assertions.assertEquals;
+public class AppPunktTest {
+    // Entfernen Sie die Punkte, wenn sie nicht benötigt werden.
+    private int punkte = 0;
+    public int getResult() {
+        return punkte;
+    }
+    @Test
+    public void testToString() {
+        Punkt p = new Punkt(3, 4);
+        String s = p.toString();
+        assertEquals("3/4", s);
+        punkte += 25;
+        System.out.println("Test 1 erfolgreich: " + s);
+    }
+    @Test
+    public void testSpiegelX() {
+        Punkt p = new Punkt(3, 4);
+        Punkt spiegelx = p.spiegelX();
+        String s = spiegelx.toString();
+        assertEquals("3/-4", s);
+        punkte += 25;
+        System.out.println("Test 2 erfolgreich: " + s);
+    }
+    @Test
+    public void testSpiegelUrsprung() {
+        Punkt p = new Punkt(3, 4);
+        Punkt spiegelUr = p.spiegelUrsprung();
+        String s = spiegelUr.toString();
+        assertEquals("-3/-4", s);
+        punkte += 50;
+        System.out.println("Test 3 erfolgreich: " + s);
+    }
+}</t>
+  </si>
+  <si>
+    <t>package de.goals.testing;
+import org.junit.Test;
+import static org.junit.Assert.*;
+public class BibVerwaltungTest {
+    @Test
+    public void testBerechneStrafgeldBuch() {
+        Buch buch = new Buch("Fussballfieber", "Manuel Neuer", 75);
+        buch.setAusleihdatum(new Datum(2020, 2, 1));
+        Datum heute = new Datum();
+        int tageUeberzogen = heute.calcDiffDays(buch.ausleihdatum) - 28;
+        double erwartetesStrafgeld = Math.max(0, tageUeberzogen) * 1.0;
+        assertEquals(erwartetesStrafgeld, buch.berechneStrafgeld(), 0.01);
+    }
+    @Test
+    public void testBerechneStrafgeldDVD() {
+        DVD dvd = new DVD("FussballfieberderFilm", "Manuel Neuer", 120);
+        dvd.setAusleihdatum(new Datum(2019, 2, 1));
+        Datum heute = new Datum();
+        int tageUeberzogen = heute.calcDiffDays(dvd.ausleihdatum) - 7;
+        double erwartetesStrafgeld = Math.max(0, tageUeberzogen) * 2.0;
+        assertEquals(erwartetesStrafgeld, dvd.berechneStrafgeld(), 0.01);
+    }
+}</t>
+  </si>
+  <si>
+    <t>package de.goals.testing; // nicht entfernen
+public class Leser {
+    // Ihre Loesung
+    public static void main(String[] args) {
+        Leser leser = new Leser(1, 12345, "Max Mustermann");
+        System.out.println("LeserID: " + leser.getLeserID());
+        System.out.println("Name: " + leser.getName());
+    }
+}</t>
+  </si>
+  <si>
+    <t>package de.goals.testing;
+import org.junit.jupiter.api.Test;
+import static org.junit.jupiter.api.Assertions.assertEquals;
+public class LeserTest {
+    @Test
+    public void testGetName() {
+        Leser l = new Leser(1, 56534, "Hoffmann");
+        String out = l.getName();
+        assertEquals("Hoffmann", out);
+        System.out.println("Test getName erfolgreich");
+    }
+    @Test
+    public void testSetName() {
+        Leser l = new Leser(1, 56534, "Hoffmann");
+        l.setName("Schneider");
+        String out = l.getName();
+        assertEquals("Schneider", out);
+        System.out.println("Test setName erfolgreich");
+    }
+    @Test
+    public void testGetLeserID() {
+        Leser l = new Leser(1, 56534, "Hoffmann");
+        int id = l.getLeserID();
+        assertEquals(1, id);
+        System.out.println("Test getLeserID erfolgreich");
+    }
+}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Im Rahmen einer Softwareentwicklung für die einheitliche Verwaltung von Flugzeugen wurde die Klasse Flugzeug entwickelt (siehe Flugzeug.java). 
+Ausgehend von dieser Klasse sind zwei Klassen Verkehrsflugzeug und Doppeldecker zu erzeugen. Diese sollen folgende Spezifikationen erfüllen:
+Klasse Verkehrsflugzeug:
+    Ein Verkehrsflugzeug ist ein Flugzeug, das genau ein Flügelpaar sowie eine zusätzliche Variable für die Anzahl der Passagiere hat. 
+    Ein Verkehrsflugzeug fliegt keine Loopings. Stellen Sie deshalb sicher, dass die Methode getLooping immer false zurückgibt, auch in allen Unterklassen von Verkehrsflugzeug.
+    Ein Verkehrsflugzeug-Objekt kann mit Angabe des Herstellers (String), der maximalen Geschwindigkeit (int), der Immatrikulationsnummer (String) und der Anzahl der Passagiere (int) erzeugt werden.
+    Die Klasse Verkehrsflugzeug hat die Methoden getAnzahlPassagiere und setAnzahlPassagiere zum Abfragen und Setzen der Anzahl der Passagiere.
+Klasse Doppeldecker:
+    Ein Doppeldecker ist ein Flugzeug, das genau zwei Flügelpaare hat.
+    Weiter ist ein Doppeldecker akrobatiktauglich, d.h. man kann damit Loopings fliegen. Für einen Looping muss der Doppeldecker eine Mindestgeschwindigkeit von 320 km/h erreichen. Definieren Sie dafür eine Konstante LOOPINGSPEED. Die Methode getLooping soll true zurückgeben, falls die zulässige max. Geschwindigkeit (maxSpeed) grösser LOOPINGSPEED ist.
+    Die Klasse Doppeldecker hat eine Variable offenesCockpit vom Typ boolean. Sie gibt an, ob der Doppeldecker ein offenes oder geschlossenes Cockpit hat. Nachdem offenesCockpit gesetzt worden ist, darf sie nicht mehr verändert werden. Der Wert des Attributes darf gelesen werden.
+    Ein Doppeldecker-Objekt kann durch 2 Konstruktoren initianlisert werden:
+        Der 1. Konstruktor hat folgende Parameter: Hersteller (String), maximale Geschwindigkeit (int), die Immatrikulationsnummer (String) und einen boolean offenesCockpit, der angibt, ob der Doppeldecker ein offenes oder geschlossenes Cockpit hat.
+        Der 2. Konstruktor hat folgende Parameter: Hersteller (String), maximale Geschwindigkeit (int), die Immatrikulationsnummer (int). Der Defaultwert für offenesCockpit bei einem Doppeldecker ist true.
+    Die Klasse Doppeldecker soll nicht erweiterbar sein.
+    Modellieren Sie die beschriebenen Klassen in einem UML-Klassendiagramm.
+    Implementieren Sie die Klassen Verkehrsflugzeug und Doppeldecker anhand der o.a. Eigenschaften.
+    Implementieren Sie eine main-Klasse Airline in der Sie beliebig Objekte der Klassen Verkehrsflugzeug und Doppeldecker anlegen. Des Weiteren legen Sie eine ArrayList flug wie folgt an:
+       ArrayList&lt;Flugzeug&gt; flug= new ArrayList&lt;Flugzeug&gt;();
+    Fügen Sie der Arraylist per flug.add() die zuvor erzeugten Objekte der Klassen Verkehrsflugzeug und Doppeldecker hinzu! Sollte dies zu Fehlern führen, dann ist ihre Implementierung der Klassen nicht korrekt!! :-) 
+    Geben Sie die Daten der in der ArrayList gespeicherten Objekten aus, in dem Sie die entsprechenden Methoden aufrufen. </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> &lt;p&gt;Im Rahmen einer Softwareentwicklung für die einheitliche Verwaltung von Flugzeugen wurde die Klasse &lt;em&gt;Flugzeug&lt;/em&gt; entwickelt (siehe Flugzeug.java).&lt;/p&gt;
+    &lt;p&gt;Ausgehend von dieser Klasse sind zwei Klassen &lt;em&gt;Verkehrsflugzeug&lt;/em&gt; und &lt;em&gt;Doppeldecker&lt;/em&gt; zu erzeugen. Diese sollen folgende Spezifikationen erfüllen:&lt;/p&gt;
+    &lt;p&gt;Klasse &lt;em&gt;Verkehrsflugzeug&lt;/em&gt;:&lt;/p&gt;
+    &lt;p&gt;- Ein Verkehrsflugzeug ist ein Flugzeug, das genau ein Flügelpaar sowie eine zusätzliche Variable für die Anzahl der Passagiere hat.&lt;/p&gt;
+    &lt;p&gt;- Ein Verkehrsflugzeug fliegt keine Loopings. Stellen Sie deshalb sicher, dass die Methode &lt;em&gt;getLooping&lt;/em&gt; immer false zurückgibt, auch in allen Unterklassen von Verkehrsflugzeug.&lt;/p&gt;
+    &lt;p&gt;- Ein Verkehrsflugzeug-Objekt kann mit Angabe des Herstellers (String), der maximalen Geschwindigkeit (int), der Immatrikulationsnummer (String) und der Anzahl der Passagiere (int) erzeugt werden.&lt;/p&gt;
+    &lt;p&gt;- Die Klasse Verkehrsflugzeug hat die Methoden &lt;em&gt;getAnzahlPassagiere&lt;/em&gt; und &lt;em&gt;setAnzahlPassagiere&lt;/em&gt; zum Abfragen und Setzen der Anzahl der Passagiere.&lt;/p&gt;
+    &lt;p&gt;Klasse &lt;em&gt;Doppeldecker&lt;/em&gt;:&lt;/p&gt;
+    &lt;p&gt;- Ein Doppeldecker ist ein Flugzeug, das genau zwei Flügelpaare hat.&lt;/p&gt;
+    &lt;p&gt;- Weiter ist ein Doppeldecker akrobatiktauglich, d.h. man kann damit Loopings fliegen. Für einen Looping muss der Doppeldecker eine Mindestgeschwindigkeit von 320 km/h erreichen. Definieren Sie dafür eine Konstante &lt;em&gt;LOOPINGSPEED&lt;/em&gt;. Die Methode &lt;em&gt;getLooping&lt;/em&gt; soll true zurückgeben, falls die zulässige max. Geschwindigkeit (&lt;em&gt;maxSpeed&lt;/em&gt;) größer LOOPINGSPEED ist.&lt;/p&gt;
+    &lt;p&gt;- Die Klasse Doppeldecker hat eine Variable &lt;em&gt;offenesCockpit&lt;/em&gt; vom Typ boolean. Sie gibt an, ob der Doppeldecker ein offenes oder geschlossenes Cockpit hat. Nachdem &lt;em&gt;offenesCockpit&lt;/em&gt; gesetzt worden ist, darf sie nicht mehr verändert werden. Der Wert des Attributes darf gelesen werden.&lt;/p&gt;
+    &lt;p&gt;- Ein Doppeldecker-Objekt kann durch 2 Konstruktoren initianlisiert werden:&lt;/p&gt;
+    &lt;p&gt;    a) Der 1. Konstruktor hat folgende Parameter: Hersteller (String), maximale Geschwindigkeit (int), die Immatrikulationsnummer (String) und einen boolean offenesCockpit, der angibt, ob der Doppeldecker ein offenes oder geschlossenes Cockpit hat.&lt;/p&gt;
+    &lt;p&gt;    b) Der 2. Konstruktor hat folgende Parameter: Hersteller (String), maximale Geschwindigkeit (int), die Immatrikulationsnummer (int). Der Defaultwert für offenesCockpit bei einem Doppeldecker ist true.&lt;/p&gt;
+    &lt;p&gt;- Die Klasse Doppeldecker soll nicht erweiterbar sein.&lt;/p&gt;
+    &lt;p&gt;1. Modellieren Sie die beschriebenen Klassen in einem UML-Klassendiagramm.&lt;/p&gt;
+    &lt;p&gt;2. Implementieren Sie die Klassen &lt;em&gt;Verkehrsflugzeug&lt;/em&gt; und &lt;em&gt;Doppeldecker&lt;/em&gt; anhand der o.a. Eigenschaften.&lt;/p&gt;
+    &lt;p&gt;3. Implementieren Sie eine main-Klasse Airline in der Sie beliebig Objekte der Klassen Verkehrsflugzeug und Doppeldecker anlegen. Des Weiteren legen Sie eine ArrayList flug wie folgt an:&lt;br /&gt;
+        &amp;nbsp; &amp;nbsp;ArrayList&amp;lt;Flugzeug&amp;gt; flug = new ArrayList&amp;lt;Flugzeug&amp;gt;();&lt;br /&gt;
+    Fügen Sie der Arraylist per flug.add() die zuvor erzeugten Objekte der Klassen Verkehrsflugzeug und Doppeldecker hinzu! Sollte dies zu Fehlern führen, dann ist ihre Implementierung der Klassen nicht korrekt!! :-)&lt;/p&gt;
+    &lt;p&gt;4. Geben Sie die Daten der in der ArrayList gespeicherten Objekten aus, in dem Sie die entsprechenden Methoden aufrufen.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>package de.goals.testing;
+import org.junit.jupiter.api.Test;
+import static org.junit.jupiter.api.Assertions.*;
+public class AirlineTest {
+    private int punkte = 0;
+    public int getResult() {
+        return punkte;
+    }
+    @Test
+    public void test1() {
+        Flugzeug f1 = new Doppeldecker("New", 123,  "98765GHS");
+        String immat = f1.getImmatNummer();
+        assertEquals("98765GHS", immat);
+        punkte += 50;
+        System.out.println("Test 1 erfolgreich");
+    }
+    @Test
+    public void test2() {
+        Flugzeug f2 = new Verkehrsflugzeug("Airbus", 900, "A8789HHU", 490);
+        int speed = f2.getMaxSpeed();
+        assertEquals(900, speed);
+        punkte += 50;
+        System.out.println("Test 2 erfolgreich");
+    }
+    @Test
+    public void test3() {
+        Verkehrsflugzeug vf = new Verkehrsflugzeug("Boeing", 500, "B1234XYZ", 320);
+        assertFalse(vf.getLooping(), "Verkehrsflugzeuge dürfen keine Loopings fliegen");
+        punkte += 50;
+        System.out.println("Test 3 erfolgreich");
+    }
+    @Test
+    public void test4() {
+        Doppeldecker dd = new Doppeldecker("Curtiss", 350, "C7890ABC");
+        assertTrue(dd.getLooping(), "Doppeldecker mit ausreichender Geschwindigkeit sollte Loopings fliegen können");
+        punkte += 50;
+        System.out.println("Test 4 erfolgreich");
+    }
+    @Test
+    public void test5() {
+        Doppeldecker ddLowSpeed = new Doppeldecker("Curtiss", 300, "C7890XYZ");
+        assertFalse(ddLowSpeed.getLooping(), "Doppeldecker mit unzureichender Geschwindigkeit sollte keine Loopings fliegen können");
+        punkte += 50;
+        System.out.println("Test 5 erfolgreich");
+    }
+}</t>
+  </si>
+  <si>
+    <t>Test erweitert und html korrigiert</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    &lt;p&gt;&lt;strong&gt;Grundlagen:&lt;/strong&gt; Eine quadratische Pyramide und ein Kegel haben eine Grundfläche, die durch die Angabe einer einzigen Länge bestimmt ist (beim Kegel der Radius), und eine Höhe. Aus diesen Größen lassen sich Volumen und Oberfläche dieser Körper berechnen.&lt;/p&gt;
+    &lt;p&gt;&lt;strong&gt;Programmieraufgabe:&lt;/strong&gt; Implementieren Sie eine geeignete abstrakte Klasse und mehrere Unterklassen, um die Volumen- und Oberflächenberechnungen durchzuführen. Folgende Klassen sind zu erstellen:&lt;/p&gt;
+    &lt;p&gt;&lt;strong&gt;Klassen und ihre Dateien:&lt;/strong&gt;&lt;/p&gt;
+    &lt;p&gt;&lt;code&gt;Koerper.java&lt;/code&gt; - Abstrakte Basis-Klasse für geometrische Körper.&lt;/p&gt;
+    &lt;p&gt;&lt;code&gt;Pyramide.java&lt;/code&gt; - Spezifische Klasse für die Pyramide.&lt;/p&gt;
+    &lt;p&gt;&lt;code&gt;Kegel.java&lt;/code&gt; - Spezifische Klasse für den Kegel.&lt;/p&gt;
+    &lt;p&gt;&lt;code&gt;Formen.java&lt;/code&gt; - Hauptklasse, die Methoden &lt;code&gt;getVolumen()&lt;/code&gt; und &lt;code&gt;getFlaeche()&lt;/code&gt; aufruft.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>package de.goals.testing; // nicht entfernen
+public class Formen {
+    public static void main(String[] args) {
+        Koerper pyramide = new Pyramide(5, 10);
+        System.out.println("Oberfläche der Pyramide: " + pyramide.getFlaeche());
+        // Hier koennen auch die anderen Klassen getestet werden
+    }
+}</t>
+  </si>
+  <si>
+    <t>Schreiben Sie ein Java-Programm MyThread.java, das die Summe aller Zahlen eines vorgegebenen int-Arrays mit Hilfe von zwei Threads berechnet. Dazu wird das Array jeweils zur Hälfte auf die beiden Threads verteilt. Jeder Thread berechnet seinen Bereich für sich. Nach Beendigung der Threads soll das Hauptprogramm die Ergebnisse aus dem Objekt lesen, die Summe berechnen und das Ergebnis ausgeben.
+Erstellen Sie eine Klasse ArrayCalc (ArrayCalc.java), die die Berechnung für einen Teil des Arrays übernimmt!
+Hinweis: Machen Sie sich mit der join()-Methode der Klasse Thread vertraut!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    &lt;p&gt;&lt;b&gt;Aufgabenstellung:&lt;/b&gt;&lt;br&gt;
+    Schreiben Sie ein Java-Programm &lt;b&gt;MyThread.java&lt;/b&gt;, das die Summe aller Zahlen eines vorgegebenen &lt;i&gt;int&lt;/i&gt;-Arrays mit Hilfe von zwei Threads berechnet. Dazu wird das Array jeweils zur Hälfte auf die beiden Threads verteilt. Jeder Thread berechnet seinen Bereich für sich. Nach Beendigung der Threads soll das Hauptprogramm die Ergebnisse aus dem Objekt lesen, die Summe berechnen und das Ergebnis ausgeben.
+    &lt;/p&gt;
+    &lt;p&gt;&lt;b&gt;Weitere Anweisungen:&lt;/b&gt;&lt;br&gt;
+    Erstellen Sie eine Klasse &lt;b&gt;ArrayCalc&lt;/b&gt; (&lt;b&gt;ArrayCalc.java&lt;/b&gt;), die die Berechnung für einen Teil des Arrays übernimmt!
+    &lt;/p&gt;
+    &lt;p&gt;&lt;b&gt;Hinweis:&lt;/b&gt;&lt;br&gt;
+    Machen Sie sich mit der &lt;b&gt;join()&lt;/b&gt;-Methode der Klasse &lt;b&gt;Thread&lt;/b&gt; vertraut!
+    &lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">package de.goals.testing;
+import org.junit.jupiter.api.Test;
+import static org.junit.jupiter.api.Assertions.assertEquals;
+public class MyThreadTest {
+    @Test
+    public void test1() {
+        int[] a = {1, 2, 3, 4, 5, 6, 7, 8, 9, 10};
+        ArrayCalc a1 = new ArrayCalc(a, 0, 4);
+        ArrayCalc a2 = new ArrayCalc(a, 5, 9);
+        Thread t1 = new Thread(a1);
+        Thread t2 = new Thread(a2);
+        t1.start();
+        t2.start();
+        try {
+            t1.join();
+            t2.join();
+        } catch (InterruptedException e) {
+            e.printStackTrace();
+        }
+        assertEquals(55, a1.getSumme() + a2.getSumme());
+        System.out.println("Test 1 erfolgreich");
+    }
+    @Test
+    public void test2() {
+        int[] a = {10, 23, 11, 18, 4, 9, 12, 21};
+        ArrayCalc a1 = new ArrayCalc(a, 0, 3);
+        ArrayCalc a2 = new ArrayCalc(a, 4, 7);
+        Thread t1 = new Thread(a1);
+        Thread t2 = new Thread(a2);
+        t1.start();
+        t2.start();
+        try {
+            t1.join();
+            t2.join();
+        } catch (InterruptedException e) {
+            e.printStackTrace();
+        }
+        assertEquals(108, a1.getSumme() + a2.getSumme());
+        System.out.println("Test 2 erfolgreich");
+    }
+}
+</t>
+  </si>
+  <si>
+    <t>&lt;p&gt; In dieser Aufgabe sollst du den Bubblesort-Algorithmus in Java implementieren. Dieser Algorithmus ist ein einfaches Verfahren zum Sortieren einer Liste von Elementen (z.B. Zahlen).&lt;/p&gt;
+&lt;br&gt;
+&lt;p&gt;Bubblesort ist ein Sortieralgorithmus, der durch wiederholtes Durchlaufen der zu sortierenden Liste arbeitet. Bei jedem Durchlauf werden benachbarte Elemente miteinander verglichen und gegebenenfalls vertauscht. Das Besondere am Bubblesort ist, dass mit jedem Durchgang das größte Element der noch zu sortierenden Elemente an das Ende der Liste "aufsteigt".&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>package de.goals.testing;
+import org.junit.jupiter.api.Test;
+import static org.junit.jupiter.api.Assertions.assertArrayEquals;
+public class BubbleSortTest {
+    @Test
+    public void testBubbleSort1() {
+        int[] arr = {64, 34, 25, 12, 22, 11, 90};
+        int[] expected = {11, 12, 22, 25, 34, 64, 90};
+        int[] sortedArray = Sortieren.bubbleSort(arr); // Sortiert das Array und gibt es zurück
+        assertArrayEquals(expected, arr); // Prüft, ob das ursprüngliche Array sortiert wurde
+    }
+    @Test
+    public void testBubbleSort2() {
+        int[] arr = {5, 1, 9, 3, 7, 6, 8, 2, 4};
+        int[] expected = {1, 2, 3, 4, 5, 6, 7, 8, 9};
+        int[] sortedArray = Sortieren.bubbleSort(arr);
+        assertArrayEquals(expected, arr);
+    }
+    @Test
+    public void testBubbleSort3() {
+        int[] arr = {10, -2, 0, -10, -20};
+        int[] expected = {-20, -10, -2, 0, 10};
+        int[] sortedArray = Sortieren.bubbleSort(arr);
+        assertArrayEquals(expected, arr);
+    }
+    @Test
+    public void testBubbleSort4() {
+        int[] arr = {1, 1, 1, 1, 1, 1};
+        int[] expected = {1, 1, 1, 1, 1, 1};
+        int[] sortedArray = Sortieren.bubbleSort(arr);
+        assertArrayEquals(expected, arr);
+    }
+}</t>
+  </si>
+  <si>
+    <t>&lt;img src="/assets/taskImgs/fahrzeugUML.png" alt="image"&gt;
+&lt;br /&gt;&lt;p&gt;
+  Schreiben Sie den Java Code für beide Klassen des UML-Diagramms.
+&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>TestFahrzeuge.java</t>
+  </si>
+  <si>
+    <t>package de.goals.testing;
+public class TestFahrzeuge {
+    public static void main(String[] args) {
+        Auto meinAuto = new Auto("Toyota", "Corolla", 2022);
+        // Ausgabe der Daten des Auto-Objekts zum Testen
+        System.out.println("Marke: " + meinAuto.getMarke());
+        System.out.println("Modell: " + meinAuto.getModell());
+        System.out.println("Jahr: " + meinAuto.getJahr());
+    }
+}</t>
+  </si>
+  <si>
+    <t>Schreiben Sie den Java Code für beide Klassen des UML-Diagramms.
+Beschreibung des Bildes mit dem UML Diagramm:
+ Klasse Fahrzeug (abstrakte Klasse):
     Attribute:
         marke: privates Attribut vom Typ String
         modell: privates Attribut vom Typ String
@@ -3124,124 +3254,12 @@
         Öffentliche Methode getJahr(): gibt einen int zurück.
 Die Klasse Auto erbt die Attribute und Methoden von der Klasse Fahrzeug. Darauf weist der Vererbungspfeil im Diagramm hin.</t>
   </si>
-  <si>
-    <t>&lt;img src="/assets/taskImgs/fahrzeugUML.png" alt="image"&gt;
-&lt;br /&gt;&lt;p&gt;
-  Schreiben Sie den Java Code für beide Klassen des UML-Diagramms, in eine Datei, erst Fahrzeug, dann Auto.
-&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>BubbleSortTest.java</t>
-  </si>
-  <si>
-    <t>FahrzeugTest.java</t>
-  </si>
-  <si>
-    <t xml:space="preserve">package de.goals.testing;
-import org.junit.jupiter.api.Test;
-import static org.junit.jupiter.api.Assertions.assertEquals;
-public class LeserTest {
-    private int punkte = 0;
-    public int getResult() {
-        return punkte;
-    }
-    @Test
-    public void test1() {
-        Leser l = new Leser(1, 56534, "Hoffmann");
-        String out = l.getName();
-        assertEquals("Hoffmann", out);
-        punkte += 100;
-        System.out.println("Test 1 erfolgreich");
-    }
-}
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">package de.goals.testing;
-import org.junit.jupiter.api.Test;
-import static org.junit.jupiter.api.Assertions.assertEquals;
-public class AppBankTest {
-    @Test
-    public void testToString() {
-        Konto konto = new Konto("Andreas", "Hoffmann", "DE232212442");
-        konto.einzahlen(100);
-        String expected = "Kunde: Andreas Hoffmann, Konto: DE232212442, Stand: 100.0, Limit: 0.0";
-        assertEquals(expected, konto.toString(), "Fehler in der toString() Methode");
-    }
-    @Test
-    public void testEinzahlen() {
-        Konto konto = new Konto("Max", "Mustermann", "DE12345678901234567890");
-        konto.einzahlen(100);
-        double expectedKontostand = 100.0;
-        assertEquals(expectedKontostand, konto.kontostand(), "Fehler in der Einzahlen-Methode");
-    }
-    @Test
-    public void testAuszahlenWithinLimit() {
-        Konto konto = new Konto("Max", "Mustermann", "DE12345678901234567890");
-        konto.einzahlen(1000);
-        konto.auszahlen(500);
-        double expectedKontostand = 500.0;
-        assertEquals(expectedKontostand, konto.kontostand(), "Fehler in der Auszahlen-Methode mit Betrag innerhalb des Limits");
-    }
-    @Test
-    public void testAuszahlenExceedingLimit() {
-        Konto konto = new Konto("Max", "Mustermann", "DE12345678901234567890");
-        konto.einzahlen(1000);
-        konto.setLimit(500); // Set the limit before withdrawing
-        konto.auszahlen(1000);
-        double expectedKontostand = konto.getLimit();
-        assertEquals(expectedKontostand, konto.kontostand(), "Fehler in der Auszahlen-Methode mit Betrag, der das Limit überschreitet");
-    }
-    @Test
-    public void testSetLimit() {
-        Konto konto = new Konto("Max", "Mustermann", "DE12345678901234567890");
-        konto.setLimit(1000);
-        double expectedLimit = 1000.0;
-        assertEquals(expectedLimit, konto.getLimit(), "Fehler in der SetLimit-Methode");
-    }
-}
-</t>
-  </si>
-  <si>
-    <t xml:space="preserve">package de.goals.testing;
-import org.junit.jupiter.api.Test;
-import static org.junit.jupiter.api.Assertions.assertEquals;
-public class AppAutoTest {
-    private int punkte = 0;
-    private KFZ porsche = new KFZ("AK-CA 740", 24500, 50, 8, 0);
-    public int getResult() {
-        return punkte;
-    }
-    @Test
-    public void testGetKMstand() {
-        assertEquals(24500, porsche.getKMstand(), "Fehler beim Aufruf der Methode getKMstand()");
-        punkte += 25;
-        System.out.println("Test 1 erfolgreich " + porsche.getKMstand());
-    }
-    @Test
-    public void testTanken() {
-        porsche.tanken(60);
-        assertEquals(50, porsche.getTankinhalt(), "Fehler beim Aufruf der Methode getTankinhalt()");
-        punkte += 25;
-        System.out.println("Test 2 erfolgreich " + porsche.getTankinhalt());
-    }
-    @Test
-    public void testFahren() {
-        porsche.tanken(60);
-        boolean ret = porsche.fahren(150);
-        assertEquals(24650, porsche.getKMstand(), "Fehler beim Aufruf der Methode getKMstand() oder fahren()");
-        punkte += 50;
-        System.out.println("Test 3 erfolgreich " + porsche.getKMstand());
-    }
-}
-</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3263,28 +3281,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF9C5700"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="24"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="24"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -3325,17 +3322,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -3348,7 +3340,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -3378,29 +3370,13 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="4">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -3417,98 +3393,77 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="3" fontId="3" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="2" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="6" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="4" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="3" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="8" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="3" fontId="4" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="2" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="2" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="2" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="9" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="11" fillId="4" borderId="1" xfId="3" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="3"/>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="3" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="3" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="3" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="2" xfId="3" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="4">
-    <cellStyle name="Gut" xfId="2" builtinId="26"/>
-    <cellStyle name="Neutral" xfId="1" builtinId="28"/>
-    <cellStyle name="Schlecht" xfId="3" builtinId="27"/>
+  <cellStyles count="3">
+    <cellStyle name="Gut" xfId="1" builtinId="26"/>
+    <cellStyle name="Schlecht" xfId="2" builtinId="27"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -3813,1595 +3768,1621 @@
     <outlinePr summaryBelow="0"/>
   </sheetPr>
   <dimension ref="A1:R39"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="31.5" x14ac:dyDescent="0.5"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="28.5" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="2" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="23.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="23.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="37.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="66.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="143.140625" style="30" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="143.140625" style="20" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="105.5703125" style="2" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="23.7109375" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="50.7109375" style="27" customWidth="1"/>
+    <col min="11" max="11" width="50.7109375" style="17" customWidth="1"/>
     <col min="12" max="12" width="49.85546875" style="2" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="74.5703125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="170.7109375" style="23" customWidth="1"/>
+    <col min="14" max="14" width="170.7109375" style="29" customWidth="1"/>
     <col min="15" max="17" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" s="12" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A1" s="14" t="s">
+    <row r="1" spans="1:18" s="6" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="A1" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="E1" s="12" t="s">
+      <c r="E1" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="F1" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="G1" s="28" t="s">
+      <c r="G1" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="H1" s="13" t="s">
+      <c r="H1" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="I1" s="12" t="s">
+      <c r="I1" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="J1" s="14" t="s">
+      <c r="J1" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="K1" s="25" t="s">
+      <c r="K1" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="L1" s="7" t="s">
+        <v>178</v>
+      </c>
+      <c r="M1" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="N1" s="29"/>
+    </row>
+    <row r="2" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="9">
+        <v>1</v>
+      </c>
+      <c r="B2" s="9">
+        <v>5</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="D2" s="9">
+        <v>34</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="F2" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="G2" s="19" t="s">
+        <v>163</v>
+      </c>
+      <c r="H2" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="J2" s="9">
+        <v>0</v>
+      </c>
+      <c r="K2" s="16" t="s">
+        <v>204</v>
+      </c>
+      <c r="L2" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="M2" s="6" t="s">
         <v>206</v>
       </c>
-      <c r="L1" s="13" t="s">
-        <v>179</v>
-      </c>
-      <c r="M1" s="12" t="s">
-        <v>180</v>
-      </c>
-      <c r="N1" s="21"/>
-    </row>
-    <row r="2" spans="1:18" s="12" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A2" s="15">
+      <c r="N2" s="29"/>
+    </row>
+    <row r="3" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="9">
+        <v>2</v>
+      </c>
+      <c r="B3" s="9">
+        <v>5</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="D3" s="9">
+        <v>36</v>
+      </c>
+      <c r="E3" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="G3" s="19" t="s">
+        <v>164</v>
+      </c>
+      <c r="H3" s="10" t="s">
+        <v>92</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="J3" s="9">
+        <v>0</v>
+      </c>
+      <c r="K3" s="16" t="s">
+        <v>204</v>
+      </c>
+      <c r="L3" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="M3" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="N3" s="29"/>
+    </row>
+    <row r="4" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="9">
+        <v>3</v>
+      </c>
+      <c r="B4" s="9">
+        <v>5</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="D4" s="9">
+        <v>34</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>94</v>
+      </c>
+      <c r="G4" s="19" t="s">
+        <v>165</v>
+      </c>
+      <c r="H4" s="10" t="s">
+        <v>281</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="J4" s="9">
+        <v>0</v>
+      </c>
+      <c r="K4" s="16" t="s">
+        <v>204</v>
+      </c>
+      <c r="L4" s="7" t="s">
+        <v>183</v>
+      </c>
+      <c r="M4" s="6">
+        <v>174</v>
+      </c>
+      <c r="N4" s="29"/>
+    </row>
+    <row r="5" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="9">
+        <v>4</v>
+      </c>
+      <c r="B5" s="9">
+        <v>5</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="D5" s="9">
+        <v>34</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="F5" s="10" t="s">
+        <v>96</v>
+      </c>
+      <c r="G5" s="11" t="s">
+        <v>166</v>
+      </c>
+      <c r="H5" s="10" t="s">
+        <v>285</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="J5" s="9">
+        <v>0</v>
+      </c>
+      <c r="K5" s="12" t="s">
+        <v>204</v>
+      </c>
+      <c r="L5" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="M5" s="6">
+        <v>47</v>
+      </c>
+      <c r="N5" s="29"/>
+    </row>
+    <row r="6" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="9">
+        <v>5</v>
+      </c>
+      <c r="B6" s="9">
+        <v>4</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="D6" s="9">
+        <v>23</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="F6" s="10" t="s">
+        <v>98</v>
+      </c>
+      <c r="G6" s="11" t="s">
+        <v>167</v>
+      </c>
+      <c r="H6" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="J6" s="9">
+        <v>0</v>
+      </c>
+      <c r="K6" s="12" t="s">
+        <v>204</v>
+      </c>
+      <c r="L6" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="M6" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="N6" s="29"/>
+    </row>
+    <row r="7" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="9">
+        <v>6</v>
+      </c>
+      <c r="B7" s="9">
+        <v>4</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="D7" s="9">
+        <v>34</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="G7" s="19" t="s">
+        <v>168</v>
+      </c>
+      <c r="H7" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="I7" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="J7" s="9">
+        <v>0</v>
+      </c>
+      <c r="K7" s="16" t="s">
+        <v>204</v>
+      </c>
+      <c r="L7" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="M7" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="N7" s="29"/>
+    </row>
+    <row r="8" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="9">
+        <v>7</v>
+      </c>
+      <c r="B8" s="9">
+        <v>4</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="D8" s="9">
+        <v>34</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="F8" s="10" t="s">
+        <v>104</v>
+      </c>
+      <c r="G8" s="19" t="s">
+        <v>169</v>
+      </c>
+      <c r="H8" s="10" t="s">
+        <v>317</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="J8" s="9">
+        <v>0</v>
+      </c>
+      <c r="K8" s="16" t="s">
+        <v>204</v>
+      </c>
+      <c r="L8" s="7" t="s">
+        <v>211</v>
+      </c>
+      <c r="M8" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="N8" s="29"/>
+    </row>
+    <row r="9" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="9">
+        <v>8</v>
+      </c>
+      <c r="B9" s="9">
+        <v>4</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="D9" s="9">
+        <v>26</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="F9" s="10" t="s">
+        <v>279</v>
+      </c>
+      <c r="G9" s="19" t="s">
+        <v>170</v>
+      </c>
+      <c r="H9" s="10" t="s">
+        <v>280</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="J9" s="9">
+        <v>0</v>
+      </c>
+      <c r="K9" s="16" t="s">
+        <v>204</v>
+      </c>
+      <c r="L9" s="7" t="s">
+        <v>213</v>
+      </c>
+      <c r="M9" s="6">
+        <v>10</v>
+      </c>
+      <c r="N9" s="29"/>
+    </row>
+    <row r="10" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="9">
+        <v>9</v>
+      </c>
+      <c r="B10" s="9">
+        <v>6</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="D10" s="9">
+        <v>63</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="F10" s="10" t="s">
+        <v>108</v>
+      </c>
+      <c r="G10" s="11" t="s">
+        <v>305</v>
+      </c>
+      <c r="H10" s="10" t="s">
+        <v>109</v>
+      </c>
+      <c r="I10" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="J10" s="9">
+        <v>0</v>
+      </c>
+      <c r="K10" s="12" t="s">
+        <v>184</v>
+      </c>
+      <c r="L10" s="7"/>
+      <c r="N10" s="29"/>
+      <c r="R10" s="7" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="9">
+        <v>10</v>
+      </c>
+      <c r="B11" s="9">
+        <v>6</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="D11" s="9">
+        <v>65</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="F11" s="10" t="s">
+        <v>268</v>
+      </c>
+      <c r="G11" s="11" t="s">
+        <v>222</v>
+      </c>
+      <c r="H11" s="10" t="s">
+        <v>269</v>
+      </c>
+      <c r="I11" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="J11" s="9">
+        <v>0</v>
+      </c>
+      <c r="K11" s="12" t="s">
+        <v>185</v>
+      </c>
+      <c r="L11" s="7"/>
+      <c r="N11" s="29"/>
+      <c r="R11" s="7" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" s="14" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="14">
+        <v>11</v>
+      </c>
+      <c r="B12" s="14">
+        <v>6</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="D12" s="14">
+        <v>63</v>
+      </c>
+      <c r="E12" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="F12" s="14" t="s">
+        <v>286</v>
+      </c>
+      <c r="G12" s="21" t="s">
+        <v>223</v>
+      </c>
+      <c r="H12" s="21" t="s">
+        <v>308</v>
+      </c>
+      <c r="I12" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="J12" s="14">
         <v>1</v>
       </c>
-      <c r="B2" s="15">
+      <c r="K12" s="14" t="s">
+        <v>186</v>
+      </c>
+      <c r="N12" s="29"/>
+      <c r="R12" s="21" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="9">
+        <v>12</v>
+      </c>
+      <c r="B13" s="9">
+        <v>6</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="D13" s="9">
+        <v>63</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="F13" s="10" t="s">
+        <v>113</v>
+      </c>
+      <c r="G13" s="11" t="s">
+        <v>224</v>
+      </c>
+      <c r="H13" s="10" t="s">
+        <v>114</v>
+      </c>
+      <c r="I13" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="J13" s="9">
+        <v>0</v>
+      </c>
+      <c r="K13" s="12" t="s">
+        <v>187</v>
+      </c>
+      <c r="L13" s="7"/>
+      <c r="N13" s="29"/>
+    </row>
+    <row r="14" spans="1:18" s="14" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="14">
+        <v>13</v>
+      </c>
+      <c r="B14" s="14">
+        <v>7</v>
+      </c>
+      <c r="C14" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="D14" s="14">
+        <v>69</v>
+      </c>
+      <c r="E14" s="14" t="s">
+        <v>115</v>
+      </c>
+      <c r="F14" s="14" t="s">
+        <v>289</v>
+      </c>
+      <c r="G14" s="14" t="s">
+        <v>225</v>
+      </c>
+      <c r="H14" s="14" t="s">
+        <v>290</v>
+      </c>
+      <c r="I14" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="J14" s="14">
+        <v>1</v>
+      </c>
+      <c r="K14" s="14" t="s">
+        <v>188</v>
+      </c>
+      <c r="N14" s="29"/>
+      <c r="R14" s="21" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="9">
+        <v>14</v>
+      </c>
+      <c r="B15" s="9">
+        <v>7</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="D15" s="9">
+        <v>70</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="F15" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>226</v>
+      </c>
+      <c r="H15" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="I15" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="J15" s="9">
+        <v>0</v>
+      </c>
+      <c r="K15" s="12" t="s">
+        <v>189</v>
+      </c>
+      <c r="L15" s="7"/>
+      <c r="N15" s="29"/>
+    </row>
+    <row r="16" spans="1:18" s="14" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="14">
+        <v>15</v>
+      </c>
+      <c r="B16" s="14">
+        <v>7</v>
+      </c>
+      <c r="C16" s="14" t="s">
+        <v>106</v>
+      </c>
+      <c r="D16" s="14">
+        <v>64</v>
+      </c>
+      <c r="E16" s="14" t="s">
+        <v>119</v>
+      </c>
+      <c r="F16" s="21" t="s">
+        <v>291</v>
+      </c>
+      <c r="G16" s="14" t="s">
+        <v>227</v>
+      </c>
+      <c r="H16" s="14" t="s">
+        <v>292</v>
+      </c>
+      <c r="I16" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="J16" s="14">
+        <v>2</v>
+      </c>
+      <c r="K16" s="14" t="s">
+        <v>190</v>
+      </c>
+      <c r="N16" s="29"/>
+    </row>
+    <row r="17" spans="1:17" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="9">
+        <v>16</v>
+      </c>
+      <c r="B17" s="9">
+        <v>8</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="D17" s="9">
+        <v>85</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="F17" s="10" t="s">
+        <v>325</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>332</v>
+      </c>
+      <c r="H17" s="10" t="s">
+        <v>326</v>
+      </c>
+      <c r="I17" s="10" t="s">
+        <v>20</v>
+      </c>
+      <c r="J17" s="9">
+        <v>0</v>
+      </c>
+      <c r="K17" s="12" t="s">
+        <v>191</v>
+      </c>
+      <c r="L17" s="7"/>
+      <c r="N17" s="21" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="9">
+        <v>17</v>
+      </c>
+      <c r="B18" s="9">
+        <v>8</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="D18" s="9">
+        <v>84</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="F18" s="10" t="s">
+        <v>270</v>
+      </c>
+      <c r="G18" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="H18" s="10" t="s">
+        <v>271</v>
+      </c>
+      <c r="I18" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="J18" s="9">
+        <v>0</v>
+      </c>
+      <c r="K18" s="12" t="s">
+        <v>192</v>
+      </c>
+      <c r="L18" s="7"/>
+      <c r="N18" s="29"/>
+    </row>
+    <row r="19" spans="1:17" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="9">
+        <v>18</v>
+      </c>
+      <c r="B19" s="9">
+        <v>8</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="D19" s="9">
+        <v>93</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="F19" s="10" t="s">
+        <v>310</v>
+      </c>
+      <c r="G19" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="H19" s="10" t="s">
+        <v>311</v>
+      </c>
+      <c r="I19" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="J19" s="9">
+        <v>0</v>
+      </c>
+      <c r="K19" s="12" t="s">
+        <v>193</v>
+      </c>
+      <c r="L19" s="7"/>
+      <c r="N19" s="29"/>
+    </row>
+    <row r="20" spans="1:17" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="22">
+        <v>19</v>
+      </c>
+      <c r="B20" s="22">
+        <v>8</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="D20" s="9">
+        <v>69</v>
+      </c>
+      <c r="E20" s="13" t="s">
+        <v>123</v>
+      </c>
+      <c r="F20" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>230</v>
+      </c>
+      <c r="H20" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="I20" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="J20" s="9">
+        <v>0</v>
+      </c>
+      <c r="K20" s="12" t="s">
+        <v>194</v>
+      </c>
+      <c r="L20" s="7"/>
+      <c r="N20" s="29"/>
+    </row>
+    <row r="21" spans="1:17" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="9">
+        <v>20</v>
+      </c>
+      <c r="B21" s="9">
+        <v>9</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="D21" s="9">
+        <v>78</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="F21" s="10" t="s">
+        <v>272</v>
+      </c>
+      <c r="G21" s="7" t="s">
+        <v>324</v>
+      </c>
+      <c r="H21" s="14" t="s">
+        <v>319</v>
+      </c>
+      <c r="I21" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="J21" s="9">
+        <v>0</v>
+      </c>
+      <c r="K21" s="12" t="s">
+        <v>195</v>
+      </c>
+      <c r="L21" s="7"/>
+      <c r="N21" s="29"/>
+    </row>
+    <row r="22" spans="1:17" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22" s="9">
+        <v>21</v>
+      </c>
+      <c r="B22" s="9">
+        <v>9</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="D22" s="9">
+        <v>75</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="F22" s="10" t="s">
+        <v>275</v>
+      </c>
+      <c r="G22" s="7" t="s">
+        <v>331</v>
+      </c>
+      <c r="H22" s="14" t="s">
+        <v>320</v>
+      </c>
+      <c r="I22" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="J22" s="9">
+        <v>0</v>
+      </c>
+      <c r="K22" s="12" t="s">
+        <v>196</v>
+      </c>
+      <c r="L22" s="7"/>
+      <c r="N22" s="21"/>
+    </row>
+    <row r="23" spans="1:17" s="24" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="23">
+        <v>22</v>
+      </c>
+      <c r="B23" s="23">
+        <v>9</v>
+      </c>
+      <c r="C23" s="24" t="s">
+        <v>106</v>
+      </c>
+      <c r="D23" s="23">
+        <v>78</v>
+      </c>
+      <c r="E23" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="F23" s="26" t="s">
+        <v>327</v>
+      </c>
+      <c r="G23" s="27" t="s">
+        <v>329</v>
+      </c>
+      <c r="H23" s="30" t="s">
+        <v>328</v>
+      </c>
+      <c r="I23" s="26" t="s">
+        <v>36</v>
+      </c>
+      <c r="J23" s="23">
+        <v>0</v>
+      </c>
+      <c r="K23" s="28" t="s">
+        <v>197</v>
+      </c>
+      <c r="L23" s="27"/>
+      <c r="N23" s="30" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="9">
+        <v>23</v>
+      </c>
+      <c r="B24" s="9">
+        <v>9</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="D24" s="9">
+        <v>75</v>
+      </c>
+      <c r="E24" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="F24" s="10" t="s">
+        <v>276</v>
+      </c>
+      <c r="G24" s="7" t="s">
+        <v>231</v>
+      </c>
+      <c r="H24" s="14" t="s">
+        <v>321</v>
+      </c>
+      <c r="I24" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="J24" s="9">
+        <v>0</v>
+      </c>
+      <c r="K24" s="12" t="s">
+        <v>198</v>
+      </c>
+      <c r="L24" s="7"/>
+      <c r="N24" s="14"/>
+    </row>
+    <row r="25" spans="1:17" s="6" customFormat="1" ht="261" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="9">
+        <v>24</v>
+      </c>
+      <c r="B25" s="9">
+        <v>11</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="D25" s="9">
+        <v>85</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="F25" s="10" t="s">
+        <v>273</v>
+      </c>
+      <c r="G25" s="7" t="s">
+        <v>334</v>
+      </c>
+      <c r="H25" s="10" t="s">
+        <v>274</v>
+      </c>
+      <c r="I25" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="J25" s="9">
+        <v>0</v>
+      </c>
+      <c r="K25" s="12" t="s">
+        <v>199</v>
+      </c>
+      <c r="L25" s="7"/>
+      <c r="N25" s="14"/>
+    </row>
+    <row r="26" spans="1:17" s="6" customFormat="1" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A26" s="9">
+        <v>25</v>
+      </c>
+      <c r="B26" s="9">
+        <v>11</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="D26" s="9">
+        <v>78</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="F26" s="10" t="s">
+        <v>335</v>
+      </c>
+      <c r="G26" s="7" t="s">
+        <v>337</v>
+      </c>
+      <c r="H26" s="10" t="s">
+        <v>336</v>
+      </c>
+      <c r="I26" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="J26" s="9">
+        <v>0</v>
+      </c>
+      <c r="K26" s="12" t="s">
+        <v>200</v>
+      </c>
+      <c r="L26" s="7"/>
+      <c r="N26" s="14" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" s="6" customFormat="1" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27" s="9">
+        <v>26</v>
+      </c>
+      <c r="B27" s="9">
+        <v>11</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="D27" s="9">
+        <v>95</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="F27" s="10" t="s">
+        <v>277</v>
+      </c>
+      <c r="G27" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="H27" s="10" t="s">
+        <v>339</v>
+      </c>
+      <c r="I27" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="J27" s="9">
+        <v>0</v>
+      </c>
+      <c r="K27" s="12" t="s">
+        <v>201</v>
+      </c>
+      <c r="L27" s="7"/>
+      <c r="N27" s="14"/>
+    </row>
+    <row r="28" spans="1:17" s="6" customFormat="1" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28" s="9">
+        <v>27</v>
+      </c>
+      <c r="B28" s="9">
+        <v>11</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="D28" s="9">
+        <v>107</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="F28" s="10" t="s">
+        <v>341</v>
+      </c>
+      <c r="G28" s="7" t="s">
+        <v>343</v>
+      </c>
+      <c r="H28" s="10" t="s">
+        <v>342</v>
+      </c>
+      <c r="I28" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="J28" s="9">
+        <v>0</v>
+      </c>
+      <c r="K28" s="12" t="s">
+        <v>202</v>
+      </c>
+      <c r="L28" s="7"/>
+      <c r="N28" s="14"/>
+    </row>
+    <row r="29" spans="1:17" s="6" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="9">
+        <v>28</v>
+      </c>
+      <c r="B29" s="9">
+        <v>0</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="D29" s="9">
+        <v>40</v>
+      </c>
+      <c r="E29" s="10" t="s">
+        <v>298</v>
+      </c>
+      <c r="F29" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="G29" s="18" t="s">
+        <v>171</v>
+      </c>
+      <c r="H29" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="I29" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="J29" s="9">
+        <v>0</v>
+      </c>
+      <c r="K29" s="16" t="s">
+        <v>204</v>
+      </c>
+      <c r="L29" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="M29" s="6">
+        <v>3</v>
+      </c>
+      <c r="N29" s="29"/>
+      <c r="P29" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q29" s="13" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17" s="24" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="23">
+        <v>29</v>
+      </c>
+      <c r="B30" s="23">
+        <v>0</v>
+      </c>
+      <c r="C30" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="D30" s="23">
+        <v>26</v>
+      </c>
+      <c r="E30" s="25" t="s">
+        <v>299</v>
+      </c>
+      <c r="F30" s="26" t="s">
+        <v>137</v>
+      </c>
+      <c r="G30" s="27" t="s">
+        <v>284</v>
+      </c>
+      <c r="H30" s="26" t="s">
+        <v>138</v>
+      </c>
+      <c r="I30" s="24" t="s">
+        <v>52</v>
+      </c>
+      <c r="J30" s="23">
+        <v>0</v>
+      </c>
+      <c r="K30" s="28" t="s">
+        <v>204</v>
+      </c>
+      <c r="L30" s="24" t="s">
+        <v>282</v>
+      </c>
+      <c r="M30" s="24" t="s">
+        <v>283</v>
+      </c>
+      <c r="N30" s="29"/>
+      <c r="P30" s="26" t="s">
+        <v>53</v>
+      </c>
+      <c r="Q30" s="25" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="31" spans="1:17" s="6" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="9">
+        <v>30</v>
+      </c>
+      <c r="B31" s="9">
+        <v>0</v>
+      </c>
+      <c r="C31" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="D31" s="9">
+        <v>34</v>
+      </c>
+      <c r="E31" s="13" t="s">
+        <v>300</v>
+      </c>
+      <c r="F31" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="G31" s="18" t="s">
+        <v>172</v>
+      </c>
+      <c r="H31" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="I31" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="J31" s="9">
+        <v>0</v>
+      </c>
+      <c r="K31" s="16" t="s">
+        <v>204</v>
+      </c>
+      <c r="L31" s="14" t="s">
+        <v>215</v>
+      </c>
+      <c r="M31" s="14" t="s">
+        <v>216</v>
+      </c>
+      <c r="N31" s="29"/>
+      <c r="P31" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q31" s="13" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="32" spans="1:17" s="6" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="9">
+        <v>31</v>
+      </c>
+      <c r="B32" s="9">
+        <v>0</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="D32" s="9">
+        <v>34</v>
+      </c>
+      <c r="E32" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="F32" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="G32" s="18" t="s">
+        <v>173</v>
+      </c>
+      <c r="H32" s="10" t="s">
+        <v>144</v>
+      </c>
+      <c r="I32" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="J32" s="9">
+        <v>0</v>
+      </c>
+      <c r="K32" s="16" t="s">
+        <v>204</v>
+      </c>
+      <c r="L32" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="M32" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="N32" s="29"/>
+      <c r="P32" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="Q32" s="13" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="33" spans="1:17" s="24" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="23">
+        <v>32</v>
+      </c>
+      <c r="B33" s="23">
+        <v>0</v>
+      </c>
+      <c r="C33" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="D33" s="23">
+        <v>26</v>
+      </c>
+      <c r="E33" s="24" t="s">
+        <v>302</v>
+      </c>
+      <c r="F33" s="26" t="s">
+        <v>146</v>
+      </c>
+      <c r="G33" s="27" t="s">
+        <v>174</v>
+      </c>
+      <c r="H33" s="26" t="s">
+        <v>147</v>
+      </c>
+      <c r="I33" s="24" t="s">
+        <v>58</v>
+      </c>
+      <c r="J33" s="23">
+        <v>0</v>
+      </c>
+      <c r="K33" s="28" t="s">
+        <v>204</v>
+      </c>
+      <c r="L33" s="27"/>
+      <c r="N33" s="29"/>
+      <c r="P33" s="26" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q33" s="25" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="34" spans="1:17" s="24" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="23">
+        <v>33</v>
+      </c>
+      <c r="B34" s="23">
+        <v>0</v>
+      </c>
+      <c r="C34" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="D34" s="23">
+        <v>28</v>
+      </c>
+      <c r="E34" s="24" t="s">
+        <v>303</v>
+      </c>
+      <c r="F34" s="26" t="s">
+        <v>149</v>
+      </c>
+      <c r="G34" s="27" t="s">
+        <v>175</v>
+      </c>
+      <c r="H34" s="26" t="s">
+        <v>150</v>
+      </c>
+      <c r="I34" s="24" t="s">
+        <v>60</v>
+      </c>
+      <c r="J34" s="23">
+        <v>0</v>
+      </c>
+      <c r="K34" s="28" t="s">
+        <v>204</v>
+      </c>
+      <c r="L34" s="27"/>
+      <c r="N34" s="29"/>
+      <c r="P34" s="26" t="s">
+        <v>61</v>
+      </c>
+      <c r="Q34" s="25" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="35" spans="1:17" s="6" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A35" s="9">
+        <v>34</v>
+      </c>
+      <c r="B35" s="9">
+        <v>0</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="D35" s="9">
+        <v>26</v>
+      </c>
+      <c r="E35" s="6" t="s">
+        <v>304</v>
+      </c>
+      <c r="F35" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="G35" s="18" t="s">
+        <v>176</v>
+      </c>
+      <c r="H35" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="I35" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="J35" s="9">
+        <v>0</v>
+      </c>
+      <c r="K35" s="16" t="s">
+        <v>204</v>
+      </c>
+      <c r="L35" s="7" t="s">
+        <v>219</v>
+      </c>
+      <c r="M35" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="N35" s="29"/>
+      <c r="P35" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="Q35" s="13" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="36" spans="1:17" s="6" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="9">
+        <v>35</v>
+      </c>
+      <c r="B36" s="9">
+        <v>0</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="D36" s="9">
+        <v>34</v>
+      </c>
+      <c r="E36" s="6" t="s">
+        <v>297</v>
+      </c>
+      <c r="F36" s="10" t="s">
+        <v>155</v>
+      </c>
+      <c r="G36" s="18" t="s">
+        <v>177</v>
+      </c>
+      <c r="H36" s="10" t="s">
+        <v>156</v>
+      </c>
+      <c r="I36" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="J36" s="9">
+        <v>0</v>
+      </c>
+      <c r="K36" s="16" t="s">
+        <v>204</v>
+      </c>
+      <c r="L36" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="M36" s="6">
         <v>5</v>
       </c>
-      <c r="C2" s="12" t="s">
-        <v>86</v>
-      </c>
-      <c r="D2" s="15">
-        <v>34</v>
-      </c>
-      <c r="E2" s="16" t="s">
-        <v>87</v>
-      </c>
-      <c r="F2" s="16" t="s">
-        <v>88</v>
-      </c>
-      <c r="G2" s="29" t="s">
-        <v>164</v>
-      </c>
-      <c r="H2" s="16" t="s">
-        <v>89</v>
-      </c>
-      <c r="I2" s="12" t="s">
-        <v>4</v>
-      </c>
-      <c r="J2" s="15">
+      <c r="N36" s="29"/>
+      <c r="P36" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q36" s="13" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="37" spans="1:17" s="6" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="9">
+        <v>36</v>
+      </c>
+      <c r="B37" s="9">
         <v>0</v>
       </c>
-      <c r="K2" s="26" t="s">
-        <v>205</v>
-      </c>
-      <c r="L2" s="13" t="s">
-        <v>181</v>
-      </c>
-      <c r="M2" s="12" t="s">
-        <v>207</v>
-      </c>
-      <c r="N2" s="21"/>
-    </row>
-    <row r="3" spans="1:18" s="12" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A3" s="15">
-        <v>2</v>
-      </c>
-      <c r="B3" s="15">
-        <v>5</v>
-      </c>
-      <c r="C3" s="12" t="s">
-        <v>86</v>
-      </c>
-      <c r="D3" s="15">
-        <v>36</v>
-      </c>
-      <c r="E3" s="19" t="s">
-        <v>90</v>
-      </c>
-      <c r="F3" s="16" t="s">
-        <v>91</v>
-      </c>
-      <c r="G3" s="29" t="s">
-        <v>165</v>
-      </c>
-      <c r="H3" s="16" t="s">
-        <v>92</v>
-      </c>
-      <c r="I3" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="J3" s="15">
+      <c r="C37" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="D37" s="9">
+        <v>97</v>
+      </c>
+      <c r="E37" s="6" t="s">
+        <v>296</v>
+      </c>
+      <c r="F37" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="G37" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="H37" s="10" t="s">
+        <v>318</v>
+      </c>
+      <c r="I37" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="J37" s="9">
         <v>0</v>
       </c>
-      <c r="K3" s="26" t="s">
-        <v>205</v>
-      </c>
-      <c r="L3" s="13" t="s">
-        <v>182</v>
-      </c>
-      <c r="M3" s="12" t="s">
-        <v>183</v>
-      </c>
-      <c r="N3" s="21"/>
-    </row>
-    <row r="4" spans="1:18" s="12" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A4" s="15">
-        <v>3</v>
-      </c>
-      <c r="B4" s="15">
-        <v>5</v>
-      </c>
-      <c r="C4" s="12" t="s">
-        <v>86</v>
-      </c>
-      <c r="D4" s="15">
-        <v>34</v>
-      </c>
-      <c r="E4" s="19" t="s">
-        <v>93</v>
-      </c>
-      <c r="F4" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="G4" s="29" t="s">
-        <v>166</v>
-      </c>
-      <c r="H4" s="16" t="s">
+      <c r="K37" s="12" t="s">
+        <v>203</v>
+      </c>
+      <c r="L37" s="7"/>
+      <c r="N37" s="14"/>
+      <c r="P37" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q37" s="13" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="38" spans="1:17" s="6" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="9">
+        <v>37</v>
+      </c>
+      <c r="B38" s="9">
+        <v>0</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="D38" s="9">
+        <v>67</v>
+      </c>
+      <c r="E38" s="6" t="s">
         <v>294</v>
       </c>
-      <c r="I4" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="J4" s="15">
+      <c r="F38" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="G38" s="7" t="s">
+        <v>345</v>
+      </c>
+      <c r="H38" s="10" t="s">
+        <v>344</v>
+      </c>
+      <c r="I38" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="J38" s="9">
         <v>0</v>
       </c>
-      <c r="K4" s="26" t="s">
-        <v>205</v>
-      </c>
-      <c r="L4" s="13" t="s">
-        <v>184</v>
-      </c>
-      <c r="M4" s="12">
-        <v>174</v>
-      </c>
-      <c r="N4" s="21"/>
-    </row>
-    <row r="5" spans="1:18" s="12" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="15">
-        <v>4</v>
-      </c>
-      <c r="B5" s="15">
-        <v>5</v>
-      </c>
-      <c r="C5" s="12" t="s">
-        <v>86</v>
-      </c>
-      <c r="D5" s="15">
-        <v>34</v>
-      </c>
-      <c r="E5" s="12" t="s">
-        <v>95</v>
-      </c>
-      <c r="F5" s="16" t="s">
-        <v>96</v>
-      </c>
-      <c r="G5" s="17" t="s">
-        <v>167</v>
-      </c>
-      <c r="H5" s="16" t="s">
-        <v>298</v>
-      </c>
-      <c r="I5" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="J5" s="15">
+      <c r="K38" s="12" t="s">
+        <v>322</v>
+      </c>
+      <c r="L38" s="7"/>
+      <c r="N38" s="14"/>
+      <c r="P38" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="Q38" s="13" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="39" spans="1:17" s="6" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="9">
+        <v>38</v>
+      </c>
+      <c r="B39" s="9">
         <v>0</v>
       </c>
-      <c r="K5" s="18" t="s">
-        <v>205</v>
-      </c>
-      <c r="L5" s="13" t="s">
-        <v>208</v>
-      </c>
-      <c r="M5" s="12">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="6" spans="1:18" s="12" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="15">
-        <v>5</v>
-      </c>
-      <c r="B6" s="15">
-        <v>4</v>
-      </c>
-      <c r="C6" s="12" t="s">
-        <v>86</v>
-      </c>
-      <c r="D6" s="15">
-        <v>23</v>
-      </c>
-      <c r="E6" s="12" t="s">
-        <v>97</v>
-      </c>
-      <c r="F6" s="16" t="s">
-        <v>98</v>
-      </c>
-      <c r="G6" s="17" t="s">
-        <v>168</v>
-      </c>
-      <c r="H6" s="16" t="s">
-        <v>99</v>
-      </c>
-      <c r="I6" s="12" t="s">
-        <v>9</v>
-      </c>
-      <c r="J6" s="15">
+      <c r="C39" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="D39" s="9">
+        <v>85</v>
+      </c>
+      <c r="E39" s="6" t="s">
+        <v>295</v>
+      </c>
+      <c r="F39" s="10" t="s">
+        <v>349</v>
+      </c>
+      <c r="G39" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="H39" s="10" t="s">
+        <v>346</v>
+      </c>
+      <c r="I39" s="10" t="s">
+        <v>347</v>
+      </c>
+      <c r="J39" s="9">
         <v>0</v>
       </c>
-      <c r="K6" s="18" t="s">
-        <v>205</v>
-      </c>
-      <c r="L6" s="13" t="s">
-        <v>209</v>
-      </c>
-      <c r="M6" s="12" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="7" spans="1:18" s="12" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A7" s="15">
-        <v>6</v>
-      </c>
-      <c r="B7" s="15">
-        <v>4</v>
-      </c>
-      <c r="C7" s="12" t="s">
-        <v>86</v>
-      </c>
-      <c r="D7" s="15">
-        <v>34</v>
-      </c>
-      <c r="E7" s="12" t="s">
-        <v>100</v>
-      </c>
-      <c r="F7" s="16" t="s">
-        <v>101</v>
-      </c>
-      <c r="G7" s="29" t="s">
-        <v>169</v>
-      </c>
-      <c r="H7" s="16" t="s">
-        <v>102</v>
-      </c>
-      <c r="I7" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="J7" s="15">
-        <v>0</v>
-      </c>
-      <c r="K7" s="26" t="s">
-        <v>205</v>
-      </c>
-      <c r="L7" s="13" t="s">
-        <v>211</v>
-      </c>
-      <c r="M7" s="12" t="s">
-        <v>291</v>
-      </c>
-      <c r="N7" s="22"/>
-    </row>
-    <row r="8" spans="1:18" s="12" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A8" s="15">
-        <v>7</v>
-      </c>
-      <c r="B8" s="15">
-        <v>4</v>
-      </c>
-      <c r="C8" s="12" t="s">
-        <v>86</v>
-      </c>
-      <c r="D8" s="15">
-        <v>34</v>
-      </c>
-      <c r="E8" s="12" t="s">
-        <v>103</v>
-      </c>
-      <c r="F8" s="16" t="s">
-        <v>104</v>
-      </c>
-      <c r="G8" s="29" t="s">
-        <v>170</v>
-      </c>
-      <c r="H8" s="16" t="s">
-        <v>330</v>
-      </c>
-      <c r="I8" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="J8" s="15">
-        <v>0</v>
-      </c>
-      <c r="K8" s="26" t="s">
-        <v>205</v>
-      </c>
-      <c r="L8" s="13" t="s">
-        <v>212</v>
-      </c>
-      <c r="M8" s="12" t="s">
-        <v>213</v>
-      </c>
-      <c r="N8" s="21"/>
-    </row>
-    <row r="9" spans="1:18" s="12" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A9" s="15">
-        <v>8</v>
-      </c>
-      <c r="B9" s="15">
-        <v>4</v>
-      </c>
-      <c r="C9" s="12" t="s">
-        <v>86</v>
-      </c>
-      <c r="D9" s="15">
-        <v>26</v>
-      </c>
-      <c r="E9" s="12" t="s">
-        <v>105</v>
-      </c>
-      <c r="F9" s="16" t="s">
-        <v>292</v>
-      </c>
-      <c r="G9" s="29" t="s">
-        <v>171</v>
-      </c>
-      <c r="H9" s="16" t="s">
-        <v>293</v>
-      </c>
-      <c r="I9" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="J9" s="15">
-        <v>0</v>
-      </c>
-      <c r="K9" s="26" t="s">
-        <v>205</v>
-      </c>
-      <c r="L9" s="13" t="s">
-        <v>214</v>
-      </c>
-      <c r="M9" s="12">
-        <v>10</v>
-      </c>
-      <c r="N9" s="21"/>
-    </row>
-    <row r="10" spans="1:18" s="12" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="15">
-        <v>9</v>
-      </c>
-      <c r="B10" s="15">
-        <v>6</v>
-      </c>
-      <c r="C10" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="D10" s="15">
-        <v>63</v>
-      </c>
-      <c r="E10" s="12" t="s">
-        <v>107</v>
-      </c>
-      <c r="F10" s="16" t="s">
-        <v>108</v>
-      </c>
-      <c r="G10" s="17" t="s">
-        <v>318</v>
-      </c>
-      <c r="H10" s="16" t="s">
-        <v>109</v>
-      </c>
-      <c r="I10" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="J10" s="15">
-        <v>0</v>
-      </c>
-      <c r="K10" s="18" t="s">
-        <v>185</v>
-      </c>
-      <c r="L10" s="13"/>
-      <c r="R10" s="13" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="11" spans="1:18" s="12" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="15">
-        <v>10</v>
-      </c>
-      <c r="B11" s="15">
-        <v>6</v>
-      </c>
-      <c r="C11" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="D11" s="15">
-        <v>65</v>
-      </c>
-      <c r="E11" s="12" t="s">
-        <v>110</v>
-      </c>
-      <c r="F11" s="16" t="s">
-        <v>276</v>
-      </c>
-      <c r="G11" s="17" t="s">
-        <v>223</v>
-      </c>
-      <c r="H11" s="16" t="s">
-        <v>277</v>
-      </c>
-      <c r="I11" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="J11" s="15">
-        <v>0</v>
-      </c>
-      <c r="K11" s="18" t="s">
-        <v>186</v>
-      </c>
-      <c r="L11" s="13"/>
-      <c r="R11" s="13" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="12" spans="1:18" s="20" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="20">
-        <v>11</v>
-      </c>
-      <c r="B12" s="20">
-        <v>6</v>
-      </c>
-      <c r="C12" s="20" t="s">
-        <v>106</v>
-      </c>
-      <c r="D12" s="20">
-        <v>63</v>
-      </c>
-      <c r="E12" s="20" t="s">
-        <v>111</v>
-      </c>
-      <c r="F12" s="20" t="s">
-        <v>299</v>
-      </c>
-      <c r="G12" s="31" t="s">
-        <v>224</v>
-      </c>
-      <c r="H12" s="31" t="s">
-        <v>321</v>
-      </c>
-      <c r="I12" s="20" t="s">
-        <v>15</v>
-      </c>
-      <c r="J12" s="20">
-        <v>1</v>
-      </c>
-      <c r="K12" s="20" t="s">
-        <v>187</v>
-      </c>
-      <c r="N12" s="12"/>
-      <c r="R12" s="31" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="13" spans="1:18" s="12" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="15">
-        <v>12</v>
-      </c>
-      <c r="B13" s="15">
-        <v>6</v>
-      </c>
-      <c r="C13" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="D13" s="15">
-        <v>63</v>
-      </c>
-      <c r="E13" s="12" t="s">
-        <v>112</v>
-      </c>
-      <c r="F13" s="16" t="s">
-        <v>113</v>
-      </c>
-      <c r="G13" s="17" t="s">
-        <v>225</v>
-      </c>
-      <c r="H13" s="16" t="s">
-        <v>114</v>
-      </c>
-      <c r="I13" s="12" t="s">
-        <v>16</v>
-      </c>
-      <c r="J13" s="15">
-        <v>0</v>
-      </c>
-      <c r="K13" s="18" t="s">
-        <v>188</v>
-      </c>
-      <c r="L13" s="13"/>
-    </row>
-    <row r="14" spans="1:18" s="20" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="20">
-        <v>13</v>
-      </c>
-      <c r="B14" s="20">
-        <v>7</v>
-      </c>
-      <c r="C14" s="20" t="s">
-        <v>106</v>
-      </c>
-      <c r="D14" s="20">
+      <c r="K39" s="12" t="s">
+        <v>323</v>
+      </c>
+      <c r="L39" s="7"/>
+      <c r="N39" s="14"/>
+      <c r="P39" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="E14" s="20" t="s">
-        <v>115</v>
-      </c>
-      <c r="F14" s="20" t="s">
-        <v>302</v>
-      </c>
-      <c r="G14" s="20" t="s">
-        <v>226</v>
-      </c>
-      <c r="H14" s="20" t="s">
-        <v>303</v>
-      </c>
-      <c r="I14" s="20" t="s">
-        <v>17</v>
-      </c>
-      <c r="J14" s="20">
-        <v>1</v>
-      </c>
-      <c r="K14" s="20" t="s">
-        <v>189</v>
-      </c>
-      <c r="N14" s="12"/>
-      <c r="R14" s="31" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="15" spans="1:18" s="12" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="15">
-        <v>14</v>
-      </c>
-      <c r="B15" s="15">
-        <v>7</v>
-      </c>
-      <c r="C15" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="D15" s="15">
-        <v>70</v>
-      </c>
-      <c r="E15" s="12" t="s">
-        <v>116</v>
-      </c>
-      <c r="F15" s="16" t="s">
-        <v>117</v>
-      </c>
-      <c r="G15" s="13" t="s">
-        <v>227</v>
-      </c>
-      <c r="H15" s="16" t="s">
-        <v>118</v>
-      </c>
-      <c r="I15" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="J15" s="15">
-        <v>0</v>
-      </c>
-      <c r="K15" s="18" t="s">
-        <v>190</v>
-      </c>
-      <c r="L15" s="13"/>
-    </row>
-    <row r="16" spans="1:18" s="20" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="20">
-        <v>15</v>
-      </c>
-      <c r="B16" s="20">
-        <v>7</v>
-      </c>
-      <c r="C16" s="20" t="s">
-        <v>106</v>
-      </c>
-      <c r="D16" s="20">
-        <v>64</v>
-      </c>
-      <c r="E16" s="20" t="s">
-        <v>119</v>
-      </c>
-      <c r="F16" s="31" t="s">
-        <v>304</v>
-      </c>
-      <c r="G16" s="20" t="s">
-        <v>228</v>
-      </c>
-      <c r="H16" s="20" t="s">
-        <v>305</v>
-      </c>
-      <c r="I16" s="20" t="s">
-        <v>19</v>
-      </c>
-      <c r="J16" s="20">
-        <v>2</v>
-      </c>
-      <c r="K16" s="20" t="s">
-        <v>191</v>
-      </c>
-      <c r="N16" s="12"/>
-    </row>
-    <row r="17" spans="1:17" s="7" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="6">
-        <v>16</v>
-      </c>
-      <c r="B17" s="6">
-        <v>8</v>
-      </c>
-      <c r="C17" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="D17" s="6">
-        <v>85</v>
-      </c>
-      <c r="E17" s="7" t="s">
-        <v>120</v>
-      </c>
-      <c r="F17" s="9" t="s">
-        <v>278</v>
-      </c>
-      <c r="G17" s="10" t="s">
-        <v>229</v>
-      </c>
-      <c r="H17" s="9" t="s">
-        <v>279</v>
-      </c>
-      <c r="I17" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="J17" s="6">
-        <v>0</v>
-      </c>
-      <c r="K17" s="11" t="s">
-        <v>192</v>
-      </c>
-      <c r="L17" s="10"/>
-      <c r="N17" s="10"/>
-    </row>
-    <row r="18" spans="1:17" s="12" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="15">
-        <v>17</v>
-      </c>
-      <c r="B18" s="15">
-        <v>8</v>
-      </c>
-      <c r="C18" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="D18" s="15">
-        <v>84</v>
-      </c>
-      <c r="E18" s="12" t="s">
-        <v>121</v>
-      </c>
-      <c r="F18" s="16" t="s">
-        <v>280</v>
-      </c>
-      <c r="G18" s="13" t="s">
-        <v>230</v>
-      </c>
-      <c r="H18" s="16" t="s">
-        <v>281</v>
-      </c>
-      <c r="I18" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="J18" s="15">
-        <v>0</v>
-      </c>
-      <c r="K18" s="18" t="s">
-        <v>193</v>
-      </c>
-      <c r="L18" s="13"/>
-    </row>
-    <row r="19" spans="1:17" s="7" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="6">
-        <v>18</v>
-      </c>
-      <c r="B19" s="6">
-        <v>8</v>
-      </c>
-      <c r="C19" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="D19" s="6">
-        <v>93</v>
-      </c>
-      <c r="E19" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="F19" s="9" t="s">
-        <v>323</v>
-      </c>
-      <c r="G19" s="10" t="s">
-        <v>231</v>
-      </c>
-      <c r="H19" s="9" t="s">
-        <v>324</v>
-      </c>
-      <c r="I19" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="J19" s="6">
-        <v>0</v>
-      </c>
-      <c r="K19" s="11" t="s">
-        <v>194</v>
-      </c>
-      <c r="L19" s="10"/>
-      <c r="N19" s="10"/>
-    </row>
-    <row r="20" spans="1:17" s="12" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="32">
-        <v>19</v>
-      </c>
-      <c r="B20" s="32">
-        <v>8</v>
-      </c>
-      <c r="C20" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="D20" s="15">
-        <v>69</v>
-      </c>
-      <c r="E20" s="19" t="s">
-        <v>123</v>
-      </c>
-      <c r="F20" s="16" t="s">
-        <v>124</v>
-      </c>
-      <c r="G20" s="13" t="s">
-        <v>232</v>
-      </c>
-      <c r="H20" s="16" t="s">
-        <v>125</v>
-      </c>
-      <c r="I20" s="19" t="s">
-        <v>30</v>
-      </c>
-      <c r="J20" s="15">
-        <v>0</v>
-      </c>
-      <c r="K20" s="18" t="s">
-        <v>195</v>
-      </c>
-      <c r="L20" s="13"/>
-      <c r="N20" s="13"/>
-    </row>
-    <row r="21" spans="1:17" s="7" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="6">
-        <v>20</v>
-      </c>
-      <c r="B21" s="6">
-        <v>9</v>
-      </c>
-      <c r="C21" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="D21" s="6">
-        <v>78</v>
-      </c>
-      <c r="E21" s="7" t="s">
-        <v>126</v>
-      </c>
-      <c r="F21" s="9" t="s">
-        <v>282</v>
-      </c>
-      <c r="G21" s="10" t="s">
-        <v>345</v>
-      </c>
-      <c r="H21" s="34" t="s">
-        <v>333</v>
-      </c>
-      <c r="I21" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="J21" s="6">
-        <v>0</v>
-      </c>
-      <c r="K21" s="11" t="s">
-        <v>196</v>
-      </c>
-      <c r="L21" s="10"/>
-    </row>
-    <row r="22" spans="1:17" s="7" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="6">
-        <v>21</v>
-      </c>
-      <c r="B22" s="6">
-        <v>9</v>
-      </c>
-      <c r="C22" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="D22" s="6">
-        <v>75</v>
-      </c>
-      <c r="E22" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="F22" s="9" t="s">
-        <v>286</v>
-      </c>
-      <c r="G22" s="10" t="s">
-        <v>233</v>
-      </c>
-      <c r="H22" s="34" t="s">
-        <v>334</v>
-      </c>
-      <c r="I22" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="J22" s="6">
-        <v>0</v>
-      </c>
-      <c r="K22" s="11" t="s">
-        <v>197</v>
-      </c>
-      <c r="L22" s="10"/>
-    </row>
-    <row r="23" spans="1:17" s="7" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="6">
-        <v>22</v>
-      </c>
-      <c r="B23" s="6">
-        <v>9</v>
-      </c>
-      <c r="C23" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="D23" s="6">
-        <v>78</v>
-      </c>
-      <c r="E23" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="F23" s="9" t="s">
-        <v>283</v>
-      </c>
-      <c r="G23" s="10" t="s">
-        <v>344</v>
-      </c>
-      <c r="H23" s="34" t="s">
-        <v>335</v>
-      </c>
-      <c r="I23" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="J23" s="6">
-        <v>0</v>
-      </c>
-      <c r="K23" s="11" t="s">
-        <v>198</v>
-      </c>
-      <c r="L23" s="10"/>
-    </row>
-    <row r="24" spans="1:17" s="7" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="6">
-        <v>23</v>
-      </c>
-      <c r="B24" s="6">
-        <v>9</v>
-      </c>
-      <c r="C24" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="D24" s="6">
-        <v>75</v>
-      </c>
-      <c r="E24" s="7" t="s">
-        <v>129</v>
-      </c>
-      <c r="F24" s="9" t="s">
-        <v>287</v>
-      </c>
-      <c r="G24" s="10" t="s">
-        <v>234</v>
-      </c>
-      <c r="H24" s="34" t="s">
-        <v>336</v>
-      </c>
-      <c r="I24" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="J24" s="6">
-        <v>0</v>
-      </c>
-      <c r="K24" s="11" t="s">
-        <v>199</v>
-      </c>
-      <c r="L24" s="10"/>
-      <c r="N24" s="33"/>
-    </row>
-    <row r="25" spans="1:17" s="7" customFormat="1" ht="261" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="6">
-        <v>24</v>
-      </c>
-      <c r="B25" s="6">
-        <v>11</v>
-      </c>
-      <c r="C25" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="D25" s="6">
-        <v>85</v>
-      </c>
-      <c r="E25" s="7" t="s">
-        <v>130</v>
-      </c>
-      <c r="F25" s="9" t="s">
-        <v>284</v>
-      </c>
-      <c r="G25" s="10" t="s">
-        <v>343</v>
-      </c>
-      <c r="H25" s="9" t="s">
-        <v>285</v>
-      </c>
-      <c r="I25" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="J25" s="6">
-        <v>0</v>
-      </c>
-      <c r="K25" s="11" t="s">
-        <v>200</v>
-      </c>
-      <c r="L25" s="10"/>
-    </row>
-    <row r="26" spans="1:17" s="7" customFormat="1" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="6">
-        <v>25</v>
-      </c>
-      <c r="B26" s="6">
-        <v>11</v>
-      </c>
-      <c r="C26" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="D26" s="6">
-        <v>78</v>
-      </c>
-      <c r="E26" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="F26" s="9" t="s">
-        <v>288</v>
-      </c>
-      <c r="G26" s="10" t="s">
-        <v>235</v>
-      </c>
-      <c r="H26" s="9" t="s">
-        <v>331</v>
-      </c>
-      <c r="I26" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="J26" s="6">
-        <v>0</v>
-      </c>
-      <c r="K26" s="11" t="s">
-        <v>201</v>
-      </c>
-      <c r="L26" s="10"/>
-    </row>
-    <row r="27" spans="1:17" s="7" customFormat="1" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="6">
-        <v>26</v>
-      </c>
-      <c r="B27" s="6">
-        <v>11</v>
-      </c>
-      <c r="C27" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="D27" s="6">
-        <v>95</v>
-      </c>
-      <c r="E27" s="7" t="s">
-        <v>132</v>
-      </c>
-      <c r="F27" s="9" t="s">
-        <v>289</v>
-      </c>
-      <c r="G27" s="10" t="s">
-        <v>236</v>
-      </c>
-      <c r="H27" s="9" t="s">
-        <v>337</v>
-      </c>
-      <c r="I27" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="J27" s="6">
-        <v>0</v>
-      </c>
-      <c r="K27" s="11" t="s">
-        <v>202</v>
-      </c>
-      <c r="L27" s="10"/>
-    </row>
-    <row r="28" spans="1:17" s="7" customFormat="1" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="6">
-        <v>27</v>
-      </c>
-      <c r="B28" s="6">
-        <v>11</v>
-      </c>
-      <c r="C28" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="D28" s="6">
-        <v>107</v>
-      </c>
-      <c r="E28" s="7" t="s">
-        <v>133</v>
-      </c>
-      <c r="F28" s="9" t="s">
-        <v>290</v>
-      </c>
-      <c r="G28" s="10" t="s">
-        <v>237</v>
-      </c>
-      <c r="H28" s="9" t="s">
-        <v>338</v>
-      </c>
-      <c r="I28" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="J28" s="6">
-        <v>0</v>
-      </c>
-      <c r="K28" s="11" t="s">
-        <v>203</v>
-      </c>
-      <c r="L28" s="10"/>
-    </row>
-    <row r="29" spans="1:17" s="12" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A29" s="15">
-        <v>28</v>
-      </c>
-      <c r="B29" s="15">
-        <v>0</v>
-      </c>
-      <c r="C29" s="12" t="s">
-        <v>86</v>
-      </c>
-      <c r="D29" s="15">
-        <v>40</v>
-      </c>
-      <c r="E29" s="16" t="s">
-        <v>311</v>
-      </c>
-      <c r="F29" s="16" t="s">
-        <v>134</v>
-      </c>
-      <c r="G29" s="28" t="s">
-        <v>172</v>
-      </c>
-      <c r="H29" s="16" t="s">
-        <v>135</v>
-      </c>
-      <c r="I29" s="12" t="s">
-        <v>50</v>
-      </c>
-      <c r="J29" s="15">
-        <v>0</v>
-      </c>
-      <c r="K29" s="26" t="s">
-        <v>205</v>
-      </c>
-      <c r="L29" s="13" t="s">
-        <v>215</v>
-      </c>
-      <c r="M29" s="12">
-        <v>3</v>
-      </c>
-      <c r="N29" s="21"/>
-      <c r="P29" s="16" t="s">
-        <v>51</v>
-      </c>
-      <c r="Q29" s="19" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="30" spans="1:17" s="36" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="35">
-        <v>29</v>
-      </c>
-      <c r="B30" s="35">
-        <v>0</v>
-      </c>
-      <c r="C30" s="36" t="s">
-        <v>86</v>
-      </c>
-      <c r="D30" s="35">
-        <v>26</v>
-      </c>
-      <c r="E30" s="37" t="s">
-        <v>312</v>
-      </c>
-      <c r="F30" s="38" t="s">
-        <v>137</v>
-      </c>
-      <c r="G30" s="39" t="s">
-        <v>297</v>
-      </c>
-      <c r="H30" s="38" t="s">
-        <v>138</v>
-      </c>
-      <c r="I30" s="36" t="s">
-        <v>52</v>
-      </c>
-      <c r="J30" s="35">
-        <v>0</v>
-      </c>
-      <c r="K30" s="40" t="s">
-        <v>205</v>
-      </c>
-      <c r="L30" s="36" t="s">
-        <v>295</v>
-      </c>
-      <c r="M30" s="36" t="s">
-        <v>296</v>
-      </c>
-      <c r="P30" s="38" t="s">
-        <v>53</v>
-      </c>
-      <c r="Q30" s="37" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="31" spans="1:17" s="12" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A31" s="15">
-        <v>30</v>
-      </c>
-      <c r="B31" s="15">
-        <v>0</v>
-      </c>
-      <c r="C31" s="12" t="s">
-        <v>86</v>
-      </c>
-      <c r="D31" s="15">
-        <v>34</v>
-      </c>
-      <c r="E31" s="19" t="s">
-        <v>313</v>
-      </c>
-      <c r="F31" s="16" t="s">
-        <v>140</v>
-      </c>
-      <c r="G31" s="28" t="s">
-        <v>173</v>
-      </c>
-      <c r="H31" s="16" t="s">
-        <v>141</v>
-      </c>
-      <c r="I31" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="J31" s="15">
-        <v>0</v>
-      </c>
-      <c r="K31" s="26" t="s">
-        <v>205</v>
-      </c>
-      <c r="L31" s="20" t="s">
-        <v>216</v>
-      </c>
-      <c r="M31" s="20" t="s">
-        <v>217</v>
-      </c>
-      <c r="N31" s="24"/>
-      <c r="P31" s="16" t="s">
-        <v>55</v>
-      </c>
-      <c r="Q31" s="19" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="32" spans="1:17" s="12" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A32" s="15">
-        <v>31</v>
-      </c>
-      <c r="B32" s="15">
-        <v>0</v>
-      </c>
-      <c r="C32" s="12" t="s">
-        <v>86</v>
-      </c>
-      <c r="D32" s="15">
-        <v>34</v>
-      </c>
-      <c r="E32" s="12" t="s">
-        <v>314</v>
-      </c>
-      <c r="F32" s="16" t="s">
-        <v>143</v>
-      </c>
-      <c r="G32" s="28" t="s">
-        <v>174</v>
-      </c>
-      <c r="H32" s="16" t="s">
-        <v>144</v>
-      </c>
-      <c r="I32" s="12" t="s">
-        <v>56</v>
-      </c>
-      <c r="J32" s="15">
-        <v>0</v>
-      </c>
-      <c r="K32" s="26" t="s">
-        <v>205</v>
-      </c>
-      <c r="L32" s="13" t="s">
-        <v>218</v>
-      </c>
-      <c r="M32" s="12" t="s">
-        <v>219</v>
-      </c>
-      <c r="N32" s="21"/>
-      <c r="P32" s="16" t="s">
-        <v>57</v>
-      </c>
-      <c r="Q32" s="19" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="33" spans="1:17" s="36" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="35">
-        <v>32</v>
-      </c>
-      <c r="B33" s="35">
-        <v>0</v>
-      </c>
-      <c r="C33" s="36" t="s">
-        <v>86</v>
-      </c>
-      <c r="D33" s="35">
-        <v>26</v>
-      </c>
-      <c r="E33" s="36" t="s">
-        <v>315</v>
-      </c>
-      <c r="F33" s="38" t="s">
-        <v>146</v>
-      </c>
-      <c r="G33" s="39" t="s">
-        <v>175</v>
-      </c>
-      <c r="H33" s="38" t="s">
-        <v>147</v>
-      </c>
-      <c r="I33" s="36" t="s">
-        <v>58</v>
-      </c>
-      <c r="J33" s="35">
-        <v>0</v>
-      </c>
-      <c r="K33" s="40" t="s">
-        <v>205</v>
-      </c>
-      <c r="L33" s="39"/>
-      <c r="P33" s="38" t="s">
-        <v>59</v>
-      </c>
-      <c r="Q33" s="37" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="34" spans="1:17" s="36" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="35">
-        <v>33</v>
-      </c>
-      <c r="B34" s="35">
-        <v>0</v>
-      </c>
-      <c r="C34" s="36" t="s">
-        <v>86</v>
-      </c>
-      <c r="D34" s="35">
-        <v>28</v>
-      </c>
-      <c r="E34" s="36" t="s">
-        <v>316</v>
-      </c>
-      <c r="F34" s="38" t="s">
-        <v>149</v>
-      </c>
-      <c r="G34" s="39" t="s">
-        <v>176</v>
-      </c>
-      <c r="H34" s="38" t="s">
-        <v>150</v>
-      </c>
-      <c r="I34" s="36" t="s">
-        <v>60</v>
-      </c>
-      <c r="J34" s="35">
-        <v>0</v>
-      </c>
-      <c r="K34" s="40" t="s">
-        <v>205</v>
-      </c>
-      <c r="L34" s="39"/>
-      <c r="P34" s="38" t="s">
-        <v>61</v>
-      </c>
-      <c r="Q34" s="37" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="35" spans="1:17" s="12" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A35" s="15">
-        <v>34</v>
-      </c>
-      <c r="B35" s="15">
-        <v>0</v>
-      </c>
-      <c r="C35" s="12" t="s">
-        <v>86</v>
-      </c>
-      <c r="D35" s="15">
-        <v>26</v>
-      </c>
-      <c r="E35" s="12" t="s">
-        <v>317</v>
-      </c>
-      <c r="F35" s="16" t="s">
-        <v>152</v>
-      </c>
-      <c r="G35" s="28" t="s">
-        <v>177</v>
-      </c>
-      <c r="H35" s="16" t="s">
-        <v>153</v>
-      </c>
-      <c r="I35" s="12" t="s">
-        <v>62</v>
-      </c>
-      <c r="J35" s="15">
-        <v>0</v>
-      </c>
-      <c r="K35" s="26" t="s">
-        <v>205</v>
-      </c>
-      <c r="L35" s="13" t="s">
-        <v>220</v>
-      </c>
-      <c r="M35" s="12" t="s">
-        <v>221</v>
-      </c>
-      <c r="N35" s="21"/>
-      <c r="P35" s="16" t="s">
-        <v>63</v>
-      </c>
-      <c r="Q35" s="19" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="36" spans="1:17" s="12" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A36" s="15">
-        <v>35</v>
-      </c>
-      <c r="B36" s="15">
-        <v>0</v>
-      </c>
-      <c r="C36" s="12" t="s">
-        <v>86</v>
-      </c>
-      <c r="D36" s="15">
-        <v>34</v>
-      </c>
-      <c r="E36" s="12" t="s">
-        <v>310</v>
-      </c>
-      <c r="F36" s="16" t="s">
-        <v>155</v>
-      </c>
-      <c r="G36" s="28" t="s">
-        <v>178</v>
-      </c>
-      <c r="H36" s="16" t="s">
-        <v>156</v>
-      </c>
-      <c r="I36" s="12" t="s">
-        <v>64</v>
-      </c>
-      <c r="J36" s="15">
-        <v>0</v>
-      </c>
-      <c r="K36" s="26" t="s">
-        <v>205</v>
-      </c>
-      <c r="L36" s="13" t="s">
-        <v>222</v>
-      </c>
-      <c r="M36" s="12">
-        <v>5</v>
-      </c>
-      <c r="N36" s="21"/>
-      <c r="P36" s="16" t="s">
-        <v>65</v>
-      </c>
-      <c r="Q36" s="19" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="37" spans="1:17" s="7" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="6">
-        <v>36</v>
-      </c>
-      <c r="B37" s="6">
-        <v>0</v>
-      </c>
-      <c r="C37" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="D37" s="6">
-        <v>97</v>
-      </c>
-      <c r="E37" s="7" t="s">
-        <v>309</v>
-      </c>
-      <c r="F37" s="9" t="s">
-        <v>158</v>
-      </c>
-      <c r="G37" s="10" t="s">
-        <v>238</v>
-      </c>
-      <c r="H37" s="9" t="s">
-        <v>332</v>
-      </c>
-      <c r="I37" s="7" t="s">
-        <v>73</v>
-      </c>
-      <c r="J37" s="6">
-        <v>0</v>
-      </c>
-      <c r="K37" s="11" t="s">
-        <v>204</v>
-      </c>
-      <c r="L37" s="10"/>
-      <c r="P37" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="Q37" s="8" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="38" spans="1:17" s="7" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="6">
-        <v>37</v>
-      </c>
-      <c r="B38" s="6">
-        <v>0</v>
-      </c>
-      <c r="C38" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="D38" s="6">
-        <v>67</v>
-      </c>
-      <c r="E38" s="7" t="s">
-        <v>307</v>
-      </c>
-      <c r="F38" s="9" t="s">
-        <v>160</v>
-      </c>
-      <c r="G38" s="10" t="s">
-        <v>239</v>
-      </c>
-      <c r="H38" s="9" t="s">
-        <v>161</v>
-      </c>
-      <c r="I38" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="J38" s="6">
-        <v>0</v>
-      </c>
-      <c r="K38" s="11" t="s">
-        <v>341</v>
-      </c>
-      <c r="L38" s="10"/>
-      <c r="P38" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="Q38" s="8" t="s">
+      <c r="Q39" s="13" t="s">
         <v>162</v>
-      </c>
-    </row>
-    <row r="39" spans="1:17" s="7" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="6">
-        <v>38</v>
-      </c>
-      <c r="B39" s="6">
-        <v>0</v>
-      </c>
-      <c r="C39" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="D39" s="6">
-        <v>85</v>
-      </c>
-      <c r="E39" s="7" t="s">
-        <v>308</v>
-      </c>
-      <c r="F39" s="9" t="s">
-        <v>339</v>
-      </c>
-      <c r="G39" s="10" t="s">
-        <v>240</v>
-      </c>
-      <c r="H39" s="9" t="s">
-        <v>340</v>
-      </c>
-      <c r="I39" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="J39" s="6">
-        <v>0</v>
-      </c>
-      <c r="K39" s="11" t="s">
-        <v>342</v>
-      </c>
-      <c r="L39" s="10"/>
-      <c r="P39" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="Q39" s="8" t="s">
-        <v>163</v>
       </c>
     </row>
   </sheetData>
@@ -5415,7 +5396,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:D63"/>
+  <dimension ref="A1:D64"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="60" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
@@ -5569,7 +5550,7 @@
         <v>13</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>325</v>
+        <v>312</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5584,7 +5565,7 @@
         <v>14</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>319</v>
+        <v>306</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5599,7 +5580,7 @@
         <v>15</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>300</v>
+        <v>287</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5614,7 +5595,7 @@
         <v>16</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5629,7 +5610,7 @@
         <v>17</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>301</v>
+        <v>288</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5644,7 +5625,7 @@
         <v>18</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5659,7 +5640,7 @@
         <v>19</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>306</v>
+        <v>293</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5674,7 +5655,7 @@
         <v>20</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>328</v>
+        <v>315</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5689,7 +5670,7 @@
         <v>21</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5704,7 +5685,7 @@
         <v>22</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5719,7 +5700,7 @@
         <v>23</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5734,7 +5715,7 @@
         <v>24</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5749,7 +5730,7 @@
         <v>25</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5764,7 +5745,7 @@
         <v>26</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5779,7 +5760,7 @@
         <v>27</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5794,7 +5775,7 @@
         <v>28</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5809,7 +5790,7 @@
         <v>29</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5824,7 +5805,7 @@
         <v>30</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>329</v>
+        <v>316</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5838,7 +5819,7 @@
         <v>31</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>252</v>
+        <v>246</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5852,7 +5833,7 @@
         <v>32</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5866,7 +5847,7 @@
         <v>33</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>254</v>
+        <v>248</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5880,7 +5861,7 @@
         <v>34</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>255</v>
+        <v>249</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5894,7 +5875,7 @@
         <v>35</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>256</v>
+        <v>250</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5908,7 +5889,7 @@
         <v>36</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>257</v>
+        <v>251</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5922,7 +5903,7 @@
         <v>37</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5936,7 +5917,7 @@
         <v>38</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5950,7 +5931,7 @@
         <v>39</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>260</v>
+        <v>333</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5964,7 +5945,7 @@
         <v>40</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>261</v>
+        <v>254</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5978,7 +5959,7 @@
         <v>41</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>262</v>
+        <v>255</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5992,7 +5973,7 @@
         <v>42</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6006,7 +5987,7 @@
         <v>43</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>264</v>
+        <v>257</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6020,7 +6001,7 @@
         <v>44</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6034,7 +6015,7 @@
         <v>45</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6048,7 +6029,7 @@
         <v>46</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>267</v>
+        <v>340</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6062,7 +6043,7 @@
         <v>47</v>
       </c>
       <c r="D44" s="5" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6076,7 +6057,7 @@
         <v>48</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>269</v>
+        <v>261</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6090,7 +6071,7 @@
         <v>49</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6216,7 +6197,7 @@
         <v>66</v>
       </c>
       <c r="D55" s="5" t="s">
-        <v>271</v>
+        <v>263</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6230,7 +6211,7 @@
         <v>68</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>272</v>
+        <v>264</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6244,7 +6225,7 @@
         <v>70</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>272</v>
+        <v>264</v>
       </c>
     </row>
     <row r="58" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6258,7 +6239,7 @@
         <v>71</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>272</v>
+        <v>264</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6272,7 +6253,7 @@
         <v>72</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>272</v>
+        <v>264</v>
       </c>
     </row>
     <row r="60" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6286,7 +6267,7 @@
         <v>73</v>
       </c>
       <c r="D60" s="5" t="s">
-        <v>273</v>
+        <v>265</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6300,7 +6281,7 @@
         <v>74</v>
       </c>
       <c r="D61" s="5" t="s">
-        <v>274</v>
+        <v>266</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6314,7 +6295,7 @@
         <v>68</v>
       </c>
       <c r="D62" s="5" t="s">
-        <v>275</v>
+        <v>267</v>
       </c>
     </row>
     <row r="63" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6328,7 +6309,21 @@
         <v>66</v>
       </c>
       <c r="D63" s="5" t="s">
-        <v>275</v>
+        <v>267</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="1">
+        <v>63</v>
+      </c>
+      <c r="B64" s="1">
+        <v>38</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>347</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>348</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Tutor Kai: All tasks work now
- Fixed remaining 3 tasks for higher functions and Java Bank Task
</commit_message>
<xml_diff>
--- a/files/programming-tasks/programmieraufgaben_JACK_SOSE23_WORKSHOP_WISE2324.xlsx
+++ b/files/programming-tasks/programmieraufgaben_JACK_SOSE23_WORKSHOP_WISE2324.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\hefl\files\programming-tasks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72D76F82-293F-48EF-B565-F7F61FF8CCC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D34F5F7-B8EF-40EA-BF9B-DFA61FAFCED5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51480" yWindow="-645" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="461" uniqueCount="350">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="354">
   <si>
     <t>id</t>
   </si>
@@ -2242,39 +2242,6 @@
   </si>
   <si>
     <t xml:space="preserve"> lambda x: math.sin(x),  lambda x: 2 * math.pi * x</t>
-  </si>
-  <si>
-    <t xml:space="preserve">import unittest
-import math
-from funktionen import concatenate_functions
-class TestConcatenateFunctions(unittest.TestCase):
-     def test_direct_math_functions(self):
-        """Testet die Verkettung von zwei direkten mathematischen Funktionen."""
-        f1 = math.sqrt  # Erste Funktion: Quadratwurzel
-        f2 = math.exp   # Zweite Funktion: Exponentialfunktion
-        concatenated_func = concatenate_functions(f1, f2)
-        x = 2  # Beispielwert
-        expected = math.sqrt(math.exp(x))
-        self.assertAlmostEqual(concatenated_func(x), expected, delta=1e-7)
-    def test_identity_function(self):
-        """Überprüft die Verkettung mit einer Identitätsfunktion."""
-        f1 = lambda x: x  # Identitätsfunktion
-        f2 = math.sin     # Zweite Funktion: Sinus
-        concatenated_func = concatenate_functions(f1, f2)
-        x = math.pi / 2  # Beispielwert
-        expected = math.sin(x)
-        self.assertEqual(concatenated_func(x), expected)
-    def test_custom_functions(self):
-        """Testet die Verkettung von benutzerdefinierten Funktionen."""
-        f1 = lambda x: x ** 2  # Quadrieren
-        f2 = lambda x: x + 2   # Addiere 2
-        concatenated_func = concatenate_functions(f1, f2)
-        x = 3  # Beispielwert
-        expected = (x + 2) ** 2
-        self.assertEqual(concatenated_func(x), expected)
-if __name__ == '__main__':
-    unittest.main()
-</t>
   </si>
   <si>
     <t xml:space="preserve">  &lt;h1&gt;Fibonacci-Folge Index Finder&lt;/h1&gt;
@@ -2844,52 +2811,6 @@
 &lt;/div&gt;</t>
   </si>
   <si>
-    <t>package de.goals.testing;
-import org.junit.jupiter.api.Test;
-import static org.junit.jupiter.api.Assertions.assertEquals;
-public class AppBankTest {
-    @Test
-    public void testToString() {
-        Konto konto = new Konto("Andreas", "Hoffmann", "DE232212442");
-        konto.einzahlen(100);
-        konto.setLimit(500);
-        String expected = "Kunde: Andreas Hoffmann, Konto: DE232212442, Stand: 100.00, Limit: 500.00";
-        assertEquals(expected, konto.toString(), "Fehler in der toString() Methode");
-    }
-    @Test
-    public void testEinzahlen() {
-        Konto konto = new Konto("Max", "Mustermann", "DE12345678901234567890");
-        konto.einzahlen(100);
-        double expectedKontostand = 100.00;
-        assertEquals(expectedKontostand, konto.getKontostand(), "Fehler in der Einzahlen-Methode");
-    }
-    @Test
-    public void testAuszahlenWithinLimit() {
-        Konto konto = new Konto("Max", "Mustermann", "DE12345678901234567890");
-        konto.einzahlen(1000);
-        konto.auszahlen(500);
-        double expectedKontostand = 500.0;
-        assertEquals(expectedKontostand, konto.getKontostand(), "Fehler in der Auszahlen-Methode mit Betrag innerhalb des Limits");
-    }
-    @Test
-    public void testAuszahlenExceedingLimit() {
-        Konto konto = new Konto("Max", "Mustermann", "DE12345678901234567890");
-        konto.einzahlen(1000);
-        konto.setLimit(500); // Set the limit before withdrawing
-        konto.auszahlen(1500); // Versucht 1500 auszuzahlen, was über das Limit geht
-        double expectedKontostand = -500.0; // Kontostand sollte -Limit sein
-        assertEquals(expectedKontostand, konto.getKontostand(), "Fehler in der Auszahlen-Methode bei Überschreitung des Limits");
-    }
-    @Test
-    public void testSetLimit() {
-        Konto konto = new Konto("Max", "Mustermann", "DE12345678901234567890");
-        konto.setLimit(1000);
-        double expectedLimit = 1000.0;
-        assertEquals(expectedLimit, konto.getLimit(), "Fehler in der SetLimit-Methode");
-    }
-}</t>
-  </si>
-  <si>
     <t>Syntaxfehler: JA, Tests: NEIN
 Tests angepasst: Erneut überprüfen</t>
   </si>
@@ -3254,12 +3175,95 @@
         Öffentliche Methode getJahr(): gibt einen int zurück.
 Die Klasse Auto erbt die Attribute und Methoden von der Klasse Fahrzeug. Darauf weist der Vererbungspfeil im Diagramm hin.</t>
   </si>
+  <si>
+    <t>package de.goals.testing;
+import org.junit.jupiter.api.Test;
+import static org.junit.jupiter.api.Assertions.assertEquals;
+public class AppBankTest {
+    @Test
+    public void testToString() {
+        Konto konto = new Konto("Andreas", "Hoffmann", "DE232212442");
+        konto.einzahlen(100);
+        konto.setLimit(500);
+        String expected = "Kunde: Andreas Hoffmann, Konto: DE232212442, Stand: 100.00, Limit: 500.00";
+        assertEquals(expected, konto.toString(), "Fehler in der toString() Methode");
+    }
+    @Test
+    public void testEinzahlen() {
+        Konto konto = new Konto("Max", "Mustermann", "DE12345678901234567890");
+        konto.einzahlen(100);
+        double expectedKontostand = 100.00;
+        assertEquals(expectedKontostand, konto.getKontostand(), "Fehler in der Einzahlen-Methode");
+    }
+    @Test
+    public void testAuszahlenWithinLimit() {
+        Konto konto = new Konto("Max", "Mustermann", "DE12345678901234567890");
+        konto.einzahlen(1000);
+        konto.auszahlen(500);
+        double expectedKontostand = 500.0;
+        assertEquals(expectedKontostand, konto.getKontostand(), "Fehler in der Auszahlen-Methode mit Betrag innerhalb des Limits");
+    }
+    @Test
+    public void testAuszahlenExceedingLimit() {
+        Konto konto = new Konto("Max", "Mustermann", "DE12345678901234567890");
+        konto.einzahlen(1000);
+        konto.setLimit(500); // Set the limit before withdrawing
+        konto.auszahlen(1500); // Versucht 1500 auszuzahlen, was über das Limit geht
+        double expectedKontostand = -500.0; // Kontostand sollte -Limit sein
+        assertEquals(expectedKontostand, konto.getKontostand(), "Fehler in der Auszahlen-Methode bei Überschreitung des Limits");
+    }
+}</t>
+  </si>
+  <si>
+    <t>import unittest
+import math
+from funktionen import concatenate_functions
+class TestConcatenateFunctions(unittest.TestCase):
+    def test_direct_math_functions(self):
+        """Testet die Verkettung von zwei direkten mathematischen Funktionen."""
+        f1 = math.sqrt  # Erste Funktion: Quadratwurzel
+        f2 = math.exp   # Zweite Funktion: Exponentialfunktion
+        concatenated_func = concatenate_functions(f1, f2)
+        x = 2  # Beispielwert
+        expected = math.sqrt(math.exp(x))
+        self.assertAlmostEqual(concatenated_func(x), expected, delta=1e-7)
+    def test_identity_function(self):
+        """Überprüft die Verkettung mit einer Identitätsfunktion."""
+        f1 = lambda x: x  # Identitätsfunktion
+        f2 = math.sin     # Zweite Funktion: Sinus
+        concatenated_func = concatenate_functions(f1, f2)
+        x = math.pi / 2  # Beispielwert
+        expected = math.sin(x)
+        self.assertEqual(concatenated_func(x), expected)
+    def test_custom_functions(self):
+        """Testet die Verkettung von benutzerdefinierten Funktionen."""
+        f1 = lambda x: x ** 2  # Quadrieren
+        f2 = lambda x: x + 2   # Addiere 2
+        concatenated_func = concatenate_functions(f1, f2)
+        x = 3  # Beispielwert
+        expected = (x + 2) ** 2
+        self.assertEqual(concatenated_func(x), expected)
+if __name__ == '__main__':
+    unittest.main()</t>
+  </si>
+  <si>
+    <t>1000, lambda betrag: steuerfunktion(betrag - freibetrag) if betrag &gt; freibetrag else 0</t>
+  </si>
+  <si>
+    <t>nutze_freibetrag</t>
+  </si>
+  <si>
+    <t>filter_liste</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lambda x: x % 2 == 0, [1, 2, 3, 4, 5, 6] </t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3314,15 +3318,8 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3332,11 +3329,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFC6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -3371,12 +3363,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -3440,30 +3431,10 @@
     <xf numFmtId="3" fontId="3" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="3" fontId="8" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="2"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="2" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="3">
+  <cellStyles count="2">
     <cellStyle name="Gut" xfId="1" builtinId="26"/>
-    <cellStyle name="Schlecht" xfId="2" builtinId="27"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -3782,7 +3753,7 @@
     <col min="11" max="11" width="50.7109375" style="17" customWidth="1"/>
     <col min="12" max="12" width="49.85546875" style="2" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="74.5703125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="170.7109375" style="29" customWidth="1"/>
+    <col min="14" max="14" width="170.7109375" style="23" customWidth="1"/>
     <col min="15" max="17" width="13.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3826,7 +3797,7 @@
       <c r="M1" s="6" t="s">
         <v>179</v>
       </c>
-      <c r="N1" s="29"/>
+      <c r="N1" s="23"/>
     </row>
     <row r="2" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="9">
@@ -3868,7 +3839,7 @@
       <c r="M2" s="6" t="s">
         <v>206</v>
       </c>
-      <c r="N2" s="29"/>
+      <c r="N2" s="23"/>
     </row>
     <row r="3" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9">
@@ -3910,7 +3881,7 @@
       <c r="M3" s="6" t="s">
         <v>182</v>
       </c>
-      <c r="N3" s="29"/>
+      <c r="N3" s="23"/>
     </row>
     <row r="4" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9">
@@ -3952,7 +3923,7 @@
       <c r="M4" s="6">
         <v>174</v>
       </c>
-      <c r="N4" s="29"/>
+      <c r="N4" s="23"/>
     </row>
     <row r="5" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="9">
@@ -3977,7 +3948,7 @@
         <v>166</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="I5" s="6" t="s">
         <v>8</v>
@@ -3994,7 +3965,7 @@
       <c r="M5" s="6">
         <v>47</v>
       </c>
-      <c r="N5" s="29"/>
+      <c r="N5" s="23"/>
     </row>
     <row r="6" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="9">
@@ -4036,7 +4007,7 @@
       <c r="M6" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="N6" s="29"/>
+      <c r="N6" s="23"/>
     </row>
     <row r="7" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="9">
@@ -4078,7 +4049,7 @@
       <c r="M7" s="6" t="s">
         <v>278</v>
       </c>
-      <c r="N7" s="29"/>
+      <c r="N7" s="23"/>
     </row>
     <row r="8" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="9">
@@ -4103,7 +4074,7 @@
         <v>169</v>
       </c>
       <c r="H8" s="10" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="I8" s="6" t="s">
         <v>11</v>
@@ -4120,7 +4091,7 @@
       <c r="M8" s="6" t="s">
         <v>212</v>
       </c>
-      <c r="N8" s="29"/>
+      <c r="N8" s="23"/>
     </row>
     <row r="9" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="9">
@@ -4162,7 +4133,7 @@
       <c r="M9" s="6">
         <v>10</v>
       </c>
-      <c r="N9" s="29"/>
+      <c r="N9" s="23"/>
     </row>
     <row r="10" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="9">
@@ -4184,7 +4155,7 @@
         <v>108</v>
       </c>
       <c r="G10" s="11" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="H10" s="10" t="s">
         <v>109</v>
@@ -4199,9 +4170,9 @@
         <v>184</v>
       </c>
       <c r="L10" s="7"/>
-      <c r="N10" s="29"/>
+      <c r="N10" s="23"/>
       <c r="R10" s="7" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="11" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4239,9 +4210,9 @@
         <v>185</v>
       </c>
       <c r="L11" s="7"/>
-      <c r="N11" s="29"/>
+      <c r="N11" s="23"/>
       <c r="R11" s="7" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="12" spans="1:18" s="14" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4261,13 +4232,13 @@
         <v>111</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="G12" s="21" t="s">
         <v>223</v>
       </c>
       <c r="H12" s="21" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="I12" s="14" t="s">
         <v>15</v>
@@ -4278,9 +4249,9 @@
       <c r="K12" s="14" t="s">
         <v>186</v>
       </c>
-      <c r="N12" s="29"/>
+      <c r="N12" s="23"/>
       <c r="R12" s="21" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="13" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4318,7 +4289,7 @@
         <v>187</v>
       </c>
       <c r="L13" s="7"/>
-      <c r="N13" s="29"/>
+      <c r="N13" s="23"/>
     </row>
     <row r="14" spans="1:18" s="14" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="14">
@@ -4337,13 +4308,13 @@
         <v>115</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="G14" s="14" t="s">
         <v>225</v>
       </c>
       <c r="H14" s="14" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="I14" s="14" t="s">
         <v>17</v>
@@ -4354,9 +4325,9 @@
       <c r="K14" s="14" t="s">
         <v>188</v>
       </c>
-      <c r="N14" s="29"/>
+      <c r="N14" s="23"/>
       <c r="R14" s="21" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="15" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4394,7 +4365,7 @@
         <v>189</v>
       </c>
       <c r="L15" s="7"/>
-      <c r="N15" s="29"/>
+      <c r="N15" s="23"/>
     </row>
     <row r="16" spans="1:18" s="14" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="14">
@@ -4413,13 +4384,13 @@
         <v>119</v>
       </c>
       <c r="F16" s="21" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="G16" s="14" t="s">
         <v>227</v>
       </c>
       <c r="H16" s="14" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="I16" s="14" t="s">
         <v>19</v>
@@ -4430,7 +4401,7 @@
       <c r="K16" s="14" t="s">
         <v>190</v>
       </c>
-      <c r="N16" s="29"/>
+      <c r="N16" s="23"/>
     </row>
     <row r="17" spans="1:17" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="9">
@@ -4449,13 +4420,13 @@
         <v>120</v>
       </c>
       <c r="F17" s="10" t="s">
+        <v>324</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>330</v>
+      </c>
+      <c r="H17" s="10" t="s">
         <v>325</v>
-      </c>
-      <c r="G17" s="7" t="s">
-        <v>332</v>
-      </c>
-      <c r="H17" s="10" t="s">
-        <v>326</v>
       </c>
       <c r="I17" s="10" t="s">
         <v>20</v>
@@ -4468,7 +4439,7 @@
       </c>
       <c r="L17" s="7"/>
       <c r="N17" s="21" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="18" spans="1:17" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4506,7 +4477,7 @@
         <v>192</v>
       </c>
       <c r="L18" s="7"/>
-      <c r="N18" s="29"/>
+      <c r="N18" s="23"/>
     </row>
     <row r="19" spans="1:17" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="9">
@@ -4525,13 +4496,13 @@
         <v>122</v>
       </c>
       <c r="F19" s="10" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="G19" s="7" t="s">
         <v>229</v>
       </c>
       <c r="H19" s="10" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="I19" s="6" t="s">
         <v>29</v>
@@ -4543,7 +4514,7 @@
         <v>193</v>
       </c>
       <c r="L19" s="7"/>
-      <c r="N19" s="29"/>
+      <c r="N19" s="23"/>
     </row>
     <row r="20" spans="1:17" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="22">
@@ -4580,7 +4551,7 @@
         <v>194</v>
       </c>
       <c r="L20" s="7"/>
-      <c r="N20" s="29"/>
+      <c r="N20" s="23"/>
     </row>
     <row r="21" spans="1:17" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="9">
@@ -4602,10 +4573,10 @@
         <v>272</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="H21" s="14" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="I21" s="6" t="s">
         <v>32</v>
@@ -4617,7 +4588,7 @@
         <v>195</v>
       </c>
       <c r="L21" s="7"/>
-      <c r="N21" s="29"/>
+      <c r="N21" s="23"/>
     </row>
     <row r="22" spans="1:17" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="9">
@@ -4639,10 +4610,10 @@
         <v>275</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="H22" s="14" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="I22" s="10" t="s">
         <v>34</v>
@@ -4656,43 +4627,43 @@
       <c r="L22" s="7"/>
       <c r="N22" s="21"/>
     </row>
-    <row r="23" spans="1:17" s="24" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="23">
+    <row r="23" spans="1:17" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="9">
         <v>22</v>
       </c>
-      <c r="B23" s="23">
+      <c r="B23" s="9">
         <v>9</v>
       </c>
-      <c r="C23" s="24" t="s">
+      <c r="C23" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="D23" s="23">
+      <c r="D23" s="9">
         <v>78</v>
       </c>
-      <c r="E23" s="24" t="s">
+      <c r="E23" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="F23" s="26" t="s">
+      <c r="F23" s="10" t="s">
+        <v>326</v>
+      </c>
+      <c r="G23" s="7" t="s">
+        <v>348</v>
+      </c>
+      <c r="H23" s="21" t="s">
         <v>327</v>
       </c>
-      <c r="G23" s="27" t="s">
-        <v>329</v>
-      </c>
-      <c r="H23" s="30" t="s">
+      <c r="I23" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="J23" s="9">
+        <v>0</v>
+      </c>
+      <c r="K23" s="12" t="s">
+        <v>197</v>
+      </c>
+      <c r="L23" s="7"/>
+      <c r="N23" s="21" t="s">
         <v>328</v>
-      </c>
-      <c r="I23" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="J23" s="23">
-        <v>0</v>
-      </c>
-      <c r="K23" s="28" t="s">
-        <v>197</v>
-      </c>
-      <c r="L23" s="27"/>
-      <c r="N23" s="30" t="s">
-        <v>330</v>
       </c>
     </row>
     <row r="24" spans="1:17" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4718,7 +4689,7 @@
         <v>231</v>
       </c>
       <c r="H24" s="14" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="I24" s="10" t="s">
         <v>38</v>
@@ -4752,7 +4723,7 @@
         <v>273</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="H25" s="10" t="s">
         <v>274</v>
@@ -4786,13 +4757,13 @@
         <v>131</v>
       </c>
       <c r="F26" s="10" t="s">
+        <v>333</v>
+      </c>
+      <c r="G26" s="7" t="s">
         <v>335</v>
       </c>
-      <c r="G26" s="7" t="s">
-        <v>337</v>
-      </c>
       <c r="H26" s="10" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="I26" s="10" t="s">
         <v>41</v>
@@ -4805,7 +4776,7 @@
       </c>
       <c r="L26" s="7"/>
       <c r="N26" s="14" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
     </row>
     <row r="27" spans="1:17" s="6" customFormat="1" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4831,7 +4802,7 @@
         <v>232</v>
       </c>
       <c r="H27" s="10" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="I27" s="10" t="s">
         <v>46</v>
@@ -4862,13 +4833,13 @@
         <v>133</v>
       </c>
       <c r="F28" s="10" t="s">
+        <v>339</v>
+      </c>
+      <c r="G28" s="7" t="s">
         <v>341</v>
       </c>
-      <c r="G28" s="7" t="s">
-        <v>343</v>
-      </c>
       <c r="H28" s="10" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="I28" s="10" t="s">
         <v>48</v>
@@ -4896,7 +4867,7 @@
         <v>40</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="F29" s="10" t="s">
         <v>134</v>
@@ -4922,7 +4893,7 @@
       <c r="M29" s="6">
         <v>3</v>
       </c>
-      <c r="N29" s="29"/>
+      <c r="N29" s="23"/>
       <c r="P29" s="10" t="s">
         <v>51</v>
       </c>
@@ -4930,51 +4901,51 @@
         <v>136</v>
       </c>
     </row>
-    <row r="30" spans="1:17" s="24" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="23">
+    <row r="30" spans="1:17" s="6" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30" s="9">
         <v>29</v>
       </c>
-      <c r="B30" s="23">
+      <c r="B30" s="9">
         <v>0</v>
       </c>
-      <c r="C30" s="24" t="s">
+      <c r="C30" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="D30" s="23">
+      <c r="D30" s="9">
         <v>26</v>
       </c>
-      <c r="E30" s="25" t="s">
-        <v>299</v>
-      </c>
-      <c r="F30" s="26" t="s">
+      <c r="E30" s="13" t="s">
+        <v>298</v>
+      </c>
+      <c r="F30" s="10" t="s">
         <v>137</v>
       </c>
-      <c r="G30" s="27" t="s">
-        <v>284</v>
-      </c>
-      <c r="H30" s="26" t="s">
+      <c r="G30" s="7" t="s">
+        <v>349</v>
+      </c>
+      <c r="H30" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="I30" s="24" t="s">
+      <c r="I30" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="J30" s="23">
+      <c r="J30" s="9">
         <v>0</v>
       </c>
-      <c r="K30" s="28" t="s">
+      <c r="K30" s="12" t="s">
         <v>204</v>
       </c>
-      <c r="L30" s="24" t="s">
+      <c r="L30" s="6" t="s">
         <v>282</v>
       </c>
-      <c r="M30" s="24" t="s">
+      <c r="M30" s="6" t="s">
         <v>283</v>
       </c>
-      <c r="N30" s="29"/>
-      <c r="P30" s="26" t="s">
+      <c r="N30" s="14"/>
+      <c r="P30" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="Q30" s="25" t="s">
+      <c r="Q30" s="13" t="s">
         <v>139</v>
       </c>
     </row>
@@ -4992,7 +4963,7 @@
         <v>34</v>
       </c>
       <c r="E31" s="13" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="F31" s="10" t="s">
         <v>140</v>
@@ -5018,7 +4989,7 @@
       <c r="M31" s="14" t="s">
         <v>216</v>
       </c>
-      <c r="N31" s="29"/>
+      <c r="N31" s="23"/>
       <c r="P31" s="10" t="s">
         <v>55</v>
       </c>
@@ -5040,7 +5011,7 @@
         <v>34</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="F32" s="10" t="s">
         <v>143</v>
@@ -5066,7 +5037,7 @@
       <c r="M32" s="6" t="s">
         <v>218</v>
       </c>
-      <c r="N32" s="29"/>
+      <c r="N32" s="23"/>
       <c r="P32" s="10" t="s">
         <v>57</v>
       </c>
@@ -5074,89 +5045,99 @@
         <v>145</v>
       </c>
     </row>
-    <row r="33" spans="1:17" s="24" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="23">
+    <row r="33" spans="1:17" s="6" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="9">
         <v>32</v>
       </c>
-      <c r="B33" s="23">
+      <c r="B33" s="9">
         <v>0</v>
       </c>
-      <c r="C33" s="24" t="s">
+      <c r="C33" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="D33" s="23">
+      <c r="D33" s="9">
         <v>26</v>
       </c>
-      <c r="E33" s="24" t="s">
+      <c r="E33" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="F33" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="G33" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="H33" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="I33" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="J33" s="9">
+        <v>0</v>
+      </c>
+      <c r="K33" s="12" t="s">
+        <v>204</v>
+      </c>
+      <c r="L33" s="7" t="s">
+        <v>351</v>
+      </c>
+      <c r="M33" s="6" t="s">
+        <v>350</v>
+      </c>
+      <c r="N33" s="14"/>
+      <c r="P33" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q33" s="13" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="34" spans="1:17" s="6" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34" s="9">
+        <v>33</v>
+      </c>
+      <c r="B34" s="9">
+        <v>0</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="D34" s="9">
+        <v>28</v>
+      </c>
+      <c r="E34" s="6" t="s">
         <v>302</v>
       </c>
-      <c r="F33" s="26" t="s">
-        <v>146</v>
-      </c>
-      <c r="G33" s="27" t="s">
-        <v>174</v>
-      </c>
-      <c r="H33" s="26" t="s">
-        <v>147</v>
-      </c>
-      <c r="I33" s="24" t="s">
-        <v>58</v>
-      </c>
-      <c r="J33" s="23">
+      <c r="F34" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="G34" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="H34" s="10" t="s">
+        <v>150</v>
+      </c>
+      <c r="I34" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="J34" s="9">
         <v>0</v>
       </c>
-      <c r="K33" s="28" t="s">
+      <c r="K34" s="12" t="s">
         <v>204</v>
       </c>
-      <c r="L33" s="27"/>
-      <c r="N33" s="29"/>
-      <c r="P33" s="26" t="s">
-        <v>59</v>
-      </c>
-      <c r="Q33" s="25" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="34" spans="1:17" s="24" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="23">
-        <v>33</v>
-      </c>
-      <c r="B34" s="23">
-        <v>0</v>
-      </c>
-      <c r="C34" s="24" t="s">
-        <v>86</v>
-      </c>
-      <c r="D34" s="23">
-        <v>28</v>
-      </c>
-      <c r="E34" s="24" t="s">
-        <v>303</v>
-      </c>
-      <c r="F34" s="26" t="s">
-        <v>149</v>
-      </c>
-      <c r="G34" s="27" t="s">
-        <v>175</v>
-      </c>
-      <c r="H34" s="26" t="s">
-        <v>150</v>
-      </c>
-      <c r="I34" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="J34" s="23">
-        <v>0</v>
-      </c>
-      <c r="K34" s="28" t="s">
-        <v>204</v>
-      </c>
-      <c r="L34" s="27"/>
-      <c r="N34" s="29"/>
-      <c r="P34" s="26" t="s">
+      <c r="L34" s="7" t="s">
+        <v>352</v>
+      </c>
+      <c r="M34" s="6" t="s">
+        <v>353</v>
+      </c>
+      <c r="N34" s="14"/>
+      <c r="P34" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="Q34" s="25" t="s">
+      <c r="Q34" s="13" t="s">
         <v>151</v>
       </c>
     </row>
@@ -5174,7 +5155,7 @@
         <v>26</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="F35" s="10" t="s">
         <v>152</v>
@@ -5200,7 +5181,7 @@
       <c r="M35" s="6" t="s">
         <v>220</v>
       </c>
-      <c r="N35" s="29"/>
+      <c r="N35" s="23"/>
       <c r="P35" s="10" t="s">
         <v>63</v>
       </c>
@@ -5222,7 +5203,7 @@
         <v>34</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F36" s="10" t="s">
         <v>155</v>
@@ -5248,7 +5229,7 @@
       <c r="M36" s="6">
         <v>5</v>
       </c>
-      <c r="N36" s="29"/>
+      <c r="N36" s="23"/>
       <c r="P36" s="10" t="s">
         <v>65</v>
       </c>
@@ -5270,7 +5251,7 @@
         <v>97</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="F37" s="10" t="s">
         <v>158</v>
@@ -5279,7 +5260,7 @@
         <v>233</v>
       </c>
       <c r="H37" s="10" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="I37" s="6" t="s">
         <v>73</v>
@@ -5313,16 +5294,16 @@
         <v>67</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F38" s="10" t="s">
         <v>160</v>
       </c>
       <c r="G38" s="7" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="H38" s="10" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="I38" s="6" t="s">
         <v>74</v>
@@ -5331,7 +5312,7 @@
         <v>0</v>
       </c>
       <c r="K38" s="12" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="L38" s="7"/>
       <c r="N38" s="14"/>
@@ -5356,25 +5337,25 @@
         <v>85</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F39" s="10" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="G39" s="7" t="s">
         <v>234</v>
       </c>
       <c r="H39" s="10" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="I39" s="10" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="J39" s="9">
         <v>0</v>
       </c>
       <c r="K39" s="12" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="L39" s="7"/>
       <c r="N39" s="14"/>
@@ -5550,7 +5531,7 @@
         <v>13</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5565,7 +5546,7 @@
         <v>14</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5580,7 +5561,7 @@
         <v>15</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5610,7 +5591,7 @@
         <v>17</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5640,7 +5621,7 @@
         <v>19</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5655,7 +5636,7 @@
         <v>20</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5805,7 +5786,7 @@
         <v>30</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5931,7 +5912,7 @@
         <v>39</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6029,7 +6010,7 @@
         <v>46</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6320,10 +6301,10 @@
         <v>38</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
workshop taks map to concept node
This was done in an old commit but was overriten
</commit_message>
<xml_diff>
--- a/files/programming-tasks/programmieraufgaben_JACK_SOSE23_WORKSHOP_WISE2324.xlsx
+++ b/files/programming-tasks/programmieraufgaben_JACK_SOSE23_WORKSHOP_WISE2324.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\hefl\files\programming-tasks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D34F5F7-B8EF-40EA-BF9B-DFA61FAFCED5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E693E1D7-D795-4FE6-BBC7-91BF9D36ED6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="51480" yWindow="-645" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3263,7 +3263,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3318,8 +3318,29 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C5700"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3329,6 +3350,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -3363,11 +3394,15 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1"/>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -3432,10 +3467,17 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="3" fontId="9" fillId="3" borderId="1" xfId="5" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="6">
     <cellStyle name="Gut" xfId="1" builtinId="26"/>
+    <cellStyle name="Gut 2" xfId="4" xr:uid="{1A463B06-9BFA-4B3E-81E4-39C4F0E07AFE}"/>
+    <cellStyle name="Neutral 2" xfId="3" xr:uid="{19014D6B-391A-4CF6-9B82-5516F796864B}"/>
+    <cellStyle name="Schlecht 2" xfId="5" xr:uid="{856DDD0E-3CB7-4286-8E4D-013EDFD66383}"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard 2" xfId="2" xr:uid="{650E2703-E298-4160-B731-FBE2C239278C}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -4858,7 +4900,7 @@
         <v>28</v>
       </c>
       <c r="B29" s="9">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="C29" s="6" t="s">
         <v>86</v>
@@ -4905,8 +4947,8 @@
       <c r="A30" s="9">
         <v>29</v>
       </c>
-      <c r="B30" s="9">
-        <v>0</v>
+      <c r="B30" s="24">
+        <v>26</v>
       </c>
       <c r="C30" s="6" t="s">
         <v>86</v>
@@ -4953,8 +4995,8 @@
       <c r="A31" s="9">
         <v>30</v>
       </c>
-      <c r="B31" s="9">
-        <v>0</v>
+      <c r="B31" s="24">
+        <v>34</v>
       </c>
       <c r="C31" s="6" t="s">
         <v>86</v>
@@ -5001,8 +5043,8 @@
       <c r="A32" s="9">
         <v>31</v>
       </c>
-      <c r="B32" s="9">
-        <v>0</v>
+      <c r="B32" s="24">
+        <v>34</v>
       </c>
       <c r="C32" s="6" t="s">
         <v>86</v>
@@ -5049,8 +5091,8 @@
       <c r="A33" s="9">
         <v>32</v>
       </c>
-      <c r="B33" s="9">
-        <v>0</v>
+      <c r="B33" s="24">
+        <v>26</v>
       </c>
       <c r="C33" s="6" t="s">
         <v>86</v>
@@ -5097,8 +5139,8 @@
       <c r="A34" s="9">
         <v>33</v>
       </c>
-      <c r="B34" s="9">
-        <v>0</v>
+      <c r="B34" s="24">
+        <v>28</v>
       </c>
       <c r="C34" s="6" t="s">
         <v>86</v>
@@ -5145,8 +5187,8 @@
       <c r="A35" s="9">
         <v>34</v>
       </c>
-      <c r="B35" s="9">
-        <v>0</v>
+      <c r="B35" s="24">
+        <v>26</v>
       </c>
       <c r="C35" s="6" t="s">
         <v>86</v>
@@ -5193,8 +5235,8 @@
       <c r="A36" s="9">
         <v>35</v>
       </c>
-      <c r="B36" s="9">
-        <v>0</v>
+      <c r="B36" s="24">
+        <v>34</v>
       </c>
       <c r="C36" s="6" t="s">
         <v>86</v>
@@ -5241,8 +5283,8 @@
       <c r="A37" s="9">
         <v>36</v>
       </c>
-      <c r="B37" s="9">
-        <v>0</v>
+      <c r="B37" s="24">
+        <v>97</v>
       </c>
       <c r="C37" s="6" t="s">
         <v>106</v>
@@ -5284,8 +5326,8 @@
       <c r="A38" s="9">
         <v>37</v>
       </c>
-      <c r="B38" s="9">
-        <v>0</v>
+      <c r="B38" s="24">
+        <v>67</v>
       </c>
       <c r="C38" s="6" t="s">
         <v>106</v>
@@ -5327,8 +5369,8 @@
       <c r="A39" s="9">
         <v>38</v>
       </c>
-      <c r="B39" s="9">
-        <v>0</v>
+      <c r="B39" s="24">
+        <v>85</v>
       </c>
       <c r="C39" s="6" t="s">
         <v>106</v>

</xml_diff>

<commit_message>
Fixed Unit-Tests for Task "Buchstabenfrequenz"
also added model solution to table
</commit_message>
<xml_diff>
--- a/files/programming-tasks/programmieraufgaben_JACK_SOSE23_WORKSHOP_WISE2324.xlsx
+++ b/files/programming-tasks/programmieraufgaben_JACK_SOSE23_WORKSHOP_WISE2324.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\hefl\files\programming-tasks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E693E1D7-D795-4FE6-BBC7-91BF9D36ED6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7DDF85F-035B-4EE6-892B-409E02337D4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51480" yWindow="-645" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Aufgaben" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="465" uniqueCount="354">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="466" uniqueCount="355">
   <si>
     <t>id</t>
   </si>
@@ -985,34 +985,6 @@
         self.assertEqual(result, 11, "Expected 11")
 if __name__ == '__main__':
     unittest.main()</t>
-  </si>
-  <si>
-    <t xml:space="preserve">import unittest
-from Buchstabenfrequenz import charFrequenz
-class TestCharFrequenz(unittest.TestCase):
-    def test_case1(self):
-        """Testcase 1"""
-        result = charFrequenz("Wie du mir so ich dir")
-        expected = [('i', 4), ('d', 2), ('r', 2), ('w', 1), ('e', 1), ('u', 1), ('m', 1), ('s', 1), ('o', 1), ('c', 1), ('h', 1)]
-        self.assertEqual(result, expected, "Expected result mismatch")
-    def test_case2(self):
-        """Testcase 2"""
-        result = charFrequenz("Ohne Pappe kein Haus!")
-        expected = [('e', 3), ('p', 3), ('h', 2), ('n', 2), ('a', 2), ('o', 1), ('k', 1), ('i', 1), ('u', 1), ('s', 1)]
-        self.assertEqual(result, expected, "Expected result mismatch")
-    def test_case3(self):
-        """Testcase 3"""
-        result = charFrequenz("Wer weiss schon was das Morgen bringen mag")
-        expected = [('s', 5), ('e', 4), ('n', 4), ('w', 3), ('r', 3), ('a', 3), ('g', 3), ('i', 2), ('o', 2), ('m', 2), ('c', 1), ('h', 1), ('d', 1), ('b', 1)]
-        self.assertEqual(result, expected, "Expected result mismatch")
-    def test_case4(self):
-        """Testcase 4"""
-        result = charFrequenz("Im Frühtau zu Berge")
-        expected = [('r', 2), ('u', 2), ('e', 2), ('i', 1), ('m', 1), ('f', 1),('ü', 1), ('h', 1), ('t', 1), ('a', 1), ('z', 1), ('b', 1), ('g', 1)]
-        self.assertEqual(result, expected, "Expected result mismatch")
-if __name__ == '__main__':
-    unittest.main()
-</t>
   </si>
   <si>
     <t xml:space="preserve">import unittest
@@ -3257,6 +3229,41 @@
   </si>
   <si>
     <t xml:space="preserve">lambda x: x % 2 == 0, [1, 2, 3, 4, 5, 6] </t>
+  </si>
+  <si>
+    <t>import unittest
+from Buchstabenfrequenz import charFrequenz
+class TestCharFrequenz(unittest.TestCase):
+    def test_case1(self):
+        result = charFrequenz("Wie du mir so ich dir")
+        expected = [('i', 4), ('d', 2), ('r', 2), ('c', 1), ('e', 1), ('h', 1), ('m', 1), ('o', 1), ('s', 1), ('u', 1), ('w', 1)]
+        self.assertEqual(result, expected)
+    def test_case2(self):
+        result = charFrequenz("Ohne Pappe kein Haus!")
+        expected = [('e', 3), ('p', 3), ('a', 2), ('h', 2), ('n', 2), ('i', 1), ('k', 1), ('o', 1), ('s', 1), ('u', 1)]
+        self.assertEqual(result, expected)
+    def test_case3(self):
+        result = charFrequenz("Wer weiss schon was das Morgen bringen mag")
+        expected = [('s', 5), ('e', 4), ('n', 4), ('a', 3), ('g', 3), ('r', 3), ('w', 3), ('i', 2), ('m', 2), ('o', 2), ('b', 1), ('c', 1), ('d', 1), ('h', 1)]
+        self.assertEqual(result, expected)
+    def test_case4(self):
+        result = charFrequenz("Im Frühtau zu Berge")
+        expected = [('e', 2), ('r', 2), ('u', 2), ('a', 1), ('b', 1), ('f', 1), ('g', 1), ('h', 1), ('i', 1), ('m', 1), ('t', 1), ('z', 1)]
+        self.assertEqual(result, expected)
+if __name__ == '__main__':
+    unittest.main()</t>
+  </si>
+  <si>
+    <t>def charFrequenz(s):
+    filtered = [char.lower() for char in s if 'a' &lt;= char.lower() &lt;= 'z']
+    frequency = {}
+    for char in filtered:
+        if char in frequency:
+            frequency[char] += 1
+        else:
+            frequency[char] = 1
+    sorted_frequency = sorted(frequency.items(), key=lambda item: (-item[1], item[0]))
+    return sorted_frequency</t>
   </si>
 </sst>
 </file>
@@ -3394,15 +3401,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="6">
+  <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1"/>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -3470,10 +3478,19 @@
     <xf numFmtId="3" fontId="9" fillId="3" borderId="1" xfId="5" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="6"/>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="0" xfId="6" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="6" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" xfId="6" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="7">
     <cellStyle name="Gut" xfId="1" builtinId="26"/>
     <cellStyle name="Gut 2" xfId="4" xr:uid="{1A463B06-9BFA-4B3E-81E4-39C4F0E07AFE}"/>
+    <cellStyle name="Neutral" xfId="6" builtinId="28"/>
     <cellStyle name="Neutral 2" xfId="3" xr:uid="{19014D6B-391A-4CF6-9B82-5516F796864B}"/>
     <cellStyle name="Schlecht 2" xfId="5" xr:uid="{856DDD0E-3CB7-4286-8E4D-013EDFD66383}"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -3797,6 +3814,7 @@
     <col min="13" max="13" width="74.5703125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="170.7109375" style="23" customWidth="1"/>
     <col min="15" max="17" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="84.140625" style="25" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" s="6" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
@@ -3831,15 +3849,16 @@
         <v>85</v>
       </c>
       <c r="K1" s="15" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="L1" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="M1" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="M1" s="6" t="s">
-        <v>179</v>
-      </c>
       <c r="N1" s="23"/>
+      <c r="R1" s="25"/>
     </row>
     <row r="2" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="9">
@@ -3873,15 +3892,16 @@
         <v>0</v>
       </c>
       <c r="K2" s="16" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="L2" s="7" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="M2" s="6" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="N2" s="23"/>
+      <c r="R2" s="25"/>
     </row>
     <row r="3" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="9">
@@ -3915,15 +3935,16 @@
         <v>0</v>
       </c>
       <c r="K3" s="16" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="L3" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="M3" s="6" t="s">
         <v>181</v>
       </c>
-      <c r="M3" s="6" t="s">
-        <v>182</v>
-      </c>
       <c r="N3" s="23"/>
+      <c r="R3" s="25"/>
     </row>
     <row r="4" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="9">
@@ -3948,7 +3969,7 @@
         <v>165</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="I4" s="6" t="s">
         <v>7</v>
@@ -3957,15 +3978,16 @@
         <v>0</v>
       </c>
       <c r="K4" s="16" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="M4" s="6">
         <v>174</v>
       </c>
       <c r="N4" s="23"/>
+      <c r="R4" s="25"/>
     </row>
     <row r="5" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="9">
@@ -3990,7 +4012,7 @@
         <v>166</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="I5" s="6" t="s">
         <v>8</v>
@@ -3999,15 +4021,16 @@
         <v>0</v>
       </c>
       <c r="K5" s="12" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="L5" s="7" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="M5" s="6">
         <v>47</v>
       </c>
       <c r="N5" s="23"/>
+      <c r="R5" s="25"/>
     </row>
     <row r="6" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="9">
@@ -4029,7 +4052,7 @@
         <v>98</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>167</v>
+        <v>353</v>
       </c>
       <c r="H6" s="10" t="s">
         <v>99</v>
@@ -4041,15 +4064,18 @@
         <v>0</v>
       </c>
       <c r="K6" s="12" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="L6" s="7" t="s">
+        <v>207</v>
+      </c>
+      <c r="M6" s="6" t="s">
         <v>208</v>
       </c>
-      <c r="M6" s="6" t="s">
-        <v>209</v>
-      </c>
       <c r="N6" s="23"/>
+      <c r="R6" s="26" t="s">
+        <v>354</v>
+      </c>
     </row>
     <row r="7" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="9">
@@ -4071,7 +4097,7 @@
         <v>101</v>
       </c>
       <c r="G7" s="19" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="H7" s="10" t="s">
         <v>102</v>
@@ -4083,15 +4109,16 @@
         <v>0</v>
       </c>
       <c r="K7" s="16" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="L7" s="7" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="M7" s="6" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="N7" s="23"/>
+      <c r="R7" s="25"/>
     </row>
     <row r="8" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="9">
@@ -4113,10 +4140,10 @@
         <v>104</v>
       </c>
       <c r="G8" s="19" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="H8" s="10" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="I8" s="6" t="s">
         <v>11</v>
@@ -4125,15 +4152,16 @@
         <v>0</v>
       </c>
       <c r="K8" s="16" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="L8" s="7" t="s">
+        <v>210</v>
+      </c>
+      <c r="M8" s="6" t="s">
         <v>211</v>
       </c>
-      <c r="M8" s="6" t="s">
-        <v>212</v>
-      </c>
       <c r="N8" s="23"/>
+      <c r="R8" s="25"/>
     </row>
     <row r="9" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="9">
@@ -4152,13 +4180,13 @@
         <v>105</v>
       </c>
       <c r="F9" s="10" t="s">
+        <v>278</v>
+      </c>
+      <c r="G9" s="19" t="s">
+        <v>169</v>
+      </c>
+      <c r="H9" s="10" t="s">
         <v>279</v>
-      </c>
-      <c r="G9" s="19" t="s">
-        <v>170</v>
-      </c>
-      <c r="H9" s="10" t="s">
-        <v>280</v>
       </c>
       <c r="I9" s="6" t="s">
         <v>12</v>
@@ -4167,15 +4195,16 @@
         <v>0</v>
       </c>
       <c r="K9" s="16" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="L9" s="7" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="M9" s="6">
         <v>10</v>
       </c>
       <c r="N9" s="23"/>
+      <c r="R9" s="25"/>
     </row>
     <row r="10" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="9">
@@ -4197,7 +4226,7 @@
         <v>108</v>
       </c>
       <c r="G10" s="11" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="H10" s="10" t="s">
         <v>109</v>
@@ -4209,12 +4238,12 @@
         <v>0</v>
       </c>
       <c r="K10" s="12" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="L10" s="7"/>
       <c r="N10" s="23"/>
-      <c r="R10" s="7" t="s">
-        <v>312</v>
+      <c r="R10" s="26" t="s">
+        <v>311</v>
       </c>
     </row>
     <row r="11" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4234,13 +4263,13 @@
         <v>110</v>
       </c>
       <c r="F11" s="10" t="s">
+        <v>267</v>
+      </c>
+      <c r="G11" s="11" t="s">
+        <v>221</v>
+      </c>
+      <c r="H11" s="10" t="s">
         <v>268</v>
-      </c>
-      <c r="G11" s="11" t="s">
-        <v>222</v>
-      </c>
-      <c r="H11" s="10" t="s">
-        <v>269</v>
       </c>
       <c r="I11" s="6" t="s">
         <v>14</v>
@@ -4249,12 +4278,12 @@
         <v>0</v>
       </c>
       <c r="K11" s="12" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="L11" s="7"/>
       <c r="N11" s="23"/>
-      <c r="R11" s="7" t="s">
-        <v>306</v>
+      <c r="R11" s="26" t="s">
+        <v>305</v>
       </c>
     </row>
     <row r="12" spans="1:18" s="14" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4274,13 +4303,13 @@
         <v>111</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="G12" s="21" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="H12" s="21" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="I12" s="14" t="s">
         <v>15</v>
@@ -4289,11 +4318,11 @@
         <v>1</v>
       </c>
       <c r="K12" s="14" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="N12" s="23"/>
-      <c r="R12" s="21" t="s">
-        <v>308</v>
+      <c r="R12" s="27" t="s">
+        <v>307</v>
       </c>
     </row>
     <row r="13" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4316,7 +4345,7 @@
         <v>113</v>
       </c>
       <c r="G13" s="11" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="H13" s="10" t="s">
         <v>114</v>
@@ -4328,10 +4357,11 @@
         <v>0</v>
       </c>
       <c r="K13" s="12" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="L13" s="7"/>
       <c r="N13" s="23"/>
+      <c r="R13" s="25"/>
     </row>
     <row r="14" spans="1:18" s="14" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="14">
@@ -4350,13 +4380,13 @@
         <v>115</v>
       </c>
       <c r="F14" s="14" t="s">
+        <v>287</v>
+      </c>
+      <c r="G14" s="14" t="s">
+        <v>224</v>
+      </c>
+      <c r="H14" s="14" t="s">
         <v>288</v>
-      </c>
-      <c r="G14" s="14" t="s">
-        <v>225</v>
-      </c>
-      <c r="H14" s="14" t="s">
-        <v>289</v>
       </c>
       <c r="I14" s="14" t="s">
         <v>17</v>
@@ -4365,11 +4395,11 @@
         <v>1</v>
       </c>
       <c r="K14" s="14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="N14" s="23"/>
-      <c r="R14" s="21" t="s">
-        <v>313</v>
+      <c r="R14" s="27" t="s">
+        <v>312</v>
       </c>
     </row>
     <row r="15" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4392,7 +4422,7 @@
         <v>117</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="H15" s="10" t="s">
         <v>118</v>
@@ -4404,10 +4434,11 @@
         <v>0</v>
       </c>
       <c r="K15" s="12" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="L15" s="7"/>
       <c r="N15" s="23"/>
+      <c r="R15" s="25"/>
     </row>
     <row r="16" spans="1:18" s="14" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="14">
@@ -4426,13 +4457,13 @@
         <v>119</v>
       </c>
       <c r="F16" s="21" t="s">
+        <v>289</v>
+      </c>
+      <c r="G16" s="14" t="s">
+        <v>226</v>
+      </c>
+      <c r="H16" s="14" t="s">
         <v>290</v>
-      </c>
-      <c r="G16" s="14" t="s">
-        <v>227</v>
-      </c>
-      <c r="H16" s="14" t="s">
-        <v>291</v>
       </c>
       <c r="I16" s="14" t="s">
         <v>19</v>
@@ -4441,11 +4472,12 @@
         <v>2</v>
       </c>
       <c r="K16" s="14" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="N16" s="23"/>
-    </row>
-    <row r="17" spans="1:17" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R16" s="28"/>
+    </row>
+    <row r="17" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="9">
         <v>16</v>
       </c>
@@ -4462,13 +4494,13 @@
         <v>120</v>
       </c>
       <c r="F17" s="10" t="s">
+        <v>323</v>
+      </c>
+      <c r="G17" s="7" t="s">
+        <v>329</v>
+      </c>
+      <c r="H17" s="10" t="s">
         <v>324</v>
-      </c>
-      <c r="G17" s="7" t="s">
-        <v>330</v>
-      </c>
-      <c r="H17" s="10" t="s">
-        <v>325</v>
       </c>
       <c r="I17" s="10" t="s">
         <v>20</v>
@@ -4477,14 +4509,15 @@
         <v>0</v>
       </c>
       <c r="K17" s="12" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="L17" s="7"/>
       <c r="N17" s="21" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="18" spans="1:17" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+        <v>327</v>
+      </c>
+      <c r="R17" s="25"/>
+    </row>
+    <row r="18" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="9">
         <v>17</v>
       </c>
@@ -4501,13 +4534,13 @@
         <v>121</v>
       </c>
       <c r="F18" s="10" t="s">
+        <v>269</v>
+      </c>
+      <c r="G18" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="H18" s="10" t="s">
         <v>270</v>
-      </c>
-      <c r="G18" s="7" t="s">
-        <v>228</v>
-      </c>
-      <c r="H18" s="10" t="s">
-        <v>271</v>
       </c>
       <c r="I18" s="6" t="s">
         <v>25</v>
@@ -4516,12 +4549,13 @@
         <v>0</v>
       </c>
       <c r="K18" s="12" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="L18" s="7"/>
       <c r="N18" s="23"/>
-    </row>
-    <row r="19" spans="1:17" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R18" s="25"/>
+    </row>
+    <row r="19" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="9">
         <v>18</v>
       </c>
@@ -4538,13 +4572,13 @@
         <v>122</v>
       </c>
       <c r="F19" s="10" t="s">
+        <v>308</v>
+      </c>
+      <c r="G19" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="H19" s="10" t="s">
         <v>309</v>
-      </c>
-      <c r="G19" s="7" t="s">
-        <v>229</v>
-      </c>
-      <c r="H19" s="10" t="s">
-        <v>310</v>
       </c>
       <c r="I19" s="6" t="s">
         <v>29</v>
@@ -4553,12 +4587,13 @@
         <v>0</v>
       </c>
       <c r="K19" s="12" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="L19" s="7"/>
       <c r="N19" s="23"/>
-    </row>
-    <row r="20" spans="1:17" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R19" s="25"/>
+    </row>
+    <row r="20" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="22">
         <v>19</v>
       </c>
@@ -4578,7 +4613,7 @@
         <v>124</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="H20" s="10" t="s">
         <v>125</v>
@@ -4590,12 +4625,13 @@
         <v>0</v>
       </c>
       <c r="K20" s="12" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="L20" s="7"/>
       <c r="N20" s="23"/>
-    </row>
-    <row r="21" spans="1:17" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R20" s="25"/>
+    </row>
+    <row r="21" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="9">
         <v>20</v>
       </c>
@@ -4612,13 +4648,13 @@
         <v>126</v>
       </c>
       <c r="F21" s="10" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="H21" s="14" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="I21" s="6" t="s">
         <v>32</v>
@@ -4627,12 +4663,13 @@
         <v>0</v>
       </c>
       <c r="K21" s="12" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="L21" s="7"/>
       <c r="N21" s="23"/>
-    </row>
-    <row r="22" spans="1:17" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R21" s="25"/>
+    </row>
+    <row r="22" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="9">
         <v>21</v>
       </c>
@@ -4649,13 +4686,13 @@
         <v>127</v>
       </c>
       <c r="F22" s="10" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="H22" s="14" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="I22" s="10" t="s">
         <v>34</v>
@@ -4664,12 +4701,13 @@
         <v>0</v>
       </c>
       <c r="K22" s="12" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="L22" s="7"/>
       <c r="N22" s="21"/>
-    </row>
-    <row r="23" spans="1:17" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R22" s="25"/>
+    </row>
+    <row r="23" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="9">
         <v>22</v>
       </c>
@@ -4686,13 +4724,13 @@
         <v>128</v>
       </c>
       <c r="F23" s="10" t="s">
+        <v>325</v>
+      </c>
+      <c r="G23" s="7" t="s">
+        <v>347</v>
+      </c>
+      <c r="H23" s="21" t="s">
         <v>326</v>
-      </c>
-      <c r="G23" s="7" t="s">
-        <v>348</v>
-      </c>
-      <c r="H23" s="21" t="s">
-        <v>327</v>
       </c>
       <c r="I23" s="10" t="s">
         <v>36</v>
@@ -4701,14 +4739,15 @@
         <v>0</v>
       </c>
       <c r="K23" s="12" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="L23" s="7"/>
       <c r="N23" s="21" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="24" spans="1:17" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+        <v>327</v>
+      </c>
+      <c r="R23" s="25"/>
+    </row>
+    <row r="24" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="9">
         <v>23</v>
       </c>
@@ -4725,13 +4764,13 @@
         <v>129</v>
       </c>
       <c r="F24" s="10" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="G24" s="7" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="H24" s="14" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="I24" s="10" t="s">
         <v>38</v>
@@ -4740,12 +4779,13 @@
         <v>0</v>
       </c>
       <c r="K24" s="12" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="L24" s="7"/>
       <c r="N24" s="14"/>
-    </row>
-    <row r="25" spans="1:17" s="6" customFormat="1" ht="261" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R24" s="25"/>
+    </row>
+    <row r="25" spans="1:18" s="6" customFormat="1" ht="261" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="9">
         <v>24</v>
       </c>
@@ -4762,13 +4802,13 @@
         <v>130</v>
       </c>
       <c r="F25" s="10" t="s">
+        <v>272</v>
+      </c>
+      <c r="G25" s="7" t="s">
+        <v>331</v>
+      </c>
+      <c r="H25" s="10" t="s">
         <v>273</v>
-      </c>
-      <c r="G25" s="7" t="s">
-        <v>332</v>
-      </c>
-      <c r="H25" s="10" t="s">
-        <v>274</v>
       </c>
       <c r="I25" s="10" t="s">
         <v>39</v>
@@ -4777,12 +4817,13 @@
         <v>0</v>
       </c>
       <c r="K25" s="12" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="L25" s="7"/>
       <c r="N25" s="14"/>
-    </row>
-    <row r="26" spans="1:17" s="6" customFormat="1" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R25" s="25"/>
+    </row>
+    <row r="26" spans="1:18" s="6" customFormat="1" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A26" s="9">
         <v>25</v>
       </c>
@@ -4799,13 +4840,13 @@
         <v>131</v>
       </c>
       <c r="F26" s="10" t="s">
+        <v>332</v>
+      </c>
+      <c r="G26" s="7" t="s">
+        <v>334</v>
+      </c>
+      <c r="H26" s="10" t="s">
         <v>333</v>
-      </c>
-      <c r="G26" s="7" t="s">
-        <v>335</v>
-      </c>
-      <c r="H26" s="10" t="s">
-        <v>334</v>
       </c>
       <c r="I26" s="10" t="s">
         <v>41</v>
@@ -4814,14 +4855,15 @@
         <v>0</v>
       </c>
       <c r="K26" s="12" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="L26" s="7"/>
       <c r="N26" s="14" t="s">
-        <v>336</v>
-      </c>
-    </row>
-    <row r="27" spans="1:17" s="6" customFormat="1" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+        <v>335</v>
+      </c>
+      <c r="R26" s="25"/>
+    </row>
+    <row r="27" spans="1:18" s="6" customFormat="1" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="9">
         <v>26</v>
       </c>
@@ -4838,13 +4880,13 @@
         <v>132</v>
       </c>
       <c r="F27" s="10" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="G27" s="7" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="H27" s="10" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="I27" s="10" t="s">
         <v>46</v>
@@ -4853,12 +4895,13 @@
         <v>0</v>
       </c>
       <c r="K27" s="12" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="L27" s="7"/>
       <c r="N27" s="14"/>
-    </row>
-    <row r="28" spans="1:17" s="6" customFormat="1" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R27" s="25"/>
+    </row>
+    <row r="28" spans="1:18" s="6" customFormat="1" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="9">
         <v>27</v>
       </c>
@@ -4875,13 +4918,13 @@
         <v>133</v>
       </c>
       <c r="F28" s="10" t="s">
+        <v>338</v>
+      </c>
+      <c r="G28" s="7" t="s">
+        <v>340</v>
+      </c>
+      <c r="H28" s="10" t="s">
         <v>339</v>
-      </c>
-      <c r="G28" s="7" t="s">
-        <v>341</v>
-      </c>
-      <c r="H28" s="10" t="s">
-        <v>340</v>
       </c>
       <c r="I28" s="10" t="s">
         <v>48</v>
@@ -4890,12 +4933,13 @@
         <v>0</v>
       </c>
       <c r="K28" s="12" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="L28" s="7"/>
       <c r="N28" s="14"/>
-    </row>
-    <row r="29" spans="1:17" s="6" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="R28" s="25"/>
+    </row>
+    <row r="29" spans="1:18" s="6" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A29" s="9">
         <v>28</v>
       </c>
@@ -4909,13 +4953,13 @@
         <v>40</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="F29" s="10" t="s">
         <v>134</v>
       </c>
       <c r="G29" s="18" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="H29" s="10" t="s">
         <v>135</v>
@@ -4927,10 +4971,10 @@
         <v>0</v>
       </c>
       <c r="K29" s="16" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="L29" s="7" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="M29" s="6">
         <v>3</v>
@@ -4942,8 +4986,9 @@
       <c r="Q29" s="13" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="30" spans="1:17" s="6" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R29" s="25"/>
+    </row>
+    <row r="30" spans="1:18" s="6" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="9">
         <v>29</v>
       </c>
@@ -4957,13 +5002,13 @@
         <v>26</v>
       </c>
       <c r="E30" s="13" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="F30" s="10" t="s">
         <v>137</v>
       </c>
       <c r="G30" s="7" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="H30" s="10" t="s">
         <v>138</v>
@@ -4975,13 +5020,13 @@
         <v>0</v>
       </c>
       <c r="K30" s="12" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="L30" s="6" t="s">
+        <v>281</v>
+      </c>
+      <c r="M30" s="6" t="s">
         <v>282</v>
-      </c>
-      <c r="M30" s="6" t="s">
-        <v>283</v>
       </c>
       <c r="N30" s="14"/>
       <c r="P30" s="10" t="s">
@@ -4990,8 +5035,9 @@
       <c r="Q30" s="13" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="31" spans="1:17" s="6" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="R30" s="25"/>
+    </row>
+    <row r="31" spans="1:18" s="6" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A31" s="9">
         <v>30</v>
       </c>
@@ -5005,13 +5051,13 @@
         <v>34</v>
       </c>
       <c r="E31" s="13" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="F31" s="10" t="s">
         <v>140</v>
       </c>
       <c r="G31" s="18" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="H31" s="10" t="s">
         <v>141</v>
@@ -5023,13 +5069,13 @@
         <v>0</v>
       </c>
       <c r="K31" s="16" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="L31" s="14" t="s">
+        <v>214</v>
+      </c>
+      <c r="M31" s="14" t="s">
         <v>215</v>
-      </c>
-      <c r="M31" s="14" t="s">
-        <v>216</v>
       </c>
       <c r="N31" s="23"/>
       <c r="P31" s="10" t="s">
@@ -5038,8 +5084,9 @@
       <c r="Q31" s="13" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="32" spans="1:17" s="6" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="R31" s="25"/>
+    </row>
+    <row r="32" spans="1:18" s="6" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="9">
         <v>31</v>
       </c>
@@ -5053,13 +5100,13 @@
         <v>34</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="F32" s="10" t="s">
         <v>143</v>
       </c>
       <c r="G32" s="18" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="H32" s="10" t="s">
         <v>144</v>
@@ -5071,13 +5118,13 @@
         <v>0</v>
       </c>
       <c r="K32" s="16" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="L32" s="7" t="s">
+        <v>216</v>
+      </c>
+      <c r="M32" s="6" t="s">
         <v>217</v>
-      </c>
-      <c r="M32" s="6" t="s">
-        <v>218</v>
       </c>
       <c r="N32" s="23"/>
       <c r="P32" s="10" t="s">
@@ -5086,8 +5133,9 @@
       <c r="Q32" s="13" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="33" spans="1:17" s="6" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R32" s="25"/>
+    </row>
+    <row r="33" spans="1:18" s="6" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="9">
         <v>32</v>
       </c>
@@ -5101,13 +5149,13 @@
         <v>26</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="F33" s="10" t="s">
         <v>146</v>
       </c>
       <c r="G33" s="7" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="H33" s="10" t="s">
         <v>147</v>
@@ -5119,13 +5167,13 @@
         <v>0</v>
       </c>
       <c r="K33" s="12" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="L33" s="7" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="M33" s="6" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="N33" s="14"/>
       <c r="P33" s="10" t="s">
@@ -5134,8 +5182,9 @@
       <c r="Q33" s="13" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="34" spans="1:17" s="6" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R33" s="25"/>
+    </row>
+    <row r="34" spans="1:18" s="6" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A34" s="9">
         <v>33</v>
       </c>
@@ -5149,13 +5198,13 @@
         <v>28</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="F34" s="10" t="s">
         <v>149</v>
       </c>
       <c r="G34" s="7" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="H34" s="10" t="s">
         <v>150</v>
@@ -5167,13 +5216,13 @@
         <v>0</v>
       </c>
       <c r="K34" s="12" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="L34" s="7" t="s">
+        <v>351</v>
+      </c>
+      <c r="M34" s="6" t="s">
         <v>352</v>
-      </c>
-      <c r="M34" s="6" t="s">
-        <v>353</v>
       </c>
       <c r="N34" s="14"/>
       <c r="P34" s="10" t="s">
@@ -5182,8 +5231,9 @@
       <c r="Q34" s="13" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="35" spans="1:17" s="6" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="R34" s="25"/>
+    </row>
+    <row r="35" spans="1:18" s="6" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A35" s="9">
         <v>34</v>
       </c>
@@ -5197,13 +5247,13 @@
         <v>26</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="F35" s="10" t="s">
         <v>152</v>
       </c>
       <c r="G35" s="18" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="H35" s="10" t="s">
         <v>153</v>
@@ -5215,13 +5265,13 @@
         <v>0</v>
       </c>
       <c r="K35" s="16" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="L35" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="M35" s="6" t="s">
         <v>219</v>
-      </c>
-      <c r="M35" s="6" t="s">
-        <v>220</v>
       </c>
       <c r="N35" s="23"/>
       <c r="P35" s="10" t="s">
@@ -5230,8 +5280,9 @@
       <c r="Q35" s="13" t="s">
         <v>154</v>
       </c>
-    </row>
-    <row r="36" spans="1:17" s="6" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="R35" s="25"/>
+    </row>
+    <row r="36" spans="1:18" s="6" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A36" s="9">
         <v>35</v>
       </c>
@@ -5245,13 +5296,13 @@
         <v>34</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="F36" s="10" t="s">
         <v>155</v>
       </c>
       <c r="G36" s="18" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="H36" s="10" t="s">
         <v>156</v>
@@ -5263,10 +5314,10 @@
         <v>0</v>
       </c>
       <c r="K36" s="16" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="L36" s="7" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="M36" s="6">
         <v>5</v>
@@ -5278,8 +5329,9 @@
       <c r="Q36" s="13" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="37" spans="1:17" s="6" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R36" s="25"/>
+    </row>
+    <row r="37" spans="1:18" s="6" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A37" s="9">
         <v>36</v>
       </c>
@@ -5293,16 +5345,16 @@
         <v>97</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="F37" s="10" t="s">
         <v>158</v>
       </c>
       <c r="G37" s="7" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="H37" s="10" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="I37" s="6" t="s">
         <v>73</v>
@@ -5311,7 +5363,7 @@
         <v>0</v>
       </c>
       <c r="K37" s="12" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="L37" s="7"/>
       <c r="N37" s="14"/>
@@ -5321,8 +5373,9 @@
       <c r="Q37" s="13" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="38" spans="1:17" s="6" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R37" s="25"/>
+    </row>
+    <row r="38" spans="1:18" s="6" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="9">
         <v>37</v>
       </c>
@@ -5336,16 +5389,16 @@
         <v>67</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="F38" s="10" t="s">
         <v>160</v>
       </c>
       <c r="G38" s="7" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="H38" s="10" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="I38" s="6" t="s">
         <v>74</v>
@@ -5354,7 +5407,7 @@
         <v>0</v>
       </c>
       <c r="K38" s="12" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="L38" s="7"/>
       <c r="N38" s="14"/>
@@ -5364,8 +5417,9 @@
       <c r="Q38" s="13" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="39" spans="1:17" s="6" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R38" s="25"/>
+    </row>
+    <row r="39" spans="1:18" s="6" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A39" s="9">
         <v>38</v>
       </c>
@@ -5379,25 +5433,25 @@
         <v>85</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="F39" s="10" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="G39" s="7" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="H39" s="10" t="s">
+        <v>343</v>
+      </c>
+      <c r="I39" s="10" t="s">
         <v>344</v>
-      </c>
-      <c r="I39" s="10" t="s">
-        <v>345</v>
       </c>
       <c r="J39" s="9">
         <v>0</v>
       </c>
       <c r="K39" s="12" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="L39" s="7"/>
       <c r="N39" s="14"/>
@@ -5407,6 +5461,7 @@
       <c r="Q39" s="13" t="s">
         <v>162</v>
       </c>
+      <c r="R39" s="25"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5573,7 +5628,7 @@
         <v>13</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5588,7 +5643,7 @@
         <v>14</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5603,7 +5658,7 @@
         <v>15</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5618,7 +5673,7 @@
         <v>16</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5633,7 +5688,7 @@
         <v>17</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5648,7 +5703,7 @@
         <v>18</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5663,7 +5718,7 @@
         <v>19</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5678,7 +5733,7 @@
         <v>20</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5693,7 +5748,7 @@
         <v>21</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5708,7 +5763,7 @@
         <v>22</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5723,7 +5778,7 @@
         <v>23</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5738,7 +5793,7 @@
         <v>24</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5753,7 +5808,7 @@
         <v>25</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5768,7 +5823,7 @@
         <v>26</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5783,7 +5838,7 @@
         <v>27</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5798,7 +5853,7 @@
         <v>28</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5813,7 +5868,7 @@
         <v>29</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5828,7 +5883,7 @@
         <v>30</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5842,7 +5897,7 @@
         <v>31</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5856,7 +5911,7 @@
         <v>32</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5870,7 +5925,7 @@
         <v>33</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5884,7 +5939,7 @@
         <v>34</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5898,7 +5953,7 @@
         <v>35</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5912,7 +5967,7 @@
         <v>36</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5926,7 +5981,7 @@
         <v>37</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5940,7 +5995,7 @@
         <v>38</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5954,7 +6009,7 @@
         <v>39</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5968,7 +6023,7 @@
         <v>40</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5982,7 +6037,7 @@
         <v>41</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5996,7 +6051,7 @@
         <v>42</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6010,7 +6065,7 @@
         <v>43</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6024,7 +6079,7 @@
         <v>44</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6038,7 +6093,7 @@
         <v>45</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6052,7 +6107,7 @@
         <v>46</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6066,7 +6121,7 @@
         <v>47</v>
       </c>
       <c r="D44" s="5" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6080,7 +6135,7 @@
         <v>48</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6094,7 +6149,7 @@
         <v>49</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6220,7 +6275,7 @@
         <v>66</v>
       </c>
       <c r="D55" s="5" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6234,7 +6289,7 @@
         <v>68</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6248,7 +6303,7 @@
         <v>70</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="58" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6262,7 +6317,7 @@
         <v>71</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6276,7 +6331,7 @@
         <v>72</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="60" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6290,7 +6345,7 @@
         <v>73</v>
       </c>
       <c r="D60" s="5" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6304,7 +6359,7 @@
         <v>74</v>
       </c>
       <c r="D61" s="5" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6318,7 +6373,7 @@
         <v>68</v>
       </c>
       <c r="D62" s="5" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="63" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6332,7 +6387,7 @@
         <v>66</v>
       </c>
       <c r="D63" s="5" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="64" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6343,10 +6398,10 @@
         <v>38</v>
       </c>
       <c r="C64" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="D64" s="2" t="s">
         <v>345</v>
-      </c>
-      <c r="D64" s="2" t="s">
-        <v>346</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Better explanation and unit-tests for task "Buchstabenfrequenz"
</commit_message>
<xml_diff>
--- a/files/programming-tasks/programmieraufgaben_JACK_SOSE23_WORKSHOP_WISE2324.xlsx
+++ b/files/programming-tasks/programmieraufgaben_JACK_SOSE23_WORKSHOP_WISE2324.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\hefl\files\programming-tasks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7DDF85F-035B-4EE6-892B-409E02337D4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99FF57EC-9EC3-426F-8EA3-5EC8A7825085}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="51480" yWindow="0" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Aufgaben" sheetId="1" r:id="rId1"/>
@@ -428,26 +428,6 @@
   </si>
   <si>
     <t>Buchstabenfrequenz</t>
-  </si>
-  <si>
-    <t>Schreiben Sie eine Funktion charFrequenz(), die die Buchstabenhäufigkeit eine Strings bestimmt. Die Häufigkeiten sollen sortiert ausgegeben werden. Sonderzeichen, Satzzeichen, Umlaute (z.B. ä, ö, ü) und Ziffern sollen nicht berückschtigt werden.
-Bsp.:
-s = "Das ist ein Teststring"
-x = charFrequenz(s)
-x wäre dann:
-[('s', 4), ('t', 4), ('i', 3), ('e', 2), ('n', 2), ('d', 1), ('a', 1), ('r', 1), ('g', 1)]</t>
-  </si>
-  <si>
-    <t>Schreiben Sie eine Funktion &lt;em&gt;charFrequenz()&lt;/em&gt;, die die Buchstabenh&amp;auml;ufigkeit eine Strings bestimmt. Die H&amp;auml;ufigkeiten sollen sortiert ausgegeben werden. Sonderzeichen, Satzzeichen, Umlaute (z.B. ä, ö, ü) und Ziffern sollen nicht ber&amp;uuml;ckschtigt werden.&lt;br /&gt;
-&lt;br /&gt;
-&lt;em&gt;Bsp.:&lt;br /&gt;
-s = "Das ist ein Teststring"&lt;br /&gt;
-x = charFrequenz(s)&lt;/em&gt;&lt;br /&gt;
-&lt;br /&gt;
-x w&amp;auml;re dann:&lt;br /&gt;
-&lt;em&gt;[(&amp;#39;s&amp;#39;, 4), (&amp;#39;t&amp;#39;, 4), (&amp;#39;i&amp;#39;, 3), (&amp;#39;e&amp;#39;, 2), (&amp;#39;n&amp;#39;, 2), (&amp;#39;d&amp;#39;, 1), (&amp;#39;a&amp;#39;, 1), (&amp;#39;r&amp;#39;, 1), (&amp;#39;g&amp;#39;, 1)]&lt;/em&gt;&lt;br /&gt;
-&lt;br /&gt;
-&amp;nbsp;</t>
   </si>
   <si>
     <t>Rekursive Summe</t>
@@ -3231,6 +3211,18 @@
     <t xml:space="preserve">lambda x: x % 2 == 0, [1, 2, 3, 4, 5, 6] </t>
   </si>
   <si>
+    <t>def charFrequenz(s):
+    filtered = [char.lower() for char in s if 'a' &lt;= char.lower() &lt;= 'z']
+    frequency = {}
+    for char in filtered:
+        if char in frequency:
+            frequency[char] += 1
+        else:
+            frequency[char] = 1
+    sorted_frequency = sorted(frequency.items(), key=lambda item: (-item[1], item[0]))
+    return sorted_frequency</t>
+  </si>
+  <si>
     <t>import unittest
 from Buchstabenfrequenz import charFrequenz
 class TestCharFrequenz(unittest.TestCase):
@@ -3254,16 +3246,32 @@
     unittest.main()</t>
   </si>
   <si>
-    <t>def charFrequenz(s):
-    filtered = [char.lower() for char in s if 'a' &lt;= char.lower() &lt;= 'z']
-    frequency = {}
-    for char in filtered:
-        if char in frequency:
-            frequency[char] += 1
-        else:
-            frequency[char] = 1
-    sorted_frequency = sorted(frequency.items(), key=lambda item: (-item[1], item[0]))
-    return sorted_frequency</t>
+    <t>&lt;p&gt;Schreiben Sie eine Funktion &lt;code&gt;charFrequenz()&lt;/code&gt;, die die Buchstabenhäufigkeit eines Strings bestimmt.Die Funktion soll:&lt;/p&gt; 
+&lt;p&gt;1. Sonderzeichen, Satzzeichen, Umlaute (z.B. ä, ö, ü) und Ziffern nicht berücksichtigen.&lt;/p&gt; 
+&lt;p&gt;2. Die Buchstabenhäufigkeiten sortiert ausgeben.&lt;/p&gt; 
+&lt;p&gt;3. Falls mehrere Buchstaben gleich oft vorkommen, diese in alphabetischer Reihenfolge ausgeben.&lt;/p&gt; 
+&lt;h2&gt;Tipps:&lt;/h2&gt; 
+&lt;p&gt;1. &lt;code&gt;sorted(s)&lt;/code&gt; sortiert die Zeichen des Strings &lt;code&gt;s&lt;/code&gt; in alphabetischer Reihenfolge und gibt eine Liste der sortierten Zeichen zurück.&lt;/p&gt; 
+&lt;p&gt;2. &lt;code&gt;s.lower()&lt;/code&gt; wandelt die Zeichen des Strings &lt;code&gt;s&lt;/code&gt; in Kleinbuchstaben um und gibt einen entsprechenden String mit Kleinbuchstaben zurück.&lt;/p&gt; 
+&lt;h2&gt;Beispiel:&lt;/h2&gt; 
+&lt;p&gt;&lt;code&gt;s = "Das ist ein Teststring 123!"&lt;/code&gt;&lt;/p&gt; 
+&lt;p&gt;&lt;code&gt;x = charFrequenz(s)&lt;/code&gt;&lt;/p&gt; &lt;p&gt;&lt;code&gt;x&lt;/code&gt; wäre dann:&lt;/p&gt; 
+&lt;p&gt;&lt;code&gt;[('s', 4), ('t', 4), ('i', 3), ('e', 2), ('n', 2), ('a', 1), ('d', 1), ('g', 1), ('r', 1)]&lt;/code&gt;&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+Schreiben Sie eine Funktion charFrequenz(), die die Buchstabenhäufigkeit eines Strings bestimmt.Die Funktion soll:
+1. Sonderzeichen, Satzzeichen, Umlaute (z.B. ä, ö, ü) und Ziffern nicht berücksichtigen.
+2. Die Buchstabenhäufigkeiten sortiert ausgeben.
+3. Falls mehrere Buchstaben gleich oft vorkommen, diese in alphabetischer Reihenfolge ausgeben.
+Tipps:
+1. sorted(s) sortiert die Zeichen des Strings s in alphabetischer Reihenfolge und gibt eine Liste der sortierten Zeichen zurück.
+2. s.lower() wandelt die Zeichen des Strings s in Kleinbuchstaben um und gibt einen entsprechenden String mit Kleinbuchstaben zurück.
+Beispiel:
+s = "Das ist ein Teststring 123!"
+x = charFrequenz(s)
+x wäre dann:
+[('s', 4), ('t', 4), ('i', 3), ('e', 2), ('n', 2), ('a', 1), ('d', 1), ('g', 1), ('r', 1)]</t>
   </si>
 </sst>
 </file>
@@ -3849,13 +3857,13 @@
         <v>85</v>
       </c>
       <c r="K1" s="15" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="M1" s="6" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="N1" s="23"/>
       <c r="R1" s="25"/>
@@ -3880,7 +3888,7 @@
         <v>88</v>
       </c>
       <c r="G2" s="19" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="H2" s="10" t="s">
         <v>89</v>
@@ -3892,13 +3900,13 @@
         <v>0</v>
       </c>
       <c r="K2" s="16" t="s">
+        <v>201</v>
+      </c>
+      <c r="L2" s="7" t="s">
+        <v>177</v>
+      </c>
+      <c r="M2" s="6" t="s">
         <v>203</v>
-      </c>
-      <c r="L2" s="7" t="s">
-        <v>179</v>
-      </c>
-      <c r="M2" s="6" t="s">
-        <v>205</v>
       </c>
       <c r="N2" s="23"/>
       <c r="R2" s="25"/>
@@ -3923,7 +3931,7 @@
         <v>91</v>
       </c>
       <c r="G3" s="19" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="H3" s="10" t="s">
         <v>92</v>
@@ -3935,13 +3943,13 @@
         <v>0</v>
       </c>
       <c r="K3" s="16" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="L3" s="7" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="M3" s="6" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="N3" s="23"/>
       <c r="R3" s="25"/>
@@ -3966,10 +3974,10 @@
         <v>94</v>
       </c>
       <c r="G4" s="19" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="I4" s="6" t="s">
         <v>7</v>
@@ -3978,10 +3986,10 @@
         <v>0</v>
       </c>
       <c r="K4" s="16" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="M4" s="6">
         <v>174</v>
@@ -4009,10 +4017,10 @@
         <v>96</v>
       </c>
       <c r="G5" s="11" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="I5" s="6" t="s">
         <v>8</v>
@@ -4021,10 +4029,10 @@
         <v>0</v>
       </c>
       <c r="K5" s="12" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="L5" s="7" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="M5" s="6">
         <v>47</v>
@@ -4049,13 +4057,13 @@
         <v>97</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>98</v>
+        <v>354</v>
       </c>
       <c r="G6" s="11" t="s">
+        <v>352</v>
+      </c>
+      <c r="H6" s="10" t="s">
         <v>353</v>
-      </c>
-      <c r="H6" s="10" t="s">
-        <v>99</v>
       </c>
       <c r="I6" s="6" t="s">
         <v>9</v>
@@ -4064,17 +4072,17 @@
         <v>0</v>
       </c>
       <c r="K6" s="12" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="L6" s="7" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="M6" s="6" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="N6" s="23"/>
       <c r="R6" s="26" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
     </row>
     <row r="7" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4091,16 +4099,16 @@
         <v>34</v>
       </c>
       <c r="E7" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="G7" s="19" t="s">
+        <v>165</v>
+      </c>
+      <c r="H7" s="10" t="s">
         <v>100</v>
-      </c>
-      <c r="F7" s="10" t="s">
-        <v>101</v>
-      </c>
-      <c r="G7" s="19" t="s">
-        <v>167</v>
-      </c>
-      <c r="H7" s="10" t="s">
-        <v>102</v>
       </c>
       <c r="I7" s="6" t="s">
         <v>10</v>
@@ -4109,13 +4117,13 @@
         <v>0</v>
       </c>
       <c r="K7" s="16" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="L7" s="7" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="M7" s="6" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="N7" s="23"/>
       <c r="R7" s="25"/>
@@ -4134,16 +4142,16 @@
         <v>34</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="G8" s="19" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="H8" s="10" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="I8" s="6" t="s">
         <v>11</v>
@@ -4152,13 +4160,13 @@
         <v>0</v>
       </c>
       <c r="K8" s="16" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="L8" s="7" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="M8" s="6" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="N8" s="23"/>
       <c r="R8" s="25"/>
@@ -4177,16 +4185,16 @@
         <v>26</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="G9" s="19" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="H9" s="10" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="I9" s="6" t="s">
         <v>12</v>
@@ -4195,10 +4203,10 @@
         <v>0</v>
       </c>
       <c r="K9" s="16" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="L9" s="7" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="M9" s="6">
         <v>10</v>
@@ -4214,22 +4222,22 @@
         <v>6</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D10" s="9">
         <v>63</v>
       </c>
       <c r="E10" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="F10" s="10" t="s">
+        <v>106</v>
+      </c>
+      <c r="G10" s="11" t="s">
+        <v>301</v>
+      </c>
+      <c r="H10" s="10" t="s">
         <v>107</v>
-      </c>
-      <c r="F10" s="10" t="s">
-        <v>108</v>
-      </c>
-      <c r="G10" s="11" t="s">
-        <v>303</v>
-      </c>
-      <c r="H10" s="10" t="s">
-        <v>109</v>
       </c>
       <c r="I10" s="6" t="s">
         <v>13</v>
@@ -4238,12 +4246,12 @@
         <v>0</v>
       </c>
       <c r="K10" s="12" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="L10" s="7"/>
       <c r="N10" s="23"/>
       <c r="R10" s="26" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
     </row>
     <row r="11" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4254,22 +4262,22 @@
         <v>6</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D11" s="9">
         <v>65</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="F11" s="10" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="G11" s="11" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="H11" s="10" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="I11" s="6" t="s">
         <v>14</v>
@@ -4278,12 +4286,12 @@
         <v>0</v>
       </c>
       <c r="K11" s="12" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="L11" s="7"/>
       <c r="N11" s="23"/>
       <c r="R11" s="26" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
     </row>
     <row r="12" spans="1:18" s="14" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4294,22 +4302,22 @@
         <v>6</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D12" s="14">
         <v>63</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="G12" s="21" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="H12" s="21" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="I12" s="14" t="s">
         <v>15</v>
@@ -4318,11 +4326,11 @@
         <v>1</v>
       </c>
       <c r="K12" s="14" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="N12" s="23"/>
       <c r="R12" s="27" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
     </row>
     <row r="13" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4333,22 +4341,22 @@
         <v>6</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D13" s="9">
         <v>63</v>
       </c>
       <c r="E13" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="F13" s="10" t="s">
+        <v>111</v>
+      </c>
+      <c r="G13" s="11" t="s">
+        <v>221</v>
+      </c>
+      <c r="H13" s="10" t="s">
         <v>112</v>
-      </c>
-      <c r="F13" s="10" t="s">
-        <v>113</v>
-      </c>
-      <c r="G13" s="11" t="s">
-        <v>223</v>
-      </c>
-      <c r="H13" s="10" t="s">
-        <v>114</v>
       </c>
       <c r="I13" s="6" t="s">
         <v>16</v>
@@ -4357,7 +4365,7 @@
         <v>0</v>
       </c>
       <c r="K13" s="12" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="L13" s="7"/>
       <c r="N13" s="23"/>
@@ -4371,22 +4379,22 @@
         <v>7</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D14" s="14">
         <v>69</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="G14" s="14" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="H14" s="14" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="I14" s="14" t="s">
         <v>17</v>
@@ -4395,11 +4403,11 @@
         <v>1</v>
       </c>
       <c r="K14" s="14" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="N14" s="23"/>
       <c r="R14" s="27" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
     </row>
     <row r="15" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4410,22 +4418,22 @@
         <v>7</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D15" s="9">
         <v>70</v>
       </c>
       <c r="E15" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="F15" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="H15" s="10" t="s">
         <v>116</v>
-      </c>
-      <c r="F15" s="10" t="s">
-        <v>117</v>
-      </c>
-      <c r="G15" s="7" t="s">
-        <v>225</v>
-      </c>
-      <c r="H15" s="10" t="s">
-        <v>118</v>
       </c>
       <c r="I15" s="6" t="s">
         <v>18</v>
@@ -4434,7 +4442,7 @@
         <v>0</v>
       </c>
       <c r="K15" s="12" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="L15" s="7"/>
       <c r="N15" s="23"/>
@@ -4448,22 +4456,22 @@
         <v>7</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D16" s="14">
         <v>64</v>
       </c>
       <c r="E16" s="14" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F16" s="21" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="G16" s="14" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="H16" s="14" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="I16" s="14" t="s">
         <v>19</v>
@@ -4472,7 +4480,7 @@
         <v>2</v>
       </c>
       <c r="K16" s="14" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="N16" s="23"/>
       <c r="R16" s="28"/>
@@ -4485,22 +4493,22 @@
         <v>8</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D17" s="9">
         <v>85</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="F17" s="10" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="H17" s="10" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="I17" s="10" t="s">
         <v>20</v>
@@ -4509,11 +4517,11 @@
         <v>0</v>
       </c>
       <c r="K17" s="12" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="L17" s="7"/>
       <c r="N17" s="21" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="R17" s="25"/>
     </row>
@@ -4525,22 +4533,22 @@
         <v>8</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D18" s="9">
         <v>84</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="F18" s="10" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="H18" s="10" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="I18" s="6" t="s">
         <v>25</v>
@@ -4549,7 +4557,7 @@
         <v>0</v>
       </c>
       <c r="K18" s="12" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="L18" s="7"/>
       <c r="N18" s="23"/>
@@ -4563,22 +4571,22 @@
         <v>8</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D19" s="9">
         <v>93</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="F19" s="10" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="H19" s="10" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="I19" s="6" t="s">
         <v>29</v>
@@ -4587,7 +4595,7 @@
         <v>0</v>
       </c>
       <c r="K19" s="12" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="L19" s="7"/>
       <c r="N19" s="23"/>
@@ -4601,22 +4609,22 @@
         <v>8</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D20" s="9">
         <v>69</v>
       </c>
       <c r="E20" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="F20" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="H20" s="10" t="s">
         <v>123</v>
-      </c>
-      <c r="F20" s="10" t="s">
-        <v>124</v>
-      </c>
-      <c r="G20" s="7" t="s">
-        <v>229</v>
-      </c>
-      <c r="H20" s="10" t="s">
-        <v>125</v>
       </c>
       <c r="I20" s="13" t="s">
         <v>30</v>
@@ -4625,7 +4633,7 @@
         <v>0</v>
       </c>
       <c r="K20" s="12" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="L20" s="7"/>
       <c r="N20" s="23"/>
@@ -4639,22 +4647,22 @@
         <v>9</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D21" s="9">
         <v>78</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="F21" s="10" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="H21" s="14" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="I21" s="6" t="s">
         <v>32</v>
@@ -4663,7 +4671,7 @@
         <v>0</v>
       </c>
       <c r="K21" s="12" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="L21" s="7"/>
       <c r="N21" s="23"/>
@@ -4677,22 +4685,22 @@
         <v>9</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D22" s="9">
         <v>75</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="F22" s="10" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="H22" s="14" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="I22" s="10" t="s">
         <v>34</v>
@@ -4701,7 +4709,7 @@
         <v>0</v>
       </c>
       <c r="K22" s="12" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="L22" s="7"/>
       <c r="N22" s="21"/>
@@ -4715,22 +4723,22 @@
         <v>9</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D23" s="9">
         <v>78</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F23" s="10" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="G23" s="7" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="H23" s="21" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="I23" s="10" t="s">
         <v>36</v>
@@ -4739,11 +4747,11 @@
         <v>0</v>
       </c>
       <c r="K23" s="12" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="L23" s="7"/>
       <c r="N23" s="21" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="R23" s="25"/>
     </row>
@@ -4755,22 +4763,22 @@
         <v>9</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D24" s="9">
         <v>75</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="F24" s="10" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="G24" s="7" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="H24" s="14" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="I24" s="10" t="s">
         <v>38</v>
@@ -4779,7 +4787,7 @@
         <v>0</v>
       </c>
       <c r="K24" s="12" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="L24" s="7"/>
       <c r="N24" s="14"/>
@@ -4793,22 +4801,22 @@
         <v>11</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D25" s="9">
         <v>85</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="F25" s="10" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="H25" s="10" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="I25" s="10" t="s">
         <v>39</v>
@@ -4817,7 +4825,7 @@
         <v>0</v>
       </c>
       <c r="K25" s="12" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="L25" s="7"/>
       <c r="N25" s="14"/>
@@ -4831,22 +4839,22 @@
         <v>11</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D26" s="9">
         <v>78</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="F26" s="10" t="s">
+        <v>330</v>
+      </c>
+      <c r="G26" s="7" t="s">
         <v>332</v>
       </c>
-      <c r="G26" s="7" t="s">
-        <v>334</v>
-      </c>
       <c r="H26" s="10" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="I26" s="10" t="s">
         <v>41</v>
@@ -4855,11 +4863,11 @@
         <v>0</v>
       </c>
       <c r="K26" s="12" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="L26" s="7"/>
       <c r="N26" s="14" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="R26" s="25"/>
     </row>
@@ -4871,22 +4879,22 @@
         <v>11</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D27" s="9">
         <v>95</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="F27" s="10" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="G27" s="7" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="H27" s="10" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="I27" s="10" t="s">
         <v>46</v>
@@ -4895,7 +4903,7 @@
         <v>0</v>
       </c>
       <c r="K27" s="12" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="L27" s="7"/>
       <c r="N27" s="14"/>
@@ -4909,22 +4917,22 @@
         <v>11</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D28" s="9">
         <v>107</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="F28" s="10" t="s">
+        <v>336</v>
+      </c>
+      <c r="G28" s="7" t="s">
         <v>338</v>
       </c>
-      <c r="G28" s="7" t="s">
-        <v>340</v>
-      </c>
       <c r="H28" s="10" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="I28" s="10" t="s">
         <v>48</v>
@@ -4933,7 +4941,7 @@
         <v>0</v>
       </c>
       <c r="K28" s="12" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="L28" s="7"/>
       <c r="N28" s="14"/>
@@ -4953,16 +4961,16 @@
         <v>40</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="F29" s="10" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="G29" s="18" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="H29" s="10" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="I29" s="6" t="s">
         <v>50</v>
@@ -4971,10 +4979,10 @@
         <v>0</v>
       </c>
       <c r="K29" s="16" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="L29" s="7" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="M29" s="6">
         <v>3</v>
@@ -4984,7 +4992,7 @@
         <v>51</v>
       </c>
       <c r="Q29" s="13" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="R29" s="25"/>
     </row>
@@ -5002,16 +5010,16 @@
         <v>26</v>
       </c>
       <c r="E30" s="13" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="F30" s="10" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="G30" s="7" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="H30" s="10" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="I30" s="6" t="s">
         <v>52</v>
@@ -5020,20 +5028,20 @@
         <v>0</v>
       </c>
       <c r="K30" s="12" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="L30" s="6" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="M30" s="6" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="N30" s="14"/>
       <c r="P30" s="10" t="s">
         <v>53</v>
       </c>
       <c r="Q30" s="13" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="R30" s="25"/>
     </row>
@@ -5051,16 +5059,16 @@
         <v>34</v>
       </c>
       <c r="E31" s="13" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="F31" s="10" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="G31" s="18" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="H31" s="10" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="I31" s="6" t="s">
         <v>54</v>
@@ -5069,20 +5077,20 @@
         <v>0</v>
       </c>
       <c r="K31" s="16" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="L31" s="14" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="M31" s="14" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="N31" s="23"/>
       <c r="P31" s="10" t="s">
         <v>55</v>
       </c>
       <c r="Q31" s="13" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="R31" s="25"/>
     </row>
@@ -5100,16 +5108,16 @@
         <v>34</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="F32" s="10" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="G32" s="18" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="H32" s="10" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="I32" s="6" t="s">
         <v>56</v>
@@ -5118,20 +5126,20 @@
         <v>0</v>
       </c>
       <c r="K32" s="16" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="L32" s="7" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="M32" s="6" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="N32" s="23"/>
       <c r="P32" s="10" t="s">
         <v>57</v>
       </c>
       <c r="Q32" s="13" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="R32" s="25"/>
     </row>
@@ -5149,16 +5157,16 @@
         <v>26</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="F33" s="10" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="G33" s="7" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="H33" s="10" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="I33" s="6" t="s">
         <v>58</v>
@@ -5167,20 +5175,20 @@
         <v>0</v>
       </c>
       <c r="K33" s="12" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="L33" s="7" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="M33" s="6" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="N33" s="14"/>
       <c r="P33" s="10" t="s">
         <v>59</v>
       </c>
       <c r="Q33" s="13" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="R33" s="25"/>
     </row>
@@ -5198,16 +5206,16 @@
         <v>28</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="F34" s="10" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="G34" s="7" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="H34" s="10" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="I34" s="6" t="s">
         <v>60</v>
@@ -5216,20 +5224,20 @@
         <v>0</v>
       </c>
       <c r="K34" s="12" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="L34" s="7" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="M34" s="6" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="N34" s="14"/>
       <c r="P34" s="10" t="s">
         <v>61</v>
       </c>
       <c r="Q34" s="13" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="R34" s="25"/>
     </row>
@@ -5247,16 +5255,16 @@
         <v>26</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="F35" s="10" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="G35" s="18" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="H35" s="10" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="I35" s="6" t="s">
         <v>62</v>
@@ -5265,20 +5273,20 @@
         <v>0</v>
       </c>
       <c r="K35" s="16" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="L35" s="7" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="M35" s="6" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="N35" s="23"/>
       <c r="P35" s="10" t="s">
         <v>63</v>
       </c>
       <c r="Q35" s="13" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="R35" s="25"/>
     </row>
@@ -5296,16 +5304,16 @@
         <v>34</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="F36" s="10" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="G36" s="18" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="H36" s="10" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="I36" s="6" t="s">
         <v>64</v>
@@ -5314,10 +5322,10 @@
         <v>0</v>
       </c>
       <c r="K36" s="16" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="L36" s="7" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="M36" s="6">
         <v>5</v>
@@ -5327,7 +5335,7 @@
         <v>65</v>
       </c>
       <c r="Q36" s="13" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="R36" s="25"/>
     </row>
@@ -5339,22 +5347,22 @@
         <v>97</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D37" s="9">
         <v>97</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="F37" s="10" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="G37" s="7" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="H37" s="10" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="I37" s="6" t="s">
         <v>73</v>
@@ -5363,7 +5371,7 @@
         <v>0</v>
       </c>
       <c r="K37" s="12" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="L37" s="7"/>
       <c r="N37" s="14"/>
@@ -5371,7 +5379,7 @@
         <v>67</v>
       </c>
       <c r="Q37" s="13" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="R37" s="25"/>
     </row>
@@ -5383,22 +5391,22 @@
         <v>67</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D38" s="9">
         <v>67</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="F38" s="10" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="G38" s="7" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="H38" s="10" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="I38" s="6" t="s">
         <v>74</v>
@@ -5407,7 +5415,7 @@
         <v>0</v>
       </c>
       <c r="K38" s="12" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="L38" s="7"/>
       <c r="N38" s="14"/>
@@ -5415,7 +5423,7 @@
         <v>75</v>
       </c>
       <c r="Q38" s="13" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="R38" s="25"/>
     </row>
@@ -5427,31 +5435,31 @@
         <v>85</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D39" s="9">
         <v>85</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="F39" s="10" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="G39" s="7" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="H39" s="10" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="I39" s="10" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="J39" s="9">
         <v>0</v>
       </c>
       <c r="K39" s="12" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="L39" s="7"/>
       <c r="N39" s="14"/>
@@ -5459,7 +5467,7 @@
         <v>69</v>
       </c>
       <c r="Q39" s="13" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="R39" s="25"/>
     </row>
@@ -5628,7 +5636,7 @@
         <v>13</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5643,7 +5651,7 @@
         <v>14</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5658,7 +5666,7 @@
         <v>15</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5673,7 +5681,7 @@
         <v>16</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5688,7 +5696,7 @@
         <v>17</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5703,7 +5711,7 @@
         <v>18</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5718,7 +5726,7 @@
         <v>19</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5733,7 +5741,7 @@
         <v>20</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5748,7 +5756,7 @@
         <v>21</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5763,7 +5771,7 @@
         <v>22</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5778,7 +5786,7 @@
         <v>23</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5793,7 +5801,7 @@
         <v>24</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5808,7 +5816,7 @@
         <v>25</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5823,7 +5831,7 @@
         <v>26</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5838,7 +5846,7 @@
         <v>27</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5853,7 +5861,7 @@
         <v>28</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5868,7 +5876,7 @@
         <v>29</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5883,7 +5891,7 @@
         <v>30</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5897,7 +5905,7 @@
         <v>31</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5911,7 +5919,7 @@
         <v>32</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5925,7 +5933,7 @@
         <v>33</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5939,7 +5947,7 @@
         <v>34</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5953,7 +5961,7 @@
         <v>35</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5967,7 +5975,7 @@
         <v>36</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5981,7 +5989,7 @@
         <v>37</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5995,7 +6003,7 @@
         <v>38</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6009,7 +6017,7 @@
         <v>39</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6023,7 +6031,7 @@
         <v>40</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6037,7 +6045,7 @@
         <v>41</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6051,7 +6059,7 @@
         <v>42</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6065,7 +6073,7 @@
         <v>43</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6079,7 +6087,7 @@
         <v>44</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6093,7 +6101,7 @@
         <v>45</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6107,7 +6115,7 @@
         <v>46</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6121,7 +6129,7 @@
         <v>47</v>
       </c>
       <c r="D44" s="5" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6135,7 +6143,7 @@
         <v>48</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6149,7 +6157,7 @@
         <v>49</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6275,7 +6283,7 @@
         <v>66</v>
       </c>
       <c r="D55" s="5" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6289,7 +6297,7 @@
         <v>68</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6303,7 +6311,7 @@
         <v>70</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
     </row>
     <row r="58" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6317,7 +6325,7 @@
         <v>71</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6331,7 +6339,7 @@
         <v>72</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
     </row>
     <row r="60" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6345,7 +6353,7 @@
         <v>73</v>
       </c>
       <c r="D60" s="5" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6359,7 +6367,7 @@
         <v>74</v>
       </c>
       <c r="D61" s="5" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6373,7 +6381,7 @@
         <v>68</v>
       </c>
       <c r="D62" s="5" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
     </row>
     <row r="63" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6387,7 +6395,7 @@
         <v>66</v>
       </c>
       <c r="D63" s="5" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
     </row>
     <row r="64" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6398,10 +6406,10 @@
         <v>38</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix Programmingasks: leser.java & schach.java
- leser.java: private method not possible for unit tests (ToDo: Change picture)
- schach.java: fixed comments
</commit_message>
<xml_diff>
--- a/files/programming-tasks/programmieraufgaben_JACK_SOSE23_WORKSHOP_WISE2324.xlsx
+++ b/files/programming-tasks/programmieraufgaben_JACK_SOSE23_WORKSHOP_WISE2324.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27531"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\hefl\files\programming-tasks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99FF57EC-9EC3-426F-8EA3-5EC8A7825085}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCC6DCA1-03E0-4579-9BD5-8B87157B2B69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="51480" yWindow="0" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Aufgaben" sheetId="1" r:id="rId1"/>
@@ -1770,23 +1770,6 @@
   </si>
   <si>
     <t>package de.goals.testing; // nicht entfernen
-import java.lang.Math;
-public class Schach
-{
-	public int felder(int cent) {
-	   //Ihre Lösung!!
-       //Rückgabe: Anzahl der Felder
-	}
-    public static void main(String[] args)
-    {
-        Schach koenigSchach= new Schach();
-        int centStuecke=1000; //Ausgabe muss bei 1000 Centstücken 9 sein.
-        System.out.println(koenigSchach.felder(centStuecke)); // Korrektur: Kai hat hier j aus dem Codegerüst von Jack mit centStuecke ersetzt
-    }    
-}</t>
-  </si>
-  <si>
-    <t>package de.goals.testing; // nicht entfernen
 public class Buch {
     // Ihre Loesung
 }</t>
@@ -2106,18 +2089,6 @@
     fahren() erhält die Strecke als Parameter und errechnet dann ob der aktuelle Tankinhalt ausreicht die Strecke zu fahren. Wenn das nicht der Fall ist, gibt die Methode false zurück. Wenn es möglich ist, dann berechnet die Methode den Kraftstoffverbrauch für die gefahrenen Kilometer und zieht die Liter von der aktuellen Kraftstoffmenge ab. Außerdem wird der Kilometerstand entsprechend erhöht. Die Methode gibt dann true zurück. 
 Implementieren Sie die Klasse KFZ in Java. Selbstverständlich können Sie auch noch weitere Methoden implementieren. 
 Implementieren Sie eine neue Test-Klasse AppAuto, in der Autos erzeugt werden und diese fahren bzw. tanken lässt. </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Betrachten Sie das folgende UML-Diagramm:
-Bild von einem Klassendiagramm der Klasse Leser: Attribute LeserID (int), Kontonr(int), Name(String). Methoden: changeKontonr(nr inr), getName(), setName(name: String), getLeserID()
-Erstellen Sie zu diesem Klassendiagramm den entsprechenden Java-Code. Beachten Sie dabei vor allem die Sichtbarkeiten!
-Implementieren Sie einen Konstruktor der alle Attribute als Argument erhält! Implementieren Sie die Rümpfe der Methoden. </t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Betrachten Sie das folgende UML-Diagramm:&lt;/p&gt;
-&lt;img src="/assets/taskImgs/UMLtoJava.png" alt="image"&gt;
-&lt;br /&gt;Erstellen Sie zu diesem Klassendiagramm den entsprechenden Java-Code. Beachten Sie dabei vor allem die Sichtbarkeiten!&lt;/p&gt;
-&lt;p&gt;Implementieren Sie einen Konstruktor der alle Attribute als Argument erh&amp;auml;lt!&amp;nbsp;Implementieren Sie die R&amp;uuml;mpfe der Methoden.&amp;nbsp;&lt;/p&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">Die Klasse Punkt soll einen Punkt in einem zweidimensionalen Koordinatensystem repräsentieren. Ein Punkt besteht aus folgenden Attribute: 
@@ -3272,6 +3243,37 @@
 x = charFrequenz(s)
 x wäre dann:
 [('s', 4), ('t', 4), ('i', 3), ('e', 2), ('n', 2), ('a', 1), ('d', 1), ('g', 1), ('r', 1)]</t>
+  </si>
+  <si>
+    <t>package de.goals.testing; // nicht entfernen
+import java.lang.Math;
+public class Schach
+{
+	public int felder(int cent) {
+	   //Ihre Lösung!!
+       //Rückgabe: Anzahl der Felder
+	}
+    public static void main(String[] args)
+    {
+        Schach koenigSchach= new Schach();
+        int centStuecke=1000; //Ausgabe muss bei 1000 Centstücken 10 sein.
+        System.out.println(koenigSchach.felder(centStuecke)); 
+    }    
+}</t>
+  </si>
+  <si>
+    <t>Betrachten Sie das folgende UML-Diagramm:
+Bild von einem Klassendiagramm der Klasse Leser: Attribute LeserID (int und protected), Kontonr(int und private), Name(String und public). Methoden: private changeKontonr(nr: int), public getName(), private setName(name: String), protected getLeserID()
+Erstellen Sie zu diesem Klassendiagramm den entsprechenden Java-Code. Beachten Sie dabei vor allem die Sichtbarkeiten!
+Implementieren Sie einen Konstruktor der alle Attribute als Argument erhält! Implementieren Sie die Rümpfe der Methoden. 
+HINWEIS VOM 12.06: Verwenden Sie public oder protected Methoden anstelle von private. Ansonsten gibt es aktuell Probleme mit unseren automatischen Tests.</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Betrachten Sie das folgende UML-Diagramm:&lt;/p&gt;
+&lt;img src="/assets/taskImgs/UMLtoJava.png" alt="image"&gt;
+&lt;br /&gt;Erstellen Sie zu diesem Klassendiagramm den entsprechenden Java-Code. Beachten Sie dabei vor allem die Sichtbarkeiten!&lt;/p&gt;
+&lt;p&gt;Implementieren Sie einen Konstruktor der alle Attribute als Argument erh&amp;auml;lt!&amp;nbsp;Implementieren Sie die R&amp;uuml;mpfe der Methoden.&amp;nbsp;&lt;/p&gt;
+&lt;p&gt;HINWEIS VOM 12.06: Verwenden Sie public oder protected Methoden anstelle von private. Ansonsten gibt es aktuell Probleme mit unseren automatischen Tests.&lt;/p&gt;</t>
   </si>
 </sst>
 </file>
@@ -3977,7 +3979,7 @@
         <v>163</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="I4" s="6" t="s">
         <v>7</v>
@@ -4020,7 +4022,7 @@
         <v>164</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="I5" s="6" t="s">
         <v>8</v>
@@ -4057,13 +4059,13 @@
         <v>97</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="H6" s="10" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="I6" s="6" t="s">
         <v>9</v>
@@ -4082,7 +4084,7 @@
       </c>
       <c r="N6" s="23"/>
       <c r="R6" s="26" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
     </row>
     <row r="7" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4123,7 +4125,7 @@
         <v>207</v>
       </c>
       <c r="M7" s="6" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="N7" s="23"/>
       <c r="R7" s="25"/>
@@ -4151,7 +4153,7 @@
         <v>166</v>
       </c>
       <c r="H8" s="10" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="I8" s="6" t="s">
         <v>11</v>
@@ -4188,13 +4190,13 @@
         <v>103</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="G9" s="19" t="s">
         <v>167</v>
       </c>
       <c r="H9" s="10" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="I9" s="6" t="s">
         <v>12</v>
@@ -4234,7 +4236,7 @@
         <v>106</v>
       </c>
       <c r="G10" s="11" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="H10" s="10" t="s">
         <v>107</v>
@@ -4251,7 +4253,7 @@
       <c r="L10" s="7"/>
       <c r="N10" s="23"/>
       <c r="R10" s="26" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
     </row>
     <row r="11" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4271,13 +4273,13 @@
         <v>108</v>
       </c>
       <c r="F11" s="10" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="G11" s="11" t="s">
         <v>219</v>
       </c>
       <c r="H11" s="10" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="I11" s="6" t="s">
         <v>14</v>
@@ -4291,7 +4293,7 @@
       <c r="L11" s="7"/>
       <c r="N11" s="23"/>
       <c r="R11" s="26" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
     </row>
     <row r="12" spans="1:18" s="14" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4311,13 +4313,13 @@
         <v>109</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="G12" s="21" t="s">
         <v>220</v>
       </c>
       <c r="H12" s="21" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="I12" s="14" t="s">
         <v>15</v>
@@ -4330,7 +4332,7 @@
       </c>
       <c r="N12" s="23"/>
       <c r="R12" s="27" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
     </row>
     <row r="13" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4388,13 +4390,13 @@
         <v>113</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="G14" s="14" t="s">
         <v>222</v>
       </c>
       <c r="H14" s="14" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="I14" s="14" t="s">
         <v>17</v>
@@ -4407,7 +4409,7 @@
       </c>
       <c r="N14" s="23"/>
       <c r="R14" s="27" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="15" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4465,13 +4467,13 @@
         <v>117</v>
       </c>
       <c r="F16" s="21" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="G16" s="14" t="s">
         <v>224</v>
       </c>
       <c r="H16" s="14" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="I16" s="14" t="s">
         <v>19</v>
@@ -4502,13 +4504,13 @@
         <v>118</v>
       </c>
       <c r="F17" s="10" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="H17" s="10" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="I17" s="10" t="s">
         <v>20</v>
@@ -4521,7 +4523,7 @@
       </c>
       <c r="L17" s="7"/>
       <c r="N17" s="21" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="R17" s="25"/>
     </row>
@@ -4542,13 +4544,13 @@
         <v>119</v>
       </c>
       <c r="F18" s="10" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="G18" s="7" t="s">
         <v>225</v>
       </c>
       <c r="H18" s="10" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="I18" s="6" t="s">
         <v>25</v>
@@ -4580,13 +4582,13 @@
         <v>120</v>
       </c>
       <c r="F19" s="10" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="G19" s="7" t="s">
         <v>226</v>
       </c>
       <c r="H19" s="10" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="I19" s="6" t="s">
         <v>29</v>
@@ -4656,13 +4658,13 @@
         <v>124</v>
       </c>
       <c r="F21" s="10" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="H21" s="14" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="I21" s="6" t="s">
         <v>32</v>
@@ -4694,13 +4696,13 @@
         <v>125</v>
       </c>
       <c r="F22" s="10" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="H22" s="14" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="I22" s="10" t="s">
         <v>34</v>
@@ -4732,13 +4734,13 @@
         <v>126</v>
       </c>
       <c r="F23" s="10" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="G23" s="7" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="H23" s="21" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="I23" s="10" t="s">
         <v>36</v>
@@ -4751,7 +4753,7 @@
       </c>
       <c r="L23" s="7"/>
       <c r="N23" s="21" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="R23" s="25"/>
     </row>
@@ -4772,13 +4774,13 @@
         <v>127</v>
       </c>
       <c r="F24" s="10" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="G24" s="7" t="s">
         <v>228</v>
       </c>
       <c r="H24" s="14" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="I24" s="10" t="s">
         <v>38</v>
@@ -4810,13 +4812,13 @@
         <v>128</v>
       </c>
       <c r="F25" s="10" t="s">
-        <v>270</v>
+        <v>353</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="H25" s="10" t="s">
-        <v>271</v>
+        <v>354</v>
       </c>
       <c r="I25" s="10" t="s">
         <v>39</v>
@@ -4848,13 +4850,13 @@
         <v>129</v>
       </c>
       <c r="F26" s="10" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="G26" s="7" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="H26" s="10" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="I26" s="10" t="s">
         <v>41</v>
@@ -4867,7 +4869,7 @@
       </c>
       <c r="L26" s="7"/>
       <c r="N26" s="14" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="R26" s="25"/>
     </row>
@@ -4888,13 +4890,13 @@
         <v>130</v>
       </c>
       <c r="F27" s="10" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="G27" s="7" t="s">
         <v>229</v>
       </c>
       <c r="H27" s="10" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="I27" s="10" t="s">
         <v>46</v>
@@ -4926,13 +4928,13 @@
         <v>131</v>
       </c>
       <c r="F28" s="10" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="H28" s="10" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="I28" s="10" t="s">
         <v>48</v>
@@ -4961,7 +4963,7 @@
         <v>40</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="F29" s="10" t="s">
         <v>132</v>
@@ -5010,13 +5012,13 @@
         <v>26</v>
       </c>
       <c r="E30" s="13" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="F30" s="10" t="s">
         <v>135</v>
       </c>
       <c r="G30" s="7" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="H30" s="10" t="s">
         <v>136</v>
@@ -5031,10 +5033,10 @@
         <v>201</v>
       </c>
       <c r="L30" s="6" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="M30" s="6" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="N30" s="14"/>
       <c r="P30" s="10" t="s">
@@ -5059,7 +5061,7 @@
         <v>34</v>
       </c>
       <c r="E31" s="13" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="F31" s="10" t="s">
         <v>138</v>
@@ -5108,7 +5110,7 @@
         <v>34</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="F32" s="10" t="s">
         <v>141</v>
@@ -5157,7 +5159,7 @@
         <v>26</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="F33" s="10" t="s">
         <v>144</v>
@@ -5178,10 +5180,10 @@
         <v>201</v>
       </c>
       <c r="L33" s="7" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="M33" s="6" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="N33" s="14"/>
       <c r="P33" s="10" t="s">
@@ -5206,7 +5208,7 @@
         <v>28</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="F34" s="10" t="s">
         <v>147</v>
@@ -5227,10 +5229,10 @@
         <v>201</v>
       </c>
       <c r="L34" s="7" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="M34" s="6" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="N34" s="14"/>
       <c r="P34" s="10" t="s">
@@ -5255,7 +5257,7 @@
         <v>26</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="F35" s="10" t="s">
         <v>150</v>
@@ -5304,7 +5306,7 @@
         <v>34</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="F36" s="10" t="s">
         <v>153</v>
@@ -5353,7 +5355,7 @@
         <v>97</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="F37" s="10" t="s">
         <v>156</v>
@@ -5362,7 +5364,7 @@
         <v>230</v>
       </c>
       <c r="H37" s="10" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="I37" s="6" t="s">
         <v>73</v>
@@ -5397,16 +5399,16 @@
         <v>67</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="F38" s="10" t="s">
         <v>158</v>
       </c>
       <c r="G38" s="7" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="H38" s="10" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="I38" s="6" t="s">
         <v>74</v>
@@ -5415,7 +5417,7 @@
         <v>0</v>
       </c>
       <c r="K38" s="12" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="L38" s="7"/>
       <c r="N38" s="14"/>
@@ -5441,25 +5443,25 @@
         <v>85</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="F39" s="10" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="G39" s="7" t="s">
         <v>231</v>
       </c>
       <c r="H39" s="10" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="I39" s="10" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="J39" s="9">
         <v>0</v>
       </c>
       <c r="K39" s="12" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="L39" s="7"/>
       <c r="N39" s="14"/>
@@ -5636,7 +5638,7 @@
         <v>13</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5651,7 +5653,7 @@
         <v>14</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5666,7 +5668,7 @@
         <v>15</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5696,7 +5698,7 @@
         <v>17</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5711,7 +5713,7 @@
         <v>18</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>233</v>
+        <v>352</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5726,7 +5728,7 @@
         <v>19</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5741,7 +5743,7 @@
         <v>20</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5756,7 +5758,7 @@
         <v>21</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5771,7 +5773,7 @@
         <v>22</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5786,7 +5788,7 @@
         <v>23</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5801,7 +5803,7 @@
         <v>24</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5816,7 +5818,7 @@
         <v>25</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5831,7 +5833,7 @@
         <v>26</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5846,7 +5848,7 @@
         <v>27</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5861,7 +5863,7 @@
         <v>28</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5876,7 +5878,7 @@
         <v>29</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5891,7 +5893,7 @@
         <v>30</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5905,7 +5907,7 @@
         <v>31</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5919,7 +5921,7 @@
         <v>32</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5933,7 +5935,7 @@
         <v>33</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5947,7 +5949,7 @@
         <v>34</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5961,7 +5963,7 @@
         <v>35</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5975,7 +5977,7 @@
         <v>36</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5989,7 +5991,7 @@
         <v>37</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6003,7 +6005,7 @@
         <v>38</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6017,7 +6019,7 @@
         <v>39</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6031,7 +6033,7 @@
         <v>40</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6045,7 +6047,7 @@
         <v>41</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6059,7 +6061,7 @@
         <v>42</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6073,7 +6075,7 @@
         <v>43</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6087,7 +6089,7 @@
         <v>44</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6101,7 +6103,7 @@
         <v>45</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6115,7 +6117,7 @@
         <v>46</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6129,7 +6131,7 @@
         <v>47</v>
       </c>
       <c r="D44" s="5" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6143,7 +6145,7 @@
         <v>48</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6157,7 +6159,7 @@
         <v>49</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6283,7 +6285,7 @@
         <v>66</v>
       </c>
       <c r="D55" s="5" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6297,7 +6299,7 @@
         <v>68</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6311,7 +6313,7 @@
         <v>70</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="58" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6325,7 +6327,7 @@
         <v>71</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6339,7 +6341,7 @@
         <v>72</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="60" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6353,7 +6355,7 @@
         <v>73</v>
       </c>
       <c r="D60" s="5" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6367,7 +6369,7 @@
         <v>74</v>
       </c>
       <c r="D61" s="5" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6381,7 +6383,7 @@
         <v>68</v>
       </c>
       <c r="D62" s="5" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="63" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6395,7 +6397,7 @@
         <v>66</v>
       </c>
       <c r="D63" s="5" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="64" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6406,10 +6408,10 @@
         <v>38</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed Bibliothek and Leser
- new UML Diagramms
- fixed Unit Test
- Mermaid Diagram Text for GPT
</commit_message>
<xml_diff>
--- a/files/programming-tasks/programmieraufgaben_JACK_SOSE23_WORKSHOP_WISE2324.xlsx
+++ b/files/programming-tasks/programmieraufgaben_JACK_SOSE23_WORKSHOP_WISE2324.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\hefl\files\programming-tasks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCC6DCA1-03E0-4579-9BD5-8B87157B2B69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC0D46B9-8D5E-4BE0-8461-EDFE268A7E27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-165" yWindow="-165" windowWidth="51930" windowHeight="21210" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Aufgaben" sheetId="1" r:id="rId1"/>
@@ -2687,26 +2687,6 @@
 </t>
   </si>
   <si>
-    <t>Betrachten Sie das folgende Klassendiagramm:
-a) Machen Sie sich mit den Eigenschaften der  Klasse Datum  vertraut, in dem Sie sich den Quelltext anschauen. Schauen Sie sich die Eigenschaften der Klasse Calendar in der Java-API an.
-b) Setzen Sie nun das oben stehende UML-Klassendiagramm in Java um, unter der Verwendung der Klasse Datum. Implementieren Sie auch die Methoden der Klassen Medium, Buch und DVD. Für die Berechnung des Strafgeldes bei Überziehung der Leihfristen gelten folgende Bestimmungen:
-- Bücher können 4 Wochen ausgeliehen werden, bei Überziehung 1 EUR Strafgeld pro angefangenen Überziehungstag.
-- DVDs können 1 Woche ausgeliehen werden, bei Überziehung 2 EUR Strafgeld pro angefangenen Überziehungstag
-Für die Berechnung der Differenztage zwischen dem Ausleihdatum und Heute implementieren Sie bitte die Methode calcDiffDays() der Klasse Datum. Nehmen Sie dazu an, dass jeder Monat 30 Tage hat und das Jahr 365 Tage.
-c) Schreiben Sie ein kleines Testprogramm (BibVerwaltung.java), das Objekte von den beiden Medien Buch und DVD erzeugt.</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Betrachten Sie das folgende Klassendiagramm:&lt;br /&gt;
-&lt;img src="/assets/taskImgs/Java_Bibliothek_Bib.jpg" alt="image"&gt;
-&lt;br /&gt;
-a) Machen Sie sich mit den&amp;nbsp;Eigenschaften der  Klasse Datum vertraut, in dem Sie sich den Quelltext anschauen. Schauen Sie sich&amp;nbsp;die Eigenschaften der Klasse Calendar in der Java-API an.&lt;/p&gt;
-&lt;p&gt;b) Setzen Sie nun das oben stehende UML-Klassendiagramm in Java um, unter der&amp;nbsp;Verwendung der Klasse Datum. Implementieren Sie auch die Methoden der Klassen&amp;nbsp;Medium, Buch und DVD. Für die Berechnung des Strafgeldes bei &amp;Uuml;berziehung der&amp;nbsp;Leihfristen gelten folgende Bestimmungen:&lt;/p&gt;
-&lt;p&gt;- Bücher k&amp;ouml;nnen 4 Wochen ausgeliehen werden, bei &amp;Uuml;berziehung 1 EUR Strafgeld pro&amp;nbsp;angefangenen &amp;Uuml;berziehungstag.&lt;br /&gt;
-- DVDs k&amp;ouml;nnen 1 Woche ausgeliehen werden, bei &amp;Uuml;berziehung 2 EUR Strafgeld pro&amp;nbsp;angefangenen &amp;Uuml;berziehungstag&lt;/p&gt;
-&lt;p&gt;Für die Berechnung der Differenztage zwischen dem Ausleihdatum und Heute&amp;nbsp;implementieren Sie bitte die Methode calcDiffDays() der Klasse Datum. Nehmen Sie&amp;nbsp;dazu an, dass jeder Monat 30 Tage hat und das Jahr 365 Tage.&lt;/p&gt;
-&lt;p&gt;c) Schreiben Sie ein kleines Testprogramm (BibVerwaltung.java), das Objekte von den&amp;nbsp;beiden Medien Buch und DVD erzeugt.&lt;/p&gt;</t>
-  </si>
-  <si>
     <t xml:space="preserve">Schreiben Sie eine Klasse Konto, die ein Bankkonto realisiert. Attribute für das Bankkonto sind der Name und Vorname des Kontoinhabers, die Kontonummer (IBAN), der Kontostand, sowie ein Limit, bis zu dem das Konto überzogen werden darf.
 Erstellen Sie einen oder mehrere geeignete Konstruktoren! Auf jeden Fall erstellen Sie einen Konstruktor:
 Konto(String Vorname, String Name, String kontonummer)
@@ -2772,31 +2752,6 @@
         assertEquals("-3/-4", s);
         punkte += 50;
         System.out.println("Test 3 erfolgreich: " + s);
-    }
-}</t>
-  </si>
-  <si>
-    <t>package de.goals.testing;
-import org.junit.Test;
-import static org.junit.Assert.*;
-public class BibVerwaltungTest {
-    @Test
-    public void testBerechneStrafgeldBuch() {
-        Buch buch = new Buch("Fussballfieber", "Manuel Neuer", 75);
-        buch.setAusleihdatum(new Datum(2020, 2, 1));
-        Datum heute = new Datum();
-        int tageUeberzogen = heute.calcDiffDays(buch.ausleihdatum) - 28;
-        double erwartetesStrafgeld = Math.max(0, tageUeberzogen) * 1.0;
-        assertEquals(erwartetesStrafgeld, buch.berechneStrafgeld(), 0.01);
-    }
-    @Test
-    public void testBerechneStrafgeldDVD() {
-        DVD dvd = new DVD("FussballfieberderFilm", "Manuel Neuer", 120);
-        dvd.setAusleihdatum(new Datum(2019, 2, 1));
-        Datum heute = new Datum();
-        int tageUeberzogen = heute.calcDiffDays(dvd.ausleihdatum) - 7;
-        double erwartetesStrafgeld = Math.max(0, tageUeberzogen) * 2.0;
-        assertEquals(erwartetesStrafgeld, dvd.berechneStrafgeld(), 0.01);
     }
 }</t>
   </si>
@@ -3262,18 +3217,112 @@
 }</t>
   </si>
   <si>
-    <t>Betrachten Sie das folgende UML-Diagramm:
-Bild von einem Klassendiagramm der Klasse Leser: Attribute LeserID (int und protected), Kontonr(int und private), Name(String und public). Methoden: private changeKontonr(nr: int), public getName(), private setName(name: String), protected getLeserID()
+    <t>package de.goals.testing;
+import org.junit.Test;
+import static org.junit.Assert.*;
+public class BibVerwaltungTest {
+    @Test
+    public void testBerechneStrafgeldBuch() {
+        Buch buch = new Buch("Fussballfieber", "Manuel Neuer", 75);
+        buch.setAusleihdatum(new Datum(2020, 2, 1));
+        Datum heute = new Datum();
+        int tageUeberzogen = heute.calcDiffDays(buch.Ausleihdatum) - 28;
+        double erwartetesStrafgeld = Math.max(0, tageUeberzogen) * 1.0;
+        assertEquals(erwartetesStrafgeld, buch.berechneStrafgeld(), 0.01);
+    }
+    @Test
+    public void testBerechneStrafgeldDVD() {
+        DVD dvd = new DVD("FussballfieberderFilm", "Manuel Neuer", 120);
+        dvd.setAusleihdatum(new Datum(2019, 2, 1));
+        Datum heute = new Datum();
+        int tageUeberzogen = heute.calcDiffDays(dvd.Ausleihdatum) - 7;
+        double erwartetesStrafgeld = Math.max(0, tageUeberzogen) * 2.0;
+        assertEquals(erwartetesStrafgeld, dvd.berechneStrafgeld(), 0.01);
+    }
+}</t>
+  </si>
+  <si>
+    <t>&lt;p&gt;Betrachten Sie das folgende Klassendiagramm:&lt;br /&gt;
+&lt;img src="/assets/taskImgs/Java_Bibliothek_Bib.svg" alt="image"&gt;
+&lt;br /&gt;
+a) Machen Sie sich mit den&amp;nbsp;Eigenschaften der  Klasse Datum vertraut, in dem Sie sich den Quelltext anschauen. Schauen Sie sich&amp;nbsp;die Eigenschaften der Klasse Calendar in der Java-API an.&lt;/p&gt;
+&lt;p&gt;b) Setzen Sie nun das oben stehende UML-Klassendiagramm in Java um, unter der&amp;nbsp;Verwendung der Klasse Datum. Implementieren Sie auch die Methoden der Klassen&amp;nbsp;Medium, Buch und DVD. Für die Berechnung des Strafgeldes bei &amp;Uuml;berziehung der&amp;nbsp;Leihfristen gelten folgende Bestimmungen:&lt;/p&gt;
+&lt;p&gt;- Bücher k&amp;ouml;nnen 4 Wochen ausgeliehen werden, bei &amp;Uuml;berziehung 1 EUR Strafgeld pro&amp;nbsp;angefangenen &amp;Uuml;berziehungstag.&lt;br /&gt;
+- DVDs k&amp;ouml;nnen 1 Woche ausgeliehen werden, bei &amp;Uuml;berziehung 2 EUR Strafgeld pro&amp;nbsp;angefangenen &amp;Uuml;berziehungstag&lt;/p&gt;
+&lt;p&gt;Für die Berechnung der Differenztage zwischen dem Ausleihdatum und Heute&amp;nbsp;implementieren Sie bitte die Methode calcDiffDays() der Klasse Datum. Nehmen Sie&amp;nbsp;dazu an, dass jeder Monat 30 Tage hat und das Jahr 365 Tage.&lt;/p&gt;
+&lt;p&gt;c) Schreiben Sie ein kleines Testprogramm (BibVerwaltung.java), das Objekte von den&amp;nbsp;beiden Medien Buch und DVD erzeugt.&lt;/p&gt;</t>
+  </si>
+  <si>
+    <t>Betrachten Sie das folgende Klassendiagramm:
+classDiagram
+    class Medium {
+        &lt;&lt;abstract&gt;&gt;
+        #Mediumtitel: String
+        #Ausleihdatum: Datum
+        #Medium(titel: String)
+        #getTitel() String
+        #berechneStrafgeld()* double (abstract)
+        #setAusleihdatum(leihdatum: Datum)
+    }
+    class Datum {
+        -Jahr: int
+        -Monat: int
+        -Tag: int
+        -Cal: Calendar
+        +Datum()
+        +Datum(jahr: int, monat: int, tag: int)
+        +getJahr() int
+        +getMonat() int
+        +getTag() int
+        +calcDiffDays(ausleih: Datum) int
+    }
+    class Buch {
+        -Buch_Autor: String
+        -Buch_Seiten: int
+        +Buch(titel: String, autor: String, seiten: int)
+        +berechneStrafgeld() double
+        +getAutor() String
+        +getSeiten() int
+    }
+    class DVD {
+        -DVD_Regisseur: String
+        -DVD_Laenge: int
+        +DVD(titel: String, regisseur: String, laenge: int)
+        +berechneStrafgeld() double
+        +getRegisseur() String
+        +getLaenge() int
+    }
+    Medium &lt;|-- Buch
+    Medium &lt;|-- DVD
+    Medium ..&gt; Datum : ausgeliehen am
+___ Ende Klassendiagramm
+a) Machen Sie sich mit den Eigenschaften der  Klasse Datum  vertraut, in dem Sie sich den Quelltext anschauen. Schauen Sie sich die Eigenschaften der Klasse Calendar in der Java-API an.
+b) Setzen Sie nun das oben stehende UML-Klassendiagramm in Java um, unter der Verwendung der Klasse Datum. Implementieren Sie auch die Methoden der Klassen Medium, Buch und DVD. Für die Berechnung des Strafgeldes bei Überziehung der Leihfristen gelten folgende Bestimmungen:
+- Bücher können 4 Wochen ausgeliehen werden, bei Überziehung 1 EUR Strafgeld pro angefangenen Überziehungstag.
+- DVDs können 1 Woche ausgeliehen werden, bei Überziehung 2 EUR Strafgeld pro angefangenen Überziehungstag
+Für die Berechnung der Differenztage zwischen dem Ausleihdatum und Heute implementieren Sie bitte die Methode calcDiffDays() der Klasse Datum. Nehmen Sie dazu an, dass jeder Monat 30 Tage hat und das Jahr 365 Tage.
+c) Schreiben Sie ein kleines Testprogramm (BibVerwaltung.java), das Objekte von den beiden Medien Buch und DVD erzeugt.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Betrachten Sie das folgende UML-Diagramm:
+classDiagram
+    class Leser {
+        #LeserID : int
+        -Kontonr : int
+        +Name : String
+        #changeKontonr(nr : int)
+        +getName() String
+        #setName(name : String)
+        #getLeserID() int
+    }
 Erstellen Sie zu diesem Klassendiagramm den entsprechenden Java-Code. Beachten Sie dabei vor allem die Sichtbarkeiten!
-Implementieren Sie einen Konstruktor der alle Attribute als Argument erhält! Implementieren Sie die Rümpfe der Methoden. 
-HINWEIS VOM 12.06: Verwenden Sie public oder protected Methoden anstelle von private. Ansonsten gibt es aktuell Probleme mit unseren automatischen Tests.</t>
+Implementieren Sie einen Konstruktor der alle Attribute als Argument erhält! Implementieren Sie die Rümpfe der Methoden. </t>
   </si>
   <si>
     <t>&lt;p&gt;Betrachten Sie das folgende UML-Diagramm:&lt;/p&gt;
-&lt;img src="/assets/taskImgs/UMLtoJava.png" alt="image"&gt;
+&lt;img src="/assets/taskImgs/UMLtoJava.svg" alt="image"&gt;
 &lt;br /&gt;Erstellen Sie zu diesem Klassendiagramm den entsprechenden Java-Code. Beachten Sie dabei vor allem die Sichtbarkeiten!&lt;/p&gt;
-&lt;p&gt;Implementieren Sie einen Konstruktor der alle Attribute als Argument erh&amp;auml;lt!&amp;nbsp;Implementieren Sie die R&amp;uuml;mpfe der Methoden.&amp;nbsp;&lt;/p&gt;
-&lt;p&gt;HINWEIS VOM 12.06: Verwenden Sie public oder protected Methoden anstelle von private. Ansonsten gibt es aktuell Probleme mit unseren automatischen Tests.&lt;/p&gt;</t>
+&lt;p&gt;Implementieren Sie einen Konstruktor der alle Attribute als Argument erh&amp;auml;lt!&amp;nbsp;Implementieren Sie die R&amp;uuml;mpfe der Methoden.&amp;nbsp;&lt;/p&gt;</t>
   </si>
 </sst>
 </file>
@@ -4059,13 +4108,13 @@
         <v>97</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="H6" s="10" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="I6" s="6" t="s">
         <v>9</v>
@@ -4084,7 +4133,7 @@
       </c>
       <c r="N6" s="23"/>
       <c r="R6" s="26" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
     </row>
     <row r="7" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4504,13 +4553,13 @@
         <v>118</v>
       </c>
       <c r="F17" s="10" t="s">
-        <v>318</v>
+        <v>352</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>324</v>
+        <v>350</v>
       </c>
       <c r="H17" s="10" t="s">
-        <v>319</v>
+        <v>351</v>
       </c>
       <c r="I17" s="10" t="s">
         <v>20</v>
@@ -4523,7 +4572,7 @@
       </c>
       <c r="L17" s="7"/>
       <c r="N17" s="21" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="R17" s="25"/>
     </row>
@@ -4699,7 +4748,7 @@
         <v>269</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="H22" s="14" t="s">
         <v>313</v>
@@ -4734,13 +4783,13 @@
         <v>126</v>
       </c>
       <c r="F23" s="10" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="G23" s="7" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="H23" s="21" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="I23" s="10" t="s">
         <v>36</v>
@@ -4753,7 +4802,7 @@
       </c>
       <c r="L23" s="7"/>
       <c r="N23" s="21" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="R23" s="25"/>
     </row>
@@ -4815,7 +4864,7 @@
         <v>353</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="H25" s="10" t="s">
         <v>354</v>
@@ -4850,13 +4899,13 @@
         <v>129</v>
       </c>
       <c r="F26" s="10" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="G26" s="7" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="H26" s="10" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
       <c r="I26" s="10" t="s">
         <v>41</v>
@@ -4869,7 +4918,7 @@
       </c>
       <c r="L26" s="7"/>
       <c r="N26" s="14" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="R26" s="25"/>
     </row>
@@ -4896,7 +4945,7 @@
         <v>229</v>
       </c>
       <c r="H27" s="10" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="I27" s="10" t="s">
         <v>46</v>
@@ -4928,13 +4977,13 @@
         <v>131</v>
       </c>
       <c r="F28" s="10" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="H28" s="10" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="I28" s="10" t="s">
         <v>48</v>
@@ -5018,7 +5067,7 @@
         <v>135</v>
       </c>
       <c r="G30" s="7" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="H30" s="10" t="s">
         <v>136</v>
@@ -5180,10 +5229,10 @@
         <v>201</v>
       </c>
       <c r="L33" s="7" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="M33" s="6" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="N33" s="14"/>
       <c r="P33" s="10" t="s">
@@ -5229,10 +5278,10 @@
         <v>201</v>
       </c>
       <c r="L34" s="7" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="M34" s="6" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="N34" s="14"/>
       <c r="P34" s="10" t="s">
@@ -5405,10 +5454,10 @@
         <v>158</v>
       </c>
       <c r="G38" s="7" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="H38" s="10" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="I38" s="6" t="s">
         <v>74</v>
@@ -5446,16 +5495,16 @@
         <v>288</v>
       </c>
       <c r="F39" s="10" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="G39" s="7" t="s">
         <v>231</v>
       </c>
       <c r="H39" s="10" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="I39" s="10" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="J39" s="9">
         <v>0</v>
@@ -5713,7 +5762,7 @@
         <v>18</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6019,7 +6068,7 @@
         <v>39</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6117,7 +6166,7 @@
         <v>46</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6408,10 +6457,10 @@
         <v>38</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
OFP CodingTask to markdown
</commit_message>
<xml_diff>
--- a/files/programming-tasks/programmieraufgaben_JACK_SOSE23_WORKSHOP_WISE2324.xlsx
+++ b/files/programming-tasks/programmieraufgaben_JACK_SOSE23_WORKSHOP_WISE2324.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\hefl\files\programming-tasks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63F2FA52-7EB1-4501-A216-5FA3AF71C1BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98CB397A-1CA3-46A1-B5B0-DFE4D1CC2426}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="870" yWindow="75" windowWidth="25875" windowHeight="20805" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-15" yWindow="90" windowWidth="25875" windowHeight="20805" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Aufgaben" sheetId="1" r:id="rId1"/>
@@ -341,19 +341,6 @@
 2. Sie brauchen das Ergebnis nicht zu formatieren oder zu runden!! </t>
   </si>
   <si>
-    <t>&lt;p&gt;Ein Kapital von 1000 Euro wird j&amp;auml;hrlich mit einem bestimmten Prozentsatz verzinst. Die rekursive&amp;nbsp;Funktion&amp;nbsp;&lt;code&gt;kapitalWert()&lt;/code&gt;&amp;nbsp;beschreibe den Kapitalwert nach n Jahren bei konstantem Zinssatz. Die Funktion gibt den Kapitalwert&amp;nbsp;(ohne Euro-Symbol oder EUR) zur&amp;uuml;ck.&amp;nbsp;&lt;br /&gt;
-&lt;br /&gt;
-&lt;strong&gt;Beispielrechnung:&lt;/strong&gt;&lt;br /&gt;
-&lt;em&gt;Startkapital: 1000.00 EUR und 5 % Zinsen&lt;br /&gt;
-Kapital nach dem 1. Jahr: 1000.00 + 0,05 *1000.00=1050.00&lt;br /&gt;
-Kapital nach dem 2. Jahr: 1050.00 + 0,05 *1050.00=1102.50&lt;br /&gt;
-...&lt;/em&gt;&lt;br /&gt;
-&lt;br /&gt;
-&lt;strong&gt;Hinweise: &lt;/strong&gt;&lt;br /&gt;
-1. Die Funktion kapitalWert sollte als Parameter den aktuellen Kapitalwert, Zinssatz und&amp;nbsp;Jahre haben!!&amp;nbsp;&lt;br /&gt;
-2. Sie brauchen das Ergebnis nicht zu formatieren oder zu runden!!&amp;nbsp;&lt;/p&gt;</t>
-  </si>
-  <si>
     <t>Python Buchhandlung</t>
   </si>
   <si>
@@ -365,42 +352,6 @@
 Schreiben Sie eine Funktion biblio(), die unter Benutzung von lambda und map, das als Ergebnis eine Liste mit Zweier-Tupeln zurückliefert. Dazu erhält die Funktion die eine Liste im o.a. Format als Argument in der Form 
 [["34587", "Learning Python, Mark Lutz", 4, 40.95], ["98762", "Programming Python, Mark Lutz", 5, 56.80], ["77226", "Head First Python, Paul Barry", 3, 32.95]]
 Die Funktion berechnet dann wie folgt: Jedes Tupel besteht aus der Bestellnummer und dem Produkt aus der Anzahl und dem Einzelpreis. Das Produkt soll jedoch um 10,- € erhöht werden, wenn der Bestellwert unter 100,00 € liegt. Die Funktion gibt dann die so errechnete Liste zurück. </t>
-  </si>
-  <si>
-    <t>&lt;p&gt;In einer Buchhandlung findet sich in einem Abrechnungsprogramm in Python eine&amp;nbsp;Liste mit Unterlisten mit folgendem Aufbau:&lt;/p&gt;
-&lt;table border="1" cellpadding="1" cellspacing="1" style="width:500px;"&gt;
-	&lt;thead&gt;
-		&lt;tr&gt;
-			&lt;th scope="col"&gt;Bestellnummer&lt;/th&gt;
-			&lt;th scope="col"&gt;Buchtitel und Autor&lt;/th&gt;
-			&lt;th scope="col"&gt;Anzahl&lt;/th&gt;
-			&lt;th scope="col"&gt;Einzelpreis&lt;/th&gt;
-		&lt;/tr&gt;
-	&lt;/thead&gt;
-	&lt;tbody&gt;
-		&lt;tr&gt;
-			&lt;td&gt;34587&lt;/td&gt;
-			&lt;td&gt;Learning Python, Mark Lutz&lt;/td&gt;
-			&lt;td&gt;4&lt;/td&gt;
-			&lt;td&gt;40.95&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td&gt;98762&lt;/td&gt;
-			&lt;td&gt;Programming Python, Mark Lutz&lt;/td&gt;
-			&lt;td&gt;5&lt;/td&gt;
-			&lt;td&gt;56.80&lt;/td&gt;
-		&lt;/tr&gt;
-		&lt;tr&gt;
-			&lt;td&gt;77226&lt;/td&gt;
-			&lt;td&gt;Head First Python, Paul Barry 3&lt;/td&gt;
-			&lt;td&gt;3&lt;/td&gt;
-			&lt;td&gt;32.00&lt;/td&gt;
-		&lt;/tr&gt;
-	&lt;/tbody&gt;
-&lt;/table&gt;
-&lt;p&gt;Schreiben Sie eine Funktion biblio(), die&amp;nbsp;unter Benutzung von lambda und map, das als Ergebnis&amp;nbsp;eine Liste mit Zweier-Tupeln zur&amp;uuml;ckliefert. Dazu erh&amp;auml;lt die Funktion die eine Liste im o.a. Format als Argument in der Form&amp;nbsp;&lt;br /&gt;
-[["34587", "Learning Python, Mark Lutz", 4, 40.95],&amp;nbsp;["98762", "Programming Python, Mark Lutz", 5, 56.80],&amp;nbsp;["77226", "Head First Python, Paul Barry", 3, 32.95]]&lt;/p&gt;
-&lt;p&gt;Die Funktion berechnet dann wie folgt:&amp;nbsp;Jedes Tupel besteht aus der Bestellnummer und&amp;nbsp;dem Produkt aus der Anzahl und dem Einzelpreis. Das Produkt soll jedoch um 10,- &amp;euro;&amp;nbsp;erh&amp;ouml;ht werden, wenn der Bestellwert unter 100,00 &amp;euro; liegt. Die Funktion gibt dann die so errechnete Liste zur&amp;uuml;ck.&amp;nbsp;&lt;/p&gt;</t>
   </si>
   <si>
     <t>Python Quersumme</t>
@@ -444,21 +395,6 @@
 </t>
   </si>
   <si>
-    <t>Erstellen Sie eine rekursive Funktion &lt;em&gt;summe&lt;/em&gt;, die zwei ganze Zahlen &lt;em&gt;m&lt;/em&gt; und &lt;em&gt;n&lt;/em&gt; als Argumente erh&amp;auml;lt und die Summe aller ganzen Zahlen zwischen &lt;em&gt;m&lt;/em&gt; und &lt;em&gt;n &lt;/em&gt;(einschlie&amp;szlig;lich) als Ergebnis liefert. Falls &lt;em&gt;m&lt;/em&gt; gr&amp;ouml;&amp;szlig;er als &lt;em&gt;n&lt;/em&gt; ist, soll das Ergebnis 0 sein.&lt;br /&gt;
-&lt;br /&gt;
-Beispiel:&lt;br /&gt;
-&lt;br /&gt;
-summe( 1, 3)&lt;br /&gt;
-6&amp;nbsp; &amp;nbsp;&lt;br /&gt;
-#Weil 1+2+3=6&lt;br /&gt;
-&lt;br /&gt;
-summe( 3, 3); &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp;&lt;br /&gt;
-3&lt;br /&gt;
-&lt;br /&gt;
-summe( 5, 3); &amp;nbsp; &amp;nbsp; &amp;nbsp; &amp;nbsp;&lt;br /&gt;
-0</t>
-  </si>
-  <si>
     <t>Euklidischer Algorithmus</t>
   </si>
   <si>
@@ -489,16 +425,6 @@
 Verwenden Sie exakt das vorgegebene Code-Gerüst und geben Sie exakt die o.a. Ausgaben an!</t>
   </si>
   <si>
-    <t>&lt;p&gt;Erg&amp;auml;nzen Sie ein gegebenes&amp;nbsp;Java-Programm (Alter.java) in dessen main-Methode eine Methode &lt;strong&gt;gibBezeichnung()&lt;/strong&gt; aufgerufen wird, die als Parameter einen int-Wert erh&amp;auml;lt der das Alter in Jahren beschreibt.&lt;/p&gt;
-&lt;p&gt;Die Methode &lt;strong&gt;gibBezeichnung()&lt;/strong&gt; sollen in Abh&amp;auml;ngigkeit des Parameters folgende Strings zur&amp;uuml;ckgeben:&lt;/p&gt;
-&lt;p&gt;&lt;i&gt;Alter in Jahren &lt;/i&gt;gr&amp;ouml;&amp;szlig;er 0 aber kleiner 18: "Du bist ja noch ein Kind!"&lt;/p&gt;
-&lt;p&gt;&lt;i&gt;Alter in Jahren &lt;/i&gt;mindestens 18 aber weniger als 67: "Du stehst mitten im Leben!"&lt;/p&gt;
-&lt;p&gt;&lt;i&gt;Alter in Jahren &lt;/i&gt;gr&amp;ouml;&amp;szlig;er gleich 67: "Als Rentner hat man es gut!"&lt;/p&gt;
-&lt;p&gt;Wenn keine der o.a. Bedingungen zutrifft (z.B. bei negativen Werten) soll der String "Mit Deinem Alter stimmt was nicht!" zur&amp;uuml;ckgegeben werden.&lt;/p&gt;
-&lt;p&gt;Verwenden Sie eine &lt;i&gt;if&lt;/i&gt;-Anweisung um die einzelnen Ausgaben in Abh&amp;auml;ngigkeit der Variable zu erzeugen. Achten Sie auf eine korrekte Angabe der Grenzen und testen Sie das Programm in dem Sie die Variable ver&amp;auml;ndern, neu kompilieren und die Ausgabe betrachten.&lt;/p&gt;
-&lt;p&gt;Verwenden Sie exakt das vorgegebene Code-Ger&amp;uuml;st und geben Sie &lt;b&gt;exakt &lt;/b&gt;die o.a. Ausgaben an!&lt;/p&gt;</t>
-  </si>
-  <si>
     <t>Java Bruchsumme</t>
   </si>
   <si>
@@ -511,11 +437,6 @@
     <t>Implementieren Sie die Methode max() der Klasse Starter im vorgegebenen Code-Gerüst (Starter.java). Die Methode max gibt die Größere der beiden natürlichen Zahlen a und b zurück. Wenn beide Zahlen gleich sind, wird dieser Wert zurückgegeben.
 Implementieren Sie nur die Methode max der Klasse Starter.
 Verwenden Sie also exakt das vorgegebene Code-Gerüst!</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Implementieren Sie die Methode &lt;i&gt;max()&amp;nbsp;&lt;/i&gt;der Klasse &lt;i&gt;Starter &lt;/i&gt;im vorgegebenen Code-Ger&amp;uuml;st (Starter.java). Die Methode &lt;i&gt;max &lt;/i&gt;gibt die Gr&amp;ouml;&amp;szlig;ere der beiden nat&amp;uuml;rlichen Zahlen &lt;i&gt;a &lt;/i&gt;und &lt;i&gt;b &lt;/i&gt;zur&amp;uuml;ck. Wenn beide Zahlen gleich sind, wird dieser Wert zur&amp;uuml;ckgegeben.&lt;/p&gt;
-&lt;p&gt;Implementieren Sie nur die Methode &lt;i&gt;max &lt;/i&gt;der Klasse &lt;i&gt;Starter&lt;/i&gt;.&lt;/p&gt;
-&lt;p&gt;&lt;strong&gt;Verwenden Sie also exakt das vorgegebene Code-Ger&amp;uuml;st!&lt;/strong&gt;&lt;/p&gt;</t>
   </si>
   <si>
     <t>Java Arrays und Schleifen</t>
@@ -534,19 +455,6 @@
 Hinweis: Schauen Sie sich die Java-API Informationen zu java.lang.Math an (https://docs.oracle.com/en/java/javase/18/). Da gibt es evtl. eine Methode die ihnen helfen kann!</t>
   </si>
   <si>
-    <t>&lt;p&gt;Nach einer alten Sage wurde der Erfinder des Schachspiels zum K&amp;ouml;nig gerufen, der ihn f&amp;uuml;r seine Erfindung belohnen wollte. Auf die Frage, was er sich w&amp;uuml;nsche, antwortete der Schachspieler, dass der K&amp;ouml;nig ihm auf das erste Feld des Schachbretts 1 Cent legen sollte, auf das zweite Feld 2 Cent, auf das dritte Feld 4 Cent, auf das vierte Feld wieder das Doppelte und so weiter.&lt;/p&gt;
-&lt;p&gt;Der K&amp;ouml;nig dachte: "Was f&amp;uuml;r ein Dummkopf! H&amp;auml;tte er sich doch Gold gew&amp;uuml;nscht und nicht nur Cent?".&lt;/p&gt;
-&lt;p&gt;Verwenden Sie das vorgegeben Code-Ger&amp;uuml;st Schach.java!&amp;nbsp;&lt;br /&gt;
-Vervollst&amp;auml;ndigen&amp;nbsp;Sie die&amp;nbsp;Methode &lt;em&gt;felder&lt;/em&gt;, mit deren Hilfe Sie das oben geschilderte Vorgehen simulieren k&amp;ouml;nnen.&amp;nbsp;&lt;/p&gt;
-&lt;pre&gt;
-public int felder(int cent)&lt;/pre&gt;
-&lt;p&gt;Der Methode &amp;uuml;bergeben Sie als Parameter die Zahl der erw&amp;uuml;nschten Cent, beispielsweise 1000, und die Methode gibt die Zahl der Felder zur&amp;uuml;ck, die der K&amp;ouml;nig mit Centst&amp;uuml;cken belegen muss, um die gew&amp;uuml;nscht Zahl zu erhalten. &lt;strong&gt;Verwenden Sie eine Schleife!&lt;/strong&gt;&lt;/p&gt;
-&lt;p&gt;F&amp;uuml;r eine gew&amp;uuml;nschte Zahl von 1.000 Centst&amp;uuml;cken sind 1 + 2 + 4 + 8 + 16 + 32 + 64 + 128 + 256 + 512 Centst&amp;uuml;cke&amp;nbsp;auf die Felder&amp;nbsp;zu legen, ben&amp;ouml;tigt werden also 10&amp;nbsp;Felder. Ein Schachbrett hat aber 8 x 8 = 64 Felder.&lt;br /&gt;
-&lt;br /&gt;
-Hinweis: Schauen Sie sich die Java-API Informationen zu java.lang.Math an (https://docs.oracle.com/en/java/javase/18/). Da gibt es evtl. eine Methode&amp;nbsp;die ihnen helfen kann!&lt;br /&gt;
-&amp;nbsp;&lt;/p&gt;</t>
-  </si>
-  <si>
     <t>Java Switch</t>
   </si>
   <si>
@@ -571,15 +479,6 @@
 C[3] = B[3]</t>
   </si>
   <si>
-    <t>&lt;p&gt;Legen Sie eine Java-Klasse &lt;em&gt;VektorWork&lt;/em&gt; an.&amp;nbsp;Schreiben Sie in dieser Klasse eine Methode &lt;em&gt;addVektor&lt;/em&gt;, die zwei int-Arrays (A und B) als Eingabe-Parameter&amp;nbsp;bekommt und als Ausgabe-Parameter ein neues int-Array C zurück gibt.&lt;/p&gt;
-&lt;p&gt;Die Methode f&amp;uuml;hrt&amp;nbsp;eine&amp;nbsp;Vektor-Addition aus ( C[0] = A[0] + B[0], C[1] = A[1] + B[1] usw. ) und gibt das Array C zur&amp;uuml;ck. Beachten Sie aber, dass die Methode Arrays unterschiedlicher Gr&amp;ouml;&amp;szlig;e beandelt, so dass auch A und B unterschiedlich gro&amp;szlig; sein k&amp;ouml;nnen.&amp;nbsp;Dazu soll&amp;nbsp;C wie folgt berechnet werden:&lt;br /&gt;
-Bsp.: Wenn A 2 Elemente besitzt und B 4 Elemente:&lt;/p&gt;
-&lt;p&gt;&lt;em&gt;C[0] = A[0] + B[0]&lt;br /&gt;
-C[1] = A[1] + B[1]&lt;br /&gt;
-C[2] = B[2]&lt;br /&gt;
-C[3] = B[3]&lt;/em&gt;&lt;/p&gt;</t>
-  </si>
-  <si>
     <t>Java_KFZ</t>
   </si>
   <si>
@@ -605,19 +504,6 @@
   </si>
   <si>
     <t>Schreiben sie ein Funktion, welche eine n x n Matrix A  als Liste von Listen erstellt, wobei der (i,j)-te Eintrag, A_{i,j}, gleich i+j ist. Verwenden sie hierfür zwei verschachtelte for-Schleifen.</t>
-  </si>
-  <si>
-    <t>&lt;p&gt; Schreiben Sie eine Funktion make_matrix, welche eine n x n Matrix A als Liste von Listen erstellt, wobei der (i, j)-te Eintrag, A&lt;sub&gt;i,j&lt;/sub&gt;, gleich i + j ist. Verwenden Sie hierfür zwei verschachtelte for-Schleifen.
- &lt;/p&gt;
-&lt;br&gt;
-Das Ergebnis für make_matrix(4) würde wie folgt aussehen:
-&lt;br&gt;
-&lt;table&gt;
-&lt;tr&gt;&lt;td&gt;0&lt;/td&gt;&lt;td&gt;1&lt;/td&gt;&lt;td&gt;2&lt;/td&gt;&lt;td&gt;3&lt;/td&gt;&lt;/tr&gt;
-&lt;tr&gt;&lt;td&gt;1&lt;/td&gt;&lt;td&gt;2&lt;/td&gt;&lt;td&gt;3&lt;/td&gt;&lt;td&gt;4&lt;/td&gt;&lt;/tr&gt;
-&lt;tr&gt;&lt;td&gt;2&lt;/td&gt;&lt;td&gt;3&lt;/td&gt;&lt;td&gt;4&lt;/td&gt;&lt;td&gt;5&lt;/td&gt;&lt;/tr&gt;
-&lt;tr&gt;&lt;td&gt;3&lt;/td&gt;&lt;td&gt;4&lt;/td&gt;&lt;td&gt;5&lt;/td&gt;&lt;td&gt;6&lt;/td&gt;&lt;/tr&gt;
-&lt;/table&gt;</t>
   </si>
   <si>
     <t>def make_matrix(n):
@@ -634,11 +520,6 @@
 &lt;/p&gt;
 &lt;br&gt;
 &lt;p&gt; Hinweis: Hierfür müssen Sie die Bibliothek "math" importieren und entsprechend nutzen.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;
-    Schreiben Sie eine Funktion "concatenate_functions", die als Eingabeargument zwei Funktionen "f1" und "f2" bekommt und als Rückgabe eine Funktion liefert, die f1(f2(x)) auswertet. Testen Sie Ihr Programm mit f1(x) = sin(x) und f2(x) = 2*pi*x. Hierfür müssen Sie die Bibliothek "math" importieren.
-  &lt;/p&gt;</t>
   </si>
   <si>
     <t>import math as m
@@ -655,11 +536,6 @@
     <t>Schreiben Sie eine Funktion namens potenz, die die Potenz von x hoch a rekursiv berechnet.</t>
   </si>
   <si>
-    <t>&lt;p&gt;
-    Schreiben Sie eine Funktion namens &lt;code&gt;potenz&lt;/code&gt;, die die Potenz von x hoch a rekursiv berechnet.
-  &lt;/p&gt;</t>
-  </si>
-  <si>
     <t>def potenz(x, a):
     if a==0:
         return 1
@@ -668,11 +544,6 @@
   </si>
   <si>
     <t>Schreiben Sie eine Funktion namens drehe_string, die einen String rekursiv umdreht.</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;
-    Schreiben Sie eine Funktion namens &lt;code&gt;drehe_string&lt;/code&gt;, die einen String rekursiv umdreht.
-  &lt;/p&gt;</t>
   </si>
   <si>
     <t>def drehe_string(s):
@@ -690,11 +561,6 @@
  werden, die die steuerfunktion auf ein Argument betrag-freibetrag anwendet.</t>
   </si>
   <si>
-    <t>&lt;p&gt;
-    Schreiben Sie eine Funktion namens &lt;code&gt;mehrwertsteuer&lt;/code&gt;, die 19% des gegebenen Betrags als Rückgabewert hat. Schreiben Sie dann eine Funktion namens &lt;code&gt;nutze_freibetrag&lt;/code&gt;, welche einen Freibetrag und eine Steuerfunktion als Eingabeparameter erhält. Innerhalb der Funktion &lt;code&gt;nutze_freibetrag&lt;/code&gt; soll eine neue Funktion definiert werden, die die Steuerfunktion auf ein Argument &lt;code&gt;(betrag - freibetrag)&lt;/code&gt; anwendet.
-  &lt;/p&gt;</t>
-  </si>
-  <si>
     <t>def mehrwertsteuer(betrag):
     return betrag*0.19
 def nutze_freibetrag(freibetrag, steuerfunktion):
@@ -711,11 +577,6 @@
     dass Listen veränderbare Variablen sind, die einen Befehl 'remove' zulassen.</t>
   </si>
   <si>
-    <t>&lt;p&gt;
-    Schreiben Sie eine Funktion höherer Ordnung namens &lt;code&gt;filter_liste&lt;/code&gt;, die eine Funktion mit boolschem Rückgabewert und eine Liste als Eingabe entgegennimmt. Sie ruft die Funktion auf jedem Element der Liste auf und entfernt diejenigen Elemente, für die die Funktion den Rückgabewert 'False' hat.
-  &lt;/p&gt;</t>
-  </si>
-  <si>
     <t>def filter_liste(funktion, liste):
     for element in list(liste):
         if not funktion(element):
@@ -730,11 +591,6 @@
     nächsten Element der Liste aufgerufen werden, bis kein Element mehr übrig ist.</t>
   </si>
   <si>
-    <t>&lt;p&gt;
-    Schreiben Sie eine Funktion höherer Ordnung namens &lt;code&gt;reduziere_liste&lt;/code&gt;, die eine Funktion mit zwei Eingabeargumenten sowie eine Liste entgegennimmt. &lt;br&gt;&lt;br&gt; Hat die Liste nur ein Element, wird dieses Element zurückgegeben. &lt;br&gt;&lt;br&gt; Für Listen mit mindestens zwei Elementen wird die Funktion auf den ersten beiden Elementen und dann iterativ immer auf dem Ergebnis und dem nächsten Element der Liste aufgerufen, bis kein Element mehr übrig ist.
-  &lt;/p&gt;</t>
-  </si>
-  <si>
     <t>def reduziere_liste(funktion, liste):
     result = liste[0]
     for i in range (1, len(liste)):
@@ -743,11 +599,6 @@
   </si>
   <si>
     <t>Schreiben Sie eine Funktion namens fib, die die n-te Zahl der Fibonacci-Folge rekursiv berechnet.</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;
-    Schreiben Sie eine Funktion namens &lt;code&gt;fib&lt;/code&gt;, die die n-te Zahl der Fibonacci-Folge rekursiv berechnet.
-  &lt;/p&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">def fib(n):
@@ -2027,15 +1878,6 @@
 Verwenden Sie eine Schleife!!!</t>
   </si>
   <si>
-    <t>&lt;p&gt;Schreiben Sie eine Java-Methode &lt;em&gt;bruchSumme()&lt;/em&gt;, die die Summe der folgenden Br&amp;uuml;che berechnet:&lt;/p&gt;
-&lt;p&gt;&lt;strong&gt;1 + 1/2 + 1/3 + 1/4 + 1/5 + ...&lt;/strong&gt;&lt;/p&gt;
-&lt;p&gt;F&amp;uuml;r n=3 w&amp;uuml;rden Sie zum Beispiel die Summe 1 + 1/2 + 1/3 = 1.8333333333333333 erhalten.&lt;br /&gt;
-&lt;br /&gt;
-Erstellen Sie eine Java-Klasse &lt;em&gt;Summenwert&lt;/em&gt; mit einer Methode &lt;em&gt;public double bruchSumme(int n)&lt;/em&gt;.&amp;nbsp;&lt;br /&gt;
-Verwenden Sie eine Schleife!!!&lt;br /&gt;
-&lt;br /&gt;</t>
-  </si>
-  <si>
     <t>Verwenden Sie das Code-Gerüst aus Java_GGT.java und implementieren Sie die Methode ggT().
 Die Methode ggT berechnet den größten gemeinsamen Teiler zweier natürlicher Zahlen a und b. Verwenden Sie dazu den folgenden Algorithmus:
 1. setze m=a und n=b
@@ -2045,18 +1887,6 @@
 5. a) falls r ungleich 0 mache weiter bei Schritt 2
     b) falls r gleich 0 dann ist m der ggT!
 Verwenden Sie exakt das vorgegebene Code-Gerüst!</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Verwenden Sie das Code-Ger&amp;uuml;st aus Java_GGT.java und implementieren Sie die Methode ggT().&lt;/p&gt;
-&lt;p&gt;Die Methode ggT berechnet den gr&amp;ouml;&amp;szlig;ten gemeinsamen Teiler zweier nat&amp;uuml;rlicher Zahlen a und b. Verwenden Sie dazu den folgenden Algorithmus:&lt;br /&gt;
-&lt;br /&gt;
-1. setze m=a und n=b&lt;br /&gt;
-2. falls m kleiner als n, dann vertausche m und n&lt;br /&gt;
-3. setze r = m-n&lt;br /&gt;
-4. setze m=n und n=r&lt;br /&gt;
-5. a) falls r ungleich 0 mache weiter bei Schritt 2&lt;br /&gt;
-&amp;nbsp;&amp;nbsp; &amp;nbsp;b) falls r gleich 0 dann ist m der ggT!&lt;/p&gt;
-&lt;p&gt;Verwenden Sie exakt das vorgegebene Code-Ger&amp;uuml;st!&lt;/p&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">Modellieren Sie Kraftfahrzeuge (KFZ) als Java-Klasse nach folgenden Festlegungen:
@@ -2120,40 +1950,10 @@
     Implementieren sie dann die Funktion sieb() mit Hilfe der Funktion vielfaches().</t>
   </si>
   <si>
-    <t>Das &lt;strong&gt;Sieb des Erathostenes&lt;/strong&gt; ist ein Algorithmus der eine Liste alle Primzahlen von &lt;em&gt;2&lt;/em&gt; bis zu einer gegebenen Zahl &lt;em&gt;n&lt;/em&gt; berechnet (siehe u.a.&amp;nbsp;&lt;em&gt;https://de.wikipedia.org/wiki/Sieb_des_Eratosthenes&lt;/em&gt;).&amp;nbsp;&lt;br /&gt;
-&lt;br /&gt;
-Implementieren Sie den Algorithmus dazu in einer Funktion &lt;em&gt;sieb()&lt;/em&gt;. Die Funktion erh&amp;auml;lt als Parameter den Wert n der angibt bis zu welcher Zahl die Primzahlen berechnet werden sollen. Die Funktion gibt die Liste mit allen Primzahlen von 2 bis n zur&amp;uuml;ck!&lt;br /&gt;
-&lt;br /&gt;
-Gehen Sie dazu wie folgt vor:
-&lt;ol&gt;
-	&lt;li&gt;Der Algorithmus berechnet jeweils die Vielfachen von 2, 3, 5 und 7 aus der gegebenen Liste und entfernt diese. Schreiben Sie deshalb zuerst eine Funktion vielfach(). Die Funktion erh&amp;auml;lt als Parameter die Zahl zu denen die Vielfachen entfernt werden sollen. Dazu die Liste auf die Operation durchgef&amp;uuml;hrt wird.&lt;br /&gt;
-	&lt;em&gt;Bsp:: vielfach(2, liste)&amp;nbsp;&lt;br /&gt;
-	Entfernt alle Vielfachen von 2 aus liste&lt;/em&gt;&lt;/li&gt;
-	&lt;li&gt;Implementieren sie dann die Funktion &lt;em&gt;sieb()&lt;/em&gt; mit Hilfe der Funktion &lt;em&gt;vielfaches()&lt;/em&gt;.&lt;/li&gt;
-&lt;/ol&gt;</t>
-  </si>
-  <si>
-    <t>Schreiben Sie &amp;nbsp;eine rekursive Funktion&amp;nbsp;&lt;code&gt;querSum(n)&lt;/code&gt;, die eine positive Ganzzahl&amp;nbsp;&lt;code&gt;n&lt;/code&gt;&amp;nbsp;als Parameter erh&amp;auml;lt und ihre Quersumme ausgibt.&lt;br /&gt;
-Hinweis:&amp;nbsp;Bsp.:&lt;br /&gt;
-&amp;gt;&amp;gt;&amp;gt;&amp;nbsp;&lt;code&gt;querSum(174)&lt;/code&gt;&amp;nbsp;&lt;br /&gt;
-&amp;gt;&amp;gt;&amp;gt;&amp;nbsp;12&lt;br /&gt;
-Weil&amp;nbsp;1+7+4=12 ist.&amp;nbsp;</t>
-  </si>
-  <si>
     <t>concatenate_functions</t>
   </si>
   <si>
     <t xml:space="preserve"> lambda x: math.sin(x),  lambda x: 2 * math.pi * x</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  &lt;h1&gt;Fibonacci-Folge Index Finder&lt;/h1&gt;
-        &lt;p&gt;Schreiben Sie eine rekursive Funktion &lt;code&gt;fib_index()&lt;/code&gt;, die den Index einer Zahl in der &lt;a href="https://de.wikipedia.org/wiki/Fibonacci-Folge" target="_blank"&gt;Fibonacci-Folge&lt;/a&gt; zurückgibt, wenn die Zahl ein Element dieser Folge ist, und &lt;code&gt;-1&lt;/code&gt; zurückgibt, wenn die Zahl nicht darin enthalten ist.&lt;/p&gt;
-        &lt;p&gt;&lt;strong&gt;Beispiel:&lt;/strong&gt;&lt;/p&gt;
-        &lt;pre&gt;&lt;code&gt;&amp;gt;&amp;gt;&amp;gt; fib_index(13)
-&amp;gt;&amp;gt;&amp;gt; 7&lt;/code&gt;&lt;/pre&gt;
-        &lt;p&gt;In der Fibonacci-Folge ist die &lt;code&gt;13&lt;/code&gt; an der &lt;code&gt;7.&lt;/code&gt; Position:
-        &lt;code&gt;0, 1, 1, 2, 3, 5, 8, 13, 21, ...&lt;/code&gt;&lt;/p&gt;
-        &lt;p&gt;&lt;strong&gt;Tipp:&lt;/strong&gt; In den Übungen haben Sie ja bereits eine Funktion zur Bestimmung der Fibonacci Folge geschrieben, die sie jetzt wiederverwenden können!&lt;/p&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">
@@ -2209,18 +2009,6 @@
 Verwenden Sie exakt das vorgegebene Code-Gerüst!</t>
   </si>
   <si>
-    <t>&lt;p&gt;Betrachten Sie den Quellcode der Datei &lt;strong&gt;ArrayWork.java&lt;/strong&gt;.&lt;/p&gt;
-&lt;p&gt;Das Programm ArrayWork.java soll verschiedene Operationen auf ein Array mit&amp;nbsp;double-Werten realisieren. Das Array ist bereits vorgegeben (double werte[]) und die&amp;nbsp;entsprechende Operation wird per Parameter als int-Wert angegeben (int arg).&lt;/p&gt;
-&lt;p&gt;Das Array und der Parameter werden einer Funktion ArrayFunc übergeben in der die&amp;nbsp;folgenden Funktionen implementiert werden sollen:&lt;/p&gt;
-&lt;p&gt;- func=1: Gib den kleinsten Wert aus dem Array zurück&lt;br /&gt;
-- func=2: Gib den gr&amp;ouml;&amp;szlig;ten Wert aus dem Array zurück&lt;br /&gt;
-- func=3: Gib den arithmetischen Mittelwert aus dem Array zurück&lt;br /&gt;
-- func=4: Addiere alle Elemente des Arrays, addiere 19 % MwSt. und gib das Ergebnis&amp;nbsp;zurück.&lt;br /&gt;
-- Für alle anderen Werte von func soll 0 zurückgegeben werden.&lt;/p&gt;
-&lt;p&gt;Implementieren Sie die gewünschte Funktionalit&amp;auml;t unter der Verwendung von Schleifen und&amp;nbsp;ggf. weiteren Funktionen.&lt;/p&gt;
-&lt;p&gt;Verwenden Sie exakt das vorgegebene Code-Gerüst!&lt;/p&gt;</t>
-  </si>
-  <si>
     <t>Vervollständigen Sie die Methode checkModulo() die als Parameter zwei int-Werte erhält, durch die Umsetzung der folgenden Bedingungen:
 Es soll zunächst der Rest der Division von i durch j berechnet werden (modulo). Implementieren Sie nun eine switch-Anweisung, die unterscheidet ob die folgenden Bedingungen erfüllt sind:
 · der Rest ist null. ("Der Rest ist null")
@@ -2228,15 +2016,6 @@
 · oder Rest ist ungerade (aber keine einstellige Primzahl) ("Der Rest ist ungerade")
 · keine der Bedingungen trifft zu. ("Keine der Aussagen trifft zu")
 In allen Fällen soll der jeweils angegebene Text (exakt diese Text!) von der Methode checkModulo urückgegeben werden. Nutzen Sie daher insbesondere die break-Anweisung!!! Verwenden Sie exakt das vorgegebene Code-Gerüst!</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Vervollständigen Sie die Methode checkModulo() die als Parameter zwei int-Werte erhält, durch die Umsetzung der folgenden Bedingungen:&lt;/p&gt;
-&lt;p&gt;Es soll zun&amp;auml;chst der Rest der Division von i durch j berechnet werden (modulo).&amp;nbsp;Implementieren Sie nun eine switch-Anweisung, die unterscheidet ob die folgenden&amp;nbsp;Bedingungen erfüllt sind:&lt;/p&gt;
-&lt;p&gt;&amp;middot; der Rest ist null. ("Der Rest ist null")&lt;br /&gt;
-&amp;middot; der Rest ist eine einstellige Primzahl ("Der Rest ist eine einstellige&amp;nbsp;Primzahl")&lt;br /&gt;
-&amp;middot; oder Rest ist ungerade (aber keine einstellige Primzahl) ("Der Rest ist ungerade")&lt;br /&gt;
-&amp;middot; keine der Bedingungen trifft zu. ("Keine der Aussagen trifft zu")&lt;/p&gt;
-&lt;p&gt;In allen F&amp;auml;llen soll der jeweils angegebene Text (exakt diese Text!) von der Methode checkModulo ur&amp;uuml;ckgegeben werden. Nutzen Sie daher insbesondere die break-Anweisung!!!&amp;nbsp;Verwenden Sie exakt das vorgegebene Code-Gerüst!&lt;/p&gt;</t>
   </si>
   <si>
     <t>package de.goals.testing; // nicht entfernen
@@ -2347,19 +2126,6 @@
         System.out.println("Summe für n=15: " + summenwert.bruchSumme(15));
     }
 }</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-&lt;p&gt;Vervollst&amp;auml;ndigen Sie die Methode &lt;i&gt;berechneRabatt() &lt;/i&gt;des Java-Programms &lt;b&gt;&lt;i&gt;Discount.java&lt;/i&gt;&lt;/b&gt;, das als Argument einen Geldbertrag erh&amp;auml;lt. Die Methode &lt;i&gt;berechneRabatt() &lt;/i&gt;erh&amp;auml;lt als Parameter einen Euro-Wert.&lt;/p&gt;
-&lt;p&gt;Falls der Betrag gr&amp;ouml;&amp;szlig;er als 1000 EUR ist, soll ein Rabatt von 8 Prozent gew&amp;auml;hrt werden. In diesem Falle soll die Methode den String "Betrag mit Rabatt:&amp;nbsp;" zur&amp;uuml;ckgeben und anschlie&amp;szlig;end den zu zahlenden Betrag (siehe Beispiele unten). Falls der Betrag kleiner oder gleich 1000 EUR ist, soll nur der Betrag zur&amp;uuml;ckgegeben werden.&lt;/p&gt;
-&lt;p&gt;Die eigentliche Ausgabe erfolgt dann im main-Part.&lt;/p&gt;
-&lt;p&gt;&lt;b&gt;Bsp. 1: &lt;/b&gt;&lt;/p&gt;
-&lt;p&gt;java Discount 1234.45&lt;/p&gt;
-&lt;p&gt;Betrag mit Rabattt:&amp;nbsp;1135.69&lt;/p&gt;
-&lt;p&gt;---------&lt;/p&gt;
-&lt;p&gt;&lt;b&gt;Bsp.: 2: &lt;/b&gt;&lt;/p&gt;
-&lt;p&gt;java Discount 999&lt;/p&gt;
-&lt;p&gt;Zu zahlender Betrag: 999.00&lt;/p&gt;</t>
   </si>
   <si>
     <t>package de.goals.testing;
@@ -2399,28 +2165,6 @@
 personal[1]=new Professor(121.40);
 personal[2]=new Mitarbeiter(40, 15);
 Berechnen Sie in einer for-Schleife die Summe der Einkommen der drei Angestellten und geben Sie die Summe in der Konsole aus!</t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Die folgende Aufgabe soll einer Universit&amp;auml;tsverwaltung&amp;nbsp;helfen die Geh&amp;auml;lter von Professoren und Mitarbeiter zu berechnen.&amp;nbsp;&lt;/p&gt;
-&lt;div&gt;a)&amp;nbsp;Erstellen Sie eine Java-Klasse &lt;em&gt;Angestellter&lt;/em&gt;, die als Attribute&lt;/div&gt;
-&lt;p style="margin-left: 40px;"&gt;&lt;em&gt;double stdProMonat&lt;/em&gt; und&lt;br /&gt;
-&lt;em&gt;double geldProStunde&lt;/em&gt;&lt;/p&gt;
-&lt;p style="margin-left: 40px;"&gt;und als Methode &lt;em&gt;public double berechneMonatseinkommen() &lt;/em&gt;besitzt.&lt;br /&gt;
-Die Methode &lt;em&gt;berechneMonatseinkommen()&lt;/em&gt; berechnet das Einkommen eines&amp;nbsp;Angestellten pro Monat und gibt dieses dann zurück.&lt;/p&gt;
-&lt;p style="margin-left: 40px;"&gt;Au&amp;szlig;erdem soll die Klasse &lt;em&gt;Angestellter&lt;/em&gt; zwei Konstruktoren besitzen:&lt;/p&gt;
-&lt;p style="margin-left: 40px;"&gt;&lt;em&gt;public Angestellter( double arbeitstdProMonat, double&amp;nbsp;gehaltProStunde&amp;nbsp;)&lt;br /&gt;
-public Angestellter()&lt;/em&gt;&lt;/p&gt;
-&lt;p&gt;b) Erstellen Sie nun eine Klasse &lt;em&gt;Professor&lt;/em&gt;, die von der Klasse &lt;em&gt;Angestellter &lt;/em&gt;erbt.&lt;/p&gt;
-&lt;p style="margin-left: 40px;"&gt;Ein Professor hat immer eine feste Arbeitszeit von 160 Stunden im Monat.&lt;br /&gt;
-Implementieren Sie den Konstruktor der Klasse &lt;em&gt;Professor.&lt;/em&gt; Falls n&amp;ouml;tig, überschreiben&amp;nbsp;Sie Methoden der Basisklasse &lt;em&gt;Angestellter &lt;/em&gt;und geben Sie die neue Implementierung&amp;nbsp;an.&lt;/p&gt;
-&lt;p&gt;c) Erstellen Sie nun eine Klasse &lt;em&gt;Mitarbeiter&lt;/em&gt;, die von der Klasse &lt;em&gt;Angestellter&lt;/em&gt; erbt.&lt;/p&gt;
-&lt;p style="margin-left: 40px;"&gt;Ein Mitarbeiter bekommt zus&amp;auml;tzlich zum jeweiligen Stundenlohn jeden Monat einen&amp;nbsp;Bonus von 500 EUR. Implementieren Sie den Konstruktor der Klasse &lt;em&gt;Mitarbeiter&lt;/em&gt;.&amp;nbsp;Falls n&amp;ouml;tig, überschreiben Sie Methoden der Basisklasse &lt;em&gt;Angestellter &lt;/em&gt;und geben Sie&amp;nbsp;die neue Implementierung an.&lt;/p&gt;
-&lt;p&gt;d) Erstellen Sie nun eine Klasse &lt;em&gt;Uni&lt;/em&gt; mit einer main()-Methode.&lt;/p&gt;
-&lt;p style="margin-left: 40px;"&gt;Erzeugen Sie ein Array von Angestellten personal mit 3 Elementen:&lt;/p&gt;
-&lt;p style="margin-left: 40px;"&gt;&lt;em&gt;personal[0]=new Angestellter(22,11.5);&lt;br /&gt;
-personal[1]=new Professor(121.40);&lt;br /&gt;
-personal[2]=new Mitarbeiter(40, 15);&lt;/em&gt;&lt;/p&gt;
-&lt;p style="margin-left: 40px;"&gt;Berechnen Sie in einer for-Schleife die Summe der Einkommen der drei Angestellten&amp;nbsp;und geben Sie die Summe in der Konsole aus!&lt;/p&gt;</t>
   </si>
   <si>
     <t>package de.goals.testing; // nicht entfernen 
@@ -2526,60 +2270,6 @@
 }</t>
   </si>
   <si>
-    <t>&lt;p&gt;Implementieren Sie den euklidischen Algorithmus zur Berechnung des "gr&amp;ouml;&amp;szlig;ten-gemeinsammen Teilers" (ggT) &lt;strong&gt;rekursiv &lt;/strong&gt;in einer Funktion ggT()&lt;/p&gt;
-&lt;p&gt;Der Euklidische Algorithmus zur Berechnung des gr&amp;ouml;&amp;szlig;ten gemeinsamen Teilers zweier positiver ganzer Zahlen a und b (ggT(a,b)) ist wie folgt rekursiv definiert:&lt;/p&gt;
-&lt;ul&gt;
-	&lt;li&gt;&lt;em&gt;ggT(a,b) = a, falls a = b&lt;/em&gt;&lt;/li&gt;
-	&lt;li&gt;&lt;em&gt;ggT(a,b) = ggT(a - b, b), falls a &gt; b&amp;nbsp;&lt;/em&gt;&lt;/li&gt;
-	&lt;li&gt;&lt;em&gt;ggT(a,b) = ggT(a, b - a), falls b &gt; a&lt;/em&gt;&lt;/li&gt;
-&lt;/ul&gt;
-&lt;p&gt;&lt;br /&gt;
-&amp;nbsp;&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>&lt;div&gt;
-  &lt;p&gt;&lt;strong&gt;Modellieren Sie Kraftfahrzeuge (KFZ) als Java-Klasse nach folgenden Festlegungen:&lt;/strong&gt;&lt;/p&gt;
-  &lt;p&gt;Zu einem KFZ werden Kennzeichen, Kilometerstand (int), Tankvolumen in Liter (float), Kraftstoffverbrauch in Liter auf 100 km (float) und Kraftstoffmenge (float) erfasst.&lt;/p&gt;
-  &lt;p&gt;Die aktuellen Werte der Attribute Kennzeichen, Kilometerstand und Tankvolumen und aktuelle Tankinhalt in Litern können mittels get-Methoden abgefragt werden. (getKennzeichen(), getKMstand(), getTankvolumen(), getTankinhalt())&lt;/p&gt;
-  &lt;p&gt;Ein KFZ soll sowohl ohne Werte als auch mit den in 1. aufgeführten Attributen erzeugt werden können.&lt;/p&gt;
-  &lt;p&gt;Ein KFZ kann tanken(Menge) und fahren(Strecke).&lt;/p&gt;
-  &lt;p&gt;tanken() erhöht die Kraftstoffmenge im Tank. Sollte die Summe Menge + aktuelle Tankmenge größer sein als das Tankvolumen, so wird die Kraftstoffmenge auf das Tankvolumen begrenzt.&lt;/p&gt;
-  &lt;p&gt;fahren() erhält die Strecke als Parameter und errechnet dann ob der aktuelle Tankinhalt ausreicht die Strecke zu fahren. Wenn das nicht der Fall ist, gibt die Methode false zurück. Wenn es möglich ist, dann berechnet die Methode den Kraftstoffverbrauch für die gefahrenen Kilometer und zieht die Liter von der aktuellen Kraftstoffmenge ab. Außerdem wird der Kilometerstand entsprechend erhöht. Die Methode gibt dann true zurück.&lt;/p&gt;
-  &lt;p&gt;Implementieren Sie die Klasse KFZ in Java. Selbstverständlich können Sie auch noch weitere Methoden implementieren.&lt;/p&gt;
-  &lt;p&gt;Implementieren Sie eine neue Test-Klasse AppAuto, in der Autos erzeugt werden und diese fahren bzw. tanken lässt.&lt;/p&gt;
-&lt;/div&gt;</t>
-  </si>
-  <si>
-    <t>&lt;div&gt;
-    &lt;p&gt;Die Klasse Punkt soll einen Punkt in einem zweidimensionalen Koordinatensystem repräsentieren. Ein Punkt besteht aus folgenden Attribute:&lt;/p&gt;
-    &lt;p&gt;&lt;strong&gt;X-Koordinate&lt;br&gt;Y-Koordinate&lt;/strong&gt;&lt;/p&gt;
-    &lt;p&gt;Ein Punkt wird in der Klasse über einen Konstruktor erzeugt, der als Parameter die x- und y-Koordinate erhält. Der Standard-Konstruktor erzeugt einen Punkt im Ursprung (0,0).&lt;/p&gt;
-    &lt;p&gt;Die Klasse Punkt soll folgende Methoden erhalten:&lt;/p&gt;
-    &lt;p&gt;&lt;strong&gt;getX()&lt;/strong&gt; und &lt;strong&gt;getY()&lt;/strong&gt;: Gibt die x- bzw. y-Koordinate des Punktes als int-Wert zurück.&lt;br&gt;&lt;strong&gt;toString()&lt;/strong&gt;: Gibt einen String in der Form x/y zurück.&lt;br&gt;&lt;strong&gt;spiegelX()&lt;/strong&gt;: Spiegelung des Punktes an der X-Achse (Ergebnis soll ein neues Objekt der Klasse Punkt sein, das zurückgegeben wird!)&lt;br&gt;&lt;strong&gt;spiegelY()&lt;/strong&gt;: Spiegelung des Punktes an der Y-Achse (Ergebnis soll ein neues Objekt der Klasse Punkt sein, das zurückgegeben wird!)&lt;br&gt;&lt;strong&gt;spiegelUrsprung()&lt;/strong&gt;: Spiegelung des Punktes am Ursprung (Ergebnis soll ein neues Objekt der Klasse Punkt sein, das zurückgegeben wird!)&lt;br&gt;&lt;strong&gt;diffUrsprung()&lt;/strong&gt;: Abstand des Punktes zum Ursprung. Gibt den Abstand in der Form x/y als String zurück.&lt;br&gt;&lt;strong&gt;diffPunkt()&lt;/strong&gt;: Abstand des Punktes zu einem anderen Punkt. Gibt den Abstand in der Form x/y als String zurück.&lt;/p&gt;
-    &lt;p&gt;Entwerfen Sie eine geeignete Klasse Punkt und implementieren Sie die Klasse Punkt in Java. Testen Sie die Klasse Punkt mit einer Main-Klasse AppPunkt.&lt;/p&gt;
-&lt;/div&gt;
-&lt;h2&gt;Umsetzung in Java&lt;/h2&gt;
-&lt;p&gt;Entwerfen Sie eine geeignete &lt;code&gt;Klasse Punkt&lt;/code&gt; und implementieren Sie die &lt;code&gt;Klasse Punkt&lt;/code&gt; in Java. Testen Sie die &lt;code&gt;Klasse Punkt&lt;/code&gt; mit einer Main-Klasse &lt;code&gt;AppPunkt&lt;/code&gt;.&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>&lt;div&gt;
-    &lt;p&gt;&lt;strong&gt;Implementieren Sie eine Klasse Radio mit folgenden Attributen:&lt;/strong&gt;&lt;/p&gt;
-    &lt;p&gt;eingeschaltet, wenn ein Radio an oder aus ist.&lt;br&gt;
-    lautstaerke, wie laut spielt das Radio Musik? (Die Lautstärke soll nur im Bereich von 0 bis 10 liegen.)&lt;br&gt;
-    frequenz, die die Frequenz des gewählten Senders angibt (Erlaubter Frequenzbereich ist zwischen 85.0 und 110.0).&lt;/p&gt;
-    &lt;p&gt;&lt;strong&gt;Implementieren Sie zu der Klasse zwei Konstruktoren der Art:&lt;/strong&gt;&lt;/p&gt;
-    &lt;p&gt;Radio()&lt;br&gt;
-    Radio(boolean istAn, int lautstaerke, double frequenz)&lt;/p&gt;
-    &lt;p&gt;Der Standardkonstruktor schaltet das Radio an mit Lautstärke 5 und der Frequenz 99.9.&lt;/p&gt;
-    &lt;p&gt;&lt;strong&gt;Zu der Klasse Radio sollen folgende Methoden implementiert werden:&lt;/strong&gt;&lt;/p&gt;
-    &lt;p&gt;lauter(), leiser(): Diese Methoden sollen die Lautstärke in dem im Parameter angegebenen Maß ändern (nur möglich im Zustand an).&lt;br&gt;
-    an(), aus(): Diese Methoden sollen den Zustand des Attributs eingeschaltet ändern.&lt;br&gt;
-    public String toString() Diese Methode soll Informationen über den internen Zustand als String zurückgeben. Es soll eine Zeichenkette der Form "Radio an: Freq=98.4, Laut=2" zurückgeben werden. (Achten Sie bitte genau auf die Form der Beispielausgabe!! Weicht die Form ab so kann Tutor Kai das Ergebnis nicht genau prüfen.&lt;/p&gt;
-    &lt;p&gt;waehleSender(double frequenz) Diese Methode soll eine Frequenz speichern. Ist die gewählte Frequenz außerhalb des erlaubten Frequenzbereichs, so soll die Frequenz 99.9 gewählt werden.&lt;/p&gt;
-    &lt;p&gt;&lt;strong&gt;Schreiben Sie eine neue Test-Klasse AppRadio die in ihrem main()-Part ein Objekt der Klasse Radio erzeugt und in der Sie dann die Methoden testweise aufrufen können.&lt;/strong&gt;&lt;/p&gt;
-&lt;/div&gt;</t>
-  </si>
-  <si>
     <t>BubbleSortTest.java</t>
   </si>
   <si>
@@ -2632,19 +2322,6 @@
     double getKontostand(): Abfrage des Kontostandes.
     setLimit(Limit): setzte das Limit auf einen neuen Betrag. 
 Erstellen Sie eine Test-Klasse AppBank in der die Konten der Kunden verwaltet werden. </t>
-  </si>
-  <si>
-    <t>&lt;div&gt;
-  &lt;p&gt;&lt;strong&gt;Schreiben Sie eine Klasse Konto, die ein Bankkonto realisiert.&lt;/strong&gt; Attribute für das Bankkonto sind der Name und Vorname des Kontoinhabers, die Kontonummer (IBAN), der Kontostand, sowie ein Limit, bis zu dem das Konto überzogen werden darf.&lt;/p&gt;
-  &lt;p&gt;&lt;strong&gt;Erstellen Sie einen oder mehrere geeignete Konstruktoren!&lt;/strong&gt; Auf jeden Fall erstellen Sie einen Konstruktor:&lt;br&gt;Konto(String Vorname, String Name, String kontonummer)&lt;br&gt;Dieser Konstruktor dient dazu einen Neukunden zu initialisieren.&lt;/p&gt;
-  &lt;p&gt;&lt;strong&gt;Erstellen Sie Methoden für folgende Operationen:&lt;/strong&gt;&lt;/p&gt;
-  &lt;p&gt;&lt;em&gt;String toString():&lt;/em&gt; Rückgabe aller Kontodaten eines Kunden in der Form (z.B.):&lt;br&gt;Kunde: Sarah Müller, Konto: DE87123456782435465711, Stand: 123.45, Limit: 1000.00&lt;/p&gt;
-  &lt;p&gt;&lt;em&gt;einzahlen(Betrag):&lt;/em&gt; Einzahlung eines Betrages&lt;/p&gt;
-  &lt;p&gt;&lt;em&gt;auszahlen():&lt;/em&gt; Auszahlung eines Betrages mit Überprüfung ob ggf. Limit überschritten wurde. In dem Falle wird dann nur die Summe bis zum Limit ausgezahlt.&lt;/p&gt;
-  &lt;p&gt;&lt;em&gt;double getKontostand():&lt;/em&gt; Abfrage des Kontostandes.&lt;/p&gt;
-  &lt;p&gt;&lt;em&gt;setLimit(Limit):&lt;/em&gt; setzte das Limit auf einen neuen Betrag.&lt;/p&gt;
-  &lt;p&gt;&lt;strong&gt;Erstellen Sie eine Test-Klasse AppBank in der die Konten der Kunden verwaltet werden.&lt;/strong&gt;&lt;/p&gt;
-&lt;/div&gt;</t>
   </si>
   <si>
     <t>Syntaxfehler: JA, Tests: NEIN
@@ -2752,29 +2429,6 @@
     Geben Sie die Daten der in der ArrayList gespeicherten Objekten aus, in dem Sie die entsprechenden Methoden aufrufen. </t>
   </si>
   <si>
-    <t xml:space="preserve"> &lt;p&gt;Im Rahmen einer Softwareentwicklung für die einheitliche Verwaltung von Flugzeugen wurde die Klasse &lt;em&gt;Flugzeug&lt;/em&gt; entwickelt (siehe Flugzeug.java).&lt;/p&gt;
-    &lt;p&gt;Ausgehend von dieser Klasse sind zwei Klassen &lt;em&gt;Verkehrsflugzeug&lt;/em&gt; und &lt;em&gt;Doppeldecker&lt;/em&gt; zu erzeugen. Diese sollen folgende Spezifikationen erfüllen:&lt;/p&gt;
-    &lt;p&gt;Klasse &lt;em&gt;Verkehrsflugzeug&lt;/em&gt;:&lt;/p&gt;
-    &lt;p&gt;- Ein Verkehrsflugzeug ist ein Flugzeug, das genau ein Flügelpaar sowie eine zusätzliche Variable für die Anzahl der Passagiere hat.&lt;/p&gt;
-    &lt;p&gt;- Ein Verkehrsflugzeug fliegt keine Loopings. Stellen Sie deshalb sicher, dass die Methode &lt;em&gt;getLooping&lt;/em&gt; immer false zurückgibt, auch in allen Unterklassen von Verkehrsflugzeug.&lt;/p&gt;
-    &lt;p&gt;- Ein Verkehrsflugzeug-Objekt kann mit Angabe des Herstellers (String), der maximalen Geschwindigkeit (int), der Immatrikulationsnummer (String) und der Anzahl der Passagiere (int) erzeugt werden.&lt;/p&gt;
-    &lt;p&gt;- Die Klasse Verkehrsflugzeug hat die Methoden &lt;em&gt;getAnzahlPassagiere&lt;/em&gt; und &lt;em&gt;setAnzahlPassagiere&lt;/em&gt; zum Abfragen und Setzen der Anzahl der Passagiere.&lt;/p&gt;
-    &lt;p&gt;Klasse &lt;em&gt;Doppeldecker&lt;/em&gt;:&lt;/p&gt;
-    &lt;p&gt;- Ein Doppeldecker ist ein Flugzeug, das genau zwei Flügelpaare hat.&lt;/p&gt;
-    &lt;p&gt;- Weiter ist ein Doppeldecker akrobatiktauglich, d.h. man kann damit Loopings fliegen. Für einen Looping muss der Doppeldecker eine Mindestgeschwindigkeit von 320 km/h erreichen. Definieren Sie dafür eine Konstante &lt;em&gt;LOOPINGSPEED&lt;/em&gt;. Die Methode &lt;em&gt;getLooping&lt;/em&gt; soll true zurückgeben, falls die zulässige max. Geschwindigkeit (&lt;em&gt;maxSpeed&lt;/em&gt;) größer LOOPINGSPEED ist.&lt;/p&gt;
-    &lt;p&gt;- Die Klasse Doppeldecker hat eine Variable &lt;em&gt;offenesCockpit&lt;/em&gt; vom Typ boolean. Sie gibt an, ob der Doppeldecker ein offenes oder geschlossenes Cockpit hat. Nachdem &lt;em&gt;offenesCockpit&lt;/em&gt; gesetzt worden ist, darf sie nicht mehr verändert werden. Der Wert des Attributes darf gelesen werden.&lt;/p&gt;
-    &lt;p&gt;- Ein Doppeldecker-Objekt kann durch 2 Konstruktoren initianlisiert werden:&lt;/p&gt;
-    &lt;p&gt;    a) Der 1. Konstruktor hat folgende Parameter: Hersteller (String), maximale Geschwindigkeit (int), die Immatrikulationsnummer (String) und einen boolean offenesCockpit, der angibt, ob der Doppeldecker ein offenes oder geschlossenes Cockpit hat.&lt;/p&gt;
-    &lt;p&gt;    b) Der 2. Konstruktor hat folgende Parameter: Hersteller (String), maximale Geschwindigkeit (int), die Immatrikulationsnummer (int). Der Defaultwert für offenesCockpit bei einem Doppeldecker ist true.&lt;/p&gt;
-    &lt;p&gt;- Die Klasse Doppeldecker soll nicht erweiterbar sein.&lt;/p&gt;
-    &lt;p&gt;1. Modellieren Sie die beschriebenen Klassen in einem UML-Klassendiagramm.&lt;/p&gt;
-    &lt;p&gt;2. Implementieren Sie die Klassen &lt;em&gt;Verkehrsflugzeug&lt;/em&gt; und &lt;em&gt;Doppeldecker&lt;/em&gt; anhand der o.a. Eigenschaften.&lt;/p&gt;
-    &lt;p&gt;3. Implementieren Sie eine main-Klasse Airline in der Sie beliebig Objekte der Klassen Verkehrsflugzeug und Doppeldecker anlegen. Des Weiteren legen Sie eine ArrayList flug wie folgt an:&lt;br /&gt;
-        &amp;nbsp; &amp;nbsp;ArrayList&amp;lt;Flugzeug&amp;gt; flug = new ArrayList&amp;lt;Flugzeug&amp;gt;();&lt;br /&gt;
-    Fügen Sie der Arraylist per flug.add() die zuvor erzeugten Objekte der Klassen Verkehrsflugzeug und Doppeldecker hinzu! Sollte dies zu Fehlern führen, dann ist ihre Implementierung der Klassen nicht korrekt!! :-)&lt;/p&gt;
-    &lt;p&gt;4. Geben Sie die Daten der in der ArrayList gespeicherten Objekten aus, in dem Sie die entsprechenden Methoden aufrufen.&lt;/p&gt;</t>
-  </si>
-  <si>
     <t>package de.goals.testing;
 import org.junit.jupiter.api.Test;
 import static org.junit.jupiter.api.Assertions.*;
@@ -2826,15 +2480,6 @@
     <t>Test erweitert und html korrigiert</t>
   </si>
   <si>
-    <t xml:space="preserve">    &lt;p&gt;&lt;strong&gt;Grundlagen:&lt;/strong&gt; Eine quadratische Pyramide und ein Kegel haben eine Grundfläche, die durch die Angabe einer einzigen Länge bestimmt ist (beim Kegel der Radius), und eine Höhe. Aus diesen Größen lassen sich Volumen und Oberfläche dieser Körper berechnen.&lt;/p&gt;
-    &lt;p&gt;&lt;strong&gt;Programmieraufgabe:&lt;/strong&gt; Implementieren Sie eine geeignete abstrakte Klasse und mehrere Unterklassen, um die Volumen- und Oberflächenberechnungen durchzuführen. Folgende Klassen sind zu erstellen:&lt;/p&gt;
-    &lt;p&gt;&lt;strong&gt;Klassen und ihre Dateien:&lt;/strong&gt;&lt;/p&gt;
-    &lt;p&gt;&lt;code&gt;Koerper.java&lt;/code&gt; - Abstrakte Basis-Klasse für geometrische Körper.&lt;/p&gt;
-    &lt;p&gt;&lt;code&gt;Pyramide.java&lt;/code&gt; - Spezifische Klasse für die Pyramide.&lt;/p&gt;
-    &lt;p&gt;&lt;code&gt;Kegel.java&lt;/code&gt; - Spezifische Klasse für den Kegel.&lt;/p&gt;
-    &lt;p&gt;&lt;code&gt;Formen.java&lt;/code&gt; - Hauptklasse, die Methoden &lt;code&gt;getVolumen()&lt;/code&gt; und &lt;code&gt;getFlaeche()&lt;/code&gt; aufruft.&lt;/p&gt;</t>
-  </si>
-  <si>
     <t>package de.goals.testing; // nicht entfernen
 public class Formen {
     public static void main(String[] args) {
@@ -2848,17 +2493,6 @@
     <t>Schreiben Sie ein Java-Programm MyThread.java, das die Summe aller Zahlen eines vorgegebenen int-Arrays mit Hilfe von zwei Threads berechnet. Dazu wird das Array jeweils zur Hälfte auf die beiden Threads verteilt. Jeder Thread berechnet seinen Bereich für sich. Nach Beendigung der Threads soll das Hauptprogramm die Ergebnisse aus dem Objekt lesen, die Summe berechnen und das Ergebnis ausgeben.
 Erstellen Sie eine Klasse ArrayCalc (ArrayCalc.java), die die Berechnung für einen Teil des Arrays übernimmt!
 Hinweis: Machen Sie sich mit der join()-Methode der Klasse Thread vertraut!</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    &lt;p&gt;&lt;b&gt;Aufgabenstellung:&lt;/b&gt;&lt;br&gt;
-    Schreiben Sie ein Java-Programm &lt;b&gt;MyThread.java&lt;/b&gt;, das die Summe aller Zahlen eines vorgegebenen &lt;i&gt;int&lt;/i&gt;-Arrays mit Hilfe von zwei Threads berechnet. Dazu wird das Array jeweils zur Hälfte auf die beiden Threads verteilt. Jeder Thread berechnet seinen Bereich für sich. Nach Beendigung der Threads soll das Hauptprogramm die Ergebnisse aus dem Objekt lesen, die Summe berechnen und das Ergebnis ausgeben.
-    &lt;/p&gt;
-    &lt;p&gt;&lt;b&gt;Weitere Anweisungen:&lt;/b&gt;&lt;br&gt;
-    Erstellen Sie eine Klasse &lt;b&gt;ArrayCalc&lt;/b&gt; (&lt;b&gt;ArrayCalc.java&lt;/b&gt;), die die Berechnung für einen Teil des Arrays übernimmt!
-    &lt;/p&gt;
-    &lt;p&gt;&lt;b&gt;Hinweis:&lt;/b&gt;&lt;br&gt;
-    Machen Sie sich mit der &lt;b&gt;join()&lt;/b&gt;-Methode der Klasse &lt;b&gt;Thread&lt;/b&gt; vertraut!
-    &lt;/p&gt;</t>
   </si>
   <si>
     <t xml:space="preserve">package de.goals.testing;
@@ -2905,11 +2539,6 @@
 </t>
   </si>
   <si>
-    <t>&lt;p&gt; In dieser Aufgabe sollst du den Bubblesort-Algorithmus in Java implementieren. Dieser Algorithmus ist ein einfaches Verfahren zum Sortieren einer Liste von Elementen (z.B. Zahlen).&lt;/p&gt;
-&lt;br&gt;
-&lt;p&gt;Bubblesort ist ein Sortieralgorithmus, der durch wiederholtes Durchlaufen der zu sortierenden Liste arbeitet. Bei jedem Durchlauf werden benachbarte Elemente miteinander verglichen und gegebenenfalls vertauscht. Das Besondere am Bubblesort ist, dass mit jedem Durchgang das größte Element der noch zu sortierenden Elemente an das Ende der Liste "aufsteigt".&lt;/p&gt;</t>
-  </si>
-  <si>
     <t>package de.goals.testing;
 import org.junit.jupiter.api.Test;
 import static org.junit.jupiter.api.Assertions.assertArrayEquals;
@@ -2943,12 +2572,6 @@
         assertArrayEquals(expected, arr);
     }
 }</t>
-  </si>
-  <si>
-    <t>&lt;img src="/assets/taskImgs/fahrzeugUML.png" alt="image"&gt;
-&lt;br /&gt;&lt;p&gt;
-  Schreiben Sie den Java Code für beide Klassen des UML-Diagramms.
-&lt;/p&gt;</t>
   </si>
   <si>
     <t>TestFahrzeuge.java</t>
@@ -3105,19 +2728,6 @@
     unittest.main()</t>
   </si>
   <si>
-    <t>&lt;p&gt;Schreiben Sie eine Funktion &lt;code&gt;charFrequenz()&lt;/code&gt;, die die Buchstabenhäufigkeit eines Strings bestimmt.Die Funktion soll:&lt;/p&gt; 
-&lt;p&gt;1. Sonderzeichen, Satzzeichen, Umlaute (z.B. ä, ö, ü) und Ziffern nicht berücksichtigen.&lt;/p&gt; 
-&lt;p&gt;2. Die Buchstabenhäufigkeiten sortiert ausgeben.&lt;/p&gt; 
-&lt;p&gt;3. Falls mehrere Buchstaben gleich oft vorkommen, diese in alphabetischer Reihenfolge ausgeben.&lt;/p&gt; 
-&lt;h2&gt;Tipps:&lt;/h2&gt; 
-&lt;p&gt;1. &lt;code&gt;sorted(s)&lt;/code&gt; sortiert die Zeichen des Strings &lt;code&gt;s&lt;/code&gt; in alphabetischer Reihenfolge und gibt eine Liste der sortierten Zeichen zurück.&lt;/p&gt; 
-&lt;p&gt;2. &lt;code&gt;s.lower()&lt;/code&gt; wandelt die Zeichen des Strings &lt;code&gt;s&lt;/code&gt; in Kleinbuchstaben um und gibt einen entsprechenden String mit Kleinbuchstaben zurück.&lt;/p&gt; 
-&lt;h2&gt;Beispiel:&lt;/h2&gt; 
-&lt;p&gt;&lt;code&gt;s = "Das ist ein Teststring 123!"&lt;/code&gt;&lt;/p&gt; 
-&lt;p&gt;&lt;code&gt;x = charFrequenz(s)&lt;/code&gt;&lt;/p&gt; &lt;p&gt;&lt;code&gt;x&lt;/code&gt; wäre dann:&lt;/p&gt; 
-&lt;p&gt;&lt;code&gt;[('s', 4), ('t', 4), ('i', 3), ('e', 2), ('n', 2), ('a', 1), ('d', 1), ('g', 1), ('r', 1)]&lt;/code&gt;&lt;/p&gt;</t>
-  </si>
-  <si>
     <t xml:space="preserve">
 Schreiben Sie eine Funktion charFrequenz(), die die Buchstabenhäufigkeit eines Strings bestimmt.Die Funktion soll:
 1. Sonderzeichen, Satzzeichen, Umlaute (z.B. ä, ö, ü) und Ziffern nicht berücksichtigen.
@@ -3175,17 +2785,6 @@
 }</t>
   </si>
   <si>
-    <t>&lt;p&gt;Betrachten Sie das folgende Klassendiagramm:&lt;br /&gt;
-&lt;img src="/assets/taskImgs/Java_Bibliothek_Bib.svg" alt="image"&gt;
-&lt;br /&gt;
-a) Machen Sie sich mit den&amp;nbsp;Eigenschaften der  Klasse Datum vertraut, in dem Sie sich den Quelltext anschauen. Schauen Sie sich&amp;nbsp;die Eigenschaften der Klasse Calendar in der Java-API an.&lt;/p&gt;
-&lt;p&gt;b) Setzen Sie nun das oben stehende UML-Klassendiagramm in Java um, unter der&amp;nbsp;Verwendung der Klasse Datum. Implementieren Sie auch die Methoden der Klassen&amp;nbsp;Medium, Buch und DVD. Für die Berechnung des Strafgeldes bei &amp;Uuml;berziehung der&amp;nbsp;Leihfristen gelten folgende Bestimmungen:&lt;/p&gt;
-&lt;p&gt;- Bücher k&amp;ouml;nnen 4 Wochen ausgeliehen werden, bei &amp;Uuml;berziehung 1 EUR Strafgeld pro&amp;nbsp;angefangenen &amp;Uuml;berziehungstag.&lt;br /&gt;
-- DVDs k&amp;ouml;nnen 1 Woche ausgeliehen werden, bei &amp;Uuml;berziehung 2 EUR Strafgeld pro&amp;nbsp;angefangenen &amp;Uuml;berziehungstag&lt;/p&gt;
-&lt;p&gt;Für die Berechnung der Differenztage zwischen dem Ausleihdatum und Heute&amp;nbsp;implementieren Sie bitte die Methode calcDiffDays() der Klasse Datum. Nehmen Sie&amp;nbsp;dazu an, dass jeder Monat 30 Tage hat und das Jahr 365 Tage.&lt;/p&gt;
-&lt;p&gt;c) Schreiben Sie ein kleines Testprogramm (BibVerwaltung.java), das Objekte von den&amp;nbsp;beiden Medien Buch und DVD erzeugt.&lt;/p&gt;</t>
-  </si>
-  <si>
     <t>Betrachten Sie das folgende Klassendiagramm:
 classDiagram
     class Medium {
@@ -3250,58 +2849,6 @@
     }
 Erstellen Sie zu diesem Klassendiagramm den entsprechenden Java-Code. Beachten Sie dabei vor allem die Sichtbarkeiten!
 Implementieren Sie einen Konstruktor der alle Attribute als Argument erhält! Implementieren Sie die Rümpfe der Methoden. </t>
-  </si>
-  <si>
-    <t>&lt;p&gt;Betrachten Sie das folgende UML-Diagramm:&lt;/p&gt;
-&lt;img src="/assets/taskImgs/UMLtoJava.svg" alt="image"&gt;
-&lt;br /&gt;Erstellen Sie zu diesem Klassendiagramm den entsprechenden Java-Code. Beachten Sie dabei vor allem die Sichtbarkeiten!&lt;/p&gt;
-&lt;p&gt;Implementieren Sie einen Konstruktor der alle Attribute als Argument erh&amp;auml;lt!&amp;nbsp;Implementieren Sie die R&amp;uuml;mpfe der Methoden.&amp;nbsp;&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>&lt;div&gt;
-    &lt;p&gt;
-    Für die Simulation eines Wettrennens sollen verschiedene Fahrzeugarten objektorientiert modelliert werden. Da alle Fahrzeugtypen gemeinsame Eigenschaften haben, definieren wir uns zunächst eine Basisklasse Fahrzeug, die als Oberklasse für die anderen Klassen dienen soll. Ein Fahrzeug hat folgende allgemeinen Merkmale:
-    &lt;/p&gt;
-    &lt;br&gt;
-    &lt;ul&gt;
-    &lt;li&gt;Seine aktuelle Position (in km und der Einfachheit halber in nur einer Dimension)&lt;/li&gt;
-    &lt;li&gt;Seine aktuelle Geschwindigkeit (in km/h)&lt;/li&gt;
-    &lt;li&gt;Es kann bewegt werden (Methode bewege). Die Methode wird mit einem double-Parameter aufgerufen, der die Anzahl der Minuten angibt, die sich das Fahrzeug mit der aktuellen Geschwindigkeit vorwärts bewegt. Der Methodenaufruf ändert natürlich die Position des Fahrzeugs, wenn es mit einer von 0 verschiedenen Geschwindigkeit bewegt wird.&lt;/li&gt;
-    &lt;li&gt;Man kann seine Geschwindigkeit setzen (Methode setzeGeschwindigkeit). Die Geschwindigkeit darf die Maximalgeschwindigkeit nicht überschreiten, eine korrekte Ausführung sollte protokolliert werden.&lt;/li&gt;
-    &lt;li&gt;Es kann seine Maximalgeschwindigkeit angeben (Methode getMaxGeschwindigkeit). Für ein Objekt der Klasse Fahrzeug soll die Maximalgeschwindigkeit 0 sein.&lt;/li&gt;
-    &lt;li&gt;Es kann die Anzahl seiner Räder angeben (Methode getAnzahlRaeder). In der Klasse Fahrzeug soll diese ebenfalls 0 sein.&lt;/li&gt;
-    &lt;/ul&gt;
-    &lt;br&gt;
-    &lt;p&gt;
-    Nun sollen einige konkrete Fahrzeuge definiert werden, indem entsprechende Klassen von Fahrzeug abgeleitet werden:
-    &lt;/p&gt;
-    &lt;br&gt;
-    &lt;ul&gt;
-    &lt;li&gt;Ein Fahrrad ist ein Fahrzeug mit 2 Rädern und Maximalgeschwindigkeit 30 km/h.&lt;/li&gt;
-    &lt;li&gt;Ein Auto ist ein Fahrzeug mit 4 Rädern und Maximalgeschwindigkeit 140 km/h.&lt;/li&gt;
-    &lt;li&gt;Ein Rennwagen ist ein Auto mit Maximalgeschwindigkeit 220 km/h.&lt;/li&gt;
-    &lt;li&gt;Ein Krankenwagen ist ein Auto mit einem zusätzlichen Blaulicht, das ein- oder ausgeschaltet sein kann (Attribut: isBlaulichtAn). Um den Zustand des Blaulichts auszugeben, wird die Methode isBlaulichtAn() benötigt. Außerdem muss der Krankenwagen Methoden zum Ein- bzw. Ausschalten des Blaulichts anbieten (blaulichtAn und blaulichtAus). &lt;/li&gt;
-    &lt;/ul&gt;
-    &lt;br&gt;
-    &lt;p&gt;
-    Definieren Sie diese Klassen und nutzen Sie dabei so weit wie möglich die Vererbung von Eigenschaften aus!
-    &lt;/p&gt;
-    &lt;br&gt;
-    &lt;p&gt;
-    Nun soll die eigentliche Simulation des Wettrennens in einer Klasse Wettrennen geschrieben werden. Erzeugen sie je ein Fahrzeug und setzen Sie dann die Geschwindigkeiten auf:
-    &lt;/p&gt;
-    &lt;br&gt;
-    &lt;ul&gt;
-    &lt;li&gt;Fahrrad: 20 km/h&lt;/li&gt;
-    &lt;li&gt;Auto: 150 km/h&lt;/li&gt;
-    &lt;li&gt;Rennwagen: 200 km/h&lt;/li&gt;
-    &lt;li&gt;Krankenwagen: 80 km/h&lt;/li&gt;
-    &lt;/ul&gt;
-    &lt;br&gt;
-    &lt;p&gt;
-    Dann sollen sich die Fahrzeuge bewegen. Der Gerechtigkeit halber geben wir dem Fahrrad einen Vorsprung von 4 Stunden. Danach lassen Sie alle Fahrzeuge eine Stunde lang mit unveränderter Geschwindigkeit vorwärts fahren. Was fällt Ihnen beim Auto auf?
-    &lt;/p&gt;
-&lt;/div&gt;</t>
   </si>
   <si>
     <t>Für die Simulation eines Wettrennens sollen verschiedene Fahrzeugarten objektorientiert modelliert werden. Da alle Fahrzeugtypen gemeinsame Eigenschaften haben, definieren wir uns zunächst eine Basisklasse Fahrzeug, die als Oberklasse für die anderen Klassen dienen soll. Ein Fahrzeug hat folgende allgemeinen Merkmale:
@@ -3323,6 +2870,384 @@
     Rennwagen 200 km/h
     Krankenwagen 80 km/h 
 Dann sollen sich die Fahrzeuge bewegen. Der Gerechtigkeit halber geben wir dem Fahrrad einen Vorsprung von 4 Stunden. Danach lassen Sie alle Fahrzeuge eine Stunde lang mit unveränderter Geschwindigkeit vorwärts fahren. Was fällt Ihnen beim Auto auf?</t>
+  </si>
+  <si>
+    <t>Ein Kapital von 1000 Euro wird jährlich mit einem bestimmten Prozentsatz verzinst. Die rekursive Funktion `kapitalWert()` beschreibt den Kapitalwert nach n Jahren bei konstantem Zinssatz. Die Funktion gibt den Kapitalwert (ohne Euro-Symbol oder EUR) zurück.
+**Beispielrechnung:**
+*Startkapital: 1000.00 EUR und 5 % Zinsen  
+Kapital nach dem 1. Jahr: 1000.00 + 0,05 * 1000.00 = 1050.00  
+Kapital nach dem 2. Jahr: 1050.00 + 0,05 * 1050.00 = 1102.50  
+...*
+**Hinweise:**  
+1. Die Funktion kapitalWert sollte als Parameter den aktuellen Kapitalwert, Zinssatz und Jahre haben!  
+2. Sie brauchen das Ergebnis nicht zu formatieren oder zu runden!</t>
+  </si>
+  <si>
+    <t>In einer Buchhandlung findet sich in einem Abrechnungsprogramm in Python eine Liste mit Unterlisten mit folgendem Aufbau:
+| Bestellnummer | Buchtitel und Autor                  | Anzahl | Einzelpreis |
+|---------------|--------------------------------------|--------|-------------|
+| 34587         | Learning Python, Mark Lutz           | 4      | 40.95       |
+| 98762         | Programming Python, Mark Lutz        | 5      | 56.80       |
+| 77226         | Head First Python, Paul Barry 3      | 3      | 32.00       |
+Schreiben Sie eine Funktion `biblio()`, die unter Benutzung von `lambda` und `map`, das als Ergebnis eine Liste mit Zweier-Tupeln zurückliefert. Dazu erhält die Funktion die eine Liste im obigen Format als Argument in der Form  
+\[["34587", "Learning Python, Mark Lutz", 4, 40.95], ["98762", "Programming Python, Mark Lutz", 5, 56.80], ["77226", "Head First Python, Paul Barry", 3, 32.95]\]
+Die Funktion berechnet dann wie folgt: Jedes Tupel besteht aus der Bestellnummer und dem Produkt aus der Anzahl und dem Einzelpreis. Das Produkt soll jedoch um 10,- € erhöht werden, wenn der Bestellwert unter 100,00 € liegt. Die Funktion gibt dann die so errechnete Liste zurück.</t>
+  </si>
+  <si>
+    <t>Schreiben Sie eine rekursive Funktion `querSum(n)`, die eine positive Ganzzahl `n` als Parameter erhält und ihre Quersumme ausgibt.
+Hinweis: Bsp.:
+``` 
+&gt;&gt; querSum(174)
+&gt;&gt; 12
+```
+Weil 1+7+4=12 ist.</t>
+  </si>
+  <si>
+    <t># Fibonacci-Folge Index Finder
+Schreiben Sie eine rekursive Funktion `fib_index()`, die den Index einer Zahl in der [Fibonacci-Folge](https://de.wikipedia.org/wiki/Fibonacci-Folge) zurückgibt, wenn die Zahl ein Element dieser Folge ist, und `-1` zurückgibt, wenn die Zahl nicht darin enthalten ist.
+**Beispiel:**
+```
+&gt;&gt;&gt; fib_index(13)
+&gt;&gt;&gt; 7
+```
+In der Fibonacci-Folge ist die `13` an der `7.` Position: `0, 1, 1, 2, 3, 5, 8, 13, 21, ...`
+**Tipp:** In den Übungen haben Sie ja bereits eine Funktion zur Bestimmung der Fibonacci Folge geschrieben, die sie jetzt wiederverwenden können!</t>
+  </si>
+  <si>
+    <t>Schreiben Sie eine Funktion `charFrequenz()`, die die Buchstabenhäufigkeit eines Strings bestimmt. Die Funktion soll:
+1. Sonderzeichen, Satzzeichen, Umlaute (z.B. ä, ö, ü) und Ziffern nicht berücksichtigen.
+2. Die Buchstabenhäufigkeiten sortiert ausgeben.
+3. Falls mehrere Buchstaben gleich oft vorkommen, diese in alphabetischer Reihenfolge ausgeben.
+## Tipps:
+1. `sorted(s)` sortiert die Zeichen des Strings `s` in alphabetischer Reihenfolge und gibt eine Liste der sortierten Zeichen zurück.
+2. `s.lower()` wandelt die Zeichen des Strings `s` in Kleinbuchstaben um und gibt einen entsprechenden String mit Kleinbuchstaben zurück.
+## Beispiel:
+```python
+s = "Das ist ein Teststring 123!"
+x = charFrequenz(s)
+```
+`x` wäre dann:
+```python
+[('s', 4), ('t', 4), ('i', 3), ('e', 2), ('n', 2), ('a', 1), ('d', 1), ('g', 1), ('r', 1)]
+```</t>
+  </si>
+  <si>
+    <t>Erstellen Sie eine rekursive Funktion *summe*, die zwei ganze Zahlen *m* und *n* als Argumente erhält und die Summe aller ganzen Zahlen zwischen *m* und *n* (einschließlich) als Ergebnis liefert. Falls *m* größer als *n* ist, soll das Ergebnis 0 sein.
+Beispiel:
+`summe(1, 3)`
+6  
+*Weil 1+2+3=6*
+`summe(3, 3)`
+3
+`summe(5, 3)`
+0</t>
+  </si>
+  <si>
+    <t>Implementieren Sie den euklidischen Algorithmus zur Berechnung des "größten-gemeinsamen Teilers" (ggT) **rekursiv** in einer Funktion ggT()
+Der Euklidische Algorithmus zur Berechnung des größten gemeinsamen Teilers zweier positiver ganzer Zahlen a und b (ggT(a,b)) ist wie folgt rekursiv definiert:
+- *ggT(a,b) = a, falls a = b*
+- *ggT(a,b) = ggT(a - b, b), falls a &gt; b*
+- *ggT(a,b) = ggT(a, b - a), falls b &gt; a*</t>
+  </si>
+  <si>
+    <t>**Das Sieb des Eratosthenes** ist ein Algorithmus, der eine Liste aller Primzahlen von *2* bis zu einer gegebenen Zahl *n* berechnet (siehe u.a. [Wikipedia](https://de.wikipedia.org/wiki/Sieb_des_Eratosthenes)).
+Implementieren Sie den Algorithmus dazu in einer Funktion *sieb()*. Die Funktion erhält als Parameter den Wert n, der angibt, bis zu welcher Zahl die Primzahlen berechnet werden sollen. Die Funktion gibt die Liste mit allen Primzahlen von 2 bis n zurück!
+Gehen Sie dazu wie folgt vor:
+1. Der Algorithmus berechnet jeweils die Vielfachen von 2, 3, 5 und 7 aus der gegebenen Liste und entfernt diese. Schreiben Sie deshalb zuerst eine Funktion vielfach(). Die Funktion erhält als Parameter die Zahl, zu denen die Vielfachen entfernt werden sollen, sowie die Liste, auf die die Operation durchgeführt wird.
+   *Beispiel: vielfach(2, liste)*  
+   Entfernt alle Vielfachen von 2 aus liste
+2. Implementieren sie dann die Funktion *sieb()* mit Hilfe der Funktion *vielfach()*.</t>
+  </si>
+  <si>
+    <t>Ergänzen Sie ein gegebenes Java-Programm (Alter.java) in dessen main-Methode eine Methode **gibBezeichnung()** aufgerufen wird, die als Parameter einen int-Wert erhält der das Alter in Jahren beschreibt.
+Die Methode **gibBezeichnung()** sollen in Abhängigkeit des Parameters folgende Strings zurückgeben:
+*Alter in Jahren* größer 0 aber kleiner 18: "Du bist ja noch ein Kind!"
+*Alter in Jahren* mindestens 18 aber weniger als 67: "Du stehst mitten im Leben!"
+*Alter in Jahren* größer gleich 67: "Als Rentner hat man es gut!"
+Wenn keine der o.a. Bedingungen zutrifft (z.B. bei negativen Werten) soll der String "Mit Deinem Alter stimmt was nicht!" zurückgegeben werden.
+Verwenden Sie eine *if*-Anweisung um die einzelnen Ausgaben in Abhängigkeit der Variable zu erzeugen. Achten Sie auf eine korrekte Angabe der Grenzen und testen Sie das Programm in dem Sie die Variable verändern, neu kompilieren und die Ausgabe betrachten.
+Verwenden Sie exakt das vorgegebene Code-Gerüst und geben Sie **exakt** die o.a. Ausgaben an!</t>
+  </si>
+  <si>
+    <t>Schreiben Sie eine Java-Methode *bruchSumme()*, die die Summe der folgenden Brüche berechnet:
+**1 + 1/2 + 1/3 + 1/4 + 1/5 + ...**
+Für n=3 würden Sie zum Beispiel die Summe 1 + 1/2 + 1/3 = 1.8333333333333333 erhalten.
+Erstellen Sie eine Java-Klasse *Summenwert* mit einer Methode *public double bruchSumme(int n)*.  
+Verwenden Sie eine Schleife!!!</t>
+  </si>
+  <si>
+    <t>Vervollständigen Sie die Methode *berechneRabatt()* des Java-Programms **Discount.java**, das als Argument einen Geldbetrag erhält. Die Methode *berechneRabatt()* erhält als Parameter einen Euro-Wert.
+Falls der Betrag größer als 1000 EUR ist, soll ein Rabatt von 8 Prozent gewährt werden. In diesem Falle soll die Methode den String "Betrag mit Rabatt: " zurückgeben und anschließend den zu zahlenden Betrag (siehe Beispiele unten). Falls der Betrag kleiner oder gleich 1000 EUR ist, soll nur der Betrag zurückgegeben werden.
+Die eigentliche Ausgabe erfolgt dann im main-Part.
+**Bsp. 1:**
+java Discount 1234.45
+Betrag mit Rabatt: 1135.69
+---------
+**Bsp.: 2:**
+java Discount 999
+Zu zahlender Betrag: 999.00</t>
+  </si>
+  <si>
+    <t>Implementieren Sie die Methode *max()* der Klasse *Starter* im vorgegebenen Code-Gerüst (Starter.java). Die Methode *max* gibt die Größere der beiden natürlichen Zahlen *a* und *b* zurück. Wenn beide Zahlen gleich sind, wird dieser Wert zurückgegeben.
+Implementieren Sie nur die Methode *max* der Klasse *Starter*.
+**Verwenden Sie also exakt das vorgegebene Code-Gerüst!**</t>
+  </si>
+  <si>
+    <t>Betrachten Sie den Quellcode der Datei **ArrayWork.java**.
+Das Programm ArrayWork.java soll verschiedene Operationen auf ein Array mit double-Werten realisieren. Das Array ist bereits vorgegeben (double werte[]) und die entsprechende Operation wird per Parameter als int-Wert angegeben (int arg).
+Das Array und der Parameter werden einer Funktion ArrayFunc übergeben in der die folgenden Funktionen implementiert werden sollen:
+- func=1: Gib den kleinsten Wert aus dem Array zurück  
+- func=2: Gib den größten Wert aus dem Array zurück  
+- func=3: Gib den arithmetischen Mittelwert aus dem Array zurück  
+- func=4: Addiere alle Elemente des Arrays, addiere 19 % MwSt. und gib das Ergebnis zurück.  
+- Für alle anderen Werte von func soll 0 zurückgegeben werden.
+Implementieren Sie die gewünschte Funktionalität unter der Verwendung von Schleifen und ggf. weiteren Funktionen.
+Verwenden Sie exakt das vorgegebene Code-Gerüst!</t>
+  </si>
+  <si>
+    <t>Nach einer alten Sage wurde der Erfinder des Schachspiels zum König gerufen, der ihn für seine Erfindung belohnen wollte. Auf die Frage, was er sich wünsche, antwortete der Schachspieler, dass der König ihm auf das erste Feld des Schachbretts 1 Cent legen sollte, auf das zweite Feld 2 Cent, auf das dritte Feld 4 Cent, auf das vierte Feld wieder das Doppelte und so weiter.
+Der König dachte: "Was für ein Dummkopf! Hätte er sich doch Gold gewünscht und nicht nur Cent?".
+Verwenden Sie das vorgegeben Code-Gerüst Schach.java!  
+Vervollständigen Sie die Methode *felder*, mit deren Hilfe Sie das oben geschilderte Vorgehen simulieren können.
+```java
+public int felder(int cent)
+```
+Der Methode übergeben Sie als Parameter die Zahl der erwünschten Cent, beispielsweise 1000, und die Methode gibt die Zahl der Felder zurück, die der König mit Centstücken belegen muss, um die gewünschte Zahl zu erhalten. **Verwenden Sie eine Schleife!**
+Für eine gewünschte Zahl von 1.000 Centstücken sind 1 + 2 + 4 + 8 + 16 + 32 + 64 + 128 + 256 + 512 Centstücke auf die Felder zu legen, benötigt werden also 10 Felder. Ein Schachbrett hat aber 8 x 8 = 64 Felder.
+Hinweis: Schauen Sie sich die Java-API Informationen zu java.lang.Math an (https://docs.oracle.com/en/java/javase/18/). Da gibt es evtl. eine Methode die ihnen helfen kann!</t>
+  </si>
+  <si>
+    <t>Vervollständigen Sie die Methode `checkModulo()`, die als Parameter zwei `int`-Werte erhält, durch die Umsetzung der folgenden Bedingungen:
+Es soll zunächst der Rest der Division von `i` durch `j` berechnet werden (modulo). Implementieren Sie nun eine `switch`-Anweisung, die unterscheidet ob die folgenden Bedingungen erfüllt sind:
+- Der Rest ist null. ("Der Rest ist null")
+- Der Rest ist eine einstellige Primzahl ("Der Rest ist eine einstellige Primzahl")
+- Der Rest ist ungerade (aber keine einstellige Primzahl) ("Der Rest ist ungerade")
+- Keine der Bedingungen trifft zu. ("Keine der Aussagen trifft zu")
+In allen Fällen soll der jeweils angegebene Text (exakt dieser Text!) von der Methode `checkModulo` zurückgegeben werden. Nutzen Sie daher insbesondere die `break`-Anweisung! Verwenden Sie exakt das vorgegebene Code-Gerüst!</t>
+  </si>
+  <si>
+    <t>Betrachten Sie das folgende Klassendiagramm:  
+![image](/assets/taskImgs/Java_Bibliothek_Bib.svg)  
+---
+a) Machen Sie sich mit den Eigenschaften der Klasse Datum vertraut, indem Sie sich den Quelltext anschauen. Schauen Sie sich die Eigenschaften der Klasse Calendar in der Java-API an.
+b) Setzen Sie nun das oben stehende UML-Klassendiagramm in Java um, unter der Verwendung der Klasse Datum. Implementieren Sie auch die Methoden der Klassen Medium, Buch und DVD. Für die Berechnung des Strafgeldes bei Überziehung der Leihfristen gelten folgende Bestimmungen:
+- Bücher können 4 Wochen ausgeliehen werden, bei Überziehung 1 EUR Strafgeld pro angefangenem Überziehungstag.
+- DVDs können 1 Woche ausgeliehen werden, bei Überziehung 2 EUR Strafgeld pro angefangenem Überziehungstag.
+Für die Berechnung der Differenztage zwischen dem Ausleihdatum und Heute implementieren Sie bitte die Methode `calcDiffDays()` der Klasse Datum. Nehmen Sie dazu an, dass jeder Monat 30 Tage hat und das Jahr 365 Tage.
+c) Schreiben Sie ein kleines Testprogramm (`BibVerwaltung.java`), das Objekte von den beiden Medien Buch und DVD erzeugt.</t>
+  </si>
+  <si>
+    <t>Verwenden Sie das Code-Gerüst aus Java_GGT.java und implementieren Sie die Methode `ggT()`.
+Die Methode `ggT` berechnet den größten gemeinsamen Teiler zweier natürlicher Zahlen `a` und `b`. Verwenden Sie dazu den folgenden Algorithmus:
+1. setze `m = a` und `n = b`
+2. falls `m` kleiner als `n`, dann vertausche `m` und `n`
+3. setze `r = m - n`
+4. setze `m = n` und `n = r`
+5. 
+   a) falls `r` ungleich 0 mache weiter bei Schritt 2  
+   b) falls `r` gleich 0 dann ist `m` der ggT!
+Verwenden Sie exakt das vorgegebene Code-Gerüst!</t>
+  </si>
+  <si>
+    <t>Die folgende Aufgabe soll einer Universitätsverwaltung helfen, die Gehälter von Professoren und Mitarbeitern zu berechnen.
+### a) Erstellen Sie eine Java-Klasse *Angestellter*, die als Attribute
+- *double stdProMonat* und
+- *double geldProStunde*
+und als Methode *public double berechneMonatseinkommen()* besitzt.  
+Die Methode *berechneMonatseinkommen()* berechnet das Einkommen eines Angestellten pro Monat und gibt dieses dann zurück.
+Außerdem soll die Klasse *Angestellter* zwei Konstruktoren besitzen:
+- *public Angestellter( double arbeitstdProMonat, double gehaltProStunde )*
+- *public Angestellter()*
+### b) Erstellen Sie nun eine Klasse *Professor*, die von der Klasse *Angestellter* erbt.
+Ein Professor hat immer eine feste Arbeitszeit von 160 Stunden im Monat.  
+Implementieren Sie den Konstruktor der Klasse *Professor*. Falls nötig, überschreiben Sie Methoden der Basisklasse *Angestellter* und geben Sie die neue Implementierung an.
+### c) Erstellen Sie nun eine Klasse *Mitarbeiter*, die von der Klasse *Angestellter* erbt.
+Ein Mitarbeiter bekommt zusätzlich zum jeweiligen Stundenlohn jeden Monat einen Bonus von 500 EUR. Implementieren Sie den Konstruktor der Klasse *Mitarbeiter*. Falls nötig, überschreiben Sie Methoden der Basisklasse *Angestellter* und geben Sie die neue Implementierung an.
+### d) Erstellen Sie nun eine Klasse *Uni* mit einer main()-Methode.
+Erzeugen Sie ein Array von Angestellten `personal` mit 3 Elementen:
+- `personal[0]=new Angestellter(22,11.5);`
+- `personal[1]=new Professor(121.40);`
+- `personal[2]=new Mitarbeiter(40, 15);`
+Berechnen Sie in einer for-Schleife die Summe der Einkommen der drei Angestellten und geben Sie die Summe in der Konsole aus!</t>
+  </si>
+  <si>
+    <t>Legen Sie eine Java-Klasse *VektorWork* an. Schreiben Sie in dieser Klasse eine Methode *addVektor*, die zwei int-Arrays (A und B) als Eingabe-Parameter bekommt und als Ausgabe-Parameter ein neues int-Array C zurück gibt.
+Die Methode führt eine Vektor-Addition aus (C[0] = A[0] + B[0], C[1] = A[1] + B[1] usw.) und gibt das Array C zurück. Beachten Sie aber, dass die Methode Arrays unterschiedlicher Größe behandelt, so dass auch A und B unterschiedlich groß sein können. Dazu soll C wie folgt berechnet werden:
+Bsp.: Wenn A 2 Elemente besitzt und B 4 Elemente:
+- *C[0] = A[0] + B[0]*
+- *C[1] = A[1] + B[1]*
+- *C[2] = B[2]*
+- *C[3] = B[3]*</t>
+  </si>
+  <si>
+    <t>**Modellieren Sie Kraftfahrzeuge (KFZ) als Java-Klasse nach folgenden Festlegungen:**
+Zu einem KFZ werden Kennzeichen, Kilometerstand (int), Tankvolumen in Liter (float), Kraftstoffverbrauch in Liter auf 100 km (float) und Kraftstoffmenge (float) erfasst.
+Die aktuellen Werte der Attribute Kennzeichen, Kilometerstand und Tankvolumen und aktuelle Tankinhalt in Litern können mittels get-Methoden abgefragt werden. (`getKennzeichen()`, `getKMstand()`, `getTankvolumen()`, `getTankinhalt()`)
+Ein KFZ soll sowohl ohne Werte als auch mit den in 1. aufgeführten Attributen erzeugt werden können.
+Ein KFZ kann `tanken(Menge)` und `fahren(Strecke)`.
+`tanken()` erhöht die Kraftstoffmenge im Tank. Sollte die Summe Menge + aktuelle Tankmenge größer sein als das Tankvolumen, so wird die Kraftstoffmenge auf das Tankvolumen begrenzt.
+`fahren()` erhält die Strecke als Parameter und errechnet dann ob der aktuelle Tankinhalt ausreicht die Strecke zu fahren. Wenn das nicht der Fall ist, gibt die Methode `false` zurück. Wenn es möglich ist, dann berechnet die Methode den Kraftstoffverbrauch für die gefahrenen Kilometer und zieht die Liter von der aktuellen Kraftstoffmenge ab. Außerdem wird der Kilometerstand entsprechend erhöht. Die Methode gibt dann `true` zurück.
+Implementieren Sie die Klasse `KFZ` in Java. Selbstverständlich können Sie auch noch weitere Methoden implementieren.
+Implementieren Sie eine neue Test-Klasse `AppAuto`, in der Autos erzeugt werden und diese fahren bzw. tanken lässt.</t>
+  </si>
+  <si>
+    <t>Die Klasse Punkt soll einen Punkt in einem zweidimensionalen Koordinatensystem repräsentieren. Ein Punkt besteht aus folgenden Attributen:
+**X-Koordinate  
+Y-Koordinate**
+Ein Punkt wird in der Klasse über einen Konstruktor erzeugt, der als Parameter die x- und y-Koordinate erhält. Der Standard-Konstruktor erzeugt einen Punkt im Ursprung (0,0).
+Die Klasse Punkt soll folgende Methoden enthalten:
+**getX()** und **getY()**: Gibt die x- bzw. y-Koordinate des Punktes als int-Wert zurück.  
+**toString()**: Gibt einen String in der Form x/y zurück.  
+**spiegelX()**: Spiegelung des Punktes an der X-Achse (Ergebnis soll ein neues Objekt der Klasse Punkt sein, das zurückgegeben wird!)  
+**spiegelY()**: Spiegelung des Punktes an der Y-Achse (Ergebnis soll ein neues Objekt der Klasse Punkt sein, das zurückgegeben wird!)  
+**spiegelUrsprung()**: Spiegelung des Punktes am Ursprung (Ergebnis soll ein neues Objekt der Klasse Punkt sein, das zurückgegeben wird!)  
+**diffUrsprung()**: Abstand des Punktes zum Ursprung. Gibt den Abstand in der Form x/y als String zurück.  
+**diffPunkt()**: Abstand des Punktes zu einem anderen Punkt. Gibt den Abstand in der Form x/y als String zurück.
+Entwerfen Sie eine geeignete Klasse Punkt und implementieren Sie die Klasse Punkt in Java. Testen Sie die Klasse Punkt mit einer Main-Klasse AppPunkt.
+## Umsetzung in Java
+Entwerfen Sie eine geeignete `Klasse Punkt` und implementieren Sie die `Klasse Punkt` in Java. Testen Sie die `Klasse Punkt` mit einer Main-Klasse `AppPunkt`.</t>
+  </si>
+  <si>
+    <t>**Schreiben Sie eine Klasse Konto, die ein Bankkonto realisiert.** Attribute für das Bankkonto sind der Name und Vorname des Kontoinhabers, die Kontonummer (IBAN), der Kontostand, sowie ein Limit, bis zu dem das Konto überzogen werden darf.
+**Erstellen Sie einen oder mehrere geeignete Konstruktoren!** Auf jeden Fall erstellen Sie einen Konstruktor:
+Konto(String Vorname, String Name, String kontonummer)
+Dieser Konstruktor dient dazu einen Neukunden zu initialisieren.
+**Erstellen Sie Methoden für folgende Operationen:**
+* *String toString():* Rückgabe aller Kontodaten eines Kunden in der Form (z.B.):  
+  Kunde: Sarah Müller, Konto: DE87123456782435465711, Stand: 123.45, Limit: 1000.00
+* *einzahlen(Betrag):* Einzahlung eines Betrages
+* *auszahlen():* Auszahlung eines Betrages mit Überprüfung ob ggf. Limit überschritten wurde. In dem Falle wird dann nur die Summe bis zum Limit ausgezahlt.
+* *double getKontostand():* Abfrage des Kontostandes.
+* *setLimit(Limit):* setze das Limit auf einen neuen Betrag.
+**Erstellen Sie eine Test-Klasse AppBank in der die Konten der Kunden verwaltet werden.**</t>
+  </si>
+  <si>
+    <t>**Implementieren Sie eine Klasse Radio mit folgenden Attributen:**
+- eingeschaltet: wenn ein Radio an oder aus ist.
+- lautstaerke: wie laut spielt das Radio Musik? (Die Lautstärke soll nur im Bereich von 0 bis 10 liegen.)
+- frequenz: die die Frequenz des gewählten Senders angibt (Erlaubter Frequenzbereich ist zwischen 85.0 und 110.0).
+**Implementieren Sie zu der Klasse zwei Konstruktoren der Art:**
+- `Radio()`
+- `Radio(boolean istAn, int lautstaerke, double frequenz)`
+Der Standardkonstruktor schaltet das Radio an mit Lautstärke 5 und der Frequenz 99.9.
+**Zu der Klasse Radio sollen folgende Methoden implementiert werden:**
+- `lauter()`, `leiser()`: Diese Methoden sollen die Lautstärke in dem im Parameter angegebenen Maß ändern (nur möglich im Zustand an).
+- `an()`, `aus()`: Diese Methoden sollen den Zustand des Attributs eingeschaltet ändern.
+- `public String toString()`: Diese Methode soll Informationen über den internen Zustand als String zurückgeben. Es soll eine Zeichenkette der Form "Radio an: Freq=98.4, Laut=2" zurückgeben werden. (Achten Sie bitte genau auf die Form der Beispielausgabe!! Weicht die Form ab, so kann Tutor Kai das Ergebnis nicht genau prüfen.)
+- `waehleSender(double frequenz)`: Diese Methode soll eine Frequenz speichern. Ist die gewählte Frequenz außerhalb des erlaubten Frequenzbereichs, so soll die Frequenz 99.9 gewählt werden.
+**Schreiben Sie eine neue Test-Klasse AppRadio, die in ihrem main()-Part ein Objekt der Klasse Radio erzeugt und in der Sie dann die Methoden testweise aufrufen können.**</t>
+  </si>
+  <si>
+    <t>Betrachten Sie das folgende UML-Diagramm:
+![image](/assets/taskImgs/UMLtoJava.svg)
+Erstellen Sie zu diesem Klassendiagramm den entsprechenden Java-Code. Beachten Sie dabei vor allem die Sichtbarkeiten!
+Implementieren Sie einen Konstruktor, der alle Attribute als Argument erhält! Implementieren Sie die Rümpfe der Methoden.</t>
+  </si>
+  <si>
+    <t>Im Rahmen einer Softwareentwicklung für die einheitliche Verwaltung von Flugzeugen wurde die Klasse *Flugzeug* entwickelt (siehe Flugzeug.java).
+Ausgehend von dieser Klasse sind zwei Klassen *Verkehrsflugzeug* und *Doppeldecker* zu erzeugen. Diese sollen folgende Spezifikationen erfüllen:
+### Klasse *Verkehrsflugzeug*:
+- Ein Verkehrsflugzeug ist ein Flugzeug, das genau ein Flügelpaar sowie eine zusätzliche Variable für die Anzahl der Passagiere hat.
+- Ein Verkehrsflugzeug fliegt keine Loopings. Stellen Sie deshalb sicher, dass die Methode *getLooping* immer `false` zurückgibt, auch in allen Unterklassen von Verkehrsflugzeug.
+- Ein Verkehrsflugzeug-Objekt kann mit Angabe des Herstellers (String), der maximalen Geschwindigkeit (int), der Immatrikulationsnummer (String) und der Anzahl der Passagiere (int) erzeugt werden.
+- Die Klasse Verkehrsflugzeug hat die Methoden *getAnzahlPassagiere* und *setAnzahlPassagiere* zum Abfragen und Setzen der Anzahl der Passagiere.
+### Klasse *Doppeldecker*:
+- Ein Doppeldecker ist ein Flugzeug, das genau zwei Flügelpaare hat.
+- Weiter ist ein Doppeldecker akrobatiktauglich, d.h. man kann damit Loopings fliegen. Für einen Looping muss der Doppeldecker eine Mindestgeschwindigkeit von 320 km/h erreichen. Definieren Sie dafür eine Konstante *LOOPINGSPEED*. Die Methode *getLooping* soll `true` zurückgeben, falls die zulässige max. Geschwindigkeit (*maxSpeed*) größer *LOOPINGSPEED* ist.
+- Die Klasse Doppeldecker hat eine Variable *offenesCockpit* vom Typ boolean. Sie gibt an, ob der Doppeldecker ein offenes oder geschlossenes Cockpit hat. Nachdem *offenesCockpit* gesetzt worden ist, darf sie nicht mehr verändert werden. Der Wert des Attributes darf gelesen werden.
+- Ein Doppeldecker-Objekt kann durch 2 Konstruktoren initianlisiert werden:
+  - a) Der 1. Konstruktor hat folgende Parameter: Hersteller (String), maximale Geschwindigkeit (int), die Immatrikulationsnummer (String) und einen boolean *offenesCockpit*, der angibt, ob der Doppeldecker ein offenes oder geschlossenes Cockpit hat.
+  - b) Der 2. Konstruktor hat folgende Parameter: Hersteller (String), maximale Geschwindigkeit (int), die Immatrikulationsnummer (int). Der Defaultwert für *offenesCockpit* bei einem Doppeldecker ist `true`.
+- Die Klasse Doppeldecker soll nicht erweiterbar sein.
+### Aufgaben
+1. Modellieren Sie die beschriebenen Klassen in einem UML-Klassendiagramm.
+2. Implementieren Sie die Klassen *Verkehrsflugzeug* und *Doppeldecker* anhand der oben genannten Eigenschaften.
+3. Implementieren Sie eine main-Klasse Airline in der Sie beliebig Objekte der Klassen Verkehrsflugzeug und Doppeldecker anlegen. Des Weiteren legen Sie eine ArrayList `flug` wie folgt an:
+   ```
+   ArrayList&lt;Flugzeug&gt; flug = new ArrayList&lt;Flugzeug&gt;();
+   ```
+   Fügen Sie der Arraylist per `flug.add()` die zuvor erzeugten Objekte der Klassen Verkehrsflugzeug und Doppeldecker hinzu! Sollte dies zu Fehlern führen, dann ist Ihre Implementierung der Klassen nicht korrekt! :-)
+4. Geben Sie die Daten der in der ArrayList gespeicherten Objekten aus, indem Sie die entsprechenden Methoden aufrufen.</t>
+  </si>
+  <si>
+    <t>**Grundlagen:** Eine quadratische Pyramide und ein Kegel haben eine Grundfläche, die durch die Angabe einer einzigen Länge bestimmt ist (beim Kegel der Radius), und eine Höhe. Aus diesen Größen lassen sich Volumen und Oberfläche dieser Körper berechnen.
+**Programmieraufgabe:** Implementieren Sie eine geeignete abstrakte Klasse und mehrere Unterklassen, um die Volumen- und Oberflächenberechnungen durchzuführen. Folgende Klassen sind zu erstellen:
+**Klassen und ihre Dateien:**
+- `Koerper.java` - Abstrakte Basis-Klasse für geometrische Körper.
+- `Pyramide.java` - Spezifische Klasse für die Pyramide.
+- `Kegel.java` - Spezifische Klasse für den Kegel.
+- `Formen.java` - Hauptklasse, die Methoden `getVolumen()` und `getFlaeche()` aufruft.</t>
+  </si>
+  <si>
+    <t>**Aufgabenstellung:**  
+Schreiben Sie ein Java-Programm **MyThread.java**, das die Summe aller Zahlen eines vorgegebenen *int*-Arrays mit Hilfe von zwei Threads berechnet. Dazu wird das Array jeweils zur Hälfte auf die beiden Threads verteilt. Jeder Thread berechnet seinen Bereich für sich. Nach Beendigung der Threads soll das Hauptprogramm die Ergebnisse aus dem Objekt lesen, die Summe berechnen und das Ergebnis ausgeben.
+**Weitere Anweisungen:**  
+Erstellen Sie eine Klasse **ArrayCalc** (**ArrayCalc.java**), die die Berechnung für einen Teil des Arrays übernimmt!
+**Hinweis:**  
+Machen Sie sich mit der **join()**-Methode der Klasse **Thread** vertraut!</t>
+  </si>
+  <si>
+    <t>Schreiben Sie eine Funktion `make_matrix`, welche eine n x n Matrix A als Liste von Listen erstellt, wobei der (i, j)-te Eintrag, \(A_{i,j}\), gleich i + j ist. Verwenden Sie hierfür zwei verschachtelte for-Schleifen.
+Das Ergebnis für `make_matrix(4)` würde wie folgt aussehen:
+|   0   |   1   |   2   |   3   |
+|-------|-------|-------|-------|
+|   1   |   2   |   3   |   4   |
+|   2   |   3   |   4   |   5   |
+|   3   |   4   |   5   |   6   |</t>
+  </si>
+  <si>
+    <t>Schreiben Sie eine Funktion **"concatenate_functions"**, die als Eingabeargument zwei Funktionen **"f1"** und **"f2"** bekommt und als Rückgabe eine Funktion liefert, die **f1(f2(x))** auswertet. Testen Sie Ihr Programm mit **f1(x) = sin(x)** und **f2(x) = 2\*pi\*x**. Hierfür müssen Sie die Bibliothek **"math"** importieren.</t>
+  </si>
+  <si>
+    <t>Schreiben Sie eine Funktion namens `potenz`, die die Potenz von x hoch a rekursiv berechnet.</t>
+  </si>
+  <si>
+    <t>Schreiben Sie eine Funktion namens `drehe_string`, die einen String rekursiv umdreht.</t>
+  </si>
+  <si>
+    <t>Schreiben Sie eine Funktion namens `mehrwertsteuer`, die 19% des gegebenen Betrags als Rückgabewert hat. 
+Schreiben Sie dann eine Funktion namens `nutze_freibetrag`, welche einen Freibetrag und eine Steuerfunktion als Eingabeparameter erhält. 
+Innerhalb der Funktion `nutze_freibetrag` soll eine neue Funktion definiert werden, die die Steuerfunktion auf ein Argument `(betrag - freibetrag)` anwendet.</t>
+  </si>
+  <si>
+    <t>Schreiben Sie eine Funktion höherer Ordnung namens `filter_liste`, die eine Funktion mit boolschem Rückgabewert und eine Liste als Eingabe entgegennimmt. Sie ruft die Funktion auf jedem Element der Liste auf und entfernt diejenigen Elemente, für die die Funktion den Rückgabewert 'False' hat.</t>
+  </si>
+  <si>
+    <t>Schreiben Sie eine Funktion höherer Ordnung namens `reduziere_liste`, die eine Funktion mit zwei Eingabeargumenten sowie eine Liste entgegennimmt.
+Hat die Liste nur ein Element, wird dieses Element zurückgegeben.
+Für Listen mit mindestens zwei Elementen wird die Funktion auf den ersten beiden Elementen und dann iterativ immer auf dem Ergebnis und dem nächsten Element der Liste aufgerufen, bis kein Element mehr übrig ist.</t>
+  </si>
+  <si>
+    <t>Schreiben Sie eine Funktion namens `fib`, die die n-te Zahl der Fibonacci-Folge rekursiv berechnet.</t>
+  </si>
+  <si>
+    <t>Für die Simulation eines Wettrennens sollen verschiedene Fahrzeugarten objektorientiert modelliert werden. Da alle Fahrzeugtypen gemeinsame Eigenschaften haben, definieren wir uns zunächst eine Basisklasse Fahrzeug, die als Oberklasse für die anderen Klassen dienen soll. Ein Fahrzeug hat folgende allgemeinen Merkmale:
+- Seine aktuelle Position (in km und der Einfachheit halber in nur einer Dimension)
+- Seine aktuelle Geschwindigkeit (in km/h)
+- Es kann bewegt werden (Methode bewege). Die Methode wird mit einem double-Parameter aufgerufen, der die Anzahl der Minuten angibt, die sich das Fahrzeug mit der aktuellen Geschwindigkeit vorwärts bewegt. Der Methodenaufruf ändert natürlich die Position des Fahrzeugs, wenn es mit einer von 0 verschiedenen Geschwindigkeit bewegt wird.
+- Man kann seine Geschwindigkeit setzen (Methode setzeGeschwindigkeit). Die Geschwindigkeit darf die Maximalgeschwindigkeit nicht überschreiten, eine korrekte Ausführung sollte protokolliert werden.
+- Es kann seine Maximalgeschwindigkeit angeben (Methode getMaxGeschwindigkeit). Für ein Objekt der Klasse Fahrzeug soll die Maximalgeschwindigkeit 0 sein.
+- Es kann die Anzahl seiner Räder angeben (Methode getAnzahlRaeder). In der Klasse Fahrzeug soll diese ebenfalls 0 sein.
+Nun sollen einige konkrete Fahrzeuge definiert werden, indem entsprechende Klassen von Fahrzeug abgeleitet werden:
+- Ein Fahrrad ist ein Fahrzeug mit 2 Rädern und Maximalgeschwindigkeit 30 km/h.
+- Ein Auto ist ein Fahrzeug mit 4 Rädern und Maximalgeschwindigkeit 140 km/h.
+- Ein Rennwagen ist ein Auto mit Maximalgeschwindigkeit 220 km/h.
+- Ein Krankenwagen ist ein Auto mit einem zusätzlichen Blaulicht, das ein- oder ausgeschaltet sein kann (Attribut: isBlaulichtAn). Um den Zustand des Blaulichts auszugeben, wird die Methode isBlaulichtAn() benötigt. Außerdem muss der Krankenwagen Methoden zum Ein- bzw. Ausschalten des Blaulichts anbieten (blaulichtAn und blaulichtAus).
+Definieren Sie diese Klassen und nutzen Sie dabei so weit wie möglich die Vererbung von Eigenschaften aus!
+Nun soll die eigentliche Simulation des Wettrennens in einer Klasse Wettrennen geschrieben werden. Erzeugen Sie je ein Fahrzeug und setzen Sie dann die Geschwindigkeiten auf:
+- Fahrrad: 20 km/h
+- Auto: 150 km/h
+- Rennwagen: 200 km/h
+- Krankenwagen: 80 km/h
+Dann sollen sich die Fahrzeuge bewegen. Der Gerechtigkeit halber geben wir dem Fahrrad einen Vorsprung von 4 Stunden. Danach lassen Sie alle Fahrzeuge eine Stunde lang mit unveränderter Geschwindigkeit vorwärts fahren. Was fällt Ihnen beim Auto auf?</t>
+  </si>
+  <si>
+    <t>In dieser Aufgabe sollst du den Bubblesort-Algorithmus in Java implementieren. Dieser Algorithmus ist ein einfaches Verfahren zum Sortieren einer Liste von Elementen (z.B. Zahlen).
+Bubblesort ist ein Sortieralgorithmus, der durch wiederholtes Durchlaufen der zu sortierenden Liste arbeitet. Bei jedem Durchlauf werden benachbarte Elemente miteinander verglichen und gegebenenfalls vertauscht. Das Besondere am Bubblesort ist, dass mit jedem Durchgang das größte Element der noch zu sortierenden Elemente an das Ende der Liste "aufsteigt".</t>
+  </si>
+  <si>
+    <t>![UML Diagram Image](https://urltodo.com/assets/taskImgs/fahrzeugUML.png)
+Schreiben Sie den Java Code für beide Klassen des UML-Diagramms.</t>
   </si>
 </sst>
 </file>
@@ -3908,13 +3833,13 @@
         <v>85</v>
       </c>
       <c r="K1" s="15" t="s">
-        <v>201</v>
+        <v>186</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>174</v>
+        <v>159</v>
       </c>
       <c r="M1" s="6" t="s">
-        <v>175</v>
+        <v>160</v>
       </c>
       <c r="N1" s="23"/>
       <c r="R1" s="25"/>
@@ -3939,10 +3864,10 @@
         <v>88</v>
       </c>
       <c r="G2" s="19" t="s">
-        <v>160</v>
-      </c>
-      <c r="H2" s="10" t="s">
-        <v>89</v>
+        <v>145</v>
+      </c>
+      <c r="H2" t="s">
+        <v>317</v>
       </c>
       <c r="I2" s="6" t="s">
         <v>4</v>
@@ -3951,13 +3876,13 @@
         <v>0</v>
       </c>
       <c r="K2" s="16" t="s">
-        <v>200</v>
+        <v>185</v>
       </c>
       <c r="L2" s="7" t="s">
-        <v>176</v>
+        <v>161</v>
       </c>
       <c r="M2" s="6" t="s">
-        <v>202</v>
+        <v>187</v>
       </c>
       <c r="N2" s="23"/>
       <c r="R2" s="25"/>
@@ -3976,16 +3901,16 @@
         <v>36</v>
       </c>
       <c r="E3" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="F3" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="F3" s="10" t="s">
-        <v>91</v>
-      </c>
       <c r="G3" s="19" t="s">
-        <v>161</v>
-      </c>
-      <c r="H3" s="10" t="s">
-        <v>92</v>
+        <v>146</v>
+      </c>
+      <c r="H3" t="s">
+        <v>318</v>
       </c>
       <c r="I3" s="6" t="s">
         <v>6</v>
@@ -3994,13 +3919,13 @@
         <v>0</v>
       </c>
       <c r="K3" s="16" t="s">
-        <v>200</v>
+        <v>185</v>
       </c>
       <c r="L3" s="7" t="s">
-        <v>177</v>
+        <v>162</v>
       </c>
       <c r="M3" s="6" t="s">
-        <v>178</v>
+        <v>163</v>
       </c>
       <c r="N3" s="23"/>
       <c r="R3" s="25"/>
@@ -4019,16 +3944,16 @@
         <v>34</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="G4" s="19" t="s">
-        <v>162</v>
-      </c>
-      <c r="H4" s="10" t="s">
-        <v>274</v>
+        <v>147</v>
+      </c>
+      <c r="H4" t="s">
+        <v>319</v>
       </c>
       <c r="I4" s="6" t="s">
         <v>7</v>
@@ -4037,10 +3962,10 @@
         <v>0</v>
       </c>
       <c r="K4" s="16" t="s">
-        <v>200</v>
+        <v>185</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>179</v>
+        <v>164</v>
       </c>
       <c r="M4" s="6">
         <v>174</v>
@@ -4062,16 +3987,16 @@
         <v>34</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="G5" s="11" t="s">
-        <v>163</v>
-      </c>
-      <c r="H5" s="10" t="s">
-        <v>277</v>
+        <v>148</v>
+      </c>
+      <c r="H5" t="s">
+        <v>320</v>
       </c>
       <c r="I5" s="6" t="s">
         <v>8</v>
@@ -4080,10 +4005,10 @@
         <v>0</v>
       </c>
       <c r="K5" s="12" t="s">
-        <v>200</v>
+        <v>185</v>
       </c>
       <c r="L5" s="7" t="s">
-        <v>203</v>
+        <v>188</v>
       </c>
       <c r="M5" s="6">
         <v>47</v>
@@ -4105,16 +4030,16 @@
         <v>23</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>346</v>
+        <v>311</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>344</v>
-      </c>
-      <c r="H6" s="10" t="s">
-        <v>345</v>
+        <v>310</v>
+      </c>
+      <c r="H6" t="s">
+        <v>321</v>
       </c>
       <c r="I6" s="6" t="s">
         <v>9</v>
@@ -4123,17 +4048,17 @@
         <v>0</v>
       </c>
       <c r="K6" s="12" t="s">
-        <v>200</v>
+        <v>185</v>
       </c>
       <c r="L6" s="7" t="s">
-        <v>204</v>
+        <v>189</v>
       </c>
       <c r="M6" s="6" t="s">
-        <v>205</v>
+        <v>190</v>
       </c>
       <c r="N6" s="23"/>
       <c r="R6" s="26" t="s">
-        <v>343</v>
+        <v>309</v>
       </c>
     </row>
     <row r="7" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4150,16 +4075,16 @@
         <v>34</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="G7" s="19" t="s">
-        <v>164</v>
-      </c>
-      <c r="H7" s="10" t="s">
-        <v>100</v>
+        <v>149</v>
+      </c>
+      <c r="H7" t="s">
+        <v>322</v>
       </c>
       <c r="I7" s="6" t="s">
         <v>10</v>
@@ -4168,13 +4093,13 @@
         <v>0</v>
       </c>
       <c r="K7" s="16" t="s">
-        <v>200</v>
+        <v>185</v>
       </c>
       <c r="L7" s="7" t="s">
-        <v>206</v>
+        <v>191</v>
       </c>
       <c r="M7" s="6" t="s">
-        <v>271</v>
+        <v>254</v>
       </c>
       <c r="N7" s="23"/>
       <c r="R7" s="25"/>
@@ -4193,16 +4118,16 @@
         <v>34</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="G8" s="19" t="s">
-        <v>165</v>
-      </c>
-      <c r="H8" s="10" t="s">
-        <v>309</v>
+        <v>150</v>
+      </c>
+      <c r="H8" t="s">
+        <v>323</v>
       </c>
       <c r="I8" s="6" t="s">
         <v>11</v>
@@ -4211,13 +4136,13 @@
         <v>0</v>
       </c>
       <c r="K8" s="16" t="s">
-        <v>200</v>
+        <v>185</v>
       </c>
       <c r="L8" s="7" t="s">
-        <v>207</v>
+        <v>192</v>
       </c>
       <c r="M8" s="6" t="s">
-        <v>208</v>
+        <v>193</v>
       </c>
       <c r="N8" s="23"/>
       <c r="R8" s="25"/>
@@ -4236,16 +4161,16 @@
         <v>26</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>272</v>
+        <v>255</v>
       </c>
       <c r="G9" s="19" t="s">
-        <v>166</v>
-      </c>
-      <c r="H9" s="10" t="s">
-        <v>273</v>
+        <v>151</v>
+      </c>
+      <c r="H9" t="s">
+        <v>324</v>
       </c>
       <c r="I9" s="6" t="s">
         <v>12</v>
@@ -4254,10 +4179,10 @@
         <v>0</v>
       </c>
       <c r="K9" s="16" t="s">
-        <v>200</v>
+        <v>185</v>
       </c>
       <c r="L9" s="7" t="s">
-        <v>209</v>
+        <v>194</v>
       </c>
       <c r="M9" s="6">
         <v>10</v>
@@ -4273,22 +4198,22 @@
         <v>6</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D10" s="9">
         <v>63</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="G10" s="11" t="s">
-        <v>297</v>
-      </c>
-      <c r="H10" s="10" t="s">
-        <v>107</v>
+        <v>275</v>
+      </c>
+      <c r="H10" t="s">
+        <v>325</v>
       </c>
       <c r="I10" s="6" t="s">
         <v>13</v>
@@ -4297,12 +4222,12 @@
         <v>0</v>
       </c>
       <c r="K10" s="12" t="s">
-        <v>180</v>
+        <v>165</v>
       </c>
       <c r="L10" s="7"/>
       <c r="N10" s="23"/>
       <c r="R10" s="26" t="s">
-        <v>305</v>
+        <v>281</v>
       </c>
     </row>
     <row r="11" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4313,22 +4238,22 @@
         <v>6</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D11" s="9">
         <v>65</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="F11" s="10" t="s">
-        <v>263</v>
+        <v>248</v>
       </c>
       <c r="G11" s="11" t="s">
-        <v>218</v>
-      </c>
-      <c r="H11" s="10" t="s">
-        <v>264</v>
+        <v>203</v>
+      </c>
+      <c r="H11" t="s">
+        <v>326</v>
       </c>
       <c r="I11" s="6" t="s">
         <v>14</v>
@@ -4337,12 +4262,12 @@
         <v>0</v>
       </c>
       <c r="K11" s="12" t="s">
-        <v>181</v>
+        <v>166</v>
       </c>
       <c r="L11" s="7"/>
       <c r="N11" s="23"/>
       <c r="R11" s="26" t="s">
-        <v>299</v>
+        <v>277</v>
       </c>
     </row>
     <row r="12" spans="1:18" s="14" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4353,22 +4278,22 @@
         <v>6</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D12" s="14">
         <v>63</v>
       </c>
       <c r="E12" s="14" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="F12" s="14" t="s">
-        <v>278</v>
+        <v>258</v>
       </c>
       <c r="G12" s="21" t="s">
-        <v>219</v>
-      </c>
-      <c r="H12" s="21" t="s">
-        <v>300</v>
+        <v>204</v>
+      </c>
+      <c r="H12" t="s">
+        <v>327</v>
       </c>
       <c r="I12" s="14" t="s">
         <v>15</v>
@@ -4377,11 +4302,11 @@
         <v>1</v>
       </c>
       <c r="K12" s="14" t="s">
-        <v>182</v>
+        <v>167</v>
       </c>
       <c r="N12" s="23"/>
       <c r="R12" s="27" t="s">
-        <v>301</v>
+        <v>278</v>
       </c>
     </row>
     <row r="13" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4392,22 +4317,22 @@
         <v>6</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D13" s="9">
         <v>63</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="F13" s="10" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="G13" s="11" t="s">
-        <v>220</v>
-      </c>
-      <c r="H13" s="10" t="s">
-        <v>112</v>
+        <v>205</v>
+      </c>
+      <c r="H13" t="s">
+        <v>328</v>
       </c>
       <c r="I13" s="6" t="s">
         <v>16</v>
@@ -4416,7 +4341,7 @@
         <v>0</v>
       </c>
       <c r="K13" s="12" t="s">
-        <v>183</v>
+        <v>168</v>
       </c>
       <c r="L13" s="7"/>
       <c r="N13" s="23"/>
@@ -4430,22 +4355,22 @@
         <v>7</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D14" s="14">
         <v>69</v>
       </c>
       <c r="E14" s="14" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="F14" s="14" t="s">
-        <v>281</v>
+        <v>261</v>
       </c>
       <c r="G14" s="14" t="s">
-        <v>221</v>
-      </c>
-      <c r="H14" s="14" t="s">
-        <v>282</v>
+        <v>206</v>
+      </c>
+      <c r="H14" t="s">
+        <v>329</v>
       </c>
       <c r="I14" s="14" t="s">
         <v>17</v>
@@ -4454,11 +4379,11 @@
         <v>1</v>
       </c>
       <c r="K14" s="14" t="s">
-        <v>184</v>
+        <v>169</v>
       </c>
       <c r="N14" s="23"/>
       <c r="R14" s="27" t="s">
-        <v>306</v>
+        <v>282</v>
       </c>
     </row>
     <row r="15" spans="1:18" s="6" customFormat="1" ht="409.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -4469,22 +4394,22 @@
         <v>7</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D15" s="9">
         <v>70</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>222</v>
-      </c>
-      <c r="H15" s="10" t="s">
-        <v>116</v>
+        <v>207</v>
+      </c>
+      <c r="H15" t="s">
+        <v>330</v>
       </c>
       <c r="I15" s="6" t="s">
         <v>18</v>
@@ -4493,7 +4418,7 @@
         <v>0</v>
       </c>
       <c r="K15" s="12" t="s">
-        <v>185</v>
+        <v>170</v>
       </c>
       <c r="L15" s="7"/>
       <c r="N15" s="23"/>
@@ -4507,22 +4432,22 @@
         <v>7</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D16" s="14">
         <v>64</v>
       </c>
       <c r="E16" s="14" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="F16" s="21" t="s">
-        <v>283</v>
+        <v>262</v>
       </c>
       <c r="G16" s="14" t="s">
-        <v>223</v>
-      </c>
-      <c r="H16" s="14" t="s">
-        <v>284</v>
+        <v>208</v>
+      </c>
+      <c r="H16" t="s">
+        <v>331</v>
       </c>
       <c r="I16" s="14" t="s">
         <v>19</v>
@@ -4531,7 +4456,7 @@
         <v>2</v>
       </c>
       <c r="K16" s="14" t="s">
-        <v>186</v>
+        <v>171</v>
       </c>
       <c r="N16" s="23"/>
       <c r="R16" s="28"/>
@@ -4544,22 +4469,22 @@
         <v>8</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D17" s="9">
         <v>85</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="F17" s="10" t="s">
-        <v>350</v>
+        <v>314</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>348</v>
-      </c>
-      <c r="H17" s="10" t="s">
-        <v>349</v>
+        <v>313</v>
+      </c>
+      <c r="H17" t="s">
+        <v>332</v>
       </c>
       <c r="I17" s="10" t="s">
         <v>20</v>
@@ -4568,11 +4493,11 @@
         <v>0</v>
       </c>
       <c r="K17" s="12" t="s">
-        <v>187</v>
+        <v>172</v>
       </c>
       <c r="L17" s="7"/>
       <c r="N17" s="21" t="s">
-        <v>318</v>
+        <v>289</v>
       </c>
       <c r="R17" s="25"/>
     </row>
@@ -4584,22 +4509,22 @@
         <v>8</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D18" s="9">
         <v>84</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="F18" s="10" t="s">
-        <v>265</v>
+        <v>249</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>224</v>
-      </c>
-      <c r="H18" s="10" t="s">
-        <v>266</v>
+        <v>209</v>
+      </c>
+      <c r="H18" t="s">
+        <v>333</v>
       </c>
       <c r="I18" s="6" t="s">
         <v>25</v>
@@ -4608,7 +4533,7 @@
         <v>0</v>
       </c>
       <c r="K18" s="12" t="s">
-        <v>188</v>
+        <v>173</v>
       </c>
       <c r="L18" s="7"/>
       <c r="N18" s="23"/>
@@ -4622,22 +4547,22 @@
         <v>8</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D19" s="9">
         <v>93</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="F19" s="10" t="s">
-        <v>302</v>
+        <v>279</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>225</v>
-      </c>
-      <c r="H19" s="10" t="s">
-        <v>303</v>
+        <v>210</v>
+      </c>
+      <c r="H19" t="s">
+        <v>334</v>
       </c>
       <c r="I19" s="6" t="s">
         <v>29</v>
@@ -4646,7 +4571,7 @@
         <v>0</v>
       </c>
       <c r="K19" s="12" t="s">
-        <v>189</v>
+        <v>174</v>
       </c>
       <c r="L19" s="7"/>
       <c r="N19" s="23"/>
@@ -4660,22 +4585,22 @@
         <v>8</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D20" s="9">
         <v>69</v>
       </c>
       <c r="E20" s="13" t="s">
-        <v>121</v>
+        <v>115</v>
       </c>
       <c r="F20" s="10" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>226</v>
-      </c>
-      <c r="H20" s="10" t="s">
-        <v>123</v>
+        <v>211</v>
+      </c>
+      <c r="H20" t="s">
+        <v>335</v>
       </c>
       <c r="I20" s="13" t="s">
         <v>30</v>
@@ -4684,7 +4609,7 @@
         <v>0</v>
       </c>
       <c r="K20" s="12" t="s">
-        <v>190</v>
+        <v>175</v>
       </c>
       <c r="L20" s="7"/>
       <c r="N20" s="23"/>
@@ -4698,22 +4623,22 @@
         <v>9</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D21" s="9">
         <v>78</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="F21" s="10" t="s">
-        <v>267</v>
+        <v>250</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>315</v>
-      </c>
-      <c r="H21" s="14" t="s">
-        <v>310</v>
+        <v>287</v>
+      </c>
+      <c r="H21" t="s">
+        <v>336</v>
       </c>
       <c r="I21" s="6" t="s">
         <v>32</v>
@@ -4722,7 +4647,7 @@
         <v>0</v>
       </c>
       <c r="K21" s="12" t="s">
-        <v>191</v>
+        <v>176</v>
       </c>
       <c r="L21" s="7"/>
       <c r="N21" s="23"/>
@@ -4736,22 +4661,22 @@
         <v>9</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D22" s="9">
         <v>75</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="F22" s="10" t="s">
-        <v>268</v>
+        <v>251</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>319</v>
-      </c>
-      <c r="H22" s="14" t="s">
-        <v>311</v>
+        <v>290</v>
+      </c>
+      <c r="H22" t="s">
+        <v>337</v>
       </c>
       <c r="I22" s="10" t="s">
         <v>34</v>
@@ -4760,7 +4685,7 @@
         <v>0</v>
       </c>
       <c r="K22" s="12" t="s">
-        <v>192</v>
+        <v>177</v>
       </c>
       <c r="L22" s="7"/>
       <c r="N22" s="21"/>
@@ -4774,22 +4699,22 @@
         <v>9</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D23" s="9">
         <v>78</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="F23" s="10" t="s">
-        <v>316</v>
+        <v>288</v>
       </c>
       <c r="G23" s="7" t="s">
-        <v>337</v>
-      </c>
-      <c r="H23" s="21" t="s">
-        <v>317</v>
+        <v>303</v>
+      </c>
+      <c r="H23" t="s">
+        <v>338</v>
       </c>
       <c r="I23" s="10" t="s">
         <v>36</v>
@@ -4798,11 +4723,11 @@
         <v>0</v>
       </c>
       <c r="K23" s="12" t="s">
-        <v>193</v>
+        <v>178</v>
       </c>
       <c r="L23" s="7"/>
       <c r="N23" s="21" t="s">
-        <v>318</v>
+        <v>289</v>
       </c>
       <c r="R23" s="25"/>
     </row>
@@ -4814,22 +4739,22 @@
         <v>9</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D24" s="9">
         <v>75</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>127</v>
+        <v>120</v>
       </c>
       <c r="F24" s="10" t="s">
-        <v>269</v>
+        <v>252</v>
       </c>
       <c r="G24" s="7" t="s">
-        <v>227</v>
-      </c>
-      <c r="H24" s="14" t="s">
-        <v>312</v>
+        <v>212</v>
+      </c>
+      <c r="H24" t="s">
+        <v>339</v>
       </c>
       <c r="I24" s="10" t="s">
         <v>38</v>
@@ -4838,7 +4763,7 @@
         <v>0</v>
       </c>
       <c r="K24" s="12" t="s">
-        <v>194</v>
+        <v>179</v>
       </c>
       <c r="L24" s="7"/>
       <c r="N24" s="14"/>
@@ -4852,22 +4777,22 @@
         <v>11</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D25" s="9">
         <v>85</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="F25" s="10" t="s">
-        <v>351</v>
+        <v>315</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>321</v>
-      </c>
-      <c r="H25" s="10" t="s">
-        <v>352</v>
+        <v>292</v>
+      </c>
+      <c r="H25" t="s">
+        <v>340</v>
       </c>
       <c r="I25" s="10" t="s">
         <v>39</v>
@@ -4876,7 +4801,7 @@
         <v>0</v>
       </c>
       <c r="K25" s="12" t="s">
-        <v>195</v>
+        <v>180</v>
       </c>
       <c r="L25" s="7"/>
       <c r="N25" s="14"/>
@@ -4890,22 +4815,22 @@
         <v>11</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D26" s="9">
         <v>78</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="F26" s="10" t="s">
-        <v>322</v>
+        <v>293</v>
       </c>
       <c r="G26" s="7" t="s">
-        <v>324</v>
-      </c>
-      <c r="H26" s="10" t="s">
-        <v>323</v>
+        <v>294</v>
+      </c>
+      <c r="H26" t="s">
+        <v>341</v>
       </c>
       <c r="I26" s="10" t="s">
         <v>41</v>
@@ -4914,11 +4839,11 @@
         <v>0</v>
       </c>
       <c r="K26" s="12" t="s">
-        <v>196</v>
+        <v>181</v>
       </c>
       <c r="L26" s="7"/>
       <c r="N26" s="14" t="s">
-        <v>325</v>
+        <v>295</v>
       </c>
       <c r="R26" s="25"/>
     </row>
@@ -4930,22 +4855,22 @@
         <v>11</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D27" s="9">
         <v>95</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="F27" s="10" t="s">
-        <v>270</v>
+        <v>253</v>
       </c>
       <c r="G27" s="7" t="s">
-        <v>228</v>
-      </c>
-      <c r="H27" s="10" t="s">
-        <v>326</v>
+        <v>213</v>
+      </c>
+      <c r="H27" t="s">
+        <v>342</v>
       </c>
       <c r="I27" s="10" t="s">
         <v>46</v>
@@ -4954,7 +4879,7 @@
         <v>0</v>
       </c>
       <c r="K27" s="12" t="s">
-        <v>197</v>
+        <v>182</v>
       </c>
       <c r="L27" s="7"/>
       <c r="N27" s="14"/>
@@ -4968,22 +4893,22 @@
         <v>11</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D28" s="9">
         <v>107</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="F28" s="10" t="s">
-        <v>328</v>
+        <v>297</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>330</v>
-      </c>
-      <c r="H28" s="10" t="s">
-        <v>329</v>
+        <v>298</v>
+      </c>
+      <c r="H28" t="s">
+        <v>343</v>
       </c>
       <c r="I28" s="10" t="s">
         <v>48</v>
@@ -4992,7 +4917,7 @@
         <v>0</v>
       </c>
       <c r="K28" s="12" t="s">
-        <v>198</v>
+        <v>183</v>
       </c>
       <c r="L28" s="7"/>
       <c r="N28" s="14"/>
@@ -5012,16 +4937,16 @@
         <v>40</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>290</v>
+        <v>268</v>
       </c>
       <c r="F29" s="10" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="G29" s="18" t="s">
-        <v>167</v>
-      </c>
-      <c r="H29" s="10" t="s">
-        <v>133</v>
+        <v>152</v>
+      </c>
+      <c r="H29" t="s">
+        <v>344</v>
       </c>
       <c r="I29" s="6" t="s">
         <v>50</v>
@@ -5030,10 +4955,10 @@
         <v>0</v>
       </c>
       <c r="K29" s="16" t="s">
-        <v>200</v>
+        <v>185</v>
       </c>
       <c r="L29" s="7" t="s">
-        <v>210</v>
+        <v>195</v>
       </c>
       <c r="M29" s="6">
         <v>3</v>
@@ -5043,7 +4968,7 @@
         <v>51</v>
       </c>
       <c r="Q29" s="13" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="R29" s="25"/>
     </row>
@@ -5061,16 +4986,16 @@
         <v>26</v>
       </c>
       <c r="E30" s="13" t="s">
-        <v>291</v>
+        <v>269</v>
       </c>
       <c r="F30" s="10" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="G30" s="7" t="s">
-        <v>338</v>
-      </c>
-      <c r="H30" s="10" t="s">
-        <v>136</v>
+        <v>304</v>
+      </c>
+      <c r="H30" t="s">
+        <v>345</v>
       </c>
       <c r="I30" s="6" t="s">
         <v>52</v>
@@ -5079,20 +5004,20 @@
         <v>0</v>
       </c>
       <c r="K30" s="12" t="s">
-        <v>200</v>
+        <v>185</v>
       </c>
       <c r="L30" s="6" t="s">
-        <v>275</v>
+        <v>256</v>
       </c>
       <c r="M30" s="6" t="s">
-        <v>276</v>
+        <v>257</v>
       </c>
       <c r="N30" s="14"/>
       <c r="P30" s="10" t="s">
         <v>53</v>
       </c>
       <c r="Q30" s="13" t="s">
-        <v>137</v>
+        <v>128</v>
       </c>
       <c r="R30" s="25"/>
     </row>
@@ -5110,16 +5035,16 @@
         <v>34</v>
       </c>
       <c r="E31" s="13" t="s">
-        <v>292</v>
+        <v>270</v>
       </c>
       <c r="F31" s="10" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="G31" s="18" t="s">
-        <v>168</v>
-      </c>
-      <c r="H31" s="10" t="s">
-        <v>139</v>
+        <v>153</v>
+      </c>
+      <c r="H31" t="s">
+        <v>346</v>
       </c>
       <c r="I31" s="6" t="s">
         <v>54</v>
@@ -5128,20 +5053,20 @@
         <v>0</v>
       </c>
       <c r="K31" s="16" t="s">
-        <v>200</v>
+        <v>185</v>
       </c>
       <c r="L31" s="14" t="s">
-        <v>211</v>
+        <v>196</v>
       </c>
       <c r="M31" s="14" t="s">
-        <v>212</v>
+        <v>197</v>
       </c>
       <c r="N31" s="23"/>
       <c r="P31" s="10" t="s">
         <v>55</v>
       </c>
       <c r="Q31" s="13" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="R31" s="25"/>
     </row>
@@ -5159,16 +5084,16 @@
         <v>34</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>293</v>
+        <v>271</v>
       </c>
       <c r="F32" s="10" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="G32" s="18" t="s">
-        <v>169</v>
-      </c>
-      <c r="H32" s="10" t="s">
-        <v>142</v>
+        <v>154</v>
+      </c>
+      <c r="H32" t="s">
+        <v>347</v>
       </c>
       <c r="I32" s="6" t="s">
         <v>56</v>
@@ -5177,20 +5102,20 @@
         <v>0</v>
       </c>
       <c r="K32" s="16" t="s">
-        <v>200</v>
+        <v>185</v>
       </c>
       <c r="L32" s="7" t="s">
-        <v>213</v>
+        <v>198</v>
       </c>
       <c r="M32" s="6" t="s">
-        <v>214</v>
+        <v>199</v>
       </c>
       <c r="N32" s="23"/>
       <c r="P32" s="10" t="s">
         <v>57</v>
       </c>
       <c r="Q32" s="13" t="s">
-        <v>143</v>
+        <v>132</v>
       </c>
       <c r="R32" s="25"/>
     </row>
@@ -5208,16 +5133,16 @@
         <v>26</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>294</v>
+        <v>272</v>
       </c>
       <c r="F33" s="10" t="s">
-        <v>144</v>
+        <v>133</v>
       </c>
       <c r="G33" s="7" t="s">
-        <v>170</v>
-      </c>
-      <c r="H33" s="10" t="s">
-        <v>145</v>
+        <v>155</v>
+      </c>
+      <c r="H33" t="s">
+        <v>348</v>
       </c>
       <c r="I33" s="6" t="s">
         <v>58</v>
@@ -5226,20 +5151,20 @@
         <v>0</v>
       </c>
       <c r="K33" s="12" t="s">
-        <v>200</v>
+        <v>185</v>
       </c>
       <c r="L33" s="7" t="s">
-        <v>340</v>
+        <v>306</v>
       </c>
       <c r="M33" s="6" t="s">
-        <v>339</v>
+        <v>305</v>
       </c>
       <c r="N33" s="14"/>
       <c r="P33" s="10" t="s">
         <v>59</v>
       </c>
       <c r="Q33" s="13" t="s">
-        <v>146</v>
+        <v>134</v>
       </c>
       <c r="R33" s="25"/>
     </row>
@@ -5257,16 +5182,16 @@
         <v>28</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>295</v>
+        <v>273</v>
       </c>
       <c r="F34" s="10" t="s">
-        <v>147</v>
+        <v>135</v>
       </c>
       <c r="G34" s="7" t="s">
-        <v>171</v>
-      </c>
-      <c r="H34" s="10" t="s">
-        <v>148</v>
+        <v>156</v>
+      </c>
+      <c r="H34" t="s">
+        <v>349</v>
       </c>
       <c r="I34" s="6" t="s">
         <v>60</v>
@@ -5275,20 +5200,20 @@
         <v>0</v>
       </c>
       <c r="K34" s="12" t="s">
-        <v>200</v>
+        <v>185</v>
       </c>
       <c r="L34" s="7" t="s">
-        <v>341</v>
+        <v>307</v>
       </c>
       <c r="M34" s="6" t="s">
-        <v>342</v>
+        <v>308</v>
       </c>
       <c r="N34" s="14"/>
       <c r="P34" s="10" t="s">
         <v>61</v>
       </c>
       <c r="Q34" s="13" t="s">
-        <v>149</v>
+        <v>136</v>
       </c>
       <c r="R34" s="25"/>
     </row>
@@ -5306,16 +5231,16 @@
         <v>26</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>296</v>
+        <v>274</v>
       </c>
       <c r="F35" s="10" t="s">
-        <v>150</v>
+        <v>137</v>
       </c>
       <c r="G35" s="18" t="s">
-        <v>172</v>
-      </c>
-      <c r="H35" s="10" t="s">
-        <v>151</v>
+        <v>157</v>
+      </c>
+      <c r="H35" t="s">
+        <v>350</v>
       </c>
       <c r="I35" s="6" t="s">
         <v>62</v>
@@ -5324,20 +5249,20 @@
         <v>0</v>
       </c>
       <c r="K35" s="16" t="s">
+        <v>185</v>
+      </c>
+      <c r="L35" s="7" t="s">
         <v>200</v>
       </c>
-      <c r="L35" s="7" t="s">
-        <v>215</v>
-      </c>
       <c r="M35" s="6" t="s">
-        <v>216</v>
+        <v>201</v>
       </c>
       <c r="N35" s="23"/>
       <c r="P35" s="10" t="s">
         <v>63</v>
       </c>
       <c r="Q35" s="13" t="s">
-        <v>152</v>
+        <v>138</v>
       </c>
       <c r="R35" s="25"/>
     </row>
@@ -5355,16 +5280,16 @@
         <v>34</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>289</v>
+        <v>267</v>
       </c>
       <c r="F36" s="10" t="s">
-        <v>153</v>
+        <v>139</v>
       </c>
       <c r="G36" s="18" t="s">
-        <v>173</v>
-      </c>
-      <c r="H36" s="10" t="s">
-        <v>154</v>
+        <v>158</v>
+      </c>
+      <c r="H36" t="s">
+        <v>351</v>
       </c>
       <c r="I36" s="6" t="s">
         <v>64</v>
@@ -5373,10 +5298,10 @@
         <v>0</v>
       </c>
       <c r="K36" s="16" t="s">
-        <v>200</v>
+        <v>185</v>
       </c>
       <c r="L36" s="7" t="s">
-        <v>217</v>
+        <v>202</v>
       </c>
       <c r="M36" s="6">
         <v>5</v>
@@ -5386,7 +5311,7 @@
         <v>65</v>
       </c>
       <c r="Q36" s="13" t="s">
-        <v>155</v>
+        <v>140</v>
       </c>
       <c r="R36" s="25"/>
     </row>
@@ -5398,22 +5323,22 @@
         <v>97</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D37" s="9">
         <v>97</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>288</v>
+        <v>266</v>
       </c>
       <c r="F37" s="10" t="s">
-        <v>354</v>
+        <v>316</v>
       </c>
       <c r="G37" s="7" t="s">
-        <v>229</v>
-      </c>
-      <c r="H37" s="10" t="s">
-        <v>353</v>
+        <v>214</v>
+      </c>
+      <c r="H37" t="s">
+        <v>352</v>
       </c>
       <c r="I37" s="6" t="s">
         <v>73</v>
@@ -5422,7 +5347,7 @@
         <v>0</v>
       </c>
       <c r="K37" s="12" t="s">
-        <v>199</v>
+        <v>184</v>
       </c>
       <c r="L37" s="7"/>
       <c r="N37" s="14"/>
@@ -5430,7 +5355,7 @@
         <v>67</v>
       </c>
       <c r="Q37" s="13" t="s">
-        <v>156</v>
+        <v>141</v>
       </c>
       <c r="R37" s="25"/>
     </row>
@@ -5442,22 +5367,22 @@
         <v>67</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D38" s="9">
         <v>67</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>286</v>
+        <v>264</v>
       </c>
       <c r="F38" s="10" t="s">
-        <v>157</v>
+        <v>142</v>
       </c>
       <c r="G38" s="7" t="s">
-        <v>332</v>
-      </c>
-      <c r="H38" s="10" t="s">
-        <v>331</v>
+        <v>299</v>
+      </c>
+      <c r="H38" t="s">
+        <v>353</v>
       </c>
       <c r="I38" s="6" t="s">
         <v>74</v>
@@ -5466,7 +5391,7 @@
         <v>0</v>
       </c>
       <c r="K38" s="12" t="s">
-        <v>313</v>
+        <v>285</v>
       </c>
       <c r="L38" s="7"/>
       <c r="N38" s="14"/>
@@ -5474,7 +5399,7 @@
         <v>75</v>
       </c>
       <c r="Q38" s="13" t="s">
-        <v>158</v>
+        <v>143</v>
       </c>
       <c r="R38" s="25"/>
     </row>
@@ -5486,31 +5411,31 @@
         <v>85</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D39" s="9">
         <v>85</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>287</v>
+        <v>265</v>
       </c>
       <c r="F39" s="10" t="s">
-        <v>336</v>
+        <v>302</v>
       </c>
       <c r="G39" s="7" t="s">
-        <v>230</v>
-      </c>
-      <c r="H39" s="10" t="s">
-        <v>333</v>
+        <v>215</v>
+      </c>
+      <c r="H39" t="s">
+        <v>354</v>
       </c>
       <c r="I39" s="10" t="s">
-        <v>334</v>
+        <v>300</v>
       </c>
       <c r="J39" s="9">
         <v>0</v>
       </c>
       <c r="K39" s="12" t="s">
-        <v>314</v>
+        <v>286</v>
       </c>
       <c r="L39" s="7"/>
       <c r="N39" s="14"/>
@@ -5518,7 +5443,7 @@
         <v>69</v>
       </c>
       <c r="Q39" s="13" t="s">
-        <v>159</v>
+        <v>144</v>
       </c>
       <c r="R39" s="25"/>
     </row>
@@ -5687,7 +5612,7 @@
         <v>13</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>304</v>
+        <v>280</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5702,7 +5627,7 @@
         <v>14</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>298</v>
+        <v>276</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5717,7 +5642,7 @@
         <v>15</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>279</v>
+        <v>259</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5732,7 +5657,7 @@
         <v>16</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>231</v>
+        <v>216</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5747,7 +5672,7 @@
         <v>17</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>280</v>
+        <v>260</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5762,7 +5687,7 @@
         <v>18</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>347</v>
+        <v>312</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5777,7 +5702,7 @@
         <v>19</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>285</v>
+        <v>263</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5792,7 +5717,7 @@
         <v>20</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>307</v>
+        <v>283</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5807,7 +5732,7 @@
         <v>21</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>232</v>
+        <v>217</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5822,7 +5747,7 @@
         <v>22</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>233</v>
+        <v>218</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5837,7 +5762,7 @@
         <v>23</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>234</v>
+        <v>219</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5852,7 +5777,7 @@
         <v>24</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>235</v>
+        <v>220</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5867,7 +5792,7 @@
         <v>25</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>236</v>
+        <v>221</v>
       </c>
     </row>
     <row r="23" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5882,7 +5807,7 @@
         <v>26</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>237</v>
+        <v>222</v>
       </c>
     </row>
     <row r="24" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5897,7 +5822,7 @@
         <v>27</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>238</v>
+        <v>223</v>
       </c>
     </row>
     <row r="25" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5912,7 +5837,7 @@
         <v>28</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>239</v>
+        <v>224</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5927,7 +5852,7 @@
         <v>29</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>240</v>
+        <v>225</v>
       </c>
     </row>
     <row r="27" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5942,7 +5867,7 @@
         <v>30</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>308</v>
+        <v>284</v>
       </c>
     </row>
     <row r="28" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5956,7 +5881,7 @@
         <v>31</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>241</v>
+        <v>226</v>
       </c>
     </row>
     <row r="29" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5970,7 +5895,7 @@
         <v>32</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>242</v>
+        <v>227</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5984,7 +5909,7 @@
         <v>33</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>243</v>
+        <v>228</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -5998,7 +5923,7 @@
         <v>34</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>244</v>
+        <v>229</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6012,7 +5937,7 @@
         <v>35</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>245</v>
+        <v>230</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6026,7 +5951,7 @@
         <v>36</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>246</v>
+        <v>231</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6040,7 +5965,7 @@
         <v>37</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>247</v>
+        <v>232</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6054,7 +5979,7 @@
         <v>38</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>248</v>
+        <v>233</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6068,7 +5993,7 @@
         <v>39</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>320</v>
+        <v>291</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6082,7 +6007,7 @@
         <v>40</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>249</v>
+        <v>234</v>
       </c>
     </row>
     <row r="38" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6096,7 +6021,7 @@
         <v>41</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>250</v>
+        <v>235</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6110,7 +6035,7 @@
         <v>42</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>251</v>
+        <v>236</v>
       </c>
     </row>
     <row r="40" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6124,7 +6049,7 @@
         <v>43</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>252</v>
+        <v>237</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6138,7 +6063,7 @@
         <v>44</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>253</v>
+        <v>238</v>
       </c>
     </row>
     <row r="42" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6152,7 +6077,7 @@
         <v>45</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>254</v>
+        <v>239</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6166,7 +6091,7 @@
         <v>46</v>
       </c>
       <c r="D43" s="5" t="s">
-        <v>327</v>
+        <v>296</v>
       </c>
     </row>
     <row r="44" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6180,7 +6105,7 @@
         <v>47</v>
       </c>
       <c r="D44" s="5" t="s">
-        <v>255</v>
+        <v>240</v>
       </c>
     </row>
     <row r="45" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6194,7 +6119,7 @@
         <v>48</v>
       </c>
       <c r="D45" s="5" t="s">
-        <v>256</v>
+        <v>241</v>
       </c>
     </row>
     <row r="46" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6208,7 +6133,7 @@
         <v>49</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>257</v>
+        <v>242</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6334,7 +6259,7 @@
         <v>66</v>
       </c>
       <c r="D55" s="5" t="s">
-        <v>258</v>
+        <v>243</v>
       </c>
     </row>
     <row r="56" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6348,7 +6273,7 @@
         <v>68</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>259</v>
+        <v>244</v>
       </c>
     </row>
     <row r="57" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6362,7 +6287,7 @@
         <v>70</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>259</v>
+        <v>244</v>
       </c>
     </row>
     <row r="58" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6376,7 +6301,7 @@
         <v>71</v>
       </c>
       <c r="D58" s="2" t="s">
-        <v>259</v>
+        <v>244</v>
       </c>
     </row>
     <row r="59" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6390,7 +6315,7 @@
         <v>72</v>
       </c>
       <c r="D59" s="2" t="s">
-        <v>259</v>
+        <v>244</v>
       </c>
     </row>
     <row r="60" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6404,7 +6329,7 @@
         <v>73</v>
       </c>
       <c r="D60" s="5" t="s">
-        <v>260</v>
+        <v>245</v>
       </c>
     </row>
     <row r="61" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6418,7 +6343,7 @@
         <v>74</v>
       </c>
       <c r="D61" s="5" t="s">
-        <v>261</v>
+        <v>246</v>
       </c>
     </row>
     <row r="62" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6432,7 +6357,7 @@
         <v>68</v>
       </c>
       <c r="D62" s="5" t="s">
-        <v>262</v>
+        <v>247</v>
       </c>
     </row>
     <row r="63" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6446,7 +6371,7 @@
         <v>66</v>
       </c>
       <c r="D63" s="5" t="s">
-        <v>262</v>
+        <v>247</v>
       </c>
     </row>
     <row r="64" spans="1:4" ht="60" customHeight="1" x14ac:dyDescent="0.25">
@@ -6457,10 +6382,10 @@
         <v>38</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>334</v>
+        <v>300</v>
       </c>
       <c r="D64" s="2" t="s">
-        <v>335</v>
+        <v>301</v>
       </c>
     </row>
   </sheetData>

</xml_diff>